<commit_message>
Expand AND voice catalog with generic operational cues
</commit_message>
<xml_diff>
--- a/docs/AND_voice_messages.xlsx
+++ b/docs/AND_voice_messages.xlsx
@@ -1,14 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci AND" sheetId="1" r:id="R9cbab2db1c4245b8"/>
+    <x:sheet name="Voci AND" sheetId="1" r:id="rId1"/>
   </x:sheets>
 </x:workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -36,7 +32,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -46,6 +42,12 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF0F4C5C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9D9D9"/>
+        <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -145,7 +147,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -195,6 +197,24 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -203,205 +223,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:C230" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="3">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:E254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:E254"/>
+  <x:tableColumns count="5">
     <x:tableColumn id="1" name="LVAR"/>
     <x:tableColumn id="2" name="nome file"/>
     <x:tableColumn id="3" name="testo del messaggio"/>
+    <x:tableColumn id="4" name="ruolo"/>
+    <x:tableColumn id="5" name="trigger (azione / tablet)"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
-  <a:themeElements>
-    <a:clrScheme name="ChatGPT">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="0E2841"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="156082"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="E97132"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="196B24"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="A02B93"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="4EA72E"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="467886"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="96607D"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="67000"/>
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="73000"/>
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="81000"/>
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="94000"/>
-                <a:lumMod val="102000"/>
-                <a:satMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:shade val="100000"/>
-                <a:lumMod val="100000"/>
-                <a:satMod val="110000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="78000"/>
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-                <a:satMod val="150000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -411,6 +243,8 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="50" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="80" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="78" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -420,8 +254,14 @@
       <x:c r="B1" s="9" t="str">
         <x:v>nome file</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="9" t="str">
         <x:v>testo del messaggio</x:v>
+      </x:c>
+      <x:c r="D1" s="9" t="str">
+        <x:v>ruolo</x:v>
+      </x:c>
+      <x:c r="E1" s="10" t="str">
+        <x:v>trigger (azione / tablet)</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
@@ -431,7 +271,7 @@
       <x:c r="B2" s="12" t="str">
         <x:v>AND.Inside.TabletAlarm2.wav</x:v>
       </x:c>
-      <x:c r="C2" s="13" t="str">
+      <x:c r="C2" s="12" t="str">
         <x:v>[Non-verbal tablet notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -442,7 +282,7 @@
       <x:c r="B3" s="12" t="str">
         <x:v>AND.NEW.DISPATCH.wav</x:v>
       </x:c>
-      <x:c r="C3" s="13" t="str">
+      <x:c r="C3" s="12" t="str">
         <x:v>[Non-verbal new-dispatch notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -453,7 +293,7 @@
       <x:c r="B4" s="12" t="str">
         <x:v>AND.NEW.DISPATCH1.wav</x:v>
       </x:c>
-      <x:c r="C4" s="13" t="str">
+      <x:c r="C4" s="12" t="str">
         <x:v>[Non-verbal new-dispatch notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -464,7 +304,7 @@
       <x:c r="B5" s="12" t="str">
         <x:v>AND.NEW.DISPATCH2.wav</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str">
+      <x:c r="C5" s="12" t="str">
         <x:v>[Non-verbal new-dispatch notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -475,7 +315,7 @@
       <x:c r="B6" s="12" t="str">
         <x:v>AND.NEW.DISPATCH3.wav</x:v>
       </x:c>
-      <x:c r="C6" s="13" t="str">
+      <x:c r="C6" s="12" t="str">
         <x:v>[Non-verbal new-dispatch notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -486,7 +326,7 @@
       <x:c r="B7" s="12" t="str">
         <x:v>AND.NEW.DISPATCH4.wav</x:v>
       </x:c>
-      <x:c r="C7" s="13" t="str">
+      <x:c r="C7" s="12" t="str">
         <x:v>[Non-verbal new-dispatch notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -497,7 +337,7 @@
       <x:c r="B8" s="12" t="str">
         <x:v>AND.NEW.MSG.wav</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="str">
+      <x:c r="C8" s="12" t="str">
         <x:v>[Non-verbal new-message notification sound.]</x:v>
       </x:c>
     </x:row>
@@ -508,7 +348,7 @@
       <x:c r="B9" s="12" t="str">
         <x:v>AND.HW1.wav</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="str">
+      <x:c r="C9" s="12" t="str">
         <x:v>We are experiencing issues with the safety straps we cannot use rescue hoist sorry we are forced to land.</x:v>
       </x:c>
     </x:row>
@@ -519,7 +359,7 @@
       <x:c r="B10" s="12" t="str">
         <x:v>AND.HW2.wav</x:v>
       </x:c>
-      <x:c r="C10" s="13" t="str">
+      <x:c r="C10" s="12" t="str">
         <x:v>Hey crew there is an emergency message from dispatcher you have to read it it's unbelievable.</x:v>
       </x:c>
     </x:row>
@@ -530,7 +370,7 @@
       <x:c r="B11" s="12" t="str">
         <x:v>AND.HW3.wav</x:v>
       </x:c>
-      <x:c r="C11" s="13" t="str">
+      <x:c r="C11" s="12" t="str">
         <x:v>Smoke and fire everywhere it seems a war movie scene out there.</x:v>
       </x:c>
     </x:row>
@@ -541,7 +381,7 @@
       <x:c r="B12" s="12" t="str">
         <x:v>AND.HW4.wav</x:v>
       </x:c>
-      <x:c r="C12" s="13" t="str">
+      <x:c r="C12" s="12" t="str">
         <x:v>Damn engine fire crew we have an engine fire.</x:v>
       </x:c>
     </x:row>
@@ -552,7 +392,7 @@
       <x:c r="B13" s="12" t="str">
         <x:v>AND.HW5.wav</x:v>
       </x:c>
-      <x:c r="C13" s="13" t="str">
+      <x:c r="C13" s="12" t="str">
         <x:v>Copilot confirmed engine two fire.</x:v>
       </x:c>
     </x:row>
@@ -563,7 +403,7 @@
       <x:c r="B14" s="12" t="str">
         <x:v>AND.HW6.wav</x:v>
       </x:c>
-      <x:c r="C14" s="13" t="str">
+      <x:c r="C14" s="12" t="str">
         <x:v>Engine two confirmed.</x:v>
       </x:c>
     </x:row>
@@ -574,7 +414,7 @@
       <x:c r="B15" s="12" t="str">
         <x:v>AND.HW7.wav</x:v>
       </x:c>
-      <x:c r="C15" s="13" t="str">
+      <x:c r="C15" s="12" t="str">
         <x:v>Engine two fire. Push bottle one and hope it goes off; crew, prepare to evacuate the helicopter.</x:v>
       </x:c>
     </x:row>
@@ -585,7 +425,7 @@
       <x:c r="B16" s="12" t="str">
         <x:v>AND.HW8.wav</x:v>
       </x:c>
-      <x:c r="C16" s="13" t="str">
+      <x:c r="C16" s="12" t="str">
         <x:v>Fire is extinguished however we have multiple failures i'm not sure we can take off again in this condition.</x:v>
       </x:c>
     </x:row>
@@ -596,7 +436,7 @@
       <x:c r="B17" s="12" t="str">
         <x:v>AND.HW9.wav</x:v>
       </x:c>
-      <x:c r="C17" s="13" t="str">
+      <x:c r="C17" s="12" t="str">
         <x:v>What the hell is happening here.</x:v>
       </x:c>
     </x:row>
@@ -607,7 +447,7 @@
       <x:c r="B18" s="12" t="str">
         <x:v>AND.HW10.wav</x:v>
       </x:c>
-      <x:c r="C18" s="13" t="str">
+      <x:c r="C18" s="12" t="str">
         <x:v>There is something bad happening in the area we have to be careful while completing tasks.</x:v>
       </x:c>
     </x:row>
@@ -618,7 +458,7 @@
       <x:c r="B19" s="12" t="str">
         <x:v>AND.HW11.wav</x:v>
       </x:c>
-      <x:c r="C19" s="13" t="str">
+      <x:c r="C19" s="12" t="str">
         <x:v>Did you see them hey what hey guys did you see them is that happening to us they are coming here are they.</x:v>
       </x:c>
     </x:row>
@@ -629,7 +469,7 @@
       <x:c r="B20" s="12" t="str">
         <x:v>AND.HW12.wav</x:v>
       </x:c>
-      <x:c r="C20" s="13" t="str">
+      <x:c r="C20" s="12" t="str">
         <x:v>We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
       </x:c>
     </x:row>
@@ -640,7 +480,7 @@
       <x:c r="B21" s="12" t="str">
         <x:v>AND.HW13.wav</x:v>
       </x:c>
-      <x:c r="C21" s="13" t="str">
+      <x:c r="C21" s="12" t="str">
         <x:v>Doc refers they have almost done we should wait for them to return.</x:v>
       </x:c>
     </x:row>
@@ -651,7 +491,7 @@
       <x:c r="B22" s="12" t="str">
         <x:v>AND.HW14.wav</x:v>
       </x:c>
-      <x:c r="C22" s="13" t="str">
+      <x:c r="C22" s="12" t="str">
         <x:v>Okay finished go away now go go go.</x:v>
       </x:c>
     </x:row>
@@ -662,7 +502,7 @@
       <x:c r="B23" s="12" t="str">
         <x:v>AND.HW15.wav</x:v>
       </x:c>
-      <x:c r="C23" s="13" t="str">
+      <x:c r="C23" s="12" t="str">
         <x:v>We're going to try and oh he i take off it will be difficult if needed be prepared for immediate evacuation.</x:v>
       </x:c>
     </x:row>
@@ -673,7 +513,7 @@
       <x:c r="B24" s="12" t="str">
         <x:v>AND.pax1.cabin.preparation.completed.wav</x:v>
       </x:c>
-      <x:c r="C24" s="13" t="str">
+      <x:c r="C24" s="12" t="str">
         <x:v>Cabin preparation completed.</x:v>
       </x:c>
     </x:row>
@@ -684,7 +524,7 @@
       <x:c r="B25" s="12" t="str">
         <x:v>AND.pax1.cabin.preparation.please.wait.wav</x:v>
       </x:c>
-      <x:c r="C25" s="13" t="str">
+      <x:c r="C25" s="12" t="str">
         <x:v>Cabin preparation please wait.</x:v>
       </x:c>
     </x:row>
@@ -695,7 +535,7 @@
       <x:c r="B26" s="12" t="str">
         <x:v>AND.pax1.cabin.secured.ready.to.fly.wav</x:v>
       </x:c>
-      <x:c r="C26" s="13" t="str">
+      <x:c r="C26" s="12" t="str">
         <x:v>Cabin secured ready to fly.</x:v>
       </x:c>
     </x:row>
@@ -706,7 +546,7 @@
       <x:c r="B27" s="12" t="str">
         <x:v>AND.pax1.hoist.1.plus.stretcher.to.helicopter.wav</x:v>
       </x:c>
-      <x:c r="C27" s="13" t="str">
+      <x:c r="C27" s="12" t="str">
         <x:v>Hoist one plus stretcher to helicopter.</x:v>
       </x:c>
     </x:row>
@@ -717,7 +557,7 @@
       <x:c r="B28" s="12" t="str">
         <x:v>AND.pax1.hoist.1.to.helicopter.patient.wav</x:v>
       </x:c>
-      <x:c r="C28" s="13" t="str">
+      <x:c r="C28" s="12" t="str">
         <x:v>Hoist one to helicopter; patient and doctor will go with ambulance.</x:v>
       </x:c>
     </x:row>
@@ -728,7 +568,7 @@
       <x:c r="B29" s="12" t="str">
         <x:v>AND.pax1.hoist.2.to.helicopter.wav</x:v>
       </x:c>
-      <x:c r="C29" s="13" t="str">
+      <x:c r="C29" s="12" t="str">
         <x:v>Hoist two to helicopter.</x:v>
       </x:c>
     </x:row>
@@ -739,7 +579,7 @@
       <x:c r="B30" s="12" t="str">
         <x:v>AND.pax1.hoist.3.to.helicopter.wav</x:v>
       </x:c>
-      <x:c r="C30" s="13" t="str">
+      <x:c r="C30" s="12" t="str">
         <x:v>Hoist three to helicopter.</x:v>
       </x:c>
     </x:row>
@@ -750,7 +590,7 @@
       <x:c r="B31" s="12" t="str">
         <x:v>AND.pax1.hoist.boom.extended.wav</x:v>
       </x:c>
-      <x:c r="C31" s="13" t="str">
+      <x:c r="C31" s="12" t="str">
         <x:v>Hoist boom extended.</x:v>
       </x:c>
     </x:row>
@@ -761,7 +601,7 @@
       <x:c r="B32" s="12" t="str">
         <x:v>AND.pax1.hoist.is.clear.wav</x:v>
       </x:c>
-      <x:c r="C32" s="13" t="str">
+      <x:c r="C32" s="12" t="str">
         <x:v>Hoist is clear.</x:v>
       </x:c>
     </x:row>
@@ -772,7 +612,7 @@
       <x:c r="B33" s="12" t="str">
         <x:v>AND.pax1.hoist.is.running.down.wav</x:v>
       </x:c>
-      <x:c r="C33" s="13" t="str">
+      <x:c r="C33" s="12" t="str">
         <x:v>Hoist is running down.</x:v>
       </x:c>
     </x:row>
@@ -783,7 +623,7 @@
       <x:c r="B34" s="12" t="str">
         <x:v>AND.pax1.hoist.is.running.up.wav</x:v>
       </x:c>
-      <x:c r="C34" s="13" t="str">
+      <x:c r="C34" s="12" t="str">
         <x:v>Hoist is running up.</x:v>
       </x:c>
     </x:row>
@@ -794,7 +634,7 @@
       <x:c r="B35" s="12" t="str">
         <x:v>AND.pax1.hoist.is.up.boom.ext.patient.is.out.wav</x:v>
       </x:c>
-      <x:c r="C35" s="13" t="str">
+      <x:c r="C35" s="12" t="str">
         <x:v>Hoist his up boom extended patient and doctor are outside hook to hoist.</x:v>
       </x:c>
     </x:row>
@@ -805,7 +645,7 @@
       <x:c r="B36" s="12" t="str">
         <x:v>AND.pax1.hoist.is.up.personnel.is.strapped.in.wav</x:v>
       </x:c>
-      <x:c r="C36" s="13" t="str">
+      <x:c r="C36" s="12" t="str">
         <x:v>Hoist his up personnel is strapped in.</x:v>
       </x:c>
     </x:row>
@@ -816,7 +656,7 @@
       <x:c r="B37" s="12" t="str">
         <x:v>AND.pax1.hoist.on.ground.personnel.getting.hooked.wav</x:v>
       </x:c>
-      <x:c r="C37" s="13" t="str">
+      <x:c r="C37" s="12" t="str">
         <x:v>Hoist on ground personnel is getting hooked.</x:v>
       </x:c>
     </x:row>
@@ -827,7 +667,7 @@
       <x:c r="B38" s="12" t="str">
         <x:v>AND.pax1.hold.position.wav</x:v>
       </x:c>
-      <x:c r="C38" s="13" t="str">
+      <x:c r="C38" s="12" t="str">
         <x:v>Hold position.</x:v>
       </x:c>
     </x:row>
@@ -838,7 +678,7 @@
       <x:c r="B39" s="12" t="str">
         <x:v>AND.pax1.hook.is.in.boom.retracted.free.to.leave.hover.wav</x:v>
       </x:c>
-      <x:c r="C39" s="13" t="str">
+      <x:c r="C39" s="12" t="str">
         <x:v>Hook is in hoist boomers retracted you're free to leave hover.</x:v>
       </x:c>
     </x:row>
@@ -849,7 +689,7 @@
       <x:c r="B40" s="12" t="str">
         <x:v>AND.pax1.medic.on.ground.and.disconnected.wav</x:v>
       </x:c>
-      <x:c r="C40" s="13" t="str">
+      <x:c r="C40" s="12" t="str">
         <x:v>Medical on ground and disconnected.</x:v>
       </x:c>
     </x:row>
@@ -860,7 +700,7 @@
       <x:c r="B41" s="12" t="str">
         <x:v>AND.pax1.patient.will.go.with.ambulance.wav</x:v>
       </x:c>
-      <x:c r="C41" s="13" t="str">
+      <x:c r="C41" s="12" t="str">
         <x:v>Patient will go with ambulance.</x:v>
       </x:c>
     </x:row>
@@ -871,7 +711,7 @@
       <x:c r="B42" s="12" t="str">
         <x:v>AND.pax1.personnel.is.on.ground.disconnected.wav</x:v>
       </x:c>
-      <x:c r="C42" s="13" t="str">
+      <x:c r="C42" s="12" t="str">
         <x:v>Personnel on ground and disconnected.</x:v>
       </x:c>
     </x:row>
@@ -882,7 +722,7 @@
       <x:c r="B43" s="12" t="str">
         <x:v>AND.pax1.position.is.good.wav</x:v>
       </x:c>
-      <x:c r="C43" s="13" t="str">
+      <x:c r="C43" s="12" t="str">
         <x:v>Position is good.</x:v>
       </x:c>
     </x:row>
@@ -893,7 +733,7 @@
       <x:c r="B44" s="12" t="str">
         <x:v>AND.pax1.ready.for.hoisting.ops.wav</x:v>
       </x:c>
-      <x:c r="C44" s="13" t="str">
+      <x:c r="C44" s="12" t="str">
         <x:v>Hold on, hoisting preparation is in progress and almost completed.</x:v>
       </x:c>
     </x:row>
@@ -904,7 +744,7 @@
       <x:c r="B45" s="12" t="str">
         <x:v>AND.pax1.set.hover.conditions.wav</x:v>
       </x:c>
-      <x:c r="C45" s="13" t="str">
+      <x:c r="C45" s="12" t="str">
         <x:v>Set hover conditions.</x:v>
       </x:c>
     </x:row>
@@ -915,7 +755,7 @@
       <x:c r="B46" s="12" t="str">
         <x:v>AND.pax1.st.comm.chk.wav</x:v>
       </x:c>
-      <x:c r="C46" s="13" t="str">
+      <x:c r="C46" s="12" t="str">
         <x:v>That's one com check.</x:v>
       </x:c>
     </x:row>
@@ -926,7 +766,7 @@
       <x:c r="B47" s="12" t="str">
         <x:v>AND.pax1.st.hoist.1.to.helicopter.wav</x:v>
       </x:c>
-      <x:c r="C47" s="13" t="str">
+      <x:c r="C47" s="12" t="str">
         <x:v>Hoist wonder helicopter.</x:v>
       </x:c>
     </x:row>
@@ -937,7 +777,7 @@
       <x:c r="B48" s="12" t="str">
         <x:v>AND.pax1.t.10.wav</x:v>
       </x:c>
-      <x:c r="C48" s="13" t="str">
+      <x:c r="C48" s="12" t="str">
         <x:v>Ten.</x:v>
       </x:c>
     </x:row>
@@ -948,7 +788,7 @@
       <x:c r="B49" s="12" t="str">
         <x:v>AND.pax1.t.20.wav</x:v>
       </x:c>
-      <x:c r="C49" s="13" t="str">
+      <x:c r="C49" s="12" t="str">
         <x:v>Twenty.</x:v>
       </x:c>
     </x:row>
@@ -959,7 +799,7 @@
       <x:c r="B50" s="12" t="str">
         <x:v>AND.pax1.t.50m.wav</x:v>
       </x:c>
-      <x:c r="C50" s="13" t="str">
+      <x:c r="C50" s="12" t="str">
         <x:v>Fifty meters.</x:v>
       </x:c>
     </x:row>
@@ -970,7 +810,7 @@
       <x:c r="B51" s="12" t="str">
         <x:v>AND.pax1.t.hi.frank.wav</x:v>
       </x:c>
-      <x:c r="C51" s="13" t="str">
+      <x:c r="C51" s="12" t="str">
         <x:v>Hey frank good morning.</x:v>
       </x:c>
     </x:row>
@@ -981,7 +821,7 @@
       <x:c r="B52" s="12" t="str">
         <x:v>AND.pax1.t.hi.sarah.wav</x:v>
       </x:c>
-      <x:c r="C52" s="13" t="str">
+      <x:c r="C52" s="12" t="str">
         <x:v>Hi sarah how are you.</x:v>
       </x:c>
     </x:row>
@@ -992,7 +832,7 @@
       <x:c r="B53" s="12" t="str">
         <x:v>AND.pax1.t.stretcher.secured.wav</x:v>
       </x:c>
-      <x:c r="C53" s="13" t="str">
+      <x:c r="C53" s="12" t="str">
         <x:v>Stretcher is secure.</x:v>
       </x:c>
     </x:row>
@@ -1003,7 +843,7 @@
       <x:c r="B54" s="12" t="str">
         <x:v>AND.pax1.t.we.are.close.set.hover.wav</x:v>
       </x:c>
-      <x:c r="C54" s="13" t="str">
+      <x:c r="C54" s="12" t="str">
         <x:v>We are reasonably close said hover is appropriate.</x:v>
       </x:c>
     </x:row>
@@ -1014,7 +854,7 @@
       <x:c r="B55" s="12" t="str">
         <x:v>AND.pax1.t.we.are.close.wav</x:v>
       </x:c>
-      <x:c r="C55" s="13" t="str">
+      <x:c r="C55" s="12" t="str">
         <x:v>We are reasonably close.</x:v>
       </x:c>
     </x:row>
@@ -1025,7 +865,7 @@
       <x:c r="B56" s="12" t="str">
         <x:v>AND.pax1.t.we.are.too.far.wav</x:v>
       </x:c>
-      <x:c r="C56" s="13" t="str">
+      <x:c r="C56" s="12" t="str">
         <x:v>We are too far.</x:v>
       </x:c>
     </x:row>
@@ -1036,7 +876,7 @@
       <x:c r="B57" s="12" t="str">
         <x:v>AND.pax1.we.are.height.is.good.wav</x:v>
       </x:c>
-      <x:c r="C57" s="13" t="str">
+      <x:c r="C57" s="12" t="str">
         <x:v>Height is good.</x:v>
       </x:c>
     </x:row>
@@ -1047,7 +887,7 @@
       <x:c r="B58" s="12" t="str">
         <x:v>AND.pax1.we.are.too.high.wav</x:v>
       </x:c>
-      <x:c r="C58" s="13" t="str">
+      <x:c r="C58" s="12" t="str">
         <x:v>We are too high.</x:v>
       </x:c>
     </x:row>
@@ -1058,7 +898,7 @@
       <x:c r="B59" s="12" t="str">
         <x:v>AND.pax1.we.are.too.low.wav</x:v>
       </x:c>
-      <x:c r="C59" s="13" t="str">
+      <x:c r="C59" s="12" t="str">
         <x:v>We are too low.</x:v>
       </x:c>
     </x:row>
@@ -1069,7 +909,7 @@
       <x:c r="B60" s="12" t="str">
         <x:v>AND.pax1.wf.doc.and.strtc.have.been.disconnected.wav</x:v>
       </x:c>
-      <x:c r="C60" s="13" t="str">
+      <x:c r="C60" s="12" t="str">
         <x:v>Doc and stretcher have been disconnected.</x:v>
       </x:c>
     </x:row>
@@ -1080,7 +920,7 @@
       <x:c r="B61" s="12" t="str">
         <x:v>AND.pax1.wf.doc.is.getting.hooked.wav</x:v>
       </x:c>
-      <x:c r="C61" s="13" t="str">
+      <x:c r="C61" s="12" t="str">
         <x:v>Doc is getting hooked.</x:v>
       </x:c>
     </x:row>
@@ -1091,7 +931,7 @@
       <x:c r="B62" s="12" t="str">
         <x:v>AND.pax1.wf.hoist.boom.extended.wav</x:v>
       </x:c>
-      <x:c r="C62" s="13" t="str">
+      <x:c r="C62" s="12" t="str">
         <x:v>Hoist storm extended.</x:v>
       </x:c>
     </x:row>
@@ -1102,7 +942,7 @@
       <x:c r="B63" s="12" t="str">
         <x:v>AND.pax1.wf.hoist.retracted.door.close.wav</x:v>
       </x:c>
-      <x:c r="C63" s="13" t="str">
+      <x:c r="C63" s="12" t="str">
         <x:v>Hoist retracted door closed cabin secured.</x:v>
       </x:c>
     </x:row>
@@ -1113,7 +953,7 @@
       <x:c r="B64" s="12" t="str">
         <x:v>AND.pax1.wf.opening.door.hoist.op.wav</x:v>
       </x:c>
-      <x:c r="C64" s="13" t="str">
+      <x:c r="C64" s="12" t="str">
         <x:v>Opening door and preparing for hoist operation.</x:v>
       </x:c>
     </x:row>
@@ -1124,7 +964,7 @@
       <x:c r="B65" s="12" t="str">
         <x:v>AND.pax1.wf.operator.has.been.disconnected.wav</x:v>
       </x:c>
-      <x:c r="C65" s="13" t="str">
+      <x:c r="C65" s="12" t="str">
         <x:v>Operator has been disconnected.</x:v>
       </x:c>
     </x:row>
@@ -1135,7 +975,7 @@
       <x:c r="B66" s="12" t="str">
         <x:v>AND.pax1.wf.operator.is.getting.hooked.wav</x:v>
       </x:c>
-      <x:c r="C66" s="13" t="str">
+      <x:c r="C66" s="12" t="str">
         <x:v>Operator is getting hooked.</x:v>
       </x:c>
     </x:row>
@@ -1146,7 +986,7 @@
       <x:c r="B67" s="12" t="str">
         <x:v>AND.pax1.wg.crew.boarded.ready.to.go.wav</x:v>
       </x:c>
-      <x:c r="C67" s="13" t="str">
+      <x:c r="C67" s="12" t="str">
         <x:v>Crew boarded cabin ready to go.</x:v>
       </x:c>
     </x:row>
@@ -1157,7 +997,7 @@
       <x:c r="B68" s="12" t="str">
         <x:v>AND.pax1.wg.helirescuer.pickup.wav</x:v>
       </x:c>
-      <x:c r="C68" s="13" t="str">
+      <x:c r="C68" s="12" t="str">
         <x:v>Due to impervious location of accident site we should evaluate to call and board expert heli-rescuers use the tablet to decide if we continue alone or if we have to pick kelly rescuers on board.</x:v>
       </x:c>
     </x:row>
@@ -1168,7 +1008,7 @@
       <x:c r="B69" s="12" t="str">
         <x:v>AND.pax1.wg.helirescuer.secured.area.wav</x:v>
       </x:c>
-      <x:c r="C69" s="13" t="str">
+      <x:c r="C69" s="12" t="str">
         <x:v>Okay heli rescuer secure the area and the casualty we are go for hosting down the other personnel.</x:v>
       </x:c>
     </x:row>
@@ -1179,7 +1019,7 @@
       <x:c r="B70" s="12" t="str">
         <x:v>AND.pax1.wg.proposed.meeting.pt.far.away.wav</x:v>
       </x:c>
-      <x:c r="C70" s="13" t="str">
+      <x:c r="C70" s="12" t="str">
         <x:v>The proposed meeting point seems far away from accident site i believe we should arrange another feasible meeting point.</x:v>
       </x:c>
     </x:row>
@@ -1190,7 +1030,7 @@
       <x:c r="B71" s="12" t="str">
         <x:v>AND.pax1.wg.we.have.to.hoist.3.to.gnd.wav</x:v>
       </x:c>
-      <x:c r="C71" s="13" t="str">
+      <x:c r="C71" s="12" t="str">
         <x:v>We have to hoist three to ground heli rescuer will be first to secure the area.</x:v>
       </x:c>
     </x:row>
@@ -1201,7 +1041,7 @@
       <x:c r="B72" s="12" t="str">
         <x:v>AND.pax1.wg.we.have.to.increase.height.speed.until.secured.wav</x:v>
       </x:c>
-      <x:c r="C72" s="13" t="str">
+      <x:c r="C72" s="12" t="str">
         <x:v>We have to increase distance and hide until the rescue area is secure.</x:v>
       </x:c>
     </x:row>
@@ -1212,7 +1052,7 @@
       <x:c r="B73" s="12" t="str">
         <x:v>AND.pax1.wg.xdoc.and.patient.with.ambu.wav</x:v>
       </x:c>
-      <x:c r="C73" s="13" t="str">
+      <x:c r="C73" s="12" t="str">
         <x:v>Dark and patient will go with the ambulance to the design hospital we have to pick him at the hospital hello pat.</x:v>
       </x:c>
     </x:row>
@@ -1223,7 +1063,7 @@
       <x:c r="B74" s="12" t="str">
         <x:v>AND.pax1.wgb.3oclock.wav</x:v>
       </x:c>
-      <x:c r="C74" s="13" t="str">
+      <x:c r="C74" s="12" t="str">
         <x:v>Three o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1234,7 +1074,7 @@
       <x:c r="B75" s="12" t="str">
         <x:v>AND.pax1.wgb.4oclock.wav</x:v>
       </x:c>
-      <x:c r="C75" s="13" t="str">
+      <x:c r="C75" s="12" t="str">
         <x:v>Four o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1245,7 +1085,7 @@
       <x:c r="B76" s="12" t="str">
         <x:v>AND.pax1.wgb.5oclock.wav</x:v>
       </x:c>
-      <x:c r="C76" s="13" t="str">
+      <x:c r="C76" s="12" t="str">
         <x:v>Five o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1256,7 +1096,7 @@
       <x:c r="B77" s="12" t="str">
         <x:v>AND.pax1.wgb.6oclock.wav</x:v>
       </x:c>
-      <x:c r="C77" s="13" t="str">
+      <x:c r="C77" s="12" t="str">
         <x:v>Six o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1267,7 +1107,7 @@
       <x:c r="B78" s="12" t="str">
         <x:v>AND.pax1.wgb.7oclock.wav</x:v>
       </x:c>
-      <x:c r="C78" s="13" t="str">
+      <x:c r="C78" s="12" t="str">
         <x:v>Seven o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1278,7 +1118,7 @@
       <x:c r="B79" s="12" t="str">
         <x:v>AND.pax1.wgb.8oclock.wav</x:v>
       </x:c>
-      <x:c r="C79" s="13" t="str">
+      <x:c r="C79" s="12" t="str">
         <x:v>Eight o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1289,7 +1129,7 @@
       <x:c r="B80" s="12" t="str">
         <x:v>AND.pax1.wgb.9oclock.wav</x:v>
       </x:c>
-      <x:c r="C80" s="13" t="str">
+      <x:c r="C80" s="12" t="str">
         <x:v>Nine o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1300,7 +1140,7 @@
       <x:c r="B81" s="12" t="str">
         <x:v>AND.pax1.wgb.10oclock.wav</x:v>
       </x:c>
-      <x:c r="C81" s="13" t="str">
+      <x:c r="C81" s="12" t="str">
         <x:v>Ten o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1311,7 +1151,7 @@
       <x:c r="B82" s="12" t="str">
         <x:v>AND.pax1.wgb.11oclock.wav</x:v>
       </x:c>
-      <x:c r="C82" s="13" t="str">
+      <x:c r="C82" s="12" t="str">
         <x:v>Eleven o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1322,7 +1162,7 @@
       <x:c r="B83" s="12" t="str">
         <x:v>AND.pax1.wgb.12oclock.wav</x:v>
       </x:c>
-      <x:c r="C83" s="13" t="str">
+      <x:c r="C83" s="12" t="str">
         <x:v>Twelve o'clock.</x:v>
       </x:c>
     </x:row>
@@ -1333,7 +1173,7 @@
       <x:c r="B84" s="12" t="str">
         <x:v>AND.pax1.wgb.are.on.the.way.to.accident.wav</x:v>
       </x:c>
-      <x:c r="C84" s="13" t="str">
+      <x:c r="C84" s="12" t="str">
         <x:v>Or on the way to the accident site.</x:v>
       </x:c>
     </x:row>
@@ -1344,7 +1184,7 @@
       <x:c r="B85" s="12" t="str">
         <x:v>AND.pax1.wgb.check.on.tablet.wav</x:v>
       </x:c>
-      <x:c r="C85" s="13" t="str">
+      <x:c r="C85" s="12" t="str">
         <x:v>Check on tablet.</x:v>
       </x:c>
     </x:row>
@@ -1355,7 +1195,7 @@
       <x:c r="B86" s="12" t="str">
         <x:v>AND.pax1.wgb.i.believe.we.found.wav</x:v>
       </x:c>
-      <x:c r="C86" s="13" t="str">
+      <x:c r="C86" s="12" t="str">
         <x:v>I believe we found something.</x:v>
       </x:c>
     </x:row>
@@ -1366,7 +1206,7 @@
       <x:c r="B87" s="12" t="str">
         <x:v>AND.pax1.wgb.its.in.front.of.us.wav</x:v>
       </x:c>
-      <x:c r="C87" s="13" t="str">
+      <x:c r="C87" s="12" t="str">
         <x:v>It's in front of us.</x:v>
       </x:c>
     </x:row>
@@ -1377,7 +1217,7 @@
       <x:c r="B88" s="12" t="str">
         <x:v>AND.pax1.wgb.yes.confirmed.we.found.target.wav</x:v>
       </x:c>
-      <x:c r="C88" s="13" t="str">
+      <x:c r="C88" s="12" t="str">
         <x:v>Yes confirmed we found our target.</x:v>
       </x:c>
     </x:row>
@@ -1388,7 +1228,7 @@
       <x:c r="B89" s="12" t="str">
         <x:v>AND.pax1.wgc.helicopter.clear.ready.to.fly.wav</x:v>
       </x:c>
-      <x:c r="C89" s="13" t="str">
+      <x:c r="C89" s="12" t="str">
         <x:v>Helicopter clear ready to fly.</x:v>
       </x:c>
     </x:row>
@@ -1399,7 +1239,7 @@
       <x:c r="B90" s="12" t="str">
         <x:v>AND.cpl.all.engine.started.successfully.wav</x:v>
       </x:c>
-      <x:c r="C90" s="13" t="str">
+      <x:c r="C90" s="12" t="str">
         <x:v>All engines started successfully.</x:v>
       </x:c>
     </x:row>
@@ -1410,7 +1250,7 @@
       <x:c r="B91" s="12" t="str">
         <x:v>AND.cpl.all.good.wav</x:v>
       </x:c>
-      <x:c r="C91" s="13" t="str">
+      <x:c r="C91" s="12" t="str">
         <x:v>Okay all good.</x:v>
       </x:c>
     </x:row>
@@ -1421,7 +1261,7 @@
       <x:c r="B92" s="12" t="str">
         <x:v>AND.cpl.area.clear.ready.to.engine.1.wav</x:v>
       </x:c>
-      <x:c r="C92" s="13" t="str">
+      <x:c r="C92" s="12" t="str">
         <x:v>Area clear ready to start engine one.</x:v>
       </x:c>
     </x:row>
@@ -1432,7 +1272,7 @@
       <x:c r="B93" s="12" t="str">
         <x:v>AND.cpl.area.clear.ready.to.engine.2.wav</x:v>
       </x:c>
-      <x:c r="C93" s="13" t="str">
+      <x:c r="C93" s="12" t="str">
         <x:v>Area clear ready to start engine two.</x:v>
       </x:c>
     </x:row>
@@ -1443,7 +1283,7 @@
       <x:c r="B94" s="12" t="str">
         <x:v>AND.cpl.comm.chk.wav</x:v>
       </x:c>
-      <x:c r="C94" s="13" t="str">
+      <x:c r="C94" s="12" t="str">
         <x:v>Co pilot hh oh comm check.</x:v>
       </x:c>
     </x:row>
@@ -1454,7 +1294,7 @@
       <x:c r="B95" s="12" t="str">
         <x:v>AND.cpl.engine.clear.wav</x:v>
       </x:c>
-      <x:c r="C95" s="13" t="str">
+      <x:c r="C95" s="12" t="str">
         <x:v>Engine clear.</x:v>
       </x:c>
     </x:row>
@@ -1465,7 +1305,7 @@
       <x:c r="B96" s="12" t="str">
         <x:v>AND.cpl.engine.fire.wav</x:v>
       </x:c>
-      <x:c r="C96" s="13" t="str">
+      <x:c r="C96" s="12" t="str">
         <x:v>Fire we have an engine fire stop engine.</x:v>
       </x:c>
     </x:row>
@@ -1476,7 +1316,7 @@
       <x:c r="B97" s="12" t="str">
         <x:v>AND.cpl.engine.started.succ.moving.to.other.wav</x:v>
       </x:c>
-      <x:c r="C97" s="13" t="str">
+      <x:c r="C97" s="12" t="str">
         <x:v>Engine started successfully moving to other engine.</x:v>
       </x:c>
     </x:row>
@@ -1487,7 +1327,7 @@
       <x:c r="B98" s="12" t="str">
         <x:v>AND.cpl.failure.wav</x:v>
       </x:c>
-      <x:c r="C98" s="13" t="str">
+      <x:c r="C98" s="12" t="str">
         <x:v>Damn we have a failure.</x:v>
       </x:c>
     </x:row>
@@ -1498,7 +1338,7 @@
       <x:c r="B99" s="12" t="str">
         <x:v>AND.cpl.holdon.performing.leak.checks.wav</x:v>
       </x:c>
-      <x:c r="C99" s="13" t="str">
+      <x:c r="C99" s="12" t="str">
         <x:v>Hold on performing leak checks.</x:v>
       </x:c>
     </x:row>
@@ -1509,7 +1349,7 @@
       <x:c r="B100" s="12" t="str">
         <x:v>AND.cpl.prepare.for.gnd.op.wav</x:v>
       </x:c>
-      <x:c r="C100" s="13" t="str">
+      <x:c r="C100" s="12" t="str">
         <x:v>Rear crew prepare for ground operation.</x:v>
       </x:c>
     </x:row>
@@ -1520,7 +1360,7 @@
       <x:c r="B101" s="12" t="str">
         <x:v>AND.cpl.prepare.for.hoist.op.wav</x:v>
       </x:c>
-      <x:c r="C101" s="13" t="str">
+      <x:c r="C101" s="12" t="str">
         <x:v>Rear crew prepare for hoist operation.</x:v>
       </x:c>
     </x:row>
@@ -1531,7 +1371,7 @@
       <x:c r="B102" s="12" t="str">
         <x:v>AND.cpl.preparing.for.engine.1.2.wav</x:v>
       </x:c>
-      <x:c r="C102" s="13" t="str">
+      <x:c r="C102" s="12" t="str">
         <x:v>Preparing for engine starting sequence one too.</x:v>
       </x:c>
     </x:row>
@@ -1542,7 +1382,7 @@
       <x:c r="B103" s="12" t="str">
         <x:v>AND.cpl.preparing.for.engine.2.1.wav</x:v>
       </x:c>
-      <x:c r="C103" s="13" t="str">
+      <x:c r="C103" s="12" t="str">
         <x:v>Preparing for engine starting sequence to one.</x:v>
       </x:c>
     </x:row>
@@ -1553,7 +1393,7 @@
       <x:c r="B104" s="12" t="str">
         <x:v>AND.cpl.rearcrew.ready.to.start.op.wav</x:v>
       </x:c>
-      <x:c r="C104" s="13" t="str">
+      <x:c r="C104" s="12" t="str">
         <x:v>Helicopter in position rear crew clear to start operation.</x:v>
       </x:c>
     </x:row>
@@ -1564,7 +1404,7 @@
       <x:c r="B105" s="12" t="str">
         <x:v>AND.cpl.rearcrew.we.are.appr.to.site.wav</x:v>
       </x:c>
-      <x:c r="C105" s="13" t="str">
+      <x:c r="C105" s="12" t="str">
         <x:v>Rear crew we are approaching the landing site.</x:v>
       </x:c>
     </x:row>
@@ -1575,7 +1415,7 @@
       <x:c r="B106" s="12" t="str">
         <x:v>AND.cpl.site.is.not.safe.for.us.wav</x:v>
       </x:c>
-      <x:c r="C106" s="13" t="str">
+      <x:c r="C106" s="12" t="str">
         <x:v>Site is not safe for us waiting for clearance.</x:v>
       </x:c>
     </x:row>
@@ -1586,7 +1426,7 @@
       <x:c r="B107" s="12" t="str">
         <x:v>AND.cpl.site.is.safe.we.can.proceed.wav</x:v>
       </x:c>
-      <x:c r="C107" s="13" t="str">
+      <x:c r="C107" s="12" t="str">
         <x:v>Site is safer operations we can proceed.</x:v>
       </x:c>
     </x:row>
@@ -1597,7 +1437,7 @@
       <x:c r="B108" s="12" t="str">
         <x:v>AND.cpl.skid.ldg.wav</x:v>
       </x:c>
-      <x:c r="C108" s="13" t="str">
+      <x:c r="C108" s="12" t="str">
         <x:v>Rear crew prepare for skid lending operation.</x:v>
       </x:c>
     </x:row>
@@ -1608,7 +1448,7 @@
       <x:c r="B109" s="12" t="str">
         <x:v>AND.cpl.t.ambulance.is.arriving.wav</x:v>
       </x:c>
-      <x:c r="C109" s="13" t="str">
+      <x:c r="C109" s="12" t="str">
         <x:v>Ambulance is arriving.</x:v>
       </x:c>
     </x:row>
@@ -1619,7 +1459,7 @@
       <x:c r="B110" s="12" t="str">
         <x:v>AND.cpl.t.ambulance.is.still.far.wav</x:v>
       </x:c>
-      <x:c r="C110" s="13" t="str">
+      <x:c r="C110" s="12" t="str">
         <x:v>Ambulance is still far away.</x:v>
       </x:c>
     </x:row>
@@ -1630,7 +1470,7 @@
       <x:c r="B111" s="12" t="str">
         <x:v>AND.cpl.t.crew.prepare.op.wav</x:v>
       </x:c>
-      <x:c r="C111" s="13" t="str">
+      <x:c r="C111" s="12" t="str">
         <x:v>Crew prepare for operation.</x:v>
       </x:c>
     </x:row>
@@ -1641,7 +1481,7 @@
       <x:c r="B112" s="12" t="str">
         <x:v>AND.cpl.t.goodmorning.frank.wav</x:v>
       </x:c>
-      <x:c r="C112" s="13" t="str">
+      <x:c r="C112" s="12" t="str">
         <x:v>Good morning frank.</x:v>
       </x:c>
     </x:row>
@@ -1652,7 +1492,7 @@
       <x:c r="B113" s="12" t="str">
         <x:v>AND.cpl.t.landing.spot.medical.crew.present.wav</x:v>
       </x:c>
-      <x:c r="C113" s="13" t="str">
+      <x:c r="C113" s="12" t="str">
         <x:v>Destination insight medical crew is ready on landing spot.</x:v>
       </x:c>
     </x:row>
@@ -1663,7 +1503,7 @@
       <x:c r="B114" s="12" t="str">
         <x:v>AND.cpl.t.we.have.to.stop.eng.wav</x:v>
       </x:c>
-      <x:c r="C114" s="13" t="str">
+      <x:c r="C114" s="12" t="str">
         <x:v>We have to stop engines and switch off the helicopter.</x:v>
       </x:c>
     </x:row>
@@ -1674,7 +1514,7 @@
       <x:c r="B115" s="12" t="str">
         <x:v>AND.cpl.u.due.to.patient.wav</x:v>
       </x:c>
-      <x:c r="C115" s="13" t="str">
+      <x:c r="C115" s="12" t="str">
         <x:v>The crew i received a call from doc due to patient conditions the ambulance arrived to an alternate hospital doc is waiting us their check location on map.</x:v>
       </x:c>
     </x:row>
@@ -1685,7 +1525,7 @@
       <x:c r="B116" s="12" t="str">
         <x:v>AND.cpl.v.above.max.hoist.wav</x:v>
       </x:c>
-      <x:c r="C116" s="13" t="str">
+      <x:c r="C116" s="12" t="str">
         <x:v>We are above maximum hoist out speed.</x:v>
       </x:c>
     </x:row>
@@ -1696,7 +1536,7 @@
       <x:c r="B117" s="12" t="str">
         <x:v>AND.cpl.v.acceleration.above.limit.wav</x:v>
       </x:c>
-      <x:c r="C117" s="13" t="str">
+      <x:c r="C117" s="12" t="str">
         <x:v>Oh acceleration is over the hoist limit.</x:v>
       </x:c>
     </x:row>
@@ -1707,7 +1547,7 @@
       <x:c r="B118" s="12" t="str">
         <x:v>AND.cpl.v.bank.angle.is.too.high.wav</x:v>
       </x:c>
-      <x:c r="C118" s="13" t="str">
+      <x:c r="C118" s="12" t="str">
         <x:v>Bank angle is too high people on hoist will have troubles if we continue.</x:v>
       </x:c>
     </x:row>
@@ -1718,7 +1558,7 @@
       <x:c r="B119" s="12" t="str">
         <x:v>AND.cpl.v.keep.bank.angle.wav</x:v>
       </x:c>
-      <x:c r="C119" s="13" t="str">
+      <x:c r="C119" s="12" t="str">
         <x:v>Keep bank angled within limits.</x:v>
       </x:c>
     </x:row>
@@ -1729,7 +1569,7 @@
       <x:c r="B120" s="12" t="str">
         <x:v>AND.cpl.v.we.are.too.fast.wav</x:v>
       </x:c>
-      <x:c r="C120" s="13" t="str">
+      <x:c r="C120" s="12" t="str">
         <x:v>We are too fast sir we risk our patient and operator life moreover we are damaging the helicopter.</x:v>
       </x:c>
     </x:row>
@@ -1740,7 +1580,7 @@
       <x:c r="B121" s="12" t="str">
         <x:v>AND.cpl.v.we.have.to.abort.wav</x:v>
       </x:c>
-      <x:c r="C121" s="13" t="str">
+      <x:c r="C121" s="12" t="str">
         <x:v>Fuck sir we have to abort mission now.</x:v>
       </x:c>
     </x:row>
@@ -1751,7 +1591,7 @@
       <x:c r="B122" s="12" t="str">
         <x:v>AND.cpl.v.we.lost.doc.and.patient.wav</x:v>
       </x:c>
-      <x:c r="C122" s="13" t="str">
+      <x:c r="C122" s="12" t="str">
         <x:v>What the fuck we lost patient and doc what are you doing.</x:v>
       </x:c>
     </x:row>
@@ -1762,7 +1602,7 @@
       <x:c r="B123" s="12" t="str">
         <x:v>AND.cpl.x.are.we.doing.aerobatic.wav</x:v>
       </x:c>
-      <x:c r="C123" s="13" t="str">
+      <x:c r="C123" s="12" t="str">
         <x:v>Ah are we doing acrobatic maneuvers with a patient on board are you serious.</x:v>
       </x:c>
     </x:row>
@@ -1773,7 +1613,7 @@
       <x:c r="B124" s="12" t="str">
         <x:v>AND.cpl.x.doc.refers.ground.ops.are.done.wav</x:v>
       </x:c>
-      <x:c r="C124" s="13" t="str">
+      <x:c r="C124" s="12" t="str">
         <x:v>Doc refers the ground operations are almost done we can either go back and have or as soon as possible or stay here and proceed with ground operation.</x:v>
       </x:c>
     </x:row>
@@ -1784,7 +1624,7 @@
       <x:c r="B125" s="12" t="str">
         <x:v>AND.cpl.x.ground.ops.will.take.time.wav</x:v>
       </x:c>
-      <x:c r="C125" s="13" t="str">
+      <x:c r="C125" s="12" t="str">
         <x:v>Round operations will take time we can leave hover and find a safe landing spot we will be advised when operations are done.</x:v>
       </x:c>
     </x:row>
@@ -1795,7 +1635,7 @@
       <x:c r="B126" s="12" t="str">
         <x:v>AND.cpl.x.hard.ldg.sarah.wav</x:v>
       </x:c>
-      <x:c r="C126" s="13" t="str">
+      <x:c r="C126" s="12" t="str">
         <x:v>Ouch it was hard landing this time sarah won't be happy.</x:v>
       </x:c>
     </x:row>
@@ -1806,7 +1646,7 @@
       <x:c r="B127" s="12" t="str">
         <x:v>AND.cpl.x.hard.ldg.wav</x:v>
       </x:c>
-      <x:c r="C127" s="13" t="str">
+      <x:c r="C127" s="12" t="str">
         <x:v>Hey it was a hard touch.</x:v>
       </x:c>
     </x:row>
@@ -1817,7 +1657,7 @@
       <x:c r="B128" s="12" t="str">
         <x:v>AND.cpl.x.nice.touch.wav</x:v>
       </x:c>
-      <x:c r="C128" s="13" t="str">
+      <x:c r="C128" s="12" t="str">
         <x:v>Wow nice touch captain.</x:v>
       </x:c>
     </x:row>
@@ -1828,7 +1668,7 @@
       <x:c r="B129" s="12" t="str">
         <x:v>AND.cpl.x.VNE.wav</x:v>
       </x:c>
-      <x:c r="C129" s="13" t="str">
+      <x:c r="C129" s="12" t="str">
         <x:v>VNE.</x:v>
       </x:c>
     </x:row>
@@ -1839,7 +1679,7 @@
       <x:c r="B130" s="12" t="str">
         <x:v>AND.cpl.x.VTOSS.wav</x:v>
       </x:c>
-      <x:c r="C130" s="13" t="str">
+      <x:c r="C130" s="12" t="str">
         <x:v>VTOSS.</x:v>
       </x:c>
     </x:row>
@@ -1850,7 +1690,7 @@
       <x:c r="B131" s="12" t="str">
         <x:v>AND.cpl.x.Vy.wav</x:v>
       </x:c>
-      <x:c r="C131" s="13" t="str">
+      <x:c r="C131" s="12" t="str">
         <x:v>Vy.</x:v>
       </x:c>
     </x:row>
@@ -1861,7 +1701,7 @@
       <x:c r="B132" s="12" t="str">
         <x:v>AND.cpl.x.we.crashed.wav</x:v>
       </x:c>
-      <x:c r="C132" s="13" t="str">
+      <x:c r="C132" s="12" t="str">
         <x:v>The a what we crashed are you all okay.</x:v>
       </x:c>
     </x:row>
@@ -1872,7 +1712,7 @@
       <x:c r="B133" s="12" t="str">
         <x:v>AND.cpl.x.wtoo.high.att.no.stretcher.wav</x:v>
       </x:c>
-      <x:c r="C133" s="13" t="str">
+      <x:c r="C133" s="12" t="str">
         <x:v>Hey hey captain that's not and aerobatic helicopter please keep calm.</x:v>
       </x:c>
     </x:row>
@@ -1883,7 +1723,7 @@
       <x:c r="B134" s="12" t="str">
         <x:v>AND.cpl.y.gnd.op.completed.set.engines.idle.or.wav</x:v>
       </x:c>
-      <x:c r="C134" s="13" t="str">
+      <x:c r="C134" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
     </x:row>
@@ -1894,7 +1734,7 @@
       <x:c r="B135" s="12" t="str">
         <x:v>AND.cpl.y.gnd.op.completed.start.engines.or.wav</x:v>
       </x:c>
-      <x:c r="C135" s="13" t="str">
+      <x:c r="C135" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
     </x:row>
@@ -1905,7 +1745,7 @@
       <x:c r="B136" s="12" t="str">
         <x:v>AND.cpl.ya.reduce.collective.wav</x:v>
       </x:c>
-      <x:c r="C136" s="13" t="str">
+      <x:c r="C136" s="12" t="str">
         <x:v>Watch out reduce collective now.</x:v>
       </x:c>
     </x:row>
@@ -1916,7 +1756,7 @@
       <x:c r="B137" s="12" t="str">
         <x:v>AND.cpl.ya.we.received.call.from.doc.modify.wav</x:v>
       </x:c>
-      <x:c r="C137" s="13" t="str">
+      <x:c r="C137" s="12" t="str">
         <x:v>A crew i just received a call from doc the ambulance has been rerouted to another hospital it seems to be better for patient conditions we have to modify our root for the new picking point location.</x:v>
       </x:c>
     </x:row>
@@ -1927,7 +1767,7 @@
       <x:c r="B138" s="12" t="str">
         <x:v>AND.cpl.yb.medical.crew.ready.ground.wav</x:v>
       </x:c>
-      <x:c r="C138" s="13" t="str">
+      <x:c r="C138" s="12" t="str">
         <x:v>Medical crew was starting ground loading procedures we have to wait here.</x:v>
       </x:c>
     </x:row>
@@ -1938,7 +1778,7 @@
       <x:c r="B139" s="12" t="str">
         <x:v>AND.cpl.yb.medical.crew.ready.hoist.forced.wav</x:v>
       </x:c>
-      <x:c r="C139" s="13" t="str">
+      <x:c r="C139" s="12" t="str">
         <x:v>Medical crew informs the due to distance we need to proceed with hoist operation crew was ready waiting us.</x:v>
       </x:c>
     </x:row>
@@ -1949,7 +1789,7 @@
       <x:c r="B140" s="12" t="str">
         <x:v>AND.cpl.yb.medical.crew.ready.hoist.wav</x:v>
       </x:c>
-      <x:c r="C140" s="13" t="str">
+      <x:c r="C140" s="12" t="str">
         <x:v>Medical crew was ready for hoist operation.</x:v>
       </x:c>
     </x:row>
@@ -1960,7 +1800,7 @@
       <x:c r="B141" s="12" t="str">
         <x:v>AND.cpl.yb.patient.will.be.transported.by.ambudoc.wav</x:v>
       </x:c>
-      <x:c r="C141" s="13" t="str">
+      <x:c r="C141" s="12" t="str">
         <x:v>Patient and doctor will be transported by ambulance and we have to pick doc and hospital.</x:v>
       </x:c>
     </x:row>
@@ -1971,7 +1811,7 @@
       <x:c r="B142" s="12" t="str">
         <x:v>AND.cpl.yb.patient.will.be.transported.by.ambulance.wav</x:v>
       </x:c>
-      <x:c r="C142" s="13" t="str">
+      <x:c r="C142" s="12" t="str">
         <x:v>Patient will be transported by ambulance we completed our task.</x:v>
       </x:c>
     </x:row>
@@ -1982,7 +1822,7 @@
       <x:c r="B143" s="12" t="str">
         <x:v>AND.cpl.yb.patient.will.be.transported.by.us.wav</x:v>
       </x:c>
-      <x:c r="C143" s="13" t="str">
+      <x:c r="C143" s="12" t="str">
         <x:v>Patient will be transported by us.</x:v>
       </x:c>
     </x:row>
@@ -1993,7 +1833,7 @@
       <x:c r="B144" s="12" t="str">
         <x:v>AND.cpl.yb.rescue.team.identified.landing.spot.wav</x:v>
       </x:c>
-      <x:c r="C144" s="13" t="str">
+      <x:c r="C144" s="12" t="str">
         <x:v>Rescue team identified a valid landing spot a marshal or is waiting us.</x:v>
       </x:c>
     </x:row>
@@ -2004,7 +1844,7 @@
       <x:c r="B145" s="12" t="str">
         <x:v>AND.cpl.yb.we.cannot.takeoff.fuel.hose.wav</x:v>
       </x:c>
-      <x:c r="C145" s="13" t="str">
+      <x:c r="C145" s="12" t="str">
         <x:v>Hey we cannot take off with fuel hose attached.</x:v>
       </x:c>
     </x:row>
@@ -2015,7 +1855,7 @@
       <x:c r="B146" s="12" t="str">
         <x:v>AND.cpl.yc.crew.ready.ldg.spot.we.can.proceed.wav</x:v>
       </x:c>
-      <x:c r="C146" s="13" t="str">
+      <x:c r="C146" s="12" t="str">
         <x:v>Crew is ready on landing spot we can proceed.</x:v>
       </x:c>
     </x:row>
@@ -2026,7 +1866,7 @@
       <x:c r="B147" s="12" t="str">
         <x:v>AND.dead.wav</x:v>
       </x:c>
-      <x:c r="C147" s="13" t="str">
+      <x:c r="C147" s="12" t="str">
         <x:v>[Non-verbal sound effect.]</x:v>
       </x:c>
     </x:row>
@@ -2037,7 +1877,7 @@
       <x:c r="B148" s="12" t="str">
         <x:v>AND.packtest.wav</x:v>
       </x:c>
-      <x:c r="C148" s="13" t="str">
+      <x:c r="C148" s="12" t="str">
         <x:v>This is the default hoist pack enjoy.</x:v>
       </x:c>
     </x:row>
@@ -2048,7 +1888,7 @@
       <x:c r="B149" s="12" t="str">
         <x:v>AND.plt.comm.check.wav</x:v>
       </x:c>
-      <x:c r="C149" s="13" t="str">
+      <x:c r="C149" s="12" t="str">
         <x:v>Through comm check please.</x:v>
       </x:c>
     </x:row>
@@ -2059,7 +1899,7 @@
       <x:c r="B150" s="12" t="str">
         <x:v>AND.plt.deboard.authorized.wav</x:v>
       </x:c>
-      <x:c r="C150" s="13" t="str">
+      <x:c r="C150" s="12" t="str">
         <x:v>Landed crew aboard authorized.</x:v>
       </x:c>
     </x:row>
@@ -2070,7 +1910,7 @@
       <x:c r="B151" s="12" t="str">
         <x:v>AND.plt.evacuate.wav</x:v>
       </x:c>
-      <x:c r="C151" s="13" t="str">
+      <x:c r="C151" s="12" t="str">
         <x:v>Evacuate helicopter now.</x:v>
       </x:c>
     </x:row>
@@ -2081,7 +1921,7 @@
       <x:c r="B152" s="12" t="str">
         <x:v>AND.plt.u.hi.sarah.wav</x:v>
       </x:c>
-      <x:c r="C152" s="13" t="str">
+      <x:c r="C152" s="12" t="str">
         <x:v>Hi sarah how you helicopter is good fuel needs to be refilled.</x:v>
       </x:c>
     </x:row>
@@ -2092,7 +1932,7 @@
       <x:c r="B153" s="12" t="str">
         <x:v>AND.plt.u.ill.chk.wav</x:v>
       </x:c>
-      <x:c r="C153" s="13" t="str">
+      <x:c r="C153" s="12" t="str">
         <x:v>I'll check.</x:v>
       </x:c>
     </x:row>
@@ -2103,7 +1943,7 @@
       <x:c r="B154" s="12" t="str">
         <x:v>AND.plt.u.mission.accomplished.wav</x:v>
       </x:c>
-      <x:c r="C154" s="13" t="str">
+      <x:c r="C154" s="12" t="str">
         <x:v>Mission accomplished.</x:v>
       </x:c>
     </x:row>
@@ -2114,7 +1954,7 @@
       <x:c r="B155" s="12" t="str">
         <x:v>AND.plt.u.thank.u.wav</x:v>
       </x:c>
-      <x:c r="C155" s="13" t="str">
+      <x:c r="C155" s="12" t="str">
         <x:v>Thank you.</x:v>
       </x:c>
     </x:row>
@@ -2125,7 +1965,7 @@
       <x:c r="B156" s="12" t="str">
         <x:v>AND.plt.u.tks.frank.wav</x:v>
       </x:c>
-      <x:c r="C156" s="13" t="str">
+      <x:c r="C156" s="12" t="str">
         <x:v>Thank you frank.</x:v>
       </x:c>
     </x:row>
@@ -2136,7 +1976,7 @@
       <x:c r="B157" s="12" t="str">
         <x:v>AND.plt.u.we.did.our.best.wav</x:v>
       </x:c>
-      <x:c r="C157" s="13" t="str">
+      <x:c r="C157" s="12" t="str">
         <x:v>We did our best unfortunately we cannot save all patients.</x:v>
       </x:c>
     </x:row>
@@ -2147,7 +1987,7 @@
       <x:c r="B158" s="12" t="str">
         <x:v>AND.plt.u.well.done.wav</x:v>
       </x:c>
-      <x:c r="C158" s="13" t="str">
+      <x:c r="C158" s="12" t="str">
         <x:v>Well done.</x:v>
       </x:c>
     </x:row>
@@ -2158,7 +1998,7 @@
       <x:c r="B159" s="12" t="str">
         <x:v>AND.plt.v.TWO.NM.accident.wav</x:v>
       </x:c>
-      <x:c r="C159" s="13" t="str">
+      <x:c r="C159" s="12" t="str">
         <x:v>Two nautical miles from accident area.</x:v>
       </x:c>
     </x:row>
@@ -2169,7 +2009,7 @@
       <x:c r="B160" s="12" t="str">
         <x:v>AND.plt.v.TWO.NM.base.wav</x:v>
       </x:c>
-      <x:c r="C160" s="13" t="str">
+      <x:c r="C160" s="12" t="str">
         <x:v>Two nautical miles from our base.</x:v>
       </x:c>
     </x:row>
@@ -2180,7 +2020,7 @@
       <x:c r="B161" s="12" t="str">
         <x:v>AND.plt.v.TWO.NM.hospital.wav</x:v>
       </x:c>
-      <x:c r="C161" s="13" t="str">
+      <x:c r="C161" s="12" t="str">
         <x:v>Two nautical miles from hospital.</x:v>
       </x:c>
     </x:row>
@@ -2191,7 +2031,7 @@
       <x:c r="B162" s="12" t="str">
         <x:v>AND.plt.v.TWO.NM.loading.wav</x:v>
       </x:c>
-      <x:c r="C162" s="13" t="str">
+      <x:c r="C162" s="12" t="str">
         <x:v>Two nautical miles from loading area.</x:v>
       </x:c>
     </x:row>
@@ -2202,7 +2042,7 @@
       <x:c r="B163" s="12" t="str">
         <x:v>AND.plt.va.engine.parameters.wav</x:v>
       </x:c>
-      <x:c r="C163" s="13" t="str">
+      <x:c r="C163" s="12" t="str">
         <x:v>Engine parameters when not good.</x:v>
       </x:c>
     </x:row>
@@ -2213,7 +2053,7 @@
       <x:c r="B164" s="12" t="str">
         <x:v>AND.plt.va.exceeded VNE.wav</x:v>
       </x:c>
-      <x:c r="C164" s="13" t="str">
+      <x:c r="C164" s="12" t="str">
         <x:v>We exceeded VNE.</x:v>
       </x:c>
     </x:row>
@@ -2224,7 +2064,7 @@
       <x:c r="B165" s="12" t="str">
         <x:v>AND.plt.va.FLI.wav</x:v>
       </x:c>
-      <x:c r="C165" s="13" t="str">
+      <x:c r="C165" s="12" t="str">
         <x:v>We exceeded the torque limits.</x:v>
       </x:c>
     </x:row>
@@ -2235,7 +2075,7 @@
       <x:c r="B166" s="12" t="str">
         <x:v>AND.plt.va.hi.sarah.bad.news.wav</x:v>
       </x:c>
-      <x:c r="C166" s="13" t="str">
+      <x:c r="C166" s="12" t="str">
         <x:v>Hi sarah i'm sorry we have some bad news for you.</x:v>
       </x:c>
     </x:row>
@@ -2246,7 +2086,7 @@
       <x:c r="B167" s="12" t="str">
         <x:v>AND.plt.va.MGB.parameters.wav</x:v>
       </x:c>
-      <x:c r="C167" s="13" t="str">
+      <x:c r="C167" s="12" t="str">
         <x:v>Main gearbox parameters were high and we felt hi vibrations.</x:v>
       </x:c>
     </x:row>
@@ -2257,7 +2097,7 @@
       <x:c r="B168" s="12" t="str">
         <x:v>AND.plt.va.TGB.parameters.wav</x:v>
       </x:c>
-      <x:c r="C168" s="13" t="str">
+      <x:c r="C168" s="12" t="str">
         <x:v>We had tail rotor gearbox parameters fluctuations.</x:v>
       </x:c>
     </x:row>
@@ -2268,7 +2108,7 @@
       <x:c r="B169" s="12" t="str">
         <x:v>AND.plt.va.we.had.failures.wav</x:v>
       </x:c>
-      <x:c r="C169" s="13" t="str">
+      <x:c r="C169" s="12" t="str">
         <x:v>We had failures they are reported in the technical log book.</x:v>
       </x:c>
     </x:row>
@@ -2279,7 +2119,7 @@
       <x:c r="B170" s="12" t="str">
         <x:v>AND.plt.va.we.had.hard.landing.wav</x:v>
       </x:c>
-      <x:c r="C170" s="13" t="str">
+      <x:c r="C170" s="12" t="str">
         <x:v>We had a hard landing.</x:v>
       </x:c>
     </x:row>
@@ -2290,7 +2130,7 @@
       <x:c r="B171" s="12" t="str">
         <x:v>AND.plt.vaa.2NM.pickup.location.wav</x:v>
       </x:c>
-      <x:c r="C171" s="13" t="str">
+      <x:c r="C171" s="12" t="str">
         <x:v>Two nautical miles from pick up location.</x:v>
       </x:c>
     </x:row>
@@ -2301,7 +2141,7 @@
       <x:c r="B172" s="12" t="str">
         <x:v>AND.plt.vaa.approaching.HR.Drop.wav</x:v>
       </x:c>
-      <x:c r="C172" s="13" t="str">
+      <x:c r="C172" s="12" t="str">
         <x:v>Hr we are now approaching to drop point thanks for the help and see you next time.</x:v>
       </x:c>
     </x:row>
@@ -2312,7 +2152,7 @@
       <x:c r="B173" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.1.wav</x:v>
       </x:c>
-      <x:c r="C173" s="13" t="str">
+      <x:c r="C173" s="12" t="str">
         <x:v>We are entering into designated SAR area it's time to start our search for the casualties.</x:v>
       </x:c>
     </x:row>
@@ -2323,7 +2163,7 @@
       <x:c r="B174" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.2.wav</x:v>
       </x:c>
-      <x:c r="C174" s="13" t="str">
+      <x:c r="C174" s="12" t="str">
         <x:v>SAR area starts here watch out and let's find our signed casualties.</x:v>
       </x:c>
     </x:row>
@@ -2334,7 +2174,7 @@
       <x:c r="B175" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.3.wav</x:v>
       </x:c>
-      <x:c r="C175" s="13" t="str">
+      <x:c r="C175" s="12" t="str">
         <x:v>Crew please stop searching for the survivor now we are entering in the assigned area.</x:v>
       </x:c>
     </x:row>
@@ -2345,7 +2185,7 @@
       <x:c r="B176" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.4.wav</x:v>
       </x:c>
-      <x:c r="C176" s="13" t="str">
+      <x:c r="C176" s="12" t="str">
         <x:v>Confirmed solve every of established the clock is ticking let's find the casualties now.</x:v>
       </x:c>
     </x:row>
@@ -2356,7 +2196,7 @@
       <x:c r="B177" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.5.wav</x:v>
       </x:c>
-      <x:c r="C177" s="13" t="str">
+      <x:c r="C177" s="12" t="str">
         <x:v>The boundary crossed let's execute the search plan and locate the survivors.</x:v>
       </x:c>
     </x:row>
@@ -2367,7 +2207,7 @@
       <x:c r="B178" s="12" t="str">
         <x:v>AND.PLT.vaa.we.are.entering.sar.area.6.wav</x:v>
       </x:c>
-      <x:c r="C178" s="13" t="str">
+      <x:c r="C178" s="12" t="str">
         <x:v>We have reached the search and rescue zone initiate the search pattern for survivors.</x:v>
       </x:c>
     </x:row>
@@ -2378,7 +2218,7 @@
       <x:c r="B179" s="12" t="str">
         <x:v>AND.plt.vab.crew.is.coming.back.wav</x:v>
       </x:c>
-      <x:c r="C179" s="13" t="str">
+      <x:c r="C179" s="12" t="str">
         <x:v>Crew is cutting back.</x:v>
       </x:c>
     </x:row>
@@ -2389,7 +2229,7 @@
       <x:c r="B180" s="12" t="str">
         <x:v>AND.plt.vab.let.s.go.wav</x:v>
       </x:c>
-      <x:c r="C180" s="13" t="str">
+      <x:c r="C180" s="12" t="str">
         <x:v>Let's go.</x:v>
       </x:c>
     </x:row>
@@ -2400,7 +2240,7 @@
       <x:c r="B181" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch.question1.wav</x:v>
       </x:c>
-      <x:c r="C181" s="13" t="str">
+      <x:c r="C181" s="12" t="str">
         <x:v>We're crew are we able to accept a new dispatch or do we need to come back to base.</x:v>
       </x:c>
     </x:row>
@@ -2411,7 +2251,7 @@
       <x:c r="B182" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch.question2.wav</x:v>
       </x:c>
-      <x:c r="C182" s="13" t="str">
+      <x:c r="C182" s="12" t="str">
         <x:v>I believe we must go back to the base before we accept new dispatches.</x:v>
       </x:c>
     </x:row>
@@ -2422,7 +2262,7 @@
       <x:c r="B183" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch1.wav</x:v>
       </x:c>
-      <x:c r="C183" s="13" t="str">
+      <x:c r="C183" s="12" t="str">
         <x:v>Hey we have a new dispatch.</x:v>
       </x:c>
     </x:row>
@@ -2433,7 +2273,7 @@
       <x:c r="B184" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch2.wav</x:v>
       </x:c>
-      <x:c r="C184" s="13" t="str">
+      <x:c r="C184" s="12" t="str">
         <x:v>How crew we have a new assignment.</x:v>
       </x:c>
     </x:row>
@@ -2444,7 +2284,7 @@
       <x:c r="B185" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch3.wav</x:v>
       </x:c>
-      <x:c r="C185" s="13" t="str">
+      <x:c r="C185" s="12" t="str">
         <x:v>How we have another dispatch.</x:v>
       </x:c>
     </x:row>
@@ -2455,7 +2295,7 @@
       <x:c r="B186" s="12" t="str">
         <x:v>AND.plt.vab.new.dispatch4.wav</x:v>
       </x:c>
-      <x:c r="C186" s="13" t="str">
+      <x:c r="C186" s="12" t="str">
         <x:v>Busy day we received a new dispatch.</x:v>
       </x:c>
     </x:row>
@@ -2466,7 +2306,7 @@
       <x:c r="B187" s="12" t="str">
         <x:v>AND.plt.vab.route.to.drop.pt.wav</x:v>
       </x:c>
-      <x:c r="C187" s="13" t="str">
+      <x:c r="C187" s="12" t="str">
         <x:v>Looks set to drop point.</x:v>
       </x:c>
     </x:row>
@@ -2477,7 +2317,7 @@
       <x:c r="B188" s="12" t="str">
         <x:v>AND.plt.vab.route.to.pick.up.wav</x:v>
       </x:c>
-      <x:c r="C188" s="13" t="str">
+      <x:c r="C188" s="12" t="str">
         <x:v>Group set to the pick up point.</x:v>
       </x:c>
     </x:row>
@@ -2488,7 +2328,7 @@
       <x:c r="B189" s="12" t="str">
         <x:v>AND.PAX2.comm.check.wav</x:v>
       </x:c>
-      <x:c r="C189" s="13" t="str">
+      <x:c r="C189" s="12" t="str">
         <x:v>Copy paramedic here comm check.</x:v>
       </x:c>
     </x:row>
@@ -2499,7 +2339,7 @@
       <x:c r="B190" s="12" t="str">
         <x:v>AND.PAX2.hi.sarah.wav</x:v>
       </x:c>
-      <x:c r="C190" s="13" t="str">
+      <x:c r="C190" s="12" t="str">
         <x:v>Hi anna nice to meet you again are you free for lunch tomorrow.</x:v>
       </x:c>
     </x:row>
@@ -2510,7 +2350,7 @@
       <x:c r="B191" s="12" t="str">
         <x:v>AND.PAX2.stretcher.secured.wav</x:v>
       </x:c>
-      <x:c r="C191" s="13" t="str">
+      <x:c r="C191" s="12" t="str">
         <x:v>Stretches secured.</x:v>
       </x:c>
     </x:row>
@@ -2521,7 +2361,7 @@
       <x:c r="B192" s="12" t="str">
         <x:v>AND.pax3.ambulance.wav</x:v>
       </x:c>
-      <x:c r="C192" s="13" t="str">
+      <x:c r="C192" s="12" t="str">
         <x:v>The ambulance with no paramedic.</x:v>
       </x:c>
     </x:row>
@@ -2532,7 +2372,7 @@
       <x:c r="B193" s="12" t="str">
         <x:v>AND.pax3.comm.chk.wav</x:v>
       </x:c>
-      <x:c r="C193" s="13" t="str">
+      <x:c r="C193" s="12" t="str">
         <x:v>Duck here comm check.</x:v>
       </x:c>
     </x:row>
@@ -2543,7 +2383,7 @@
       <x:c r="B194" s="12" t="str">
         <x:v>AND.pax3.confirmed.onscene.wav</x:v>
       </x:c>
-      <x:c r="C194" s="13" t="str">
+      <x:c r="C194" s="12" t="str">
         <x:v>Confirmed on scene.</x:v>
       </x:c>
     </x:row>
@@ -2554,7 +2394,7 @@
       <x:c r="B195" s="12" t="str">
         <x:v>AND.pax3.fire.engine.wav</x:v>
       </x:c>
-      <x:c r="C195" s="13" t="str">
+      <x:c r="C195" s="12" t="str">
         <x:v>Fire engine.</x:v>
       </x:c>
     </x:row>
@@ -2565,7 +2405,7 @@
       <x:c r="B196" s="12" t="str">
         <x:v>AND.pax3.gnd.ops.pls.standby.wav</x:v>
       </x:c>
-      <x:c r="C196" s="13" t="str">
+      <x:c r="C196" s="12" t="str">
         <x:v>We need time for ground operations please stand by.</x:v>
       </x:c>
     </x:row>
@@ -2576,7 +2416,7 @@
       <x:c r="B197" s="12" t="str">
         <x:v>AND.pax3.hosppital.proposal.wav</x:v>
       </x:c>
-      <x:c r="C197" s="13" t="str">
+      <x:c r="C197" s="12" t="str">
         <x:v>I said of possible hospital destination for our patient info available on tablet we can confirm or change later.</x:v>
       </x:c>
     </x:row>
@@ -2587,7 +2427,7 @@
       <x:c r="B198" s="12" t="str">
         <x:v>AND.pax3.patient.has.died.wav</x:v>
       </x:c>
-      <x:c r="C198" s="13" t="str">
+      <x:c r="C198" s="12" t="str">
         <x:v>Patient has died.</x:v>
       </x:c>
     </x:row>
@@ -2598,7 +2438,7 @@
       <x:c r="B199" s="12" t="str">
         <x:v>AND.pax3.patient.life.signs.fading.wav</x:v>
       </x:c>
-      <x:c r="C199" s="13" t="str">
+      <x:c r="C199" s="12" t="str">
         <x:v>Patient life signs of fading.</x:v>
       </x:c>
     </x:row>
@@ -2609,7 +2449,7 @@
       <x:c r="B200" s="12" t="str">
         <x:v>AND.pax3.patient.midway.wav</x:v>
       </x:c>
-      <x:c r="C200" s="13" t="str">
+      <x:c r="C200" s="12" t="str">
         <x:v>Patient location is far away ambulance crew on seen may transport patient to the meeting point proposed on tablet please confirm if we want to meet midway.</x:v>
       </x:c>
     </x:row>
@@ -2620,7 +2460,7 @@
       <x:c r="B201" s="12" t="str">
         <x:v>AND.pax3.patient.onboard.wav</x:v>
       </x:c>
-      <x:c r="C201" s="13" t="str">
+      <x:c r="C201" s="12" t="str">
         <x:v>Patient on board take care.</x:v>
       </x:c>
     </x:row>
@@ -2631,7 +2471,7 @@
       <x:c r="B202" s="12" t="str">
         <x:v>AND.pax3.patient.safe.wav</x:v>
       </x:c>
-      <x:c r="C202" s="13" t="str">
+      <x:c r="C202" s="12" t="str">
         <x:v>Patient has been the board to the hospital key is safe.</x:v>
       </x:c>
     </x:row>
@@ -2642,7 +2482,7 @@
       <x:c r="B203" s="12" t="str">
         <x:v>AND.pax3.police.wav</x:v>
       </x:c>
-      <x:c r="C203" s="13" t="str">
+      <x:c r="C203" s="12" t="str">
         <x:v>Police.</x:v>
       </x:c>
     </x:row>
@@ -2653,7 +2493,7 @@
       <x:c r="B204" s="12" t="str">
         <x:v>AND.pax3.qpatient.safe.wav</x:v>
       </x:c>
-      <x:c r="C204" s="13" t="str">
+      <x:c r="C204" s="12" t="str">
         <x:v>Patients has been deboarded to the hospital.</x:v>
       </x:c>
     </x:row>
@@ -2664,7 +2504,7 @@
       <x:c r="B205" s="12" t="str">
         <x:v>AND.pax3.we.will.be.first.on.scene.wav</x:v>
       </x:c>
-      <x:c r="C205" s="13" t="str">
+      <x:c r="C205" s="12" t="str">
         <x:v>We will be first on scene.</x:v>
       </x:c>
     </x:row>
@@ -2675,7 +2515,7 @@
       <x:c r="B206" s="12" t="str">
         <x:v>AND.pax3.we.will.find.ambulance.not.far.away.wav</x:v>
       </x:c>
-      <x:c r="C206" s="13" t="str">
+      <x:c r="C206" s="12" t="str">
         <x:v>We will find an ambulance not far away from accident site they are unable to reach the site.</x:v>
       </x:c>
     </x:row>
@@ -2686,7 +2526,7 @@
       <x:c r="B207" s="12" t="str">
         <x:v>AND.PAX3.wea.CPR.in.progress.wav</x:v>
       </x:c>
-      <x:c r="C207" s="13" t="str">
+      <x:c r="C207" s="12" t="str">
         <x:v>Cpr in progress please stand by it may take time.</x:v>
       </x:c>
     </x:row>
@@ -2697,7 +2537,7 @@
       <x:c r="B208" s="12" t="str">
         <x:v>AND.PAX3.wea.lost.patient.wav</x:v>
       </x:c>
-      <x:c r="C208" s="13" t="str">
+      <x:c r="C208" s="12" t="str">
         <x:v>We lost the patient we have to record the time of the death please stand by until we secure the cabin.</x:v>
       </x:c>
     </x:row>
@@ -2708,7 +2548,7 @@
       <x:c r="B209" s="12" t="str">
         <x:v>AND.PAX3.wea.patient.CPR.successful.wav</x:v>
       </x:c>
-      <x:c r="C209" s="13" t="str">
+      <x:c r="C209" s="12" t="str">
         <x:v>Good cpr successfully reanimated patient we are now securing him for the flight please wait for clearance.</x:v>
       </x:c>
     </x:row>
@@ -2719,7 +2559,7 @@
       <x:c r="B210" s="12" t="str">
         <x:v>AND.pax3.weneed.extra.time.for.transport.wav</x:v>
       </x:c>
-      <x:c r="C210" s="13" t="str">
+      <x:c r="C210" s="12" t="str">
         <x:v>Patient conditions are critical we need extra time to stabilize for transport please wait.</x:v>
       </x:c>
     </x:row>
@@ -2730,7 +2570,7 @@
       <x:c r="B211" s="12" t="str">
         <x:v>AND.pax3.weo.lost.organ.wav</x:v>
       </x:c>
-      <x:c r="C211" s="13" t="str">
+      <x:c r="C211" s="12" t="str">
         <x:v>I believe we lost the organ it's too degraded.</x:v>
       </x:c>
     </x:row>
@@ -2741,7 +2581,7 @@
       <x:c r="B212" s="12" t="str">
         <x:v>AND.pax3.weo.organ.degraded.wav</x:v>
       </x:c>
-      <x:c r="C212" s="13" t="str">
+      <x:c r="C212" s="12" t="str">
         <x:v>Organs data seems to be degrading.</x:v>
       </x:c>
     </x:row>
@@ -2752,7 +2592,7 @@
       <x:c r="B213" s="12" t="str">
         <x:v>AND.pax3.weo.wbriefing.wav</x:v>
       </x:c>
-      <x:c r="C213" s="13" t="str">
+      <x:c r="C213" s="12" t="str">
         <x:v>Let's proceed with a small briefing about our next operations as soon as we arrive h i will proceed to the scene securing the area after their clearance our crew will join them to perform the medical operation at the end of rescue operations the medical cruel board followed by hr in case the engine has to be transported with hoist out i will be boarded first all clear.</x:v>
       </x:c>
     </x:row>
@@ -2763,7 +2603,7 @@
       <x:c r="B214" s="12" t="str">
         <x:v>AND.pax3.weo.welcome.wav</x:v>
       </x:c>
-      <x:c r="C214" s="13" t="str">
+      <x:c r="C214" s="12" t="str">
         <x:v>Welcome onboard hello his viewers.</x:v>
       </x:c>
     </x:row>
@@ -2774,7 +2614,7 @@
       <x:c r="B215" s="12" t="str">
         <x:v>AND.frank.doyou.need.fuel.wav</x:v>
       </x:c>
-      <x:c r="C215" s="13" t="str">
+      <x:c r="C215" s="12" t="str">
         <x:v>If you need refueling please ask.</x:v>
       </x:c>
     </x:row>
@@ -2785,7 +2625,7 @@
       <x:c r="B216" s="12" t="str">
         <x:v>AND.frank.fuel.as.requested.wav</x:v>
       </x:c>
-      <x:c r="C216" s="13" t="str">
+      <x:c r="C216" s="12" t="str">
         <x:v>Fuel is as you requested.</x:v>
       </x:c>
     </x:row>
@@ -2796,7 +2636,7 @@
       <x:c r="B217" s="12" t="str">
         <x:v>AND.frank.fuel.full.wav</x:v>
       </x:c>
-      <x:c r="C217" s="13" t="str">
+      <x:c r="C217" s="12" t="str">
         <x:v>Fuel tanks are almost full.</x:v>
       </x:c>
     </x:row>
@@ -2807,7 +2647,7 @@
       <x:c r="B218" s="12" t="str">
         <x:v>AND.frank.fuel.low.wav</x:v>
       </x:c>
-      <x:c r="C218" s="13" t="str">
+      <x:c r="C218" s="12" t="str">
         <x:v>Refueling has not been performed and fuel level is low.</x:v>
       </x:c>
     </x:row>
@@ -2818,7 +2658,7 @@
       <x:c r="B219" s="12" t="str">
         <x:v>AND.frank.GPU.disco.wav</x:v>
       </x:c>
-      <x:c r="C219" s="13" t="str">
+      <x:c r="C219" s="12" t="str">
         <x:v>Gp you disconnected ready to go good day.</x:v>
       </x:c>
     </x:row>
@@ -2829,7 +2669,7 @@
       <x:c r="B220" s="12" t="str">
         <x:v>AND.frank.helicopter.clear.logbook.signed.wav</x:v>
       </x:c>
-      <x:c r="C220" s="13" t="str">
+      <x:c r="C220" s="12" t="str">
         <x:v>I kept captain helicopter is ready to fly law book filled and signed.</x:v>
       </x:c>
     </x:row>
@@ -2840,7 +2680,7 @@
       <x:c r="B221" s="12" t="str">
         <x:v>AND.frank.hi.all.wav</x:v>
       </x:c>
-      <x:c r="C221" s="13" t="str">
+      <x:c r="C221" s="12" t="str">
         <x:v>Hey good morning all ready for the missions.</x:v>
       </x:c>
     </x:row>
@@ -2851,7 +2691,7 @@
       <x:c r="B222" s="12" t="str">
         <x:v>AND.frank.ready.for.GPU.wav</x:v>
       </x:c>
-      <x:c r="C222" s="13" t="str">
+      <x:c r="C222" s="12" t="str">
         <x:v>Really to supply external power at your request.</x:v>
       </x:c>
     </x:row>
@@ -2862,7 +2702,7 @@
       <x:c r="B223" s="12" t="str">
         <x:v>AND.Sarah.bye.wav</x:v>
       </x:c>
-      <x:c r="C223" s="13" t="str">
+      <x:c r="C223" s="12" t="str">
         <x:v>Bye see you tomorrow.</x:v>
       </x:c>
     </x:row>
@@ -2873,7 +2713,7 @@
       <x:c r="B224" s="12" t="str">
         <x:v>AND.Sarah.everything.good.wav</x:v>
       </x:c>
-      <x:c r="C224" s="13" t="str">
+      <x:c r="C224" s="12" t="str">
         <x:v>How was the last mission was everything good with the helicopter.</x:v>
       </x:c>
     </x:row>
@@ -2884,7 +2724,7 @@
       <x:c r="B225" s="12" t="str">
         <x:v>AND.Sarah.helicopter.in.precious.hands.wav</x:v>
       </x:c>
-      <x:c r="C225" s="13" t="str">
+      <x:c r="C225" s="12" t="str">
         <x:v>Don't worry the helicopter is now in my precious hands it will be ready to fly for the next mission.</x:v>
       </x:c>
     </x:row>
@@ -2895,7 +2735,7 @@
       <x:c r="B226" s="12" t="str">
         <x:v>AND.Sarah.hi.guys.wav</x:v>
       </x:c>
-      <x:c r="C226" s="13" t="str">
+      <x:c r="C226" s="12" t="str">
         <x:v>Oh my preferred cray hi guys.</x:v>
       </x:c>
     </x:row>
@@ -2906,7 +2746,7 @@
       <x:c r="B227" s="12" t="str">
         <x:v>AND.Sarah.it.seems.i.have.to.work.wav</x:v>
       </x:c>
-      <x:c r="C227" s="13" t="str">
+      <x:c r="C227" s="12" t="str">
         <x:v>It seems i have to work a lot on it.</x:v>
       </x:c>
     </x:row>
@@ -2917,7 +2757,7 @@
       <x:c r="B228" s="12" t="str">
         <x:v>AND.Sarah.tomorrow.there.is.a.restaurant.wav</x:v>
       </x:c>
-      <x:c r="C228" s="13" t="str">
+      <x:c r="C228" s="12" t="str">
         <x:v>Hi tomorrow okay there is a good restaurant just out of here.</x:v>
       </x:c>
     </x:row>
@@ -2928,25 +2768,433 @@
       <x:c r="B229" s="12" t="str">
         <x:v>AND.Sarah.what.you.did.wav</x:v>
       </x:c>
-      <x:c r="C229" s="13" t="str">
+      <x:c r="C229" s="12" t="str">
         <x:v>Hey what you did to the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="230" ht="15" hidden="0" customHeight="1">
-      <x:c r="A230" s="18" t="str">
+      <x:c r="A230" s="17" t="str">
         <x:v>L:ANDFOOL</x:v>
       </x:c>
-      <x:c r="B230" s="15" t="str">
+      <x:c r="B230" s="12" t="str">
         <x:v>stayngalive.wav</x:v>
       </x:c>
-      <x:c r="C230" s="16" t="str">
+      <x:c r="C230" s="12" t="str">
         <x:v>[Excerpt from “Stayin’ Alive”; lyrics omitted.]</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231" ht="42" customHeight="1">
+      <x:c r="A231" s="19" t="str">
+        <x:v>L:ANDMARSHALLEFT</x:v>
+      </x:c>
+      <x:c r="B231" s="20" t="str">
+        <x:v>AND.marshal.move.left.wav</x:v>
+      </x:c>
+      <x:c r="C231" s="20" t="str">
+        <x:v>Move left slowly.</x:v>
+      </x:c>
+      <x:c r="D231" s="20" t="str">
+        <x:v>Marshal</x:v>
+      </x:c>
+      <x:c r="E231" s="21" t="str">
+        <x:v>Shared marshall/pisteur3 controller selects the left correction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="42" customHeight="1">
+      <x:c r="A232" s="19" t="str">
+        <x:v>L:ANDMARSHALRIGHT</x:v>
+      </x:c>
+      <x:c r="B232" s="20" t="str">
+        <x:v>AND.marshal.move.right.wav</x:v>
+      </x:c>
+      <x:c r="C232" s="20" t="str">
+        <x:v>Move right slowly.</x:v>
+      </x:c>
+      <x:c r="D232" s="20" t="str">
+        <x:v>Marshal</x:v>
+      </x:c>
+      <x:c r="E232" s="21" t="str">
+        <x:v>Shared marshall/pisteur3 controller selects the right correction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="42" customHeight="1">
+      <x:c r="A233" s="19" t="str">
+        <x:v>L:ANDMARSHALFORWARD</x:v>
+      </x:c>
+      <x:c r="B233" s="20" t="str">
+        <x:v>AND.marshal.come.forward.wav</x:v>
+      </x:c>
+      <x:c r="C233" s="20" t="str">
+        <x:v>Come forward slowly.</x:v>
+      </x:c>
+      <x:c r="D233" s="20" t="str">
+        <x:v>Marshal</x:v>
+      </x:c>
+      <x:c r="E233" s="21" t="str">
+        <x:v>Shared marshal controller commands the forward approach.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="42" customHeight="1">
+      <x:c r="A234" s="19" t="str">
+        <x:v>L:ANDMARSHALHOLD</x:v>
+      </x:c>
+      <x:c r="B234" s="20" t="str">
+        <x:v>AND.marshal.hold.position.wav</x:v>
+      </x:c>
+      <x:c r="C234" s="20" t="str">
+        <x:v>Hold position.</x:v>
+      </x:c>
+      <x:c r="D234" s="20" t="str">
+        <x:v>Marshal</x:v>
+      </x:c>
+      <x:c r="E234" s="21" t="str">
+        <x:v>Marshal controller enters the hold or safety-buffer state.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="42" customHeight="1">
+      <x:c r="A235" s="19" t="str">
+        <x:v>L:ANDMARSHALLANDCLEAR</x:v>
+      </x:c>
+      <x:c r="B235" s="20" t="str">
+        <x:v>AND.marshal.landing.area.clear.wav</x:v>
+      </x:c>
+      <x:c r="C235" s="20" t="str">
+        <x:v>Landing area clear. You are cleared to land.</x:v>
+      </x:c>
+      <x:c r="D235" s="20" t="str">
+        <x:v>Marshal</x:v>
+      </x:c>
+      <x:c r="E235" s="21" t="str">
+        <x:v>A valid landing is committed inside the configured landing area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="42" customHeight="1">
+      <x:c r="A236" s="19" t="str">
+        <x:v>L:ANDMEDASSESSMENT</x:v>
+      </x:c>
+      <x:c r="B236" s="20" t="str">
+        <x:v>AND.medical.assessment.in.progress.wav</x:v>
+      </x:c>
+      <x:c r="C236" s="20" t="str">
+        <x:v>Patient assessment in progress. Stand by for the treatment decision.</x:v>
+      </x:c>
+      <x:c r="D236" s="20" t="str">
+        <x:v>Medical crew</x:v>
+      </x:c>
+      <x:c r="E236" s="21" t="str">
+        <x:v>Crew visit begins and the tablet starts revealing clinical data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="42" customHeight="1">
+      <x:c r="A237" s="19" t="str">
+        <x:v>L:ANDMEDCRITICAL</x:v>
+      </x:c>
+      <x:c r="B237" s="20" t="str">
+        <x:v>AND.medical.critical.vital.signs.wav</x:v>
+      </x:c>
+      <x:c r="C237" s="20" t="str">
+        <x:v>Critical vital signs. Prepare for immediate transport.</x:v>
+      </x:c>
+      <x:c r="D237" s="20" t="str">
+        <x:v>Medical crew</x:v>
+      </x:c>
+      <x:c r="E237" s="21" t="str">
+        <x:v>Critical-vitals indicators turn red, patient deterioration requires an urgent transport decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="42" customHeight="1">
+      <x:c r="A238" s="19" t="str">
+        <x:v>L:ANDMEDTRANSPORT</x:v>
+      </x:c>
+      <x:c r="B238" s="20" t="str">
+        <x:v>AND.medical.patient.ready.for.transport.wav</x:v>
+      </x:c>
+      <x:c r="C238" s="20" t="str">
+        <x:v>Patient stabilized for transport. Prepare the cabin for loading.</x:v>
+      </x:c>
+      <x:c r="D238" s="20" t="str">
+        <x:v>Medical crew</x:v>
+      </x:c>
+      <x:c r="E238" s="21" t="str">
+        <x:v>Treatment result allows the loading or transport branch to start.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="42" customHeight="1">
+      <x:c r="A239" s="19" t="str">
+        <x:v>L:ANDCPRAWAITLAND</x:v>
+      </x:c>
+      <x:c r="B239" s="20" t="str">
+        <x:v>AND.medical.cpr.awaiting.landing.wav</x:v>
+      </x:c>
+      <x:c r="C239" s="20" t="str">
+        <x:v>CPR is required. Land as soon as safely possible before treatment can start.</x:v>
+      </x:c>
+      <x:c r="D239" s="20" t="str">
+        <x:v>Medical crew</x:v>
+      </x:c>
+      <x:c r="E239" s="21" t="str">
+        <x:v>L:CPR becomes 1 while airborne and MCPR_ONBOARD is disabled.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="42" customHeight="1">
+      <x:c r="A240" s="19" t="str">
+        <x:v>L:ANDCPRSTOPPED</x:v>
+      </x:c>
+      <x:c r="B240" s="20" t="str">
+        <x:v>AND.medical.cpr.stopped.wav</x:v>
+      </x:c>
+      <x:c r="C240" s="20" t="str">
+        <x:v>CPR has been stopped. Continue monitoring and follow the clinical plan.</x:v>
+      </x:c>
+      <x:c r="D240" s="20" t="str">
+        <x:v>Medical crew</x:v>
+      </x:c>
+      <x:c r="E240" s="21" t="str">
+        <x:v>The tablet STOP CPR action sets L:CPR to 5.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="42" customHeight="1">
+      <x:c r="A241" s="19" t="str">
+        <x:v>L:ANDAMBUHANDOVER</x:v>
+      </x:c>
+      <x:c r="B241" s="20" t="str">
+        <x:v>AND.ground.ambulance.handover.ready.wav</x:v>
+      </x:c>
+      <x:c r="C241" s="20" t="str">
+        <x:v>Ambulance is on scene. Prepare for patient handover.</x:v>
+      </x:c>
+      <x:c r="D241" s="20" t="str">
+        <x:v>Ground support</x:v>
+      </x:c>
+      <x:c r="E241" s="21" t="str">
+        <x:v>Ambulance arrival completes, before the patient-transfer branch begins.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="42" customHeight="1">
+      <x:c r="A242" s="19" t="str">
+        <x:v>L:ANDSECONDAMBULANCE</x:v>
+      </x:c>
+      <x:c r="B242" s="20" t="str">
+        <x:v>AND.ground.second.ambulance.assigned.wav</x:v>
+      </x:c>
+      <x:c r="C242" s="20" t="str">
+        <x:v>A second ambulance is managing another patient. Keep the landing area clear.</x:v>
+      </x:c>
+      <x:c r="D242" s="20" t="str">
+        <x:v>Ground support</x:v>
+      </x:c>
+      <x:c r="E242" s="21" t="str">
+        <x:v>Secondary-rescue flow assigns ambulance 2 to patient 2 or patient 3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="42" customHeight="1">
+      <x:c r="A243" s="19" t="str">
+        <x:v>L:ANDPOLICESECURING</x:v>
+      </x:c>
+      <x:c r="B243" s="20" t="str">
+        <x:v>AND.ground.police.securing.scene.wav</x:v>
+      </x:c>
+      <x:c r="C243" s="20" t="str">
+        <x:v>Police are securing the scene. Stay clear until the area is released.</x:v>
+      </x:c>
+      <x:c r="D243" s="20" t="str">
+        <x:v>Ground support</x:v>
+      </x:c>
+      <x:c r="E243" s="21" t="str">
+        <x:v>Police arrival and the scene-security/privacy-screen path begin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="42" customHeight="1">
+      <x:c r="A244" s="19" t="str">
+        <x:v>L:ANDFIREHAZARD</x:v>
+      </x:c>
+      <x:c r="B244" s="20" t="str">
+        <x:v>AND.ground.fire.service.hazard.wav</x:v>
+      </x:c>
+      <x:c r="C244" s="20" t="str">
+        <x:v>Fire service is controlling a hazard. Do not land until cleared.</x:v>
+      </x:c>
+      <x:c r="D244" s="20" t="str">
+        <x:v>Ground support</x:v>
+      </x:c>
+      <x:c r="E244" s="21" t="str">
+        <x:v>Fire-engine or fire-hazard branch is active.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="42" customHeight="1">
+      <x:c r="A245" s="19" t="str">
+        <x:v>L:ANDOPSGROUNDDELAY</x:v>
+      </x:c>
+      <x:c r="B245" s="20" t="str">
+        <x:v>AND.ops.ground.operations.delayed.wav</x:v>
+      </x:c>
+      <x:c r="C245" s="20" t="str">
+        <x:v>Ground operations are delayed. Check the Dispatch page for the current status.</x:v>
+      </x:c>
+      <x:c r="D245" s="20" t="str">
+        <x:v>Flight or ground crew</x:v>
+      </x:c>
+      <x:c r="E245" s="21" t="str">
+        <x:v>ops_progress_warning becomes 1 after 120 seconds without progress; tablet shows the orange Dispatch warning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="42" customHeight="1">
+      <x:c r="A246" s="19" t="str">
+        <x:v>L:ANDHOISTPAUSE</x:v>
+      </x:c>
+      <x:c r="B246" s="20" t="str">
+        <x:v>AND.hoist.operation.paused.wav</x:v>
+      </x:c>
+      <x:c r="C246" s="20" t="str">
+        <x:v>Hold position. Hoist operation is paused until the aircraft is stable.</x:v>
+      </x:c>
+      <x:c r="D246" s="20" t="str">
+        <x:v>Hoist operator</x:v>
+      </x:c>
+      <x:c r="E246" s="21" t="str">
+        <x:v>A speed, acceleration, or bank-angle limit requires a temporary hoist pause.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="42" customHeight="1">
+      <x:c r="A247" s="19" t="str">
+        <x:v>L:ANDHOISTABORT</x:v>
+      </x:c>
+      <x:c r="B247" s="20" t="str">
+        <x:v>AND.hoist.operation.abort.wav</x:v>
+      </x:c>
+      <x:c r="C247" s="20" t="str">
+        <x:v>Abort the hoist operation. Recover the crew only when conditions are safe.</x:v>
+      </x:c>
+      <x:c r="D247" s="20" t="str">
+        <x:v>Hoist operator</x:v>
+      </x:c>
+      <x:c r="E247" s="21" t="str">
+        <x:v>An unsafe hoist state requires abort and recovery rather than continuation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="42" customHeight="1">
+      <x:c r="A248" s="19" t="str">
+        <x:v>L:ANDROUTEUNAVAILABLE</x:v>
+      </x:c>
+      <x:c r="B248" s="20" t="str">
+        <x:v>AND.route.unavailable.check.tablet.wav</x:v>
+      </x:c>
+      <x:c r="C248" s="20" t="str">
+        <x:v>Route is unavailable. Select or confirm the destination on the tablet.</x:v>
+      </x:c>
+      <x:c r="D248" s="20" t="str">
+        <x:v>Pilot or copilot</x:v>
+      </x:c>
+      <x:c r="E248" s="21" t="str">
+        <x:v>routeupdate records a missing or failed destination after its retry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="42" customHeight="1">
+      <x:c r="A249" s="19" t="str">
+        <x:v>L:ANDROUTECHANGED</x:v>
+      </x:c>
+      <x:c r="B249" s="20" t="str">
+        <x:v>AND.route.changed.check.tablet.wav</x:v>
+      </x:c>
+      <x:c r="C249" s="20" t="str">
+        <x:v>Destination changed. Check the revised route on the tablet.</x:v>
+      </x:c>
+      <x:c r="D249" s="20" t="str">
+        <x:v>Pilot or copilot</x:v>
+      </x:c>
+      <x:c r="E249" s="21" t="str">
+        <x:v>Hospital, pickup, or custom target changes and the route is recalculated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="42" customHeight="1">
+      <x:c r="A250" s="19" t="str">
+        <x:v>L:ANDDISPATCHCANCELLED</x:v>
+      </x:c>
+      <x:c r="B250" s="20" t="str">
+        <x:v>AND.dispatch.cancelled.await.tasking.wav</x:v>
+      </x:c>
+      <x:c r="C250" s="20" t="str">
+        <x:v>Dispatch cancelled. Follow the instructions on the tablet and await reassignment.</x:v>
+      </x:c>
+      <x:c r="D250" s="20" t="str">
+        <x:v>Dispatch</x:v>
+      </x:c>
+      <x:c r="E250" s="21" t="str">
+        <x:v>Cancellation criteria end the current dispatch; HEMS must not continue intervention.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="42" customHeight="1">
+      <x:c r="A251" s="19" t="str">
+        <x:v>L:ANDSTARTUPBLOCKED</x:v>
+      </x:c>
+      <x:c r="B251" s="20" t="str">
+        <x:v>AND.cockpit.engine.start.hold.wav</x:v>
+      </x:c>
+      <x:c r="C251" s="20" t="str">
+        <x:v>Hold engine start. Ground operations are still in progress.</x:v>
+      </x:c>
+      <x:c r="D251" s="20" t="str">
+        <x:v>Pilot or copilot</x:v>
+      </x:c>
+      <x:c r="E251" s="21" t="str">
+        <x:v>marshall_ground_ops_active or pisteur3_guidance_active blocks a first-pump start request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="42" customHeight="1">
+      <x:c r="A252" s="19" t="str">
+        <x:v>L:ANDMAINTENANCEHOLD</x:v>
+      </x:c>
+      <x:c r="B252" s="20" t="str">
+        <x:v>AND.technical.inspection.required.wav</x:v>
+      </x:c>
+      <x:c r="C252" s="20" t="str">
+        <x:v>Aircraft requires inspection. Do not depart until maintenance releases it.</x:v>
+      </x:c>
+      <x:c r="D252" s="20" t="str">
+        <x:v>Technician</x:v>
+      </x:c>
+      <x:c r="E252" s="21" t="str">
+        <x:v>A failure or hard landing requires inspection before the next release.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="42" customHeight="1">
+      <x:c r="A253" s="19" t="str">
+        <x:v>L:ANDMULTIPLEPATIENTS</x:v>
+      </x:c>
+      <x:c r="B253" s="20" t="str">
+        <x:v>AND.medical.additional.patients.on.scene.wav</x:v>
+      </x:c>
+      <x:c r="C253" s="20" t="str">
+        <x:v>Additional patients remain on scene. Await tasking before departure.</x:v>
+      </x:c>
+      <x:c r="D253" s="20" t="str">
+        <x:v>Crew chief</x:v>
+      </x:c>
+      <x:c r="E253" s="21" t="str">
+        <x:v>Patient 2 or 3 remains active, or secondary rescue begins.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="42" customHeight="1">
+      <x:c r="A254" s="22" t="str">
+        <x:v>L:ANDCREWRETURNING</x:v>
+      </x:c>
+      <x:c r="B254" s="23" t="str">
+        <x:v>AND.crew.returning.to.aircraft.wav</x:v>
+      </x:c>
+      <x:c r="C254" s="23" t="str">
+        <x:v>Ground crew is returning to the aircraft. Keep the landing area clear.</x:v>
+      </x:c>
+      <x:c r="D254" s="23" t="str">
+        <x:v>Crew chief</x:v>
+      </x:c>
+      <x:c r="E254" s="24" t="str">
+        <x:v>Post-visit, post-load, or post-hoist crew-return flow begins.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R497f1c4128384866"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add voice correction alternatives to AND catalog
</commit_message>
<xml_diff>
--- a/docs/AND_voice_messages.xlsx
+++ b/docs/AND_voice_messages.xlsx
@@ -147,7 +147,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +215,12 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -223,14 +229,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:E254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:E254"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:F254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F254"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="LVAR"/>
     <x:tableColumn id="2" name="nome file"/>
     <x:tableColumn id="3" name="testo del messaggio"/>
     <x:tableColumn id="4" name="ruolo"/>
     <x:tableColumn id="5" name="trigger (azione / tablet)"/>
+    <x:tableColumn id="6" name="correzioni proposte"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -245,6 +252,7 @@
     <x:col min="3" max="3" width="80" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="78" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="112" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -260,8 +268,11 @@
       <x:c r="D1" s="9" t="str">
         <x:v>ruolo</x:v>
       </x:c>
-      <x:c r="E1" s="10" t="str">
+      <x:c r="E1" s="9" t="str">
         <x:v>trigger (azione / tablet)</x:v>
+      </x:c>
+      <x:c r="F1" s="10" t="str">
+        <x:v>correzioni proposte</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
@@ -341,7 +352,7 @@
         <x:v>[Non-verbal new-message notification sound.]</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" ht="120" hidden="0" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>L:ANDHW1</x:v>
       </x:c>
@@ -351,8 +362,13 @@
       <x:c r="C9" s="12" t="str">
         <x:v>We are experiencing issues with the safety straps we cannot use rescue hoist sorry we are forced to land.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="F9" s="25" t="str">
+        <x:v>1) We have a problem with the safety straps. We cannot use the rescue hoist and must land.
+2) We have a problem with the safety straps. We can't use the rescue hoist and must land.
+3) Attention: we have a problem with the safety straps. We cannot use the rescue hoist and must land.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="120" hidden="0" customHeight="1">
       <x:c r="A10" s="17" t="str">
         <x:v>L:ANDHW2</x:v>
       </x:c>
@@ -362,8 +378,13 @@
       <x:c r="C10" s="12" t="str">
         <x:v>Hey crew there is an emergency message from dispatcher you have to read it it's unbelievable.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="F10" s="25" t="str">
+        <x:v>1) Crew, there is an emergency message from Dispatch. Please read it.
+2) Be advised: crew, there is an emergency message from Dispatch. Please read it.
+3) All crew, there is an emergency message from Dispatch. Please read it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="120" hidden="0" customHeight="1">
       <x:c r="A11" s="17" t="str">
         <x:v>L:ANDHW3</x:v>
       </x:c>
@@ -373,8 +394,13 @@
       <x:c r="C11" s="12" t="str">
         <x:v>Smoke and fire everywhere it seems a war movie scene out there.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="F11" s="25" t="str">
+        <x:v>1) Smoke and fire everywhere. It looks like a war zone out there.
+2) Be advised: smoke and fire everywhere. It looks like a war zone out there.
+3) Attention: smoke and fire everywhere. It looks like a war zone out there.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="120" hidden="0" customHeight="1">
       <x:c r="A12" s="17" t="str">
         <x:v>L:ANDHW4</x:v>
       </x:c>
@@ -384,8 +410,13 @@
       <x:c r="C12" s="12" t="str">
         <x:v>Damn engine fire crew we have an engine fire.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="F12" s="25" t="str">
+        <x:v>1) Crew, we have an engine fire.
+2) Be advised: crew, we have an engine fire.
+3) All crew, we have an engine fire.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" hidden="0" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>L:ANDHW5</x:v>
       </x:c>
@@ -395,8 +426,13 @@
       <x:c r="C13" s="12" t="str">
         <x:v>Copilot confirmed engine two fire.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="F13" s="25" t="str">
+        <x:v>1) Copilot confirms an engine two fire.
+2) Be advised: copilot confirms an engine two fire.
+3) Attention: copilot confirms an engine two fire.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" hidden="0" customHeight="1">
       <x:c r="A14" s="17" t="str">
         <x:v>L:ANDHW6</x:v>
       </x:c>
@@ -406,8 +442,13 @@
       <x:c r="C14" s="12" t="str">
         <x:v>Engine two confirmed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="F14" s="25" t="str">
+        <x:v>1) Engine two fire confirmed.
+2) Be advised: engine two fire confirmed.
+3) Attention: engine two fire confirmed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="120" hidden="0" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>L:ANDHW7</x:v>
       </x:c>
@@ -417,8 +458,13 @@
       <x:c r="C15" s="12" t="str">
         <x:v>Engine two fire. Push bottle one and hope it goes off; crew, prepare to evacuate the helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="F15" s="25" t="str">
+        <x:v>1) Engine two fire. Discharge bottle one; crew, prepare to evacuate.
+2) Be advised: engine two fire. Discharge bottle one; crew, prepare to evacuate.
+3) Attention: engine two fire. Discharge bottle one; crew, prepare to evacuate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="120" hidden="0" customHeight="1">
       <x:c r="A16" s="17" t="str">
         <x:v>L:ANDHW8</x:v>
       </x:c>
@@ -428,8 +474,13 @@
       <x:c r="C16" s="12" t="str">
         <x:v>Fire is extinguished however we have multiple failures i'm not sure we can take off again in this condition.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="F16" s="25" t="str">
+        <x:v>1) The fire is out, but we have multiple failures. I am not sure we can take off again.
+2) The fire is out, but we have multiple failures. I'm not sure we can take off again.
+3) Attention: the fire is out, but we have multiple failures. I am not sure we can take off again.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="120" hidden="0" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>L:ANDHW9</x:v>
       </x:c>
@@ -439,8 +490,13 @@
       <x:c r="C17" s="12" t="str">
         <x:v>What the hell is happening here.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="F17" s="25" t="str">
+        <x:v>1) What the hell is happening here.
+2) Be advised: what the hell is happening here.
+3) Attention: what the hell is happening here.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="120" hidden="0" customHeight="1">
       <x:c r="A18" s="17" t="str">
         <x:v>L:ANDHW10</x:v>
       </x:c>
@@ -450,8 +506,13 @@
       <x:c r="C18" s="12" t="str">
         <x:v>There is something bad happening in the area we have to be careful while completing tasks.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="F18" s="25" t="str">
+        <x:v>1) Something is wrong in the area. Remain alert while completing the mission.
+2) Be advised: something is wrong in the area. Remain alert while completing the mission.
+3) Attention: something is wrong in the area. Remain alert while completing the mission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="120" hidden="0" customHeight="1">
       <x:c r="A19" s="17" t="str">
         <x:v>L:ANDHW11</x:v>
       </x:c>
@@ -461,8 +522,13 @@
       <x:c r="C19" s="12" t="str">
         <x:v>Did you see them hey what hey guys did you see them is that happening to us they are coming here are they.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="F19" s="25" t="str">
+        <x:v>1) Did you see that? Guys, are they coming toward us?
+2) Can you confirm: did you see that? Guys, are they coming toward us?
+3) Please confirm: did you see that? Guys, are they coming toward us?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="120" hidden="0" customHeight="1">
       <x:c r="A20" s="17" t="str">
         <x:v>L:ANDHW12</x:v>
       </x:c>
@@ -472,8 +538,13 @@
       <x:c r="C20" s="12" t="str">
         <x:v>We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="F20" s="25" t="str">
+        <x:v>1) We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
+2) Be advised: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
+3) Attention: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="120" hidden="0" customHeight="1">
       <x:c r="A21" s="17" t="str">
         <x:v>L:ANDHW13</x:v>
       </x:c>
@@ -483,8 +554,13 @@
       <x:c r="C21" s="12" t="str">
         <x:v>Doc refers they have almost done we should wait for them to return.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="F21" s="25" t="str">
+        <x:v>1) The doctor says they are almost finished. We should wait for their return.
+2) Be advised: the doctor says they are almost finished. We should wait for their return.
+3) Attention: the doctor says they are almost finished. We should wait for their return.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="120" hidden="0" customHeight="1">
       <x:c r="A22" s="17" t="str">
         <x:v>L:ANDHW14</x:v>
       </x:c>
@@ -494,8 +570,13 @@
       <x:c r="C22" s="12" t="str">
         <x:v>Okay finished go away now go go go.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="F22" s="25" t="str">
+        <x:v>1) Okay, finished. Move away now; go, go, go.
+2) Be advised: okay, finished. Move away now; go, go, go.
+3) Attention: okay, finished. Move away now; go, go, go.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="120" hidden="0" customHeight="1">
       <x:c r="A23" s="17" t="str">
         <x:v>L:ANDHW15</x:v>
       </x:c>
@@ -505,8 +586,13 @@
       <x:c r="C23" s="12" t="str">
         <x:v>We're going to try and oh he i take off it will be difficult if needed be prepared for immediate evacuation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="F23" s="25" t="str">
+        <x:v>1) We are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
+2) We're going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
+3) Attention: we are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="120" hidden="0" customHeight="1">
       <x:c r="A24" s="17" t="str">
         <x:v>L:AND1</x:v>
       </x:c>
@@ -516,8 +602,13 @@
       <x:c r="C24" s="12" t="str">
         <x:v>Cabin preparation completed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="F24" s="25" t="str">
+        <x:v>1) Cabin preparation completed.
+2) Be advised: cabin preparation completed.
+3) Attention: cabin preparation completed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="120" hidden="0" customHeight="1">
       <x:c r="A25" s="17" t="str">
         <x:v>L:AND2</x:v>
       </x:c>
@@ -527,8 +618,13 @@
       <x:c r="C25" s="12" t="str">
         <x:v>Cabin preparation please wait.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="F25" s="25" t="str">
+        <x:v>1) Cabin preparation is in progress. Please wait.
+2) Be advised: cabin preparation is in progress. Please wait.
+3) Attention: cabin preparation is in progress. Please wait.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="120" hidden="0" customHeight="1">
       <x:c r="A26" s="17" t="str">
         <x:v>L:AND3</x:v>
       </x:c>
@@ -538,8 +634,13 @@
       <x:c r="C26" s="12" t="str">
         <x:v>Cabin secured ready to fly.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="F26" s="25" t="str">
+        <x:v>1) Cabin secured and ready for flight.
+2) Be advised: cabin secured and ready for flight.
+3) Attention: cabin secured and ready for flight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="120" hidden="0" customHeight="1">
       <x:c r="A27" s="17" t="str">
         <x:v>L:AND5</x:v>
       </x:c>
@@ -549,8 +650,13 @@
       <x:c r="C27" s="12" t="str">
         <x:v>Hoist one plus stretcher to helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="F27" s="25" t="str">
+        <x:v>1) Bring hoist one and the stretcher to the helicopter.
+2) Be advised: bring hoist one and the stretcher to the helicopter.
+3) Attention: bring hoist one and the stretcher to the helicopter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="120" hidden="0" customHeight="1">
       <x:c r="A28" s="17" t="str">
         <x:v>L:AND6</x:v>
       </x:c>
@@ -560,8 +666,13 @@
       <x:c r="C28" s="12" t="str">
         <x:v>Hoist one to helicopter; patient and doctor will go with ambulance.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="F28" s="25" t="str">
+        <x:v>1) Hoist one to the helicopter. The patient and doctor will travel by ambulance.
+2) Be advised: hoist one to the helicopter. The patient and doctor will travel by ambulance.
+3) Attention: hoist one to the helicopter. The patient and doctor will travel by ambulance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="120" hidden="0" customHeight="1">
       <x:c r="A29" s="17" t="str">
         <x:v>L:AND7</x:v>
       </x:c>
@@ -571,8 +682,13 @@
       <x:c r="C29" s="12" t="str">
         <x:v>Hoist two to helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="F29" s="25" t="str">
+        <x:v>1) Hoist two to helicopter.
+2) Be advised: hoist two to helicopter.
+3) Attention: hoist two to helicopter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="120" hidden="0" customHeight="1">
       <x:c r="A30" s="17" t="str">
         <x:v>L:AND8</x:v>
       </x:c>
@@ -582,8 +698,13 @@
       <x:c r="C30" s="12" t="str">
         <x:v>Hoist three to helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="F30" s="25" t="str">
+        <x:v>1) Hoist three to helicopter.
+2) Be advised: hoist three to helicopter.
+3) Attention: hoist three to helicopter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="120" hidden="0" customHeight="1">
       <x:c r="A31" s="17" t="str">
         <x:v>L:AND9</x:v>
       </x:c>
@@ -593,8 +714,13 @@
       <x:c r="C31" s="12" t="str">
         <x:v>Hoist boom extended.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="F31" s="25" t="str">
+        <x:v>1) Hoist boom extended.
+2) Be advised: hoist boom extended.
+3) Attention: hoist boom extended.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="120" hidden="0" customHeight="1">
       <x:c r="A32" s="17" t="str">
         <x:v>L:AND10</x:v>
       </x:c>
@@ -604,8 +730,13 @@
       <x:c r="C32" s="12" t="str">
         <x:v>Hoist is clear.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="F32" s="25" t="str">
+        <x:v>1) Hoist is clear.
+2) Be advised: hoist is clear.
+3) Attention: hoist is clear.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="120" hidden="0" customHeight="1">
       <x:c r="A33" s="17" t="str">
         <x:v>L:AND11</x:v>
       </x:c>
@@ -615,8 +746,13 @@
       <x:c r="C33" s="12" t="str">
         <x:v>Hoist is running down.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="F33" s="25" t="str">
+        <x:v>1) Hoist is running down.
+2) Be advised: hoist is running down.
+3) Attention: hoist is running down.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="120" hidden="0" customHeight="1">
       <x:c r="A34" s="17" t="str">
         <x:v>L:AND12</x:v>
       </x:c>
@@ -626,8 +762,13 @@
       <x:c r="C34" s="12" t="str">
         <x:v>Hoist is running up.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="F34" s="25" t="str">
+        <x:v>1) Hoist is running up.
+2) Be advised: hoist is running up.
+3) Attention: hoist is running up.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="120" hidden="0" customHeight="1">
       <x:c r="A35" s="17" t="str">
         <x:v>L:AND13</x:v>
       </x:c>
@@ -637,8 +778,13 @@
       <x:c r="C35" s="12" t="str">
         <x:v>Hoist his up boom extended patient and doctor are outside hook to hoist.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="F35" s="25" t="str">
+        <x:v>1) Hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
+2) Be advised: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
+3) Attention: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="120" hidden="0" customHeight="1">
       <x:c r="A36" s="17" t="str">
         <x:v>L:AND14</x:v>
       </x:c>
@@ -648,8 +794,13 @@
       <x:c r="C36" s="12" t="str">
         <x:v>Hoist his up personnel is strapped in.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="F36" s="25" t="str">
+        <x:v>1) Hoist is up; personnel are strapped in.
+2) Be advised: hoist is up; personnel are strapped in.
+3) Attention: hoist is up; personnel are strapped in.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="120" hidden="0" customHeight="1">
       <x:c r="A37" s="17" t="str">
         <x:v>L:AND15</x:v>
       </x:c>
@@ -659,8 +810,13 @@
       <x:c r="C37" s="12" t="str">
         <x:v>Hoist on ground personnel is getting hooked.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="F37" s="25" t="str">
+        <x:v>1) Hoist is on the ground. Personnel are being hooked on.
+2) Be advised: hoist is on the ground. Personnel are being hooked on.
+3) Attention: hoist is on the ground. Personnel are being hooked on.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="120" hidden="0" customHeight="1">
       <x:c r="A38" s="17" t="str">
         <x:v>L:AND16</x:v>
       </x:c>
@@ -670,8 +826,13 @@
       <x:c r="C38" s="12" t="str">
         <x:v>Hold position.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="F38" s="25" t="str">
+        <x:v>1) Hold position.
+2) Maintain position.
+3) Maintain your position.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="120" hidden="0" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>L:AND18</x:v>
       </x:c>
@@ -681,8 +842,13 @@
       <x:c r="C39" s="12" t="str">
         <x:v>Hook is in hoist boomers retracted you're free to leave hover.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="F39" s="25" t="str">
+        <x:v>1) Hook is in and boom retracted. You are clear to leave the hover.
+2) Hook is in and boom retracted. You're clear to leave the hover.
+3) Attention: hook is in and boom retracted. You are clear to leave the hover.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="120" hidden="0" customHeight="1">
       <x:c r="A40" s="17" t="str">
         <x:v>L:AND19</x:v>
       </x:c>
@@ -692,8 +858,13 @@
       <x:c r="C40" s="12" t="str">
         <x:v>Medical on ground and disconnected.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="F40" s="25" t="str">
+        <x:v>1) Medic is on the ground and disconnected.
+2) Be advised: medic is on the ground and disconnected.
+3) Attention: medic is on the ground and disconnected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="120" hidden="0" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>L:AND20</x:v>
       </x:c>
@@ -703,8 +874,13 @@
       <x:c r="C41" s="12" t="str">
         <x:v>Patient will go with ambulance.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="F41" s="25" t="str">
+        <x:v>1) The patient will travel by ambulance.
+2) Be advised: the patient will travel by ambulance.
+3) Attention: the patient will travel by ambulance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="120" hidden="0" customHeight="1">
       <x:c r="A42" s="17" t="str">
         <x:v>L:AND21</x:v>
       </x:c>
@@ -714,8 +890,13 @@
       <x:c r="C42" s="12" t="str">
         <x:v>Personnel on ground and disconnected.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="F42" s="25" t="str">
+        <x:v>1) Personnel are on the ground and disconnected.
+2) Be advised: personnel are on the ground and disconnected.
+3) Attention: personnel are on the ground and disconnected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="120" hidden="0" customHeight="1">
       <x:c r="A43" s="17" t="str">
         <x:v>L:AND22</x:v>
       </x:c>
@@ -725,8 +906,13 @@
       <x:c r="C43" s="12" t="str">
         <x:v>Position is good.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="F43" s="25" t="str">
+        <x:v>1) Position is good.
+2) Be advised: position is good.
+3) Attention: position is good.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="120" hidden="0" customHeight="1">
       <x:c r="A44" s="17" t="str">
         <x:v>L:AND23</x:v>
       </x:c>
@@ -736,8 +922,13 @@
       <x:c r="C44" s="12" t="str">
         <x:v>Hold on, hoisting preparation is in progress and almost completed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="F44" s="25" t="str">
+        <x:v>1) Hold on, hoisting preparation is in progress and almost completed.
+2) Be advised: hold on, hoisting preparation is in progress and almost completed.
+3) Attention: hold on, hoisting preparation is in progress and almost completed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="120" hidden="0" customHeight="1">
       <x:c r="A45" s="17" t="str">
         <x:v>L:AND24</x:v>
       </x:c>
@@ -747,8 +938,13 @@
       <x:c r="C45" s="12" t="str">
         <x:v>Set hover conditions.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="F45" s="25" t="str">
+        <x:v>1) Set hover conditions.
+2) Be advised: set hover conditions.
+3) Attention: set hover conditions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="120" hidden="0" customHeight="1">
       <x:c r="A46" s="17" t="str">
         <x:v>L:AND25</x:v>
       </x:c>
@@ -758,8 +954,13 @@
       <x:c r="C46" s="12" t="str">
         <x:v>That's one com check.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="F46" s="25" t="str">
+        <x:v>1) This is a communications check.
+2) Be advised: this is a communications check.
+3) Attention: this is a communications check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="120" hidden="0" customHeight="1">
       <x:c r="A47" s="17" t="str">
         <x:v>L:AND26</x:v>
       </x:c>
@@ -769,8 +970,13 @@
       <x:c r="C47" s="12" t="str">
         <x:v>Hoist wonder helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="F47" s="25" t="str">
+        <x:v>1) Hoist one to the helicopter.
+2) Be advised: hoist one to the helicopter.
+3) Attention: hoist one to the helicopter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="120" hidden="0" customHeight="1">
       <x:c r="A48" s="17" t="str">
         <x:v>L:AND32</x:v>
       </x:c>
@@ -780,8 +986,13 @@
       <x:c r="C48" s="12" t="str">
         <x:v>Ten.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="F48" s="25" t="str">
+        <x:v>1) Ten.
+2) Be advised: ten.
+3) Attention: ten.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="120" hidden="0" customHeight="1">
       <x:c r="A49" s="17" t="str">
         <x:v>L:AND33</x:v>
       </x:c>
@@ -791,8 +1002,13 @@
       <x:c r="C49" s="12" t="str">
         <x:v>Twenty.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="F49" s="25" t="str">
+        <x:v>1) Twenty.
+2) Be advised: twenty.
+3) Attention: twenty.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="120" hidden="0" customHeight="1">
       <x:c r="A50" s="17" t="str">
         <x:v>L:AND34</x:v>
       </x:c>
@@ -802,8 +1018,13 @@
       <x:c r="C50" s="12" t="str">
         <x:v>Fifty meters.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="F50" s="25" t="str">
+        <x:v>1) Fifty meters.
+2) Be advised: fifty meters.
+3) Attention: fifty meters.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="120" hidden="0" customHeight="1">
       <x:c r="A51" s="17" t="str">
         <x:v>L:AND37</x:v>
       </x:c>
@@ -813,8 +1034,13 @@
       <x:c r="C51" s="12" t="str">
         <x:v>Hey frank good morning.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="F51" s="25" t="str">
+        <x:v>1) Hey frank good morning.
+2) Be advised: hey frank good morning.
+3) Attention: hey frank good morning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="120" hidden="0" customHeight="1">
       <x:c r="A52" s="17" t="str">
         <x:v>L:AND38</x:v>
       </x:c>
@@ -824,8 +1050,13 @@
       <x:c r="C52" s="12" t="str">
         <x:v>Hi sarah how are you.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="F52" s="25" t="str">
+        <x:v>1) Hi sarah how are you.
+2) Be advised: hi sarah how are you.
+3) Attention: hi sarah how are you.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="120" hidden="0" customHeight="1">
       <x:c r="A53" s="17" t="str">
         <x:v>L:AND42</x:v>
       </x:c>
@@ -835,8 +1066,13 @@
       <x:c r="C53" s="12" t="str">
         <x:v>Stretcher is secure.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="F53" s="25" t="str">
+        <x:v>1) Stretcher is secure.
+2) Be advised: stretcher is secure.
+3) Attention: stretcher is secure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="120" hidden="0" customHeight="1">
       <x:c r="A54" s="17" t="str">
         <x:v>L:AND43</x:v>
       </x:c>
@@ -846,8 +1082,13 @@
       <x:c r="C54" s="12" t="str">
         <x:v>We are reasonably close said hover is appropriate.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="F54" s="25" t="str">
+        <x:v>1) We are close enough; set hover conditions.
+2) We're close enough; set hover conditions.
+3) Attention: we are close enough; set hover conditions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="120" hidden="0" customHeight="1">
       <x:c r="A55" s="17" t="str">
         <x:v>L:AND44</x:v>
       </x:c>
@@ -857,8 +1098,13 @@
       <x:c r="C55" s="12" t="str">
         <x:v>We are reasonably close.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="56" ht="15" hidden="0" customHeight="1">
+      <x:c r="F55" s="25" t="str">
+        <x:v>1) We are reasonably close.
+2) We're reasonably close.
+3) Attention: we are reasonably close.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="120" hidden="0" customHeight="1">
       <x:c r="A56" s="17" t="str">
         <x:v>L:AND45</x:v>
       </x:c>
@@ -868,8 +1114,13 @@
       <x:c r="C56" s="12" t="str">
         <x:v>We are too far.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="F56" s="25" t="str">
+        <x:v>1) We are too far.
+2) We're too far.
+3) Attention: we are too far.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="120" hidden="0" customHeight="1">
       <x:c r="A57" s="17" t="str">
         <x:v>L:AND46</x:v>
       </x:c>
@@ -879,8 +1130,13 @@
       <x:c r="C57" s="12" t="str">
         <x:v>Height is good.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="F57" s="25" t="str">
+        <x:v>1) Height is good.
+2) Be advised: height is good.
+3) Attention: height is good.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="120" hidden="0" customHeight="1">
       <x:c r="A58" s="17" t="str">
         <x:v>L:AND47</x:v>
       </x:c>
@@ -890,8 +1146,13 @@
       <x:c r="C58" s="12" t="str">
         <x:v>We are too high.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="F58" s="25" t="str">
+        <x:v>1) We are too high.
+2) We're too high.
+3) Attention: we are too high.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="120" hidden="0" customHeight="1">
       <x:c r="A59" s="17" t="str">
         <x:v>L:AND48</x:v>
       </x:c>
@@ -901,8 +1162,13 @@
       <x:c r="C59" s="12" t="str">
         <x:v>We are too low.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="F59" s="25" t="str">
+        <x:v>1) We are too low.
+2) We're too low.
+3) Attention: we are too low.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="120" hidden="0" customHeight="1">
       <x:c r="A60" s="17" t="str">
         <x:v>L:AND49</x:v>
       </x:c>
@@ -912,8 +1178,13 @@
       <x:c r="C60" s="12" t="str">
         <x:v>Doc and stretcher have been disconnected.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="F60" s="25" t="str">
+        <x:v>1) The doctor and stretcher are disconnected.
+2) Be advised: the doctor and stretcher are disconnected.
+3) Attention: the doctor and stretcher are disconnected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="120" hidden="0" customHeight="1">
       <x:c r="A61" s="17" t="str">
         <x:v>L:AND51</x:v>
       </x:c>
@@ -923,8 +1194,13 @@
       <x:c r="C61" s="12" t="str">
         <x:v>Doc is getting hooked.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="F61" s="25" t="str">
+        <x:v>1) Doc is getting hooked.
+2) Be advised: doc is getting hooked.
+3) Attention: doc is getting hooked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="120" hidden="0" customHeight="1">
       <x:c r="A62" s="17" t="str">
         <x:v>L:AND52</x:v>
       </x:c>
@@ -934,8 +1210,13 @@
       <x:c r="C62" s="12" t="str">
         <x:v>Hoist storm extended.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="F62" s="25" t="str">
+        <x:v>1) Hoist boom extended.
+2) Be advised: hoist boom extended.
+3) Attention: hoist boom extended.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="120" hidden="0" customHeight="1">
       <x:c r="A63" s="17" t="str">
         <x:v>L:AND54</x:v>
       </x:c>
@@ -945,8 +1226,13 @@
       <x:c r="C63" s="12" t="str">
         <x:v>Hoist retracted door closed cabin secured.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="F63" s="25" t="str">
+        <x:v>1) Hoist retracted, door closed, cabin secured.
+2) Be advised: hoist retracted, door closed, cabin secured.
+3) Attention: hoist retracted, door closed, cabin secured.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="120" hidden="0" customHeight="1">
       <x:c r="A64" s="17" t="str">
         <x:v>L:AND55</x:v>
       </x:c>
@@ -956,8 +1242,13 @@
       <x:c r="C64" s="12" t="str">
         <x:v>Opening door and preparing for hoist operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="F64" s="25" t="str">
+        <x:v>1) Opening door and preparing for hoist operation.
+2) Be advised: opening door and preparing for hoist operation.
+3) Attention: opening door and preparing for hoist operation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="120" hidden="0" customHeight="1">
       <x:c r="A65" s="17" t="str">
         <x:v>L:AND56</x:v>
       </x:c>
@@ -967,8 +1258,13 @@
       <x:c r="C65" s="12" t="str">
         <x:v>Operator has been disconnected.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="F65" s="25" t="str">
+        <x:v>1) Operator has been disconnected.
+2) Be advised: operator has been disconnected.
+3) Attention: operator has been disconnected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="120" hidden="0" customHeight="1">
       <x:c r="A66" s="17" t="str">
         <x:v>L:AND57</x:v>
       </x:c>
@@ -978,8 +1274,13 @@
       <x:c r="C66" s="12" t="str">
         <x:v>Operator is getting hooked.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="F66" s="25" t="str">
+        <x:v>1) Operator is getting hooked.
+2) Be advised: operator is getting hooked.
+3) Attention: operator is getting hooked.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="120" hidden="0" customHeight="1">
       <x:c r="A67" s="17" t="str">
         <x:v>L:AND59</x:v>
       </x:c>
@@ -988,6 +1289,11 @@
       </x:c>
       <x:c r="C67" s="12" t="str">
         <x:v>Crew boarded cabin ready to go.</x:v>
+      </x:c>
+      <x:c r="F67" s="25" t="str">
+        <x:v>1) Crew boarded, cabin ready to go.
+2) Be advised: crew boarded, cabin ready to go.
+3) Attention: crew boarded, cabin ready to go.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" hidden="0" customHeight="1">
@@ -1000,8 +1306,13 @@
       <x:c r="C68" s="12" t="str">
         <x:v>Due to impervious location of accident site we should evaluate to call and board expert heli-rescuers use the tablet to decide if we continue alone or if we have to pick kelly rescuers on board.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="F68" s="25" t="str">
+        <x:v>1) The accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
+2) Be advised: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
+3) Attention: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="120" hidden="0" customHeight="1">
       <x:c r="A69" s="17" t="str">
         <x:v>L:AND61</x:v>
       </x:c>
@@ -1010,6 +1321,11 @@
       </x:c>
       <x:c r="C69" s="12" t="str">
         <x:v>Okay heli rescuer secure the area and the casualty we are go for hosting down the other personnel.</x:v>
+      </x:c>
+      <x:c r="F69" s="25" t="str">
+        <x:v>1) The heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
+2) Be advised: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
+3) Attention: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="24" hidden="0" customHeight="1">
@@ -1022,8 +1338,13 @@
       <x:c r="C70" s="12" t="str">
         <x:v>The proposed meeting point seems far away from accident site i believe we should arrange another feasible meeting point.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="F70" s="25" t="str">
+        <x:v>1) The proposed meeting point is far from the accident site. We should arrange a more practical point.
+2) Be advised: the proposed meeting point is far from the accident site. We should arrange a more practical point.
+3) Attention: the proposed meeting point is far from the accident site. We should arrange a more practical point.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="120" hidden="0" customHeight="1">
       <x:c r="A71" s="17" t="str">
         <x:v>L:AND63</x:v>
       </x:c>
@@ -1033,8 +1354,13 @@
       <x:c r="C71" s="12" t="str">
         <x:v>We have to hoist three to ground heli rescuer will be first to secure the area.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="F71" s="25" t="str">
+        <x:v>1) We need to hoist three people to the ground. The heli-rescuer will secure the area first.
+2) Be advised: we need to hoist three people to the ground. The heli-rescuer will secure the area first.
+3) Attention: we need to hoist three people to the ground. The heli-rescuer will secure the area first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="120" hidden="0" customHeight="1">
       <x:c r="A72" s="17" t="str">
         <x:v>L:AND64</x:v>
       </x:c>
@@ -1044,8 +1370,13 @@
       <x:c r="C72" s="12" t="str">
         <x:v>We have to increase distance and hide until the rescue area is secure.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="F72" s="25" t="str">
+        <x:v>1) Increase distance and altitude until the rescue area is secure.
+2) Be advised: increase distance and altitude until the rescue area is secure.
+3) Attention: increase distance and altitude until the rescue area is secure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="120" hidden="0" customHeight="1">
       <x:c r="A73" s="17" t="str">
         <x:v>L:AND65</x:v>
       </x:c>
@@ -1055,8 +1386,13 @@
       <x:c r="C73" s="12" t="str">
         <x:v>Dark and patient will go with the ambulance to the design hospital we have to pick him at the hospital hello pat.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="F73" s="25" t="str">
+        <x:v>1) The doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
+2) Be advised: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
+3) Attention: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="120" hidden="0" customHeight="1">
       <x:c r="A74" s="17" t="str">
         <x:v>L:AND66</x:v>
       </x:c>
@@ -1066,8 +1402,13 @@
       <x:c r="C74" s="12" t="str">
         <x:v>Three o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="F74" s="25" t="str">
+        <x:v>1) Three o'clock.
+2) Be advised: three o'clock.
+3) Attention: three o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="120" hidden="0" customHeight="1">
       <x:c r="A75" s="17" t="str">
         <x:v>L:AND67</x:v>
       </x:c>
@@ -1077,8 +1418,13 @@
       <x:c r="C75" s="12" t="str">
         <x:v>Four o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="F75" s="25" t="str">
+        <x:v>1) Four o'clock.
+2) Be advised: four o'clock.
+3) Attention: four o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="120" hidden="0" customHeight="1">
       <x:c r="A76" s="17" t="str">
         <x:v>L:AND68</x:v>
       </x:c>
@@ -1088,8 +1434,13 @@
       <x:c r="C76" s="12" t="str">
         <x:v>Five o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="F76" s="25" t="str">
+        <x:v>1) Five o'clock.
+2) Be advised: five o'clock.
+3) Attention: five o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="120" hidden="0" customHeight="1">
       <x:c r="A77" s="17" t="str">
         <x:v>L:AND69</x:v>
       </x:c>
@@ -1099,8 +1450,13 @@
       <x:c r="C77" s="12" t="str">
         <x:v>Six o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="F77" s="25" t="str">
+        <x:v>1) Six o'clock.
+2) Be advised: six o'clock.
+3) Attention: six o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="120" hidden="0" customHeight="1">
       <x:c r="A78" s="17" t="str">
         <x:v>L:AND70</x:v>
       </x:c>
@@ -1110,8 +1466,13 @@
       <x:c r="C78" s="12" t="str">
         <x:v>Seven o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="F78" s="25" t="str">
+        <x:v>1) Seven o'clock.
+2) Be advised: seven o'clock.
+3) Attention: seven o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="120" hidden="0" customHeight="1">
       <x:c r="A79" s="17" t="str">
         <x:v>L:AND71</x:v>
       </x:c>
@@ -1121,8 +1482,13 @@
       <x:c r="C79" s="12" t="str">
         <x:v>Eight o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="F79" s="25" t="str">
+        <x:v>1) Eight o'clock.
+2) Be advised: eight o'clock.
+3) Attention: eight o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="120" hidden="0" customHeight="1">
       <x:c r="A80" s="17" t="str">
         <x:v>L:AND72</x:v>
       </x:c>
@@ -1132,8 +1498,13 @@
       <x:c r="C80" s="12" t="str">
         <x:v>Nine o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="F80" s="25" t="str">
+        <x:v>1) Nine o'clock.
+2) Be advised: nine o'clock.
+3) Attention: nine o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="120" hidden="0" customHeight="1">
       <x:c r="A81" s="17" t="str">
         <x:v>L:AND73</x:v>
       </x:c>
@@ -1143,8 +1514,13 @@
       <x:c r="C81" s="12" t="str">
         <x:v>Ten o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="F81" s="25" t="str">
+        <x:v>1) Ten o'clock.
+2) Be advised: ten o'clock.
+3) Attention: ten o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="120" hidden="0" customHeight="1">
       <x:c r="A82" s="17" t="str">
         <x:v>L:AND74</x:v>
       </x:c>
@@ -1154,8 +1530,13 @@
       <x:c r="C82" s="12" t="str">
         <x:v>Eleven o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="F82" s="25" t="str">
+        <x:v>1) Eleven o'clock.
+2) Be advised: eleven o'clock.
+3) Attention: eleven o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="120" hidden="0" customHeight="1">
       <x:c r="A83" s="17" t="str">
         <x:v>L:AND75</x:v>
       </x:c>
@@ -1165,8 +1546,13 @@
       <x:c r="C83" s="12" t="str">
         <x:v>Twelve o'clock.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="F83" s="25" t="str">
+        <x:v>1) Twelve o'clock.
+2) Be advised: twelve o'clock.
+3) Attention: twelve o'clock.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="120" hidden="0" customHeight="1">
       <x:c r="A84" s="17" t="str">
         <x:v>L:AND76</x:v>
       </x:c>
@@ -1176,8 +1562,13 @@
       <x:c r="C84" s="12" t="str">
         <x:v>Or on the way to the accident site.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="F84" s="25" t="str">
+        <x:v>1) We are on the way to the accident site.
+2) We're on the way to the accident site.
+3) Attention: we are on the way to the accident site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="120" hidden="0" customHeight="1">
       <x:c r="A85" s="17" t="str">
         <x:v>L:AND77</x:v>
       </x:c>
@@ -1187,8 +1578,13 @@
       <x:c r="C85" s="12" t="str">
         <x:v>Check on tablet.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="86" ht="15" hidden="0" customHeight="1">
+      <x:c r="F85" s="25" t="str">
+        <x:v>1) Check the tablet.
+2) Review the tablet.
+3) Please review the tablet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="120" hidden="0" customHeight="1">
       <x:c r="A86" s="17" t="str">
         <x:v>L:AND78</x:v>
       </x:c>
@@ -1198,8 +1594,13 @@
       <x:c r="C86" s="12" t="str">
         <x:v>I believe we found something.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="87" ht="15" hidden="0" customHeight="1">
+      <x:c r="F86" s="25" t="str">
+        <x:v>1) I believe we found something.
+2) Be advised: i believe we found something.
+3) Attention: i believe we found something.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="120" hidden="0" customHeight="1">
       <x:c r="A87" s="17" t="str">
         <x:v>L:AND79</x:v>
       </x:c>
@@ -1209,8 +1610,13 @@
       <x:c r="C87" s="12" t="str">
         <x:v>It's in front of us.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="88" ht="15" hidden="0" customHeight="1">
+      <x:c r="F87" s="25" t="str">
+        <x:v>1) It's in front of us.
+2) Be advised: it's in front of us.
+3) Attention: it's in front of us.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="120" hidden="0" customHeight="1">
       <x:c r="A88" s="17" t="str">
         <x:v>L:AND80</x:v>
       </x:c>
@@ -1220,8 +1626,13 @@
       <x:c r="C88" s="12" t="str">
         <x:v>Yes confirmed we found our target.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="89" ht="15" hidden="0" customHeight="1">
+      <x:c r="F88" s="25" t="str">
+        <x:v>1) Confirmed. We found the target.
+2) Be advised: confirmed. We found the target.
+3) Attention: confirmed. We found the target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="120" hidden="0" customHeight="1">
       <x:c r="A89" s="17" t="str">
         <x:v>L:AND81</x:v>
       </x:c>
@@ -1231,8 +1642,13 @@
       <x:c r="C89" s="12" t="str">
         <x:v>Helicopter clear ready to fly.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="90" ht="15" hidden="0" customHeight="1">
+      <x:c r="F89" s="25" t="str">
+        <x:v>1) Helicopter clear and ready for flight.
+2) Be advised: helicopter clear and ready for flight.
+3) Attention: helicopter clear and ready for flight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="120" hidden="0" customHeight="1">
       <x:c r="A90" s="17" t="str">
         <x:v>L:CPLAND1</x:v>
       </x:c>
@@ -1242,8 +1658,13 @@
       <x:c r="C90" s="12" t="str">
         <x:v>All engines started successfully.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="91" ht="15" hidden="0" customHeight="1">
+      <x:c r="F90" s="25" t="str">
+        <x:v>1) Both engines started successfully.
+2) Be advised: both engines started successfully.
+3) Attention: both engines started successfully.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="120" hidden="0" customHeight="1">
       <x:c r="A91" s="17" t="str">
         <x:v>L:CPLAND2</x:v>
       </x:c>
@@ -1253,8 +1674,13 @@
       <x:c r="C91" s="12" t="str">
         <x:v>Okay all good.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="92" ht="15" hidden="0" customHeight="1">
+      <x:c r="F91" s="25" t="str">
+        <x:v>1) Okay, all good.
+2) Be advised: okay, all good.
+3) Attention: okay, all good.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="120" hidden="0" customHeight="1">
       <x:c r="A92" s="17" t="str">
         <x:v>L:CPLAND3</x:v>
       </x:c>
@@ -1264,8 +1690,13 @@
       <x:c r="C92" s="12" t="str">
         <x:v>Area clear ready to start engine one.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="93" ht="15" hidden="0" customHeight="1">
+      <x:c r="F92" s="25" t="str">
+        <x:v>1) Area clear. Ready to start engine one.
+2) Be advised: area clear. Ready to start engine one.
+3) Attention: area clear. Ready to start engine one.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="120" hidden="0" customHeight="1">
       <x:c r="A93" s="17" t="str">
         <x:v>L:CPLAND4</x:v>
       </x:c>
@@ -1275,8 +1706,13 @@
       <x:c r="C93" s="12" t="str">
         <x:v>Area clear ready to start engine two.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="94" ht="15" hidden="0" customHeight="1">
+      <x:c r="F93" s="25" t="str">
+        <x:v>1) Area clear. Ready to start engine two.
+2) Be advised: area clear. Ready to start engine two.
+3) Attention: area clear. Ready to start engine two.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="120" hidden="0" customHeight="1">
       <x:c r="A94" s="17" t="str">
         <x:v>L:CPLAND5</x:v>
       </x:c>
@@ -1286,8 +1722,13 @@
       <x:c r="C94" s="12" t="str">
         <x:v>Co pilot hh oh comm check.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="95" ht="15" hidden="0" customHeight="1">
+      <x:c r="F94" s="25" t="str">
+        <x:v>1) Copilot here, communications check.
+2) Be advised: copilot here, communications check.
+3) Attention: copilot here, communications check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="120" hidden="0" customHeight="1">
       <x:c r="A95" s="17" t="str">
         <x:v>L:CPLAND6</x:v>
       </x:c>
@@ -1297,8 +1738,13 @@
       <x:c r="C95" s="12" t="str">
         <x:v>Engine clear.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="96" ht="15" hidden="0" customHeight="1">
+      <x:c r="F95" s="25" t="str">
+        <x:v>1) Engine area clear.
+2) Be advised: engine area clear.
+3) Attention: engine area clear.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="120" hidden="0" customHeight="1">
       <x:c r="A96" s="17" t="str">
         <x:v>L:CPLAND7</x:v>
       </x:c>
@@ -1308,8 +1754,13 @@
       <x:c r="C96" s="12" t="str">
         <x:v>Fire we have an engine fire stop engine.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="97" ht="15" hidden="0" customHeight="1">
+      <x:c r="F96" s="25" t="str">
+        <x:v>1) Engine fire. Stop the engine.
+2) Be advised: engine fire. Stop the engine.
+3) Attention: engine fire. Stop the engine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="120" hidden="0" customHeight="1">
       <x:c r="A97" s="17" t="str">
         <x:v>L:CPLAND8</x:v>
       </x:c>
@@ -1319,8 +1770,13 @@
       <x:c r="C97" s="12" t="str">
         <x:v>Engine started successfully moving to other engine.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="98" ht="15" hidden="0" customHeight="1">
+      <x:c r="F97" s="25" t="str">
+        <x:v>1) Engine started successfully. Moving to the other engine.
+2) Be advised: engine started successfully. Moving to the other engine.
+3) Attention: engine started successfully. Moving to the other engine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="120" hidden="0" customHeight="1">
       <x:c r="A98" s="17" t="str">
         <x:v>L:CPLAND9</x:v>
       </x:c>
@@ -1330,8 +1786,13 @@
       <x:c r="C98" s="12" t="str">
         <x:v>Damn we have a failure.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="99" ht="15" hidden="0" customHeight="1">
+      <x:c r="F98" s="25" t="str">
+        <x:v>1) Damn we have a failure.
+2) Be advised: damn we have a failure.
+3) Attention: damn we have a failure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="120" hidden="0" customHeight="1">
       <x:c r="A99" s="17" t="str">
         <x:v>L:CPLAND10</x:v>
       </x:c>
@@ -1341,8 +1802,13 @@
       <x:c r="C99" s="12" t="str">
         <x:v>Hold on performing leak checks.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="100" ht="15" hidden="0" customHeight="1">
+      <x:c r="F99" s="25" t="str">
+        <x:v>1) Hold on. Performing leak checks.
+2) Be advised: hold on. Performing leak checks.
+3) Attention: hold on. Performing leak checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="120" hidden="0" customHeight="1">
       <x:c r="A100" s="17" t="str">
         <x:v>L:CPLAND11</x:v>
       </x:c>
@@ -1352,8 +1818,13 @@
       <x:c r="C100" s="12" t="str">
         <x:v>Rear crew prepare for ground operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="101" ht="15" hidden="0" customHeight="1">
+      <x:c r="F100" s="25" t="str">
+        <x:v>1) Rear crew, prepare for ground operations.
+2) Be advised: rear crew, prepare for ground operations.
+3) Attention: rear crew, prepare for ground operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="120" hidden="0" customHeight="1">
       <x:c r="A101" s="17" t="str">
         <x:v>L:CPLAND12</x:v>
       </x:c>
@@ -1363,8 +1834,13 @@
       <x:c r="C101" s="12" t="str">
         <x:v>Rear crew prepare for hoist operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="102" ht="15" hidden="0" customHeight="1">
+      <x:c r="F101" s="25" t="str">
+        <x:v>1) Rear crew, prepare for hoist operations.
+2) Be advised: rear crew, prepare for hoist operations.
+3) Attention: rear crew, prepare for hoist operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="120" hidden="0" customHeight="1">
       <x:c r="A102" s="17" t="str">
         <x:v>L:CPLAND13</x:v>
       </x:c>
@@ -1374,8 +1850,13 @@
       <x:c r="C102" s="12" t="str">
         <x:v>Preparing for engine starting sequence one too.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="103" ht="15" hidden="0" customHeight="1">
+      <x:c r="F102" s="25" t="str">
+        <x:v>1) Preparing for engine-start sequence one, then two.
+2) Be advised: preparing for engine-start sequence one, then two.
+3) Attention: preparing for engine-start sequence one, then two.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="120" hidden="0" customHeight="1">
       <x:c r="A103" s="17" t="str">
         <x:v>L:CPLAND14</x:v>
       </x:c>
@@ -1385,8 +1866,13 @@
       <x:c r="C103" s="12" t="str">
         <x:v>Preparing for engine starting sequence to one.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="104" ht="15" hidden="0" customHeight="1">
+      <x:c r="F103" s="25" t="str">
+        <x:v>1) Preparing for engine-start sequence two, then one.
+2) Be advised: preparing for engine-start sequence two, then one.
+3) Attention: preparing for engine-start sequence two, then one.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="120" hidden="0" customHeight="1">
       <x:c r="A104" s="17" t="str">
         <x:v>L:CPLAND15</x:v>
       </x:c>
@@ -1396,8 +1882,13 @@
       <x:c r="C104" s="12" t="str">
         <x:v>Helicopter in position rear crew clear to start operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="105" ht="15" hidden="0" customHeight="1">
+      <x:c r="F104" s="25" t="str">
+        <x:v>1) Helicopter in position. Rear crew, clear to start operations.
+2) Be advised: helicopter in position. Rear crew, clear to start operations.
+3) Attention: helicopter in position. Rear crew, clear to start operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="120" hidden="0" customHeight="1">
       <x:c r="A105" s="17" t="str">
         <x:v>L:CPLAND16</x:v>
       </x:c>
@@ -1407,8 +1898,13 @@
       <x:c r="C105" s="12" t="str">
         <x:v>Rear crew we are approaching the landing site.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="106" ht="15" hidden="0" customHeight="1">
+      <x:c r="F105" s="25" t="str">
+        <x:v>1) Rear crew, we are approaching the landing site.
+2) Be advised: rear crew, we are approaching the landing site.
+3) Attention: rear crew, we are approaching the landing site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="120" hidden="0" customHeight="1">
       <x:c r="A106" s="17" t="str">
         <x:v>L:CPLAND17</x:v>
       </x:c>
@@ -1418,8 +1914,13 @@
       <x:c r="C106" s="12" t="str">
         <x:v>Site is not safe for us waiting for clearance.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="107" ht="15" hidden="0" customHeight="1">
+      <x:c r="F106" s="25" t="str">
+        <x:v>1) The site is not safe. Waiting for clearance.
+2) Be advised: the site is not safe. Waiting for clearance.
+3) Attention: the site is not safe. Waiting for clearance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="120" hidden="0" customHeight="1">
       <x:c r="A107" s="17" t="str">
         <x:v>L:CPLAND18</x:v>
       </x:c>
@@ -1429,8 +1930,13 @@
       <x:c r="C107" s="12" t="str">
         <x:v>Site is safer operations we can proceed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="108" ht="15" hidden="0" customHeight="1">
+      <x:c r="F107" s="25" t="str">
+        <x:v>1) The site is safe. Operations may proceed.
+2) Be advised: the site is safe. Operations may proceed.
+3) Attention: the site is safe. Operations may proceed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="120" hidden="0" customHeight="1">
       <x:c r="A108" s="17" t="str">
         <x:v>L:CPLAND19</x:v>
       </x:c>
@@ -1440,8 +1946,13 @@
       <x:c r="C108" s="12" t="str">
         <x:v>Rear crew prepare for skid lending operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="109" ht="15" hidden="0" customHeight="1">
+      <x:c r="F108" s="25" t="str">
+        <x:v>1) Rear crew, prepare for skid landing operations.
+2) Be advised: rear crew, prepare for skid landing operations.
+3) Attention: rear crew, prepare for skid landing operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="120" hidden="0" customHeight="1">
       <x:c r="A109" s="17" t="str">
         <x:v>L:CPLAND20</x:v>
       </x:c>
@@ -1451,8 +1962,13 @@
       <x:c r="C109" s="12" t="str">
         <x:v>Ambulance is arriving.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="110" ht="15" hidden="0" customHeight="1">
+      <x:c r="F109" s="25" t="str">
+        <x:v>1) Ambulance is arriving.
+2) Be advised: ambulance is arriving.
+3) Attention: ambulance is arriving.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="120" hidden="0" customHeight="1">
       <x:c r="A110" s="17" t="str">
         <x:v>L:CPLAND21</x:v>
       </x:c>
@@ -1462,8 +1978,13 @@
       <x:c r="C110" s="12" t="str">
         <x:v>Ambulance is still far away.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="111" ht="15" hidden="0" customHeight="1">
+      <x:c r="F110" s="25" t="str">
+        <x:v>1) Ambulance is still far away.
+2) Be advised: ambulance is still far away.
+3) Attention: ambulance is still far away.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="120" hidden="0" customHeight="1">
       <x:c r="A111" s="17" t="str">
         <x:v>L:CPLAND22</x:v>
       </x:c>
@@ -1473,8 +1994,13 @@
       <x:c r="C111" s="12" t="str">
         <x:v>Crew prepare for operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="112" ht="15" hidden="0" customHeight="1">
+      <x:c r="F111" s="25" t="str">
+        <x:v>1) Crew, prepare for operations.
+2) Be advised: crew, prepare for operations.
+3) All crew, prepare for operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="120" hidden="0" customHeight="1">
       <x:c r="A112" s="17" t="str">
         <x:v>L:CPLAND23</x:v>
       </x:c>
@@ -1484,8 +2010,13 @@
       <x:c r="C112" s="12" t="str">
         <x:v>Good morning frank.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="113" ht="15" hidden="0" customHeight="1">
+      <x:c r="F112" s="25" t="str">
+        <x:v>1) Good morning frank.
+2) Be advised: good morning frank.
+3) Attention: good morning frank.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="120" hidden="0" customHeight="1">
       <x:c r="A113" s="17" t="str">
         <x:v>L:CPLAND24</x:v>
       </x:c>
@@ -1495,8 +2026,13 @@
       <x:c r="C113" s="12" t="str">
         <x:v>Destination insight medical crew is ready on landing spot.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="114" ht="15" hidden="0" customHeight="1">
+      <x:c r="F113" s="25" t="str">
+        <x:v>1) Landing site in sight. Medical crew is ready at the landing area.
+2) Be advised: landing site in sight. Medical crew is ready at the landing area.
+3) Attention: landing site in sight. Medical crew is ready at the landing area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="120" hidden="0" customHeight="1">
       <x:c r="A114" s="17" t="str">
         <x:v>L:CPLAND25</x:v>
       </x:c>
@@ -1505,6 +2041,11 @@
       </x:c>
       <x:c r="C114" s="12" t="str">
         <x:v>We have to stop engines and switch off the helicopter.</x:v>
+      </x:c>
+      <x:c r="F114" s="25" t="str">
+        <x:v>1) We have to stop the engines and shut down the helicopter.
+2) Be advised: we have to stop the engines and shut down the helicopter.
+3) Attention: we have to stop the engines and shut down the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="24" hidden="0" customHeight="1">
@@ -1517,8 +2058,13 @@
       <x:c r="C115" s="12" t="str">
         <x:v>The crew i received a call from doc due to patient conditions the ambulance arrived to an alternate hospital doc is waiting us their check location on map.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="116" ht="15" hidden="0" customHeight="1">
+      <x:c r="F115" s="25" t="str">
+        <x:v>1) Crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
+2) Be advised: crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
+3) All crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="116" ht="120" hidden="0" customHeight="1">
       <x:c r="A116" s="17" t="str">
         <x:v>L:CPLAND27</x:v>
       </x:c>
@@ -1528,8 +2074,13 @@
       <x:c r="C116" s="12" t="str">
         <x:v>We are above maximum hoist out speed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="117" ht="15" hidden="0" customHeight="1">
+      <x:c r="F116" s="25" t="str">
+        <x:v>1) We are above maximum hoist-out speed.
+2) We're above maximum hoist-out speed.
+3) Attention: we are above maximum hoist-out speed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="117" ht="120" hidden="0" customHeight="1">
       <x:c r="A117" s="17" t="str">
         <x:v>L:CPLAND28</x:v>
       </x:c>
@@ -1539,8 +2090,13 @@
       <x:c r="C117" s="12" t="str">
         <x:v>Oh acceleration is over the hoist limit.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="118" ht="15" hidden="0" customHeight="1">
+      <x:c r="F117" s="25" t="str">
+        <x:v>1) Acceleration is above the hoist limit.
+2) Be advised: acceleration is above the hoist limit.
+3) Attention: acceleration is above the hoist limit.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="118" ht="120" hidden="0" customHeight="1">
       <x:c r="A118" s="17" t="str">
         <x:v>L:CPLAND29</x:v>
       </x:c>
@@ -1550,8 +2106,13 @@
       <x:c r="C118" s="12" t="str">
         <x:v>Bank angle is too high people on hoist will have troubles if we continue.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="119" ht="15" hidden="0" customHeight="1">
+      <x:c r="F118" s="25" t="str">
+        <x:v>1) Bank angle is too high. Continuing would endanger the patient and hoist operator.
+2) Be advised: bank angle is too high. Continuing would endanger the patient and hoist operator.
+3) Attention: bank angle is too high. Continuing would endanger the patient and hoist operator.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119" ht="120" hidden="0" customHeight="1">
       <x:c r="A119" s="17" t="str">
         <x:v>L:CPLAND30</x:v>
       </x:c>
@@ -1561,8 +2122,13 @@
       <x:c r="C119" s="12" t="str">
         <x:v>Keep bank angled within limits.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="120" ht="15" hidden="0" customHeight="1">
+      <x:c r="F119" s="25" t="str">
+        <x:v>1) Keep the bank angle within limits.
+2) Be advised: keep the bank angle within limits.
+3) Attention: keep the bank angle within limits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="120" hidden="0" customHeight="1">
       <x:c r="A120" s="17" t="str">
         <x:v>L:CPLAND31</x:v>
       </x:c>
@@ -1572,8 +2138,13 @@
       <x:c r="C120" s="12" t="str">
         <x:v>We are too fast sir we risk our patient and operator life moreover we are damaging the helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="121" ht="15" hidden="0" customHeight="1">
+      <x:c r="F120" s="25" t="str">
+        <x:v>1) We are too fast. We risk the patient, the operator, and the helicopter.
+2) We're too fast. We risk the patient, the operator, and the helicopter.
+3) Attention: we are too fast. We risk the patient, the operator, and the helicopter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121" ht="120" hidden="0" customHeight="1">
       <x:c r="A121" s="17" t="str">
         <x:v>L:CPLAND32</x:v>
       </x:c>
@@ -1583,8 +2154,13 @@
       <x:c r="C121" s="12" t="str">
         <x:v>Fuck sir we have to abort mission now.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="122" ht="15" hidden="0" customHeight="1">
+      <x:c r="F121" s="25" t="str">
+        <x:v>1) We have to abort the mission now.
+2) Be advised: we have to abort the mission now.
+3) Attention: we have to abort the mission now.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122" ht="120" hidden="0" customHeight="1">
       <x:c r="A122" s="17" t="str">
         <x:v>L:CPLAND33</x:v>
       </x:c>
@@ -1594,8 +2170,13 @@
       <x:c r="C122" s="12" t="str">
         <x:v>What the fuck we lost patient and doc what are you doing.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="123" ht="15" hidden="0" customHeight="1">
+      <x:c r="F122" s="25" t="str">
+        <x:v>1) We lost the doctor and patient. What are you doing?
+2) Can you confirm: we lost the doctor and patient. What are you doing?
+3) Please confirm: we lost the doctor and patient. What are you doing?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123" ht="120" hidden="0" customHeight="1">
       <x:c r="A123" s="17" t="str">
         <x:v>L:CPLAND36</x:v>
       </x:c>
@@ -1604,6 +2185,11 @@
       </x:c>
       <x:c r="C123" s="12" t="str">
         <x:v>Ah are we doing acrobatic maneuvers with a patient on board are you serious.</x:v>
+      </x:c>
+      <x:c r="F123" s="25" t="str">
+        <x:v>1) Are we doing aerobatics with a patient on board?
+2) Can you confirm: are we doing aerobatics with a patient on board?
+3) Please confirm: are we doing aerobatics with a patient on board?</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="24" hidden="0" customHeight="1">
@@ -1616,6 +2202,11 @@
       <x:c r="C124" s="12" t="str">
         <x:v>Doc refers the ground operations are almost done we can either go back and have or as soon as possible or stay here and proceed with ground operation.</x:v>
       </x:c>
+      <x:c r="F124" s="25" t="str">
+        <x:v>1) The doctor says ground operations are almost complete. We can return to base or wait to proceed.
+2) Be advised: the doctor says ground operations are almost complete. We can return to base or wait to proceed.
+3) Attention: the doctor says ground operations are almost complete. We can return to base or wait to proceed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="125" ht="24" hidden="0" customHeight="1">
       <x:c r="A125" s="17" t="str">
@@ -1627,8 +2218,13 @@
       <x:c r="C125" s="12" t="str">
         <x:v>Round operations will take time we can leave hover and find a safe landing spot we will be advised when operations are done.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="126" ht="15" hidden="0" customHeight="1">
+      <x:c r="F125" s="25" t="str">
+        <x:v>1) Ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
+2) Be advised: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
+3) Attention: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="120" hidden="0" customHeight="1">
       <x:c r="A126" s="17" t="str">
         <x:v>L:CPLAND39</x:v>
       </x:c>
@@ -1638,8 +2234,13 @@
       <x:c r="C126" s="12" t="str">
         <x:v>Ouch it was hard landing this time sarah won't be happy.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="127" ht="15" hidden="0" customHeight="1">
+      <x:c r="F126" s="25" t="str">
+        <x:v>1) That was a hard landing. Sarah will not be happy.
+2) Be advised: that was a hard landing. Sarah will not be happy.
+3) Attention: that was a hard landing. Sarah will not be happy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127" ht="120" hidden="0" customHeight="1">
       <x:c r="A127" s="17" t="str">
         <x:v>L:CPLAND40</x:v>
       </x:c>
@@ -1649,8 +2250,13 @@
       <x:c r="C127" s="12" t="str">
         <x:v>Hey it was a hard touch.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="128" ht="15" hidden="0" customHeight="1">
+      <x:c r="F127" s="25" t="str">
+        <x:v>1) That was a hard touch.
+2) Be advised: that was a hard touch.
+3) Attention: that was a hard touch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="128" ht="120" hidden="0" customHeight="1">
       <x:c r="A128" s="17" t="str">
         <x:v>L:CPLAND41</x:v>
       </x:c>
@@ -1660,8 +2266,13 @@
       <x:c r="C128" s="12" t="str">
         <x:v>Wow nice touch captain.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="129" ht="15" hidden="0" customHeight="1">
+      <x:c r="F128" s="25" t="str">
+        <x:v>1) Wow nice touch captain.
+2) Be advised: wow nice touch captain.
+3) Attention: wow nice touch captain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129" ht="120" hidden="0" customHeight="1">
       <x:c r="A129" s="17" t="str">
         <x:v>L:CPLAND42</x:v>
       </x:c>
@@ -1671,8 +2282,13 @@
       <x:c r="C129" s="12" t="str">
         <x:v>VNE.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="130" ht="15" hidden="0" customHeight="1">
+      <x:c r="F129" s="25" t="str">
+        <x:v>1) VNE.
+2) Be advised: vNE.
+3) Attention: vNE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="130" ht="120" hidden="0" customHeight="1">
       <x:c r="A130" s="17" t="str">
         <x:v>L:CPLAND43</x:v>
       </x:c>
@@ -1682,8 +2298,13 @@
       <x:c r="C130" s="12" t="str">
         <x:v>VTOSS.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="131" ht="15" hidden="0" customHeight="1">
+      <x:c r="F130" s="25" t="str">
+        <x:v>1) VTOSS.
+2) Be advised: vTOSS.
+3) Attention: vTOSS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131" ht="120" hidden="0" customHeight="1">
       <x:c r="A131" s="17" t="str">
         <x:v>L:CPLAND44</x:v>
       </x:c>
@@ -1693,8 +2314,13 @@
       <x:c r="C131" s="12" t="str">
         <x:v>Vy.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="132" ht="15" hidden="0" customHeight="1">
+      <x:c r="F131" s="25" t="str">
+        <x:v>1) Vy.
+2) Be advised: vy.
+3) Attention: vy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132" ht="120" hidden="0" customHeight="1">
       <x:c r="A132" s="17" t="str">
         <x:v>L:CPLAND45</x:v>
       </x:c>
@@ -1704,8 +2330,13 @@
       <x:c r="C132" s="12" t="str">
         <x:v>The a what we crashed are you all okay.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="133" ht="15" hidden="0" customHeight="1">
+      <x:c r="F132" s="25" t="str">
+        <x:v>1) We crashed. Is everyone okay?
+2) Can you confirm: we crashed. Is everyone okay?
+3) Please confirm: we crashed. Is everyone okay?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="120" hidden="0" customHeight="1">
       <x:c r="A133" s="17" t="str">
         <x:v>L:CPLAND46</x:v>
       </x:c>
@@ -1714,6 +2345,11 @@
       </x:c>
       <x:c r="C133" s="12" t="str">
         <x:v>Hey hey captain that's not and aerobatic helicopter please keep calm.</x:v>
+      </x:c>
+      <x:c r="F133" s="25" t="str">
+        <x:v>1) Captain, this is not an aerobatic helicopter. Please keep it calm.
+2) Be advised: captain, this is not an aerobatic helicopter. Please keep it calm.
+3) Attention: captain, this is not an aerobatic helicopter. Please keep it calm.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="36" hidden="0" customHeight="1">
@@ -1726,6 +2362,11 @@
       <x:c r="C134" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
+      <x:c r="F134" s="25" t="str">
+        <x:v>1) Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
+2) Be advised: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
+3) Attention: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
+      </x:c>
     </x:row>
     <x:row r="135" ht="24" hidden="0" customHeight="1">
       <x:c r="A135" s="17" t="str">
@@ -1737,8 +2378,13 @@
       <x:c r="C135" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="136" ht="15" hidden="0" customHeight="1">
+      <x:c r="F135" s="25" t="str">
+        <x:v>1) Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
+2) Be advised: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
+3) Attention: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136" ht="120" hidden="0" customHeight="1">
       <x:c r="A136" s="17" t="str">
         <x:v>L:CPLAND51</x:v>
       </x:c>
@@ -1747,6 +2393,11 @@
       </x:c>
       <x:c r="C136" s="12" t="str">
         <x:v>Watch out reduce collective now.</x:v>
+      </x:c>
+      <x:c r="F136" s="25" t="str">
+        <x:v>1) Watch out. Reduce collective now.
+2) Be advised: watch out. Reduce collective now.
+3) Attention: watch out. Reduce collective now.</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="24" hidden="0" customHeight="1">
@@ -1759,8 +2410,13 @@
       <x:c r="C137" s="12" t="str">
         <x:v>A crew i just received a call from doc the ambulance has been rerouted to another hospital it seems to be better for patient conditions we have to modify our root for the new picking point location.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="138" ht="15" hidden="0" customHeight="1">
+      <x:c r="F137" s="25" t="str">
+        <x:v>1) Crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
+2) Be advised: crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
+3) All crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138" ht="120" hidden="0" customHeight="1">
       <x:c r="A138" s="17" t="str">
         <x:v>L:CPLAND53</x:v>
       </x:c>
@@ -1770,8 +2426,13 @@
       <x:c r="C138" s="12" t="str">
         <x:v>Medical crew was starting ground loading procedures we have to wait here.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="139" ht="15" hidden="0" customHeight="1">
+      <x:c r="F138" s="25" t="str">
+        <x:v>1) Medical crew has started ground-loading procedures. We must wait here.
+2) Be advised: medical crew has started ground-loading procedures. We must wait here.
+3) Attention: medical crew has started ground-loading procedures. We must wait here.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139" ht="120" hidden="0" customHeight="1">
       <x:c r="A139" s="17" t="str">
         <x:v>L:CPLAND54</x:v>
       </x:c>
@@ -1781,8 +2442,13 @@
       <x:c r="C139" s="12" t="str">
         <x:v>Medical crew informs the due to distance we need to proceed with hoist operation crew was ready waiting us.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="140" ht="15" hidden="0" customHeight="1">
+      <x:c r="F139" s="25" t="str">
+        <x:v>1) Medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
+2) Be advised: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
+3) Attention: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140" ht="120" hidden="0" customHeight="1">
       <x:c r="A140" s="17" t="str">
         <x:v>L:CPLAND55</x:v>
       </x:c>
@@ -1792,8 +2458,13 @@
       <x:c r="C140" s="12" t="str">
         <x:v>Medical crew was ready for hoist operation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="141" ht="15" hidden="0" customHeight="1">
+      <x:c r="F140" s="25" t="str">
+        <x:v>1) Medical crew is ready for hoist operations.
+2) Be advised: medical crew is ready for hoist operations.
+3) Attention: medical crew is ready for hoist operations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141" ht="120" hidden="0" customHeight="1">
       <x:c r="A141" s="17" t="str">
         <x:v>L:CPLAND56</x:v>
       </x:c>
@@ -1803,8 +2474,13 @@
       <x:c r="C141" s="12" t="str">
         <x:v>Patient and doctor will be transported by ambulance and we have to pick doc and hospital.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="142" ht="15" hidden="0" customHeight="1">
+      <x:c r="F141" s="25" t="str">
+        <x:v>1) The patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
+2) Be advised: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
+3) Attention: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142" ht="120" hidden="0" customHeight="1">
       <x:c r="A142" s="17" t="str">
         <x:v>L:CPLAND57</x:v>
       </x:c>
@@ -1814,8 +2490,13 @@
       <x:c r="C142" s="12" t="str">
         <x:v>Patient will be transported by ambulance we completed our task.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="143" ht="15" hidden="0" customHeight="1">
+      <x:c r="F142" s="25" t="str">
+        <x:v>1) The patient will travel by ambulance. Our task is complete.
+2) Be advised: the patient will travel by ambulance. Our task is complete.
+3) Attention: the patient will travel by ambulance. Our task is complete.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143" ht="120" hidden="0" customHeight="1">
       <x:c r="A143" s="17" t="str">
         <x:v>L:CPLAND58</x:v>
       </x:c>
@@ -1825,8 +2506,13 @@
       <x:c r="C143" s="12" t="str">
         <x:v>Patient will be transported by us.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="144" ht="15" hidden="0" customHeight="1">
+      <x:c r="F143" s="25" t="str">
+        <x:v>1) The patient will be transported by us.
+2) Be advised: the patient will be transported by us.
+3) Attention: the patient will be transported by us.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="120" hidden="0" customHeight="1">
       <x:c r="A144" s="17" t="str">
         <x:v>L:CPLAND59</x:v>
       </x:c>
@@ -1836,8 +2522,13 @@
       <x:c r="C144" s="12" t="str">
         <x:v>Rescue team identified a valid landing spot a marshal or is waiting us.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="145" ht="15" hidden="0" customHeight="1">
+      <x:c r="F144" s="25" t="str">
+        <x:v>1) The rescue team identified a valid landing spot. A marshal is waiting for us.
+2) Be advised: the rescue team identified a valid landing spot. A marshal is waiting for us.
+3) Attention: the rescue team identified a valid landing spot. A marshal is waiting for us.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145" ht="120" hidden="0" customHeight="1">
       <x:c r="A145" s="17" t="str">
         <x:v>L:CPLAND60</x:v>
       </x:c>
@@ -1847,8 +2538,13 @@
       <x:c r="C145" s="12" t="str">
         <x:v>Hey we cannot take off with fuel hose attached.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="146" ht="15" hidden="0" customHeight="1">
+      <x:c r="F145" s="25" t="str">
+        <x:v>1) We cannot take off with the fuel hose attached.
+2) We can't take off with the fuel hose attached.
+3) Attention: we cannot take off with the fuel hose attached.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146" ht="120" hidden="0" customHeight="1">
       <x:c r="A146" s="17" t="str">
         <x:v>L:CPLAND61</x:v>
       </x:c>
@@ -1857,6 +2553,11 @@
       </x:c>
       <x:c r="C146" s="12" t="str">
         <x:v>Crew is ready on landing spot we can proceed.</x:v>
+      </x:c>
+      <x:c r="F146" s="25" t="str">
+        <x:v>1) Crew is ready at the landing site. We can proceed.
+2) Be advised: crew is ready at the landing site. We can proceed.
+3) Attention: crew is ready at the landing site. We can proceed.</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="15" hidden="0" customHeight="1">
@@ -1870,7 +2571,7 @@
         <x:v>[Non-verbal sound effect.]</x:v>
       </x:c>
     </x:row>
-    <x:row r="148" ht="15" hidden="0" customHeight="1">
+    <x:row r="148" ht="120" hidden="0" customHeight="1">
       <x:c r="A148" s="17" t="str">
         <x:v>L:ANDTEST1</x:v>
       </x:c>
@@ -1880,8 +2581,13 @@
       <x:c r="C148" s="12" t="str">
         <x:v>This is the default hoist pack enjoy.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="149" ht="15" hidden="0" customHeight="1">
+      <x:c r="F148" s="25" t="str">
+        <x:v>1) This is the default hoist pack enjoy.
+2) Be advised: this is the default hoist pack enjoy.
+3) Attention: this is the default hoist pack enjoy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149" ht="120" hidden="0" customHeight="1">
       <x:c r="A149" s="17" t="str">
         <x:v>L:PLTAND1</x:v>
       </x:c>
@@ -1891,8 +2597,13 @@
       <x:c r="C149" s="12" t="str">
         <x:v>Through comm check please.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="150" ht="15" hidden="0" customHeight="1">
+      <x:c r="F149" s="25" t="str">
+        <x:v>1) Pilot, communications check.
+2) Be advised: pilot, communications check.
+3) Attention: pilot, communications check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150" ht="120" hidden="0" customHeight="1">
       <x:c r="A150" s="17" t="str">
         <x:v>L:PLTAND2</x:v>
       </x:c>
@@ -1902,8 +2613,13 @@
       <x:c r="C150" s="12" t="str">
         <x:v>Landed crew aboard authorized.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="151" ht="15" hidden="0" customHeight="1">
+      <x:c r="F150" s="25" t="str">
+        <x:v>1) Landed. Crew, board when authorized.
+2) Be advised: landed. Crew, board when authorized.
+3) Attention: landed. Crew, board when authorized.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151" ht="120" hidden="0" customHeight="1">
       <x:c r="A151" s="17" t="str">
         <x:v>L:PLTAND3</x:v>
       </x:c>
@@ -1913,8 +2629,13 @@
       <x:c r="C151" s="12" t="str">
         <x:v>Evacuate helicopter now.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="152" ht="15" hidden="0" customHeight="1">
+      <x:c r="F151" s="25" t="str">
+        <x:v>1) Evacuate helicopter now.
+2) Be advised: evacuate helicopter now.
+3) Attention: evacuate helicopter now.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152" ht="120" hidden="0" customHeight="1">
       <x:c r="A152" s="17" t="str">
         <x:v>L:PLTAND5</x:v>
       </x:c>
@@ -1924,8 +2645,13 @@
       <x:c r="C152" s="12" t="str">
         <x:v>Hi sarah how you helicopter is good fuel needs to be refilled.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="153" ht="15" hidden="0" customHeight="1">
+      <x:c r="F152" s="25" t="str">
+        <x:v>1) Hi Sarah, how are you? The helicopter is good, but it needs refuelling.
+2) Be advised: hi Sarah, how are you? The helicopter is good, but it needs refuelling.
+3) Attention: hi Sarah, how are you? The helicopter is good, but it needs refuelling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153" ht="120" hidden="0" customHeight="1">
       <x:c r="A153" s="17" t="str">
         <x:v>L:PLTAND6</x:v>
       </x:c>
@@ -1935,8 +2661,13 @@
       <x:c r="C153" s="12" t="str">
         <x:v>I'll check.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="154" ht="15" hidden="0" customHeight="1">
+      <x:c r="F153" s="25" t="str">
+        <x:v>1) I'll check.
+2) Be advised: i'll check.
+3) Attention: i'll check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154" ht="120" hidden="0" customHeight="1">
       <x:c r="A154" s="17" t="str">
         <x:v>L:PLTAND7</x:v>
       </x:c>
@@ -1946,8 +2677,13 @@
       <x:c r="C154" s="12" t="str">
         <x:v>Mission accomplished.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="155" ht="15" hidden="0" customHeight="1">
+      <x:c r="F154" s="25" t="str">
+        <x:v>1) Mission accomplished.
+2) Be advised: mission accomplished.
+3) Attention: mission accomplished.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" ht="120" hidden="0" customHeight="1">
       <x:c r="A155" s="17" t="str">
         <x:v>L:PLTAND8</x:v>
       </x:c>
@@ -1957,8 +2693,13 @@
       <x:c r="C155" s="12" t="str">
         <x:v>Thank you.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="156" ht="15" hidden="0" customHeight="1">
+      <x:c r="F155" s="25" t="str">
+        <x:v>1) Thank you.
+2) Be advised: thank you.
+3) Attention: thank you.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156" ht="120" hidden="0" customHeight="1">
       <x:c r="A156" s="17" t="str">
         <x:v>L:PLTAND9</x:v>
       </x:c>
@@ -1968,8 +2709,13 @@
       <x:c r="C156" s="12" t="str">
         <x:v>Thank you frank.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="157" ht="15" hidden="0" customHeight="1">
+      <x:c r="F156" s="25" t="str">
+        <x:v>1) Thank you, Frank.
+2) Be advised: thank you, Frank.
+3) Attention: thank you, Frank.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157" ht="120" hidden="0" customHeight="1">
       <x:c r="A157" s="17" t="str">
         <x:v>L:PLTAND10</x:v>
       </x:c>
@@ -1979,8 +2725,13 @@
       <x:c r="C157" s="12" t="str">
         <x:v>We did our best unfortunately we cannot save all patients.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="158" ht="15" hidden="0" customHeight="1">
+      <x:c r="F157" s="25" t="str">
+        <x:v>1) We did our best. Unfortunately, we could not save every patient.
+2) Be advised: we did our best. Unfortunately, we could not save every patient.
+3) Attention: we did our best. Unfortunately, we could not save every patient.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="158" ht="120" hidden="0" customHeight="1">
       <x:c r="A158" s="17" t="str">
         <x:v>L:PLTAND11</x:v>
       </x:c>
@@ -1990,8 +2741,13 @@
       <x:c r="C158" s="12" t="str">
         <x:v>Well done.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="159" ht="15" hidden="0" customHeight="1">
+      <x:c r="F158" s="25" t="str">
+        <x:v>1) Well done.
+2) Be advised: well done.
+3) Attention: well done.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159" ht="120" hidden="0" customHeight="1">
       <x:c r="A159" s="17" t="str">
         <x:v>L:PLTAND13</x:v>
       </x:c>
@@ -2001,8 +2757,13 @@
       <x:c r="C159" s="12" t="str">
         <x:v>Two nautical miles from accident area.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="160" ht="15" hidden="0" customHeight="1">
+      <x:c r="F159" s="25" t="str">
+        <x:v>1) Two nautical miles from the accident area.
+2) Be advised: two nautical miles from the accident area.
+3) Attention: two nautical miles from the accident area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="160" ht="120" hidden="0" customHeight="1">
       <x:c r="A160" s="17" t="str">
         <x:v>L:PLTAND14</x:v>
       </x:c>
@@ -2012,8 +2773,13 @@
       <x:c r="C160" s="12" t="str">
         <x:v>Two nautical miles from our base.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="161" ht="15" hidden="0" customHeight="1">
+      <x:c r="F160" s="25" t="str">
+        <x:v>1) Two nautical miles from our base.
+2) Be advised: two nautical miles from our base.
+3) Attention: two nautical miles from our base.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161" ht="120" hidden="0" customHeight="1">
       <x:c r="A161" s="17" t="str">
         <x:v>L:PLTAND15</x:v>
       </x:c>
@@ -2023,8 +2789,13 @@
       <x:c r="C161" s="12" t="str">
         <x:v>Two nautical miles from hospital.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="162" ht="15" hidden="0" customHeight="1">
+      <x:c r="F161" s="25" t="str">
+        <x:v>1) Two nautical miles from hospital.
+2) Be advised: two nautical miles from hospital.
+3) Attention: two nautical miles from hospital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162" ht="120" hidden="0" customHeight="1">
       <x:c r="A162" s="17" t="str">
         <x:v>L:PLTAND16</x:v>
       </x:c>
@@ -2034,8 +2805,13 @@
       <x:c r="C162" s="12" t="str">
         <x:v>Two nautical miles from loading area.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="163" ht="15" hidden="0" customHeight="1">
+      <x:c r="F162" s="25" t="str">
+        <x:v>1) Two nautical miles from the loading area.
+2) Be advised: two nautical miles from the loading area.
+3) Attention: two nautical miles from the loading area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163" ht="120" hidden="0" customHeight="1">
       <x:c r="A163" s="17" t="str">
         <x:v>L:PLTAND17</x:v>
       </x:c>
@@ -2045,8 +2821,13 @@
       <x:c r="C163" s="12" t="str">
         <x:v>Engine parameters when not good.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="164" ht="15" hidden="0" customHeight="1">
+      <x:c r="F163" s="25" t="str">
+        <x:v>1) Engine parameters are not good.
+2) Be advised: engine parameters are not good.
+3) Attention: engine parameters are not good.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164" ht="120" hidden="0" customHeight="1">
       <x:c r="A164" s="17" t="str">
         <x:v>L:PLTAND19</x:v>
       </x:c>
@@ -2056,8 +2837,13 @@
       <x:c r="C164" s="12" t="str">
         <x:v>We exceeded VNE.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="165" ht="15" hidden="0" customHeight="1">
+      <x:c r="F164" s="25" t="str">
+        <x:v>1) We exceeded VNE.
+2) Be advised: we exceeded VNE.
+3) Attention: we exceeded VNE.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165" ht="120" hidden="0" customHeight="1">
       <x:c r="A165" s="17" t="str">
         <x:v>L:PLTAND20</x:v>
       </x:c>
@@ -2067,8 +2853,13 @@
       <x:c r="C165" s="12" t="str">
         <x:v>We exceeded the torque limits.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="166" ht="15" hidden="0" customHeight="1">
+      <x:c r="F165" s="25" t="str">
+        <x:v>1) We exceeded the torque limits.
+2) Be advised: we exceeded the torque limits.
+3) Attention: we exceeded the torque limits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166" ht="120" hidden="0" customHeight="1">
       <x:c r="A166" s="17" t="str">
         <x:v>L:PLTAND21</x:v>
       </x:c>
@@ -2078,8 +2869,13 @@
       <x:c r="C166" s="12" t="str">
         <x:v>Hi sarah i'm sorry we have some bad news for you.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="167" ht="15" hidden="0" customHeight="1">
+      <x:c r="F166" s="25" t="str">
+        <x:v>1) Hi sarah i'm sorry we have some bad news for you.
+2) Be advised: hi sarah i'm sorry we have some bad news for you.
+3) Attention: hi sarah i'm sorry we have some bad news for you.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167" ht="120" hidden="0" customHeight="1">
       <x:c r="A167" s="17" t="str">
         <x:v>L:PLTAND24</x:v>
       </x:c>
@@ -2089,8 +2885,13 @@
       <x:c r="C167" s="12" t="str">
         <x:v>Main gearbox parameters were high and we felt hi vibrations.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="168" ht="15" hidden="0" customHeight="1">
+      <x:c r="F167" s="25" t="str">
+        <x:v>1) Main gearbox parameters were high, and we felt strong vibrations.
+2) Be advised: main gearbox parameters were high, and we felt strong vibrations.
+3) Attention: main gearbox parameters were high, and we felt strong vibrations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168" ht="120" hidden="0" customHeight="1">
       <x:c r="A168" s="17" t="str">
         <x:v>L:PLTAND25</x:v>
       </x:c>
@@ -2100,8 +2901,13 @@
       <x:c r="C168" s="12" t="str">
         <x:v>We had tail rotor gearbox parameters fluctuations.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="169" ht="15" hidden="0" customHeight="1">
+      <x:c r="F168" s="25" t="str">
+        <x:v>1) Tail-rotor gearbox parameters fluctuated.
+2) Be advised: tail-rotor gearbox parameters fluctuated.
+3) Attention: tail-rotor gearbox parameters fluctuated.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" ht="120" hidden="0" customHeight="1">
       <x:c r="A169" s="17" t="str">
         <x:v>L:PLTAND26</x:v>
       </x:c>
@@ -2111,8 +2917,13 @@
       <x:c r="C169" s="12" t="str">
         <x:v>We had failures they are reported in the technical log book.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="170" ht="15" hidden="0" customHeight="1">
+      <x:c r="F169" s="25" t="str">
+        <x:v>1) We had failures. They are recorded in the technical logbook.
+2) Be advised: we had failures. They are recorded in the technical logbook.
+3) Attention: we had failures. They are recorded in the technical logbook.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170" ht="120" hidden="0" customHeight="1">
       <x:c r="A170" s="17" t="str">
         <x:v>L:PLTAND27</x:v>
       </x:c>
@@ -2122,8 +2933,13 @@
       <x:c r="C170" s="12" t="str">
         <x:v>We had a hard landing.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="171" ht="15" hidden="0" customHeight="1">
+      <x:c r="F170" s="25" t="str">
+        <x:v>1) We had a hard landing.
+2) Be advised: we had a hard landing.
+3) Attention: we had a hard landing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171" ht="120" hidden="0" customHeight="1">
       <x:c r="A171" s="17" t="str">
         <x:v>L:PLTAND28</x:v>
       </x:c>
@@ -2133,8 +2949,13 @@
       <x:c r="C171" s="12" t="str">
         <x:v>Two nautical miles from pick up location.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="172" ht="15" hidden="0" customHeight="1">
+      <x:c r="F171" s="25" t="str">
+        <x:v>1) Two nautical miles from the pickup location.
+2) Be advised: two nautical miles from the pickup location.
+3) Attention: two nautical miles from the pickup location.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172" ht="120" hidden="0" customHeight="1">
       <x:c r="A172" s="17" t="str">
         <x:v>L:PLTAND29</x:v>
       </x:c>
@@ -2144,8 +2965,13 @@
       <x:c r="C172" s="12" t="str">
         <x:v>Hr we are now approaching to drop point thanks for the help and see you next time.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="173" ht="15" hidden="0" customHeight="1">
+      <x:c r="F172" s="25" t="str">
+        <x:v>1) Heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
+2) Be advised: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
+3) Attention: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173" ht="120" hidden="0" customHeight="1">
       <x:c r="A173" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2155,8 +2981,13 @@
       <x:c r="C173" s="12" t="str">
         <x:v>We are entering into designated SAR area it's time to start our search for the casualties.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="174" ht="15" hidden="0" customHeight="1">
+      <x:c r="F173" s="25" t="str">
+        <x:v>1) We are entering the designated SAR area. Start the search for casualties.
+2) We're entering the designated SAR area. Start the search for casualties.
+3) Attention: we are entering the designated SAR area. Start the search for casualties.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174" ht="120" hidden="0" customHeight="1">
       <x:c r="A174" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2166,8 +2997,13 @@
       <x:c r="C174" s="12" t="str">
         <x:v>SAR area starts here watch out and let's find our signed casualties.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="175" ht="15" hidden="0" customHeight="1">
+      <x:c r="F174" s="25" t="str">
+        <x:v>1) The SAR area starts here. Stay alert and search for casualties.
+2) Be advised: the SAR area starts here. Stay alert and search for casualties.
+3) Attention: the SAR area starts here. Stay alert and search for casualties.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175" ht="120" hidden="0" customHeight="1">
       <x:c r="A175" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2177,8 +3013,13 @@
       <x:c r="C175" s="12" t="str">
         <x:v>Crew please stop searching for the survivor now we are entering in the assigned area.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="176" ht="15" hidden="0" customHeight="1">
+      <x:c r="F175" s="25" t="str">
+        <x:v>1) Crew, stop searching. We are now entering the assigned area.
+2) Crew, stop searching. We're now entering the assigned area.
+3) All crew, stop searching. We are now entering the assigned area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176" ht="120" hidden="0" customHeight="1">
       <x:c r="A176" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2188,8 +3029,13 @@
       <x:c r="C176" s="12" t="str">
         <x:v>Confirmed solve every of established the clock is ticking let's find the casualties now.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="177" ht="15" hidden="0" customHeight="1">
+      <x:c r="F176" s="25" t="str">
+        <x:v>1) Confirmed. The clock is ticking; start the search now.
+2) Be advised: confirmed. The clock is ticking; start the search now.
+3) Attention: confirmed. The clock is ticking; start the search now.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177" ht="120" hidden="0" customHeight="1">
       <x:c r="A177" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2199,8 +3045,13 @@
       <x:c r="C177" s="12" t="str">
         <x:v>The boundary crossed let's execute the search plan and locate the survivors.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="178" ht="15" hidden="0" customHeight="1">
+      <x:c r="F177" s="25" t="str">
+        <x:v>1) Boundary crossed. Execute the search plan and locate the survivors.
+2) Be advised: boundary crossed. Execute the search plan and locate the survivors.
+3) Attention: boundary crossed. Execute the search plan and locate the survivors.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178" ht="120" hidden="0" customHeight="1">
       <x:c r="A178" s="17" t="str">
         <x:v>L:PLTAND30</x:v>
       </x:c>
@@ -2210,8 +3061,13 @@
       <x:c r="C178" s="12" t="str">
         <x:v>We have reached the search and rescue zone initiate the search pattern for survivors.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="179" ht="15" hidden="0" customHeight="1">
+      <x:c r="F178" s="25" t="str">
+        <x:v>1) We have reached the search-and-rescue zone. Begin the search pattern for survivors.
+2) We've reached the search-and-rescue zone. Begin the search pattern for survivors.
+3) Attention: we have reached the search-and-rescue zone. Begin the search pattern for survivors.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179" ht="120" hidden="0" customHeight="1">
       <x:c r="A179" s="17" t="str">
         <x:v>L:PLTAND36</x:v>
       </x:c>
@@ -2221,8 +3077,13 @@
       <x:c r="C179" s="12" t="str">
         <x:v>Crew is cutting back.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="180" ht="15" hidden="0" customHeight="1">
+      <x:c r="F179" s="25" t="str">
+        <x:v>1) Crew is coming back.
+2) Be advised: crew is coming back.
+3) Attention: crew is coming back.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180" ht="120" hidden="0" customHeight="1">
       <x:c r="A180" s="17" t="str">
         <x:v>L:PLTAND37</x:v>
       </x:c>
@@ -2232,8 +3093,13 @@
       <x:c r="C180" s="12" t="str">
         <x:v>Let's go.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="181" ht="15" hidden="0" customHeight="1">
+      <x:c r="F180" s="25" t="str">
+        <x:v>1) Let's go.
+2) Be advised: let's go.
+3) Attention: let's go.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181" ht="120" hidden="0" customHeight="1">
       <x:c r="A181" s="17" t="str">
         <x:v>L:PLTAND38</x:v>
       </x:c>
@@ -2243,8 +3109,13 @@
       <x:c r="C181" s="12" t="str">
         <x:v>We're crew are we able to accept a new dispatch or do we need to come back to base.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="182" ht="15" hidden="0" customHeight="1">
+      <x:c r="F181" s="25" t="str">
+        <x:v>1) Crew, can we accept a new dispatch, or do we need to return to base?
+2) Can you confirm: crew, can we accept a new dispatch, or do we need to return to base?
+3) All crew, can we accept a new dispatch, or do we need to return to base?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182" ht="120" hidden="0" customHeight="1">
       <x:c r="A182" s="17" t="str">
         <x:v>L:PLTAND38</x:v>
       </x:c>
@@ -2254,8 +3125,13 @@
       <x:c r="C182" s="12" t="str">
         <x:v>I believe we must go back to the base before we accept new dispatches.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="183" ht="15" hidden="0" customHeight="1">
+      <x:c r="F182" s="25" t="str">
+        <x:v>1) I believe we should return to base before accepting another dispatch.
+2) Be advised: i believe we should return to base before accepting another dispatch.
+3) Attention: i believe we should return to base before accepting another dispatch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183" ht="120" hidden="0" customHeight="1">
       <x:c r="A183" s="17" t="str">
         <x:v>L:PLTAND40</x:v>
       </x:c>
@@ -2265,8 +3141,13 @@
       <x:c r="C183" s="12" t="str">
         <x:v>Hey we have a new dispatch.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="184" ht="15" hidden="0" customHeight="1">
+      <x:c r="F183" s="25" t="str">
+        <x:v>1) We have a new dispatch.
+2) Be advised: we have a new dispatch.
+3) Attention: we have a new dispatch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184" ht="120" hidden="0" customHeight="1">
       <x:c r="A184" s="17" t="str">
         <x:v>L:PLTAND40</x:v>
       </x:c>
@@ -2276,8 +3157,13 @@
       <x:c r="C184" s="12" t="str">
         <x:v>How crew we have a new assignment.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="185" ht="15" hidden="0" customHeight="1">
+      <x:c r="F184" s="25" t="str">
+        <x:v>1) Crew, we have a new assignment.
+2) Be advised: crew, we have a new assignment.
+3) All crew, we have a new assignment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="185" ht="120" hidden="0" customHeight="1">
       <x:c r="A185" s="17" t="str">
         <x:v>L:PLTAND40</x:v>
       </x:c>
@@ -2287,8 +3173,13 @@
       <x:c r="C185" s="12" t="str">
         <x:v>How we have another dispatch.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="186" ht="15" hidden="0" customHeight="1">
+      <x:c r="F185" s="25" t="str">
+        <x:v>1) We have another dispatch.
+2) Be advised: we have another dispatch.
+3) Attention: we have another dispatch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186" ht="120" hidden="0" customHeight="1">
       <x:c r="A186" s="17" t="str">
         <x:v>L:PLTAND40</x:v>
       </x:c>
@@ -2298,8 +3189,13 @@
       <x:c r="C186" s="12" t="str">
         <x:v>Busy day we received a new dispatch.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="187" ht="15" hidden="0" customHeight="1">
+      <x:c r="F186" s="25" t="str">
+        <x:v>1) Busy day we received a new dispatch.
+2) Be advised: busy day we received a new dispatch.
+3) Attention: busy day we received a new dispatch.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="187" ht="120" hidden="0" customHeight="1">
       <x:c r="A187" s="17" t="str">
         <x:v>L:PLTAND44</x:v>
       </x:c>
@@ -2309,8 +3205,13 @@
       <x:c r="C187" s="12" t="str">
         <x:v>Looks set to drop point.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="188" ht="15" hidden="0" customHeight="1">
+      <x:c r="F187" s="25" t="str">
+        <x:v>1) Route set to the drop point.
+2) Be advised: route set to the drop point.
+3) Attention: route set to the drop point.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188" ht="120" hidden="0" customHeight="1">
       <x:c r="A188" s="17" t="str">
         <x:v>L:PLTAND45</x:v>
       </x:c>
@@ -2320,8 +3221,13 @@
       <x:c r="C188" s="12" t="str">
         <x:v>Group set to the pick up point.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="189" ht="15" hidden="0" customHeight="1">
+      <x:c r="F188" s="25" t="str">
+        <x:v>1) Route set to the pickup point.
+2) Be advised: route set to the pickup point.
+3) Attention: route set to the pickup point.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189" ht="120" hidden="0" customHeight="1">
       <x:c r="A189" s="17" t="str">
         <x:v>L:PAX2AND1</x:v>
       </x:c>
@@ -2331,8 +3237,13 @@
       <x:c r="C189" s="12" t="str">
         <x:v>Copy paramedic here comm check.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="190" ht="15" hidden="0" customHeight="1">
+      <x:c r="F189" s="25" t="str">
+        <x:v>1) Copy, paramedic here. Communications check.
+2) Be advised: copy, paramedic here. Communications check.
+3) Attention: copy, paramedic here. Communications check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190" ht="120" hidden="0" customHeight="1">
       <x:c r="A190" s="17" t="str">
         <x:v>L:PAX2AND3</x:v>
       </x:c>
@@ -2342,8 +3253,13 @@
       <x:c r="C190" s="12" t="str">
         <x:v>Hi anna nice to meet you again are you free for lunch tomorrow.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="191" ht="15" hidden="0" customHeight="1">
+      <x:c r="F190" s="25" t="str">
+        <x:v>1) Hi Anna, nice to meet you again. Are you free for lunch tomorrow?
+2) Can you confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?
+3) Please confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191" ht="120" hidden="0" customHeight="1">
       <x:c r="A191" s="17" t="str">
         <x:v>L:PAX2AND4</x:v>
       </x:c>
@@ -2353,8 +3269,13 @@
       <x:c r="C191" s="12" t="str">
         <x:v>Stretches secured.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="192" ht="15" hidden="0" customHeight="1">
+      <x:c r="F191" s="25" t="str">
+        <x:v>1) Stretcher secured.
+2) Be advised: stretcher secured.
+3) Attention: stretcher secured.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192" ht="120" hidden="0" customHeight="1">
       <x:c r="A192" s="17" t="str">
         <x:v>L:PAX3AND1</x:v>
       </x:c>
@@ -2364,8 +3285,13 @@
       <x:c r="C192" s="12" t="str">
         <x:v>The ambulance with no paramedic.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="193" ht="15" hidden="0" customHeight="1">
+      <x:c r="F192" s="25" t="str">
+        <x:v>1) An ambulance is on scene, but no paramedic is present.
+2) Be advised: an ambulance is on scene, but no paramedic is present.
+3) Attention: an ambulance is on scene, but no paramedic is present.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193" ht="120" hidden="0" customHeight="1">
       <x:c r="A193" s="17" t="str">
         <x:v>L:PAX3AND2</x:v>
       </x:c>
@@ -2375,8 +3301,13 @@
       <x:c r="C193" s="12" t="str">
         <x:v>Duck here comm check.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="194" ht="15" hidden="0" customHeight="1">
+      <x:c r="F193" s="25" t="str">
+        <x:v>1) Medic here. Communications check.
+2) Be advised: medic here. Communications check.
+3) Attention: medic here. Communications check.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194" ht="120" hidden="0" customHeight="1">
       <x:c r="A194" s="17" t="str">
         <x:v>L:PAX3AND3</x:v>
       </x:c>
@@ -2386,8 +3317,13 @@
       <x:c r="C194" s="12" t="str">
         <x:v>Confirmed on scene.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="195" ht="15" hidden="0" customHeight="1">
+      <x:c r="F194" s="25" t="str">
+        <x:v>1) Confirmed on scene.
+2) Be advised: confirmed on scene.
+3) Attention: confirmed on scene.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="195" ht="120" hidden="0" customHeight="1">
       <x:c r="A195" s="17" t="str">
         <x:v>L:PAX3AND4</x:v>
       </x:c>
@@ -2397,8 +3333,13 @@
       <x:c r="C195" s="12" t="str">
         <x:v>Fire engine.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="196" ht="15" hidden="0" customHeight="1">
+      <x:c r="F195" s="25" t="str">
+        <x:v>1) Fire engine.
+2) Be advised: fire engine.
+3) Attention: fire engine.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="196" ht="120" hidden="0" customHeight="1">
       <x:c r="A196" s="17" t="str">
         <x:v>L:PAX3AND5</x:v>
       </x:c>
@@ -2408,8 +3349,13 @@
       <x:c r="C196" s="12" t="str">
         <x:v>We need time for ground operations please stand by.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="197" ht="15" hidden="0" customHeight="1">
+      <x:c r="F196" s="25" t="str">
+        <x:v>1) We need time for ground operations. Please stand by.
+2) Be advised: we need time for ground operations. Please stand by.
+3) Attention: we need time for ground operations. Please stand by.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="197" ht="120" hidden="0" customHeight="1">
       <x:c r="A197" s="17" t="str">
         <x:v>L:PAX3AND6</x:v>
       </x:c>
@@ -2419,8 +3365,13 @@
       <x:c r="C197" s="12" t="str">
         <x:v>I said of possible hospital destination for our patient info available on tablet we can confirm or change later.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="198" ht="15" hidden="0" customHeight="1">
+      <x:c r="F197" s="25" t="str">
+        <x:v>1) A possible hospital destination is available on the tablet. We can confirm or change it later.
+2) Be advised: a possible hospital destination is available on the tablet. We can confirm or change it later.
+3) Attention: a possible hospital destination is available on the tablet. We can confirm or change it later.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="198" ht="120" hidden="0" customHeight="1">
       <x:c r="A198" s="17" t="str">
         <x:v>L:PAX3AND7</x:v>
       </x:c>
@@ -2430,8 +3381,13 @@
       <x:c r="C198" s="12" t="str">
         <x:v>Patient has died.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="199" ht="15" hidden="0" customHeight="1">
+      <x:c r="F198" s="25" t="str">
+        <x:v>1) Patient has died.
+2) Be advised: patient has died.
+3) Attention: patient has died.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="199" ht="120" hidden="0" customHeight="1">
       <x:c r="A199" s="17" t="str">
         <x:v>L:PAX3AND8</x:v>
       </x:c>
@@ -2440,6 +3396,11 @@
       </x:c>
       <x:c r="C199" s="12" t="str">
         <x:v>Patient life signs of fading.</x:v>
+      </x:c>
+      <x:c r="F199" s="25" t="str">
+        <x:v>1) The patient's vital signs are fading.
+2) Be advised: the patient's vital signs are fading.
+3) Attention: the patient's vital signs are fading.</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="24" hidden="0" customHeight="1">
@@ -2452,8 +3413,13 @@
       <x:c r="C200" s="12" t="str">
         <x:v>Patient location is far away ambulance crew on seen may transport patient to the meeting point proposed on tablet please confirm if we want to meet midway.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="201" ht="15" hidden="0" customHeight="1">
+      <x:c r="F200" s="25" t="str">
+        <x:v>1) The patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
+2) Be advised: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
+3) Attention: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="201" ht="120" hidden="0" customHeight="1">
       <x:c r="A201" s="17" t="str">
         <x:v>L:PAX3AND10</x:v>
       </x:c>
@@ -2463,8 +3429,13 @@
       <x:c r="C201" s="12" t="str">
         <x:v>Patient on board take care.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="202" ht="15" hidden="0" customHeight="1">
+      <x:c r="F201" s="25" t="str">
+        <x:v>1) Patient on board. Take care.
+2) Be advised: patient on board. Take care.
+3) The patient is on board. Take care.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202" ht="120" hidden="0" customHeight="1">
       <x:c r="A202" s="17" t="str">
         <x:v>L:PAX3AND11</x:v>
       </x:c>
@@ -2474,8 +3445,13 @@
       <x:c r="C202" s="12" t="str">
         <x:v>Patient has been the board to the hospital key is safe.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="203" ht="15" hidden="0" customHeight="1">
+      <x:c r="F202" s="25" t="str">
+        <x:v>1) The patient has been delivered to the hospital and is safe.
+2) Be advised: the patient has been delivered to the hospital and is safe.
+3) Attention: the patient has been delivered to the hospital and is safe.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203" ht="120" hidden="0" customHeight="1">
       <x:c r="A203" s="17" t="str">
         <x:v>L:PAX3AND12</x:v>
       </x:c>
@@ -2485,8 +3461,13 @@
       <x:c r="C203" s="12" t="str">
         <x:v>Police.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="204" ht="15" hidden="0" customHeight="1">
+      <x:c r="F203" s="25" t="str">
+        <x:v>1) Police.
+2) Be advised: police.
+3) Attention: police.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204" ht="120" hidden="0" customHeight="1">
       <x:c r="A204" s="17" t="str">
         <x:v>L:PAX3AND13</x:v>
       </x:c>
@@ -2496,8 +3477,13 @@
       <x:c r="C204" s="12" t="str">
         <x:v>Patients has been deboarded to the hospital.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="205" ht="15" hidden="0" customHeight="1">
+      <x:c r="F204" s="25" t="str">
+        <x:v>1) The patient has been deboarded at the hospital.
+2) Be advised: the patient has been deboarded at the hospital.
+3) Attention: the patient has been deboarded at the hospital.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205" ht="120" hidden="0" customHeight="1">
       <x:c r="A205" s="17" t="str">
         <x:v>L:PAX3AND15</x:v>
       </x:c>
@@ -2507,8 +3493,13 @@
       <x:c r="C205" s="12" t="str">
         <x:v>We will be first on scene.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="206" ht="15" hidden="0" customHeight="1">
+      <x:c r="F205" s="25" t="str">
+        <x:v>1) We will be first on scene.
+2) Be advised: we will be first on scene.
+3) Attention: we will be first on scene.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206" ht="120" hidden="0" customHeight="1">
       <x:c r="A206" s="17" t="str">
         <x:v>L:PAX3AND16</x:v>
       </x:c>
@@ -2518,8 +3509,13 @@
       <x:c r="C206" s="12" t="str">
         <x:v>We will find an ambulance not far away from accident site they are unable to reach the site.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="207" ht="15" hidden="0" customHeight="1">
+      <x:c r="F206" s="25" t="str">
+        <x:v>1) We will find an ambulance near the accident site; it cannot reach the scene.
+2) We will find an ambulance near the accident site; it can't reach the scene.
+3) Attention: we will find an ambulance near the accident site; it cannot reach the scene.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207" ht="120" hidden="0" customHeight="1">
       <x:c r="A207" s="17" t="str">
         <x:v>L:PAX3AND17</x:v>
       </x:c>
@@ -2529,8 +3525,13 @@
       <x:c r="C207" s="12" t="str">
         <x:v>Cpr in progress please stand by it may take time.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="208" ht="15" hidden="0" customHeight="1">
+      <x:c r="F207" s="25" t="str">
+        <x:v>1) CPR in progress. Please stand by; it may take time.
+2) Be advised: cPR in progress. Please stand by; it may take time.
+3) Attention: cPR in progress. Please stand by; it may take time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208" ht="120" hidden="0" customHeight="1">
       <x:c r="A208" s="17" t="str">
         <x:v>L:PAX3AND19</x:v>
       </x:c>
@@ -2540,8 +3541,13 @@
       <x:c r="C208" s="12" t="str">
         <x:v>We lost the patient we have to record the time of the death please stand by until we secure the cabin.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="209" ht="15" hidden="0" customHeight="1">
+      <x:c r="F208" s="25" t="str">
+        <x:v>1) We lost the patient. Record the time of death and stand by while we secure the cabin.
+2) Be advised: we lost the patient. Record the time of death and stand by while we secure the cabin.
+3) Attention: we lost the patient. Record the time of death and stand by while we secure the cabin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209" ht="120" hidden="0" customHeight="1">
       <x:c r="A209" s="17" t="str">
         <x:v>L:PAX3AND20</x:v>
       </x:c>
@@ -2551,8 +3557,13 @@
       <x:c r="C209" s="12" t="str">
         <x:v>Good cpr successfully reanimated patient we are now securing him for the flight please wait for clearance.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="210" ht="15" hidden="0" customHeight="1">
+      <x:c r="F209" s="25" t="str">
+        <x:v>1) CPR was successful. The patient has been resuscitated; we are securing them for flight.
+2) Be advised: cPR was successful. The patient has been resuscitated; we are securing them for flight.
+3) Attention: cPR was successful. The patient has been resuscitated; we are securing them for flight.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="210" ht="120" hidden="0" customHeight="1">
       <x:c r="A210" s="17" t="str">
         <x:v>L:PAX3AND22</x:v>
       </x:c>
@@ -2562,8 +3573,13 @@
       <x:c r="C210" s="12" t="str">
         <x:v>Patient conditions are critical we need extra time to stabilize for transport please wait.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="211" ht="15" hidden="0" customHeight="1">
+      <x:c r="F210" s="25" t="str">
+        <x:v>1) The patient is critical. We need extra time to stabilize them for transport.
+2) Be advised: the patient is critical. We need extra time to stabilize them for transport.
+3) Attention: the patient is critical. We need extra time to stabilize them for transport.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="211" ht="120" hidden="0" customHeight="1">
       <x:c r="A211" s="17" t="str">
         <x:v>L:PAX3AND23</x:v>
       </x:c>
@@ -2573,8 +3589,13 @@
       <x:c r="C211" s="12" t="str">
         <x:v>I believe we lost the organ it's too degraded.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="212" ht="15" hidden="0" customHeight="1">
+      <x:c r="F211" s="25" t="str">
+        <x:v>1) We lost the organ; it is too degraded.
+2) Be advised: we lost the organ; it is too degraded.
+3) Attention: we lost the organ; it is too degraded.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="212" ht="120" hidden="0" customHeight="1">
       <x:c r="A212" s="17" t="str">
         <x:v>L:PAX3AND24</x:v>
       </x:c>
@@ -2583,6 +3604,11 @@
       </x:c>
       <x:c r="C212" s="12" t="str">
         <x:v>Organs data seems to be degrading.</x:v>
+      </x:c>
+      <x:c r="F212" s="25" t="str">
+        <x:v>1) The organ's condition is deteriorating.
+2) Be advised: the organ's condition is deteriorating.
+3) Attention: the organ's condition is deteriorating.</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="36" hidden="0" customHeight="1">
@@ -2595,8 +3621,13 @@
       <x:c r="C213" s="12" t="str">
         <x:v>Let's proceed with a small briefing about our next operations as soon as we arrive h i will proceed to the scene securing the area after their clearance our crew will join them to perform the medical operation at the end of rescue operations the medical cruel board followed by hr in case the engine has to be transported with hoist out i will be boarded first all clear.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="214" ht="15" hidden="0" customHeight="1">
+      <x:c r="F213" s="25" t="str">
+        <x:v>1) Briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
+2) Be advised: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
+3) Attention: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="214" ht="120" hidden="0" customHeight="1">
       <x:c r="A214" s="17" t="str">
         <x:v>L:PAX3AND26</x:v>
       </x:c>
@@ -2606,8 +3637,13 @@
       <x:c r="C214" s="12" t="str">
         <x:v>Welcome onboard hello his viewers.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="215" ht="15" hidden="0" customHeight="1">
+      <x:c r="F214" s="25" t="str">
+        <x:v>1) Welcome on board, heli-rescuer.
+2) Be advised: welcome on board, heli-rescuer.
+3) Attention: welcome on board, heli-rescuer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="215" ht="120" hidden="0" customHeight="1">
       <x:c r="A215" s="17" t="str">
         <x:v>L:FRAAND1</x:v>
       </x:c>
@@ -2617,8 +3653,13 @@
       <x:c r="C215" s="12" t="str">
         <x:v>If you need refueling please ask.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="216" ht="15" hidden="0" customHeight="1">
+      <x:c r="F215" s="25" t="str">
+        <x:v>1) If you need refueling please ask.
+2) Be advised: if you need refueling please ask.
+3) Attention: if you need refueling please ask.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="216" ht="120" hidden="0" customHeight="1">
       <x:c r="A216" s="17" t="str">
         <x:v>L:FRAAND2</x:v>
       </x:c>
@@ -2628,8 +3669,13 @@
       <x:c r="C216" s="12" t="str">
         <x:v>Fuel is as you requested.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="217" ht="15" hidden="0" customHeight="1">
+      <x:c r="F216" s="25" t="str">
+        <x:v>1) Fuel is as you requested.
+2) Be advised: fuel is as you requested.
+3) Attention: fuel is as you requested.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="217" ht="120" hidden="0" customHeight="1">
       <x:c r="A217" s="17" t="str">
         <x:v>L:FRAAND3</x:v>
       </x:c>
@@ -2639,8 +3685,13 @@
       <x:c r="C217" s="12" t="str">
         <x:v>Fuel tanks are almost full.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="218" ht="15" hidden="0" customHeight="1">
+      <x:c r="F217" s="25" t="str">
+        <x:v>1) Fuel tanks are almost full.
+2) Be advised: fuel tanks are almost full.
+3) Attention: fuel tanks are almost full.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="218" ht="120" hidden="0" customHeight="1">
       <x:c r="A218" s="17" t="str">
         <x:v>L:FRAAND4</x:v>
       </x:c>
@@ -2650,8 +3701,13 @@
       <x:c r="C218" s="12" t="str">
         <x:v>Refueling has not been performed and fuel level is low.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="219" ht="15" hidden="0" customHeight="1">
+      <x:c r="F218" s="25" t="str">
+        <x:v>1) Refueling has not been performed and fuel level is low.
+2) Be advised: refueling has not been performed and fuel level is low.
+3) Attention: refueling has not been performed and fuel level is low.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="219" ht="120" hidden="0" customHeight="1">
       <x:c r="A219" s="17" t="str">
         <x:v>L:FRAAND5</x:v>
       </x:c>
@@ -2661,8 +3717,13 @@
       <x:c r="C219" s="12" t="str">
         <x:v>Gp you disconnected ready to go good day.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="220" ht="15" hidden="0" customHeight="1">
+      <x:c r="F219" s="25" t="str">
+        <x:v>1) GPU disconnected. Ready to go. Good day.
+2) Be advised: gPU disconnected. Ready to go. Good day.
+3) Attention: gPU disconnected. Ready to go. Good day.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="220" ht="120" hidden="0" customHeight="1">
       <x:c r="A220" s="17" t="str">
         <x:v>L:FRAAND6</x:v>
       </x:c>
@@ -2672,8 +3733,13 @@
       <x:c r="C220" s="12" t="str">
         <x:v>I kept captain helicopter is ready to fly law book filled and signed.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="221" ht="15" hidden="0" customHeight="1">
+      <x:c r="F220" s="25" t="str">
+        <x:v>1) Captain, the helicopter is ready for flight. The logbook is completed and signed.
+2) Be advised: captain, the helicopter is ready for flight. The logbook is completed and signed.
+3) Attention: captain, the helicopter is ready for flight. The logbook is completed and signed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="221" ht="120" hidden="0" customHeight="1">
       <x:c r="A221" s="17" t="str">
         <x:v>L:FRAAND7</x:v>
       </x:c>
@@ -2683,8 +3749,13 @@
       <x:c r="C221" s="12" t="str">
         <x:v>Hey good morning all ready for the missions.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="222" ht="15" hidden="0" customHeight="1">
+      <x:c r="F221" s="25" t="str">
+        <x:v>1) Good morning, everyone. Ready for the mission?
+2) Can you confirm: good morning, everyone. Ready for the mission?
+3) Please confirm: good morning, everyone. Ready for the mission?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="222" ht="120" hidden="0" customHeight="1">
       <x:c r="A222" s="17" t="str">
         <x:v>L:FRAAND8</x:v>
       </x:c>
@@ -2694,8 +3765,13 @@
       <x:c r="C222" s="12" t="str">
         <x:v>Really to supply external power at your request.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="223" ht="15" hidden="0" customHeight="1">
+      <x:c r="F222" s="25" t="str">
+        <x:v>1) Ready to provide external power at your request.
+2) Be advised: ready to provide external power at your request.
+3) Attention: ready to provide external power at your request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223" ht="120" hidden="0" customHeight="1">
       <x:c r="A223" s="17" t="str">
         <x:v>L:SARAAND1</x:v>
       </x:c>
@@ -2705,8 +3781,13 @@
       <x:c r="C223" s="12" t="str">
         <x:v>Bye see you tomorrow.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="224" ht="15" hidden="0" customHeight="1">
+      <x:c r="F223" s="25" t="str">
+        <x:v>1) Bye see you tomorrow.
+2) Be advised: bye see you tomorrow.
+3) Attention: bye see you tomorrow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224" ht="120" hidden="0" customHeight="1">
       <x:c r="A224" s="17" t="str">
         <x:v>L:SARAAND2</x:v>
       </x:c>
@@ -2716,8 +3797,13 @@
       <x:c r="C224" s="12" t="str">
         <x:v>How was the last mission was everything good with the helicopter.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="225" ht="15" hidden="0" customHeight="1">
+      <x:c r="F224" s="25" t="str">
+        <x:v>1) How was the last mission? Was everything all right with the helicopter?
+2) Can you confirm: how was the last mission? Was everything all right with the helicopter?
+3) Please confirm: how was the last mission? Was everything all right with the helicopter?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225" ht="120" hidden="0" customHeight="1">
       <x:c r="A225" s="17" t="str">
         <x:v>L:SARAAND4</x:v>
       </x:c>
@@ -2727,8 +3813,13 @@
       <x:c r="C225" s="12" t="str">
         <x:v>Don't worry the helicopter is now in my precious hands it will be ready to fly for the next mission.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="226" ht="15" hidden="0" customHeight="1">
+      <x:c r="F225" s="25" t="str">
+        <x:v>1) Do not worry; the helicopter is in good hands and will be ready for the next mission.
+2) Be advised: do not worry; the helicopter is in good hands and will be ready for the next mission.
+3) Attention: do not worry; the helicopter is in good hands and will be ready for the next mission.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226" ht="120" hidden="0" customHeight="1">
       <x:c r="A226" s="17" t="str">
         <x:v>L:SARAAND5</x:v>
       </x:c>
@@ -2738,8 +3829,13 @@
       <x:c r="C226" s="12" t="str">
         <x:v>Oh my preferred cray hi guys.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="227" ht="15" hidden="0" customHeight="1">
+      <x:c r="F226" s="25" t="str">
+        <x:v>1) Hi, guys.
+2) Be advised: hi, guys.
+3) Attention: hi, guys.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227" ht="120" hidden="0" customHeight="1">
       <x:c r="A227" s="17" t="str">
         <x:v>L:SARAAND6</x:v>
       </x:c>
@@ -2749,8 +3845,13 @@
       <x:c r="C227" s="12" t="str">
         <x:v>It seems i have to work a lot on it.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="228" ht="15" hidden="0" customHeight="1">
+      <x:c r="F227" s="25" t="str">
+        <x:v>1) It looks like I have a lot of work to do.
+2) Be advised: it looks like I have a lot of work to do.
+3) Attention: it looks like I have a lot of work to do.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228" ht="120" hidden="0" customHeight="1">
       <x:c r="A228" s="17" t="str">
         <x:v>L:SARAAND7</x:v>
       </x:c>
@@ -2760,8 +3861,13 @@
       <x:c r="C228" s="12" t="str">
         <x:v>Hi tomorrow okay there is a good restaurant just out of here.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="229" ht="15" hidden="0" customHeight="1">
+      <x:c r="F228" s="25" t="str">
+        <x:v>1) Tomorrow there is a good restaurant just outside. Would you like to go?
+2) Can you confirm: tomorrow there is a good restaurant just outside. Would you like to go?
+3) Please confirm: tomorrow there is a good restaurant just outside. Would you like to go?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229" ht="120" hidden="0" customHeight="1">
       <x:c r="A229" s="17" t="str">
         <x:v>L:SARAAND8</x:v>
       </x:c>
@@ -2770,6 +3876,11 @@
       </x:c>
       <x:c r="C229" s="12" t="str">
         <x:v>Hey what you did to the helicopter.</x:v>
+      </x:c>
+      <x:c r="F229" s="25" t="str">
+        <x:v>1) What did you do to the helicopter?
+2) Can you confirm: what did you do to the helicopter?
+3) Please confirm: what did you do to the helicopter?</x:v>
       </x:c>
     </x:row>
     <x:row r="230" ht="15" hidden="0" customHeight="1">
@@ -2783,7 +3894,7 @@
         <x:v>[Excerpt from “Stayin’ Alive”; lyrics omitted.]</x:v>
       </x:c>
     </x:row>
-    <x:row r="231" ht="42" customHeight="1">
+    <x:row r="231" ht="120" customHeight="1">
       <x:c r="A231" s="19" t="str">
         <x:v>L:ANDMARSHALLEFT</x:v>
       </x:c>
@@ -2796,11 +3907,16 @@
       <x:c r="D231" s="20" t="str">
         <x:v>Marshal</x:v>
       </x:c>
-      <x:c r="E231" s="21" t="str">
+      <x:c r="E231" s="20" t="str">
         <x:v>Shared marshall/pisteur3 controller selects the left correction.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="232" ht="42" customHeight="1">
+      <x:c r="F231" s="25" t="str">
+        <x:v>1) Move left slowly.
+2) Be advised: move left slowly.
+3) Attention: move left slowly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232" ht="120" customHeight="1">
       <x:c r="A232" s="19" t="str">
         <x:v>L:ANDMARSHALRIGHT</x:v>
       </x:c>
@@ -2813,11 +3929,16 @@
       <x:c r="D232" s="20" t="str">
         <x:v>Marshal</x:v>
       </x:c>
-      <x:c r="E232" s="21" t="str">
+      <x:c r="E232" s="20" t="str">
         <x:v>Shared marshall/pisteur3 controller selects the right correction.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="233" ht="42" customHeight="1">
+      <x:c r="F232" s="25" t="str">
+        <x:v>1) Move right slowly.
+2) Be advised: move right slowly.
+3) Attention: move right slowly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233" ht="120" customHeight="1">
       <x:c r="A233" s="19" t="str">
         <x:v>L:ANDMARSHALFORWARD</x:v>
       </x:c>
@@ -2830,11 +3951,16 @@
       <x:c r="D233" s="20" t="str">
         <x:v>Marshal</x:v>
       </x:c>
-      <x:c r="E233" s="21" t="str">
+      <x:c r="E233" s="20" t="str">
         <x:v>Shared marshal controller commands the forward approach.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="234" ht="42" customHeight="1">
+      <x:c r="F233" s="25" t="str">
+        <x:v>1) Come forward slowly.
+2) Be advised: come forward slowly.
+3) Attention: come forward slowly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234" ht="120" customHeight="1">
       <x:c r="A234" s="19" t="str">
         <x:v>L:ANDMARSHALHOLD</x:v>
       </x:c>
@@ -2847,11 +3973,16 @@
       <x:c r="D234" s="20" t="str">
         <x:v>Marshal</x:v>
       </x:c>
-      <x:c r="E234" s="21" t="str">
+      <x:c r="E234" s="20" t="str">
         <x:v>Marshal controller enters the hold or safety-buffer state.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="235" ht="42" customHeight="1">
+      <x:c r="F234" s="25" t="str">
+        <x:v>1) Hold position.
+2) Maintain position.
+3) Maintain your position.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235" ht="120" customHeight="1">
       <x:c r="A235" s="19" t="str">
         <x:v>L:ANDMARSHALLANDCLEAR</x:v>
       </x:c>
@@ -2864,11 +3995,16 @@
       <x:c r="D235" s="20" t="str">
         <x:v>Marshal</x:v>
       </x:c>
-      <x:c r="E235" s="21" t="str">
+      <x:c r="E235" s="20" t="str">
         <x:v>A valid landing is committed inside the configured landing area.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="236" ht="42" customHeight="1">
+      <x:c r="F235" s="25" t="str">
+        <x:v>1) Landing area clear. You are cleared to land.
+2) Landing area clear. You're cleared to land.
+3) Attention: landing area clear. You are cleared to land.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236" ht="120" customHeight="1">
       <x:c r="A236" s="19" t="str">
         <x:v>L:ANDMEDASSESSMENT</x:v>
       </x:c>
@@ -2881,11 +4017,16 @@
       <x:c r="D236" s="20" t="str">
         <x:v>Medical crew</x:v>
       </x:c>
-      <x:c r="E236" s="21" t="str">
+      <x:c r="E236" s="20" t="str">
         <x:v>Crew visit begins and the tablet starts revealing clinical data.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="237" ht="42" customHeight="1">
+      <x:c r="F236" s="25" t="str">
+        <x:v>1) Patient assessment in progress. Stand by for the treatment decision.
+2) Be advised: patient assessment in progress. Stand by for the treatment decision.
+3) Attention: patient assessment in progress. Stand by for the treatment decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237" ht="120" customHeight="1">
       <x:c r="A237" s="19" t="str">
         <x:v>L:ANDMEDCRITICAL</x:v>
       </x:c>
@@ -2898,11 +4039,16 @@
       <x:c r="D237" s="20" t="str">
         <x:v>Medical crew</x:v>
       </x:c>
-      <x:c r="E237" s="21" t="str">
+      <x:c r="E237" s="20" t="str">
         <x:v>Critical-vitals indicators turn red, patient deterioration requires an urgent transport decision.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="238" ht="42" customHeight="1">
+      <x:c r="F237" s="25" t="str">
+        <x:v>1) Critical vital signs. Prepare for immediate transport.
+2) Be advised: critical vital signs. Prepare for immediate transport.
+3) Attention: critical vital signs. Prepare for immediate transport.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238" ht="120" customHeight="1">
       <x:c r="A238" s="19" t="str">
         <x:v>L:ANDMEDTRANSPORT</x:v>
       </x:c>
@@ -2915,11 +4061,16 @@
       <x:c r="D238" s="20" t="str">
         <x:v>Medical crew</x:v>
       </x:c>
-      <x:c r="E238" s="21" t="str">
+      <x:c r="E238" s="20" t="str">
         <x:v>Treatment result allows the loading or transport branch to start.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="239" ht="42" customHeight="1">
+      <x:c r="F238" s="25" t="str">
+        <x:v>1) Patient stabilized for transport. Prepare the cabin for loading.
+2) Be advised: patient stabilized for transport. Prepare the cabin for loading.
+3) Attention: patient stabilized for transport. Prepare the cabin for loading.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239" ht="120" customHeight="1">
       <x:c r="A239" s="19" t="str">
         <x:v>L:ANDCPRAWAITLAND</x:v>
       </x:c>
@@ -2932,11 +4083,16 @@
       <x:c r="D239" s="20" t="str">
         <x:v>Medical crew</x:v>
       </x:c>
-      <x:c r="E239" s="21" t="str">
+      <x:c r="E239" s="20" t="str">
         <x:v>L:CPR becomes 1 while airborne and MCPR_ONBOARD is disabled.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="240" ht="42" customHeight="1">
+      <x:c r="F239" s="25" t="str">
+        <x:v>1) CPR is required. Land as soon as safely possible before treatment can start.
+2) Be advised: cPR is required. Land as soon as safely possible before treatment can start.
+3) Attention: cPR is required. Land as soon as safely possible before treatment can start.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240" ht="120" customHeight="1">
       <x:c r="A240" s="19" t="str">
         <x:v>L:ANDCPRSTOPPED</x:v>
       </x:c>
@@ -2949,11 +4105,16 @@
       <x:c r="D240" s="20" t="str">
         <x:v>Medical crew</x:v>
       </x:c>
-      <x:c r="E240" s="21" t="str">
+      <x:c r="E240" s="20" t="str">
         <x:v>The tablet STOP CPR action sets L:CPR to 5.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="241" ht="42" customHeight="1">
+      <x:c r="F240" s="25" t="str">
+        <x:v>1) CPR has been stopped. Continue monitoring and follow the clinical plan.
+2) Be advised: cPR has been stopped. Continue monitoring and follow the clinical plan.
+3) Attention: cPR has been stopped. Continue monitoring and follow the clinical plan.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241" ht="120" customHeight="1">
       <x:c r="A241" s="19" t="str">
         <x:v>L:ANDAMBUHANDOVER</x:v>
       </x:c>
@@ -2966,11 +4127,16 @@
       <x:c r="D241" s="20" t="str">
         <x:v>Ground support</x:v>
       </x:c>
-      <x:c r="E241" s="21" t="str">
+      <x:c r="E241" s="20" t="str">
         <x:v>Ambulance arrival completes, before the patient-transfer branch begins.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="242" ht="42" customHeight="1">
+      <x:c r="F241" s="25" t="str">
+        <x:v>1) Ambulance is on scene. Prepare for patient handover.
+2) Be advised: ambulance is on scene. Prepare for patient handover.
+3) Attention: ambulance is on scene. Prepare for patient handover.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242" ht="120" customHeight="1">
       <x:c r="A242" s="19" t="str">
         <x:v>L:ANDSECONDAMBULANCE</x:v>
       </x:c>
@@ -2983,11 +4149,16 @@
       <x:c r="D242" s="20" t="str">
         <x:v>Ground support</x:v>
       </x:c>
-      <x:c r="E242" s="21" t="str">
+      <x:c r="E242" s="20" t="str">
         <x:v>Secondary-rescue flow assigns ambulance 2 to patient 2 or patient 3.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="243" ht="42" customHeight="1">
+      <x:c r="F242" s="25" t="str">
+        <x:v>1) A second ambulance is managing another patient. Keep the landing area clear.
+2) Be advised: a second ambulance is managing another patient. Keep the landing area clear.
+3) Attention: a second ambulance is managing another patient. Keep the landing area clear.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243" ht="120" customHeight="1">
       <x:c r="A243" s="19" t="str">
         <x:v>L:ANDPOLICESECURING</x:v>
       </x:c>
@@ -3000,11 +4171,16 @@
       <x:c r="D243" s="20" t="str">
         <x:v>Ground support</x:v>
       </x:c>
-      <x:c r="E243" s="21" t="str">
+      <x:c r="E243" s="20" t="str">
         <x:v>Police arrival and the scene-security/privacy-screen path begin.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="244" ht="42" customHeight="1">
+      <x:c r="F243" s="25" t="str">
+        <x:v>1) Police are securing the scene. Stay clear until the area is released.
+2) Be advised: police are securing the scene. Stay clear until the area is released.
+3) Attention: police are securing the scene. Stay clear until the area is released.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244" ht="120" customHeight="1">
       <x:c r="A244" s="19" t="str">
         <x:v>L:ANDFIREHAZARD</x:v>
       </x:c>
@@ -3017,11 +4193,16 @@
       <x:c r="D244" s="20" t="str">
         <x:v>Ground support</x:v>
       </x:c>
-      <x:c r="E244" s="21" t="str">
+      <x:c r="E244" s="20" t="str">
         <x:v>Fire-engine or fire-hazard branch is active.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="245" ht="42" customHeight="1">
+      <x:c r="F244" s="25" t="str">
+        <x:v>1) Fire service is controlling a hazard. Do not land until cleared.
+2) Be advised: fire service is controlling a hazard. Do not land until cleared.
+3) Attention: fire service is controlling a hazard. Do not land until cleared.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245" ht="120" customHeight="1">
       <x:c r="A245" s="19" t="str">
         <x:v>L:ANDOPSGROUNDDELAY</x:v>
       </x:c>
@@ -3034,11 +4215,16 @@
       <x:c r="D245" s="20" t="str">
         <x:v>Flight or ground crew</x:v>
       </x:c>
-      <x:c r="E245" s="21" t="str">
+      <x:c r="E245" s="20" t="str">
         <x:v>ops_progress_warning becomes 1 after 120 seconds without progress; tablet shows the orange Dispatch warning.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="246" ht="42" customHeight="1">
+      <x:c r="F245" s="25" t="str">
+        <x:v>1) Ground operations are delayed. Check the Dispatch page for the current status.
+2) Be advised: ground operations are delayed. Check the Dispatch page for the current status.
+3) Attention: ground operations are delayed. Check the Dispatch page for the current status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246" ht="120" customHeight="1">
       <x:c r="A246" s="19" t="str">
         <x:v>L:ANDHOISTPAUSE</x:v>
       </x:c>
@@ -3051,11 +4237,16 @@
       <x:c r="D246" s="20" t="str">
         <x:v>Hoist operator</x:v>
       </x:c>
-      <x:c r="E246" s="21" t="str">
+      <x:c r="E246" s="20" t="str">
         <x:v>A speed, acceleration, or bank-angle limit requires a temporary hoist pause.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="247" ht="42" customHeight="1">
+      <x:c r="F246" s="25" t="str">
+        <x:v>1) Hold position. Hoist operation is paused until the aircraft is stable.
+2) Maintain position. Hoist operation is paused until the aircraft is stable.
+3) Maintain your position. Hoist operation is paused until the aircraft is stable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247" ht="120" customHeight="1">
       <x:c r="A247" s="19" t="str">
         <x:v>L:ANDHOISTABORT</x:v>
       </x:c>
@@ -3068,11 +4259,16 @@
       <x:c r="D247" s="20" t="str">
         <x:v>Hoist operator</x:v>
       </x:c>
-      <x:c r="E247" s="21" t="str">
+      <x:c r="E247" s="20" t="str">
         <x:v>An unsafe hoist state requires abort and recovery rather than continuation.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="248" ht="42" customHeight="1">
+      <x:c r="F247" s="25" t="str">
+        <x:v>1) Abort the hoist operation. Recover the crew only when conditions are safe.
+2) Be advised: abort the hoist operation. Recover the crew only when conditions are safe.
+3) Attention: abort the hoist operation. Recover the crew only when conditions are safe.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248" ht="120" customHeight="1">
       <x:c r="A248" s="19" t="str">
         <x:v>L:ANDROUTEUNAVAILABLE</x:v>
       </x:c>
@@ -3085,11 +4281,16 @@
       <x:c r="D248" s="20" t="str">
         <x:v>Pilot or copilot</x:v>
       </x:c>
-      <x:c r="E248" s="21" t="str">
+      <x:c r="E248" s="20" t="str">
         <x:v>routeupdate records a missing or failed destination after its retry.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="249" ht="42" customHeight="1">
+      <x:c r="F248" s="25" t="str">
+        <x:v>1) Route is unavailable. Select or confirm the destination on the tablet.
+2) Be advised: route is unavailable. Select or confirm the destination on the tablet.
+3) Attention: route is unavailable. Select or confirm the destination on the tablet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249" ht="120" customHeight="1">
       <x:c r="A249" s="19" t="str">
         <x:v>L:ANDROUTECHANGED</x:v>
       </x:c>
@@ -3102,11 +4303,16 @@
       <x:c r="D249" s="20" t="str">
         <x:v>Pilot or copilot</x:v>
       </x:c>
-      <x:c r="E249" s="21" t="str">
+      <x:c r="E249" s="20" t="str">
         <x:v>Hospital, pickup, or custom target changes and the route is recalculated.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="250" ht="42" customHeight="1">
+      <x:c r="F249" s="25" t="str">
+        <x:v>1) Destination changed. Check the revised route on the tablet.
+2) Be advised: destination changed. Check the revised route on the tablet.
+3) Attention: destination changed. Check the revised route on the tablet.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250" ht="120" customHeight="1">
       <x:c r="A250" s="19" t="str">
         <x:v>L:ANDDISPATCHCANCELLED</x:v>
       </x:c>
@@ -3119,11 +4325,16 @@
       <x:c r="D250" s="20" t="str">
         <x:v>Dispatch</x:v>
       </x:c>
-      <x:c r="E250" s="21" t="str">
+      <x:c r="E250" s="20" t="str">
         <x:v>Cancellation criteria end the current dispatch; HEMS must not continue intervention.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="251" ht="42" customHeight="1">
+      <x:c r="F250" s="25" t="str">
+        <x:v>1) Dispatch cancelled. Follow the instructions on the tablet and await reassignment.
+2) Be advised: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
+3) Attention: dispatch cancelled. Follow the instructions on the tablet and await reassignment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251" ht="120" customHeight="1">
       <x:c r="A251" s="19" t="str">
         <x:v>L:ANDSTARTUPBLOCKED</x:v>
       </x:c>
@@ -3136,11 +4347,16 @@
       <x:c r="D251" s="20" t="str">
         <x:v>Pilot or copilot</x:v>
       </x:c>
-      <x:c r="E251" s="21" t="str">
+      <x:c r="E251" s="20" t="str">
         <x:v>marshall_ground_ops_active or pisteur3_guidance_active blocks a first-pump start request.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="252" ht="42" customHeight="1">
+      <x:c r="F251" s="25" t="str">
+        <x:v>1) Hold engine start. Ground operations are still in progress.
+2) Be advised: hold engine start. Ground operations are still in progress.
+3) Attention: hold engine start. Ground operations are still in progress.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252" ht="120" customHeight="1">
       <x:c r="A252" s="19" t="str">
         <x:v>L:ANDMAINTENANCEHOLD</x:v>
       </x:c>
@@ -3153,11 +4369,16 @@
       <x:c r="D252" s="20" t="str">
         <x:v>Technician</x:v>
       </x:c>
-      <x:c r="E252" s="21" t="str">
+      <x:c r="E252" s="20" t="str">
         <x:v>A failure or hard landing requires inspection before the next release.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="253" ht="42" customHeight="1">
+      <x:c r="F252" s="25" t="str">
+        <x:v>1) Aircraft requires inspection. Do not depart until maintenance releases it.
+2) Be advised: aircraft requires inspection. Do not depart until maintenance releases it.
+3) Attention: aircraft requires inspection. Do not depart until maintenance releases it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253" ht="120" customHeight="1">
       <x:c r="A253" s="19" t="str">
         <x:v>L:ANDMULTIPLEPATIENTS</x:v>
       </x:c>
@@ -3170,11 +4391,16 @@
       <x:c r="D253" s="20" t="str">
         <x:v>Crew chief</x:v>
       </x:c>
-      <x:c r="E253" s="21" t="str">
+      <x:c r="E253" s="20" t="str">
         <x:v>Patient 2 or 3 remains active, or secondary rescue begins.</x:v>
       </x:c>
-    </x:row>
-    <x:row r="254" ht="42" customHeight="1">
+      <x:c r="F253" s="25" t="str">
+        <x:v>1) Additional patients remain on scene. Await tasking before departure.
+2) Be advised: additional patients remain on scene. Await tasking before departure.
+3) Attention: additional patients remain on scene. Await tasking before departure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254" ht="120" customHeight="1">
       <x:c r="A254" s="22" t="str">
         <x:v>L:ANDCREWRETURNING</x:v>
       </x:c>
@@ -3187,8 +4413,13 @@
       <x:c r="D254" s="23" t="str">
         <x:v>Crew chief</x:v>
       </x:c>
-      <x:c r="E254" s="24" t="str">
+      <x:c r="E254" s="23" t="str">
         <x:v>Post-visit, post-load, or post-hoist crew-return flow begins.</x:v>
+      </x:c>
+      <x:c r="F254" s="26" t="str">
+        <x:v>1) Ground crew is returning to the aircraft. Keep the landing area clear.
+2) Be advised: ground crew is returning to the aircraft. Keep the landing area clear.
+3) Attention: ground crew is returning to the aircraft. Keep the landing area clear.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Separate corrections from alternative voice proposals
</commit_message>
<xml_diff>
--- a/docs/AND_voice_messages.xlsx
+++ b/docs/AND_voice_messages.xlsx
@@ -229,15 +229,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:F254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F254"/>
-  <x:tableColumns count="6">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndVoiceMessages" displayName="AndVoiceMessages" ref="A1:G254" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:G254"/>
+  <x:tableColumns count="7">
     <x:tableColumn id="1" name="LVAR"/>
     <x:tableColumn id="2" name="nome file"/>
     <x:tableColumn id="3" name="testo del messaggio"/>
     <x:tableColumn id="4" name="ruolo"/>
     <x:tableColumn id="5" name="trigger (azione / tablet)"/>
     <x:tableColumn id="6" name="correzioni proposte"/>
+    <x:tableColumn id="7" name="proposte alternative"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -253,6 +254,7 @@
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="78" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="112" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="108" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -272,7 +274,10 @@
         <x:v>trigger (azione / tablet)</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>correzioni proposte</x:v>
+        <x:v>correzione proposta</x:v>
+      </x:c>
+      <x:c r="G1" s="10" t="str">
+        <x:v>proposte alternative</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
@@ -363,9 +368,12 @@
         <x:v>We are experiencing issues with the safety straps we cannot use rescue hoist sorry we are forced to land.</x:v>
       </x:c>
       <x:c r="F9" s="25" t="str">
-        <x:v>1) We have a problem with the safety straps. We cannot use the rescue hoist and must land.
-2) We have a problem with the safety straps. We can't use the rescue hoist and must land.
-3) Attention: we have a problem with the safety straps. We cannot use the rescue hoist and must land.</x:v>
+        <x:v>We have a problem with the safety straps. We cannot use the rescue hoist and must land.</x:v>
+      </x:c>
+      <x:c r="G9" s="25" t="str">
+        <x:v>1) We have a problem with the safety straps. We can't use the rescue hoist and must land.
+2) Attention: we have a problem with the safety straps. We cannot use the rescue hoist and must land.
+3) For information: we have a problem with the safety straps. We cannot use the rescue hoist and must land.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="120" hidden="0" customHeight="1">
@@ -379,9 +387,12 @@
         <x:v>Hey crew there is an emergency message from dispatcher you have to read it it's unbelievable.</x:v>
       </x:c>
       <x:c r="F10" s="25" t="str">
-        <x:v>1) Crew, there is an emergency message from Dispatch. Please read it.
-2) Be advised: crew, there is an emergency message from Dispatch. Please read it.
-3) All crew, there is an emergency message from Dispatch. Please read it.</x:v>
+        <x:v>Crew, there is an emergency message from Dispatch. Please read it.</x:v>
+      </x:c>
+      <x:c r="G10" s="25" t="str">
+        <x:v>1) Be advised: crew, there is an emergency message from Dispatch. Please read it.
+2) All crew, there is an emergency message from Dispatch. Please read it.
+3) For information: crew, there is an emergency message from Dispatch. Please read it.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="120" hidden="0" customHeight="1">
@@ -395,9 +406,12 @@
         <x:v>Smoke and fire everywhere it seems a war movie scene out there.</x:v>
       </x:c>
       <x:c r="F11" s="25" t="str">
-        <x:v>1) Smoke and fire everywhere. It looks like a war zone out there.
-2) Be advised: smoke and fire everywhere. It looks like a war zone out there.
-3) Attention: smoke and fire everywhere. It looks like a war zone out there.</x:v>
+        <x:v>Smoke and fire everywhere. It looks like a war zone out there.</x:v>
+      </x:c>
+      <x:c r="G11" s="25" t="str">
+        <x:v>1) Be advised: smoke and fire everywhere. It looks like a war zone out there.
+2) Attention: smoke and fire everywhere. It looks like a war zone out there.
+3) For information: smoke and fire everywhere. It looks like a war zone out there.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="120" hidden="0" customHeight="1">
@@ -411,9 +425,12 @@
         <x:v>Damn engine fire crew we have an engine fire.</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
-        <x:v>1) Crew, we have an engine fire.
-2) Be advised: crew, we have an engine fire.
-3) All crew, we have an engine fire.</x:v>
+        <x:v>Crew, we have an engine fire.</x:v>
+      </x:c>
+      <x:c r="G12" s="25" t="str">
+        <x:v>1) Be advised: crew, we have an engine fire.
+2) All crew, we have an engine fire.
+3) For information: crew, we have an engine fire.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="120" hidden="0" customHeight="1">
@@ -427,9 +444,12 @@
         <x:v>Copilot confirmed engine two fire.</x:v>
       </x:c>
       <x:c r="F13" s="25" t="str">
-        <x:v>1) Copilot confirms an engine two fire.
-2) Be advised: copilot confirms an engine two fire.
-3) Attention: copilot confirms an engine two fire.</x:v>
+        <x:v>Copilot confirms an engine two fire.</x:v>
+      </x:c>
+      <x:c r="G13" s="25" t="str">
+        <x:v>1) Be advised: copilot confirms an engine two fire.
+2) Attention: copilot confirms an engine two fire.
+3) For information: copilot confirms an engine two fire.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="120" hidden="0" customHeight="1">
@@ -443,9 +463,12 @@
         <x:v>Engine two confirmed.</x:v>
       </x:c>
       <x:c r="F14" s="25" t="str">
-        <x:v>1) Engine two fire confirmed.
-2) Be advised: engine two fire confirmed.
-3) Attention: engine two fire confirmed.</x:v>
+        <x:v>Engine two fire confirmed.</x:v>
+      </x:c>
+      <x:c r="G14" s="25" t="str">
+        <x:v>1) Be advised: engine two fire confirmed.
+2) Attention: engine two fire confirmed.
+3) For information: engine two fire confirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="120" hidden="0" customHeight="1">
@@ -459,9 +482,12 @@
         <x:v>Engine two fire. Push bottle one and hope it goes off; crew, prepare to evacuate the helicopter.</x:v>
       </x:c>
       <x:c r="F15" s="25" t="str">
-        <x:v>1) Engine two fire. Discharge bottle one; crew, prepare to evacuate.
-2) Be advised: engine two fire. Discharge bottle one; crew, prepare to evacuate.
-3) Attention: engine two fire. Discharge bottle one; crew, prepare to evacuate.</x:v>
+        <x:v>Engine two fire. Discharge bottle one; crew, prepare to evacuate.</x:v>
+      </x:c>
+      <x:c r="G15" s="25" t="str">
+        <x:v>1) Be advised: engine two fire. Discharge bottle one; crew, prepare to evacuate.
+2) Attention: engine two fire. Discharge bottle one; crew, prepare to evacuate.
+3) For information: engine two fire. Discharge bottle one; crew, prepare to evacuate.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="120" hidden="0" customHeight="1">
@@ -475,9 +501,12 @@
         <x:v>Fire is extinguished however we have multiple failures i'm not sure we can take off again in this condition.</x:v>
       </x:c>
       <x:c r="F16" s="25" t="str">
-        <x:v>1) The fire is out, but we have multiple failures. I am not sure we can take off again.
-2) The fire is out, but we have multiple failures. I'm not sure we can take off again.
-3) Attention: the fire is out, but we have multiple failures. I am not sure we can take off again.</x:v>
+        <x:v>The fire is out, but we have multiple failures. I am not sure we can take off again.</x:v>
+      </x:c>
+      <x:c r="G16" s="25" t="str">
+        <x:v>1) The fire is out, but we have multiple failures. I'm not sure we can take off again.
+2) Attention: the fire is out, but we have multiple failures. I am not sure we can take off again.
+3) For information: the fire is out, but we have multiple failures. I am not sure we can take off again.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="120" hidden="0" customHeight="1">
@@ -491,9 +520,12 @@
         <x:v>What the hell is happening here.</x:v>
       </x:c>
       <x:c r="F17" s="25" t="str">
-        <x:v>1) What the hell is happening here.
-2) Be advised: what the hell is happening here.
-3) Attention: what the hell is happening here.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G17" s="25" t="str">
+        <x:v>1) Be advised: what the hell is happening here.
+2) Attention: what the hell is happening here.
+3) For information: what the hell is happening here.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="120" hidden="0" customHeight="1">
@@ -507,9 +539,12 @@
         <x:v>There is something bad happening in the area we have to be careful while completing tasks.</x:v>
       </x:c>
       <x:c r="F18" s="25" t="str">
-        <x:v>1) Something is wrong in the area. Remain alert while completing the mission.
-2) Be advised: something is wrong in the area. Remain alert while completing the mission.
-3) Attention: something is wrong in the area. Remain alert while completing the mission.</x:v>
+        <x:v>Something is wrong in the area. Remain alert while completing the mission.</x:v>
+      </x:c>
+      <x:c r="G18" s="25" t="str">
+        <x:v>1) Be advised: something is wrong in the area. Remain alert while completing the mission.
+2) Attention: something is wrong in the area. Remain alert while completing the mission.
+3) For information: something is wrong in the area. Remain alert while completing the mission.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="120" hidden="0" customHeight="1">
@@ -523,9 +558,12 @@
         <x:v>Did you see them hey what hey guys did you see them is that happening to us they are coming here are they.</x:v>
       </x:c>
       <x:c r="F19" s="25" t="str">
-        <x:v>1) Did you see that? Guys, are they coming toward us?
-2) Can you confirm: did you see that? Guys, are they coming toward us?
-3) Please confirm: did you see that? Guys, are they coming toward us?</x:v>
+        <x:v>Did you see that? Guys, are they coming toward us?</x:v>
+      </x:c>
+      <x:c r="G19" s="25" t="str">
+        <x:v>1) Can you confirm: did you see that? Guys, are they coming toward us?
+2) Please confirm: did you see that? Guys, are they coming toward us?
+3) Message update: did you see that? Guys, are they coming toward us?</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="120" hidden="0" customHeight="1">
@@ -539,9 +577,12 @@
         <x:v>We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
       </x:c>
       <x:c r="F20" s="25" t="str">
-        <x:v>1) We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
-2) Be advised: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
-3) Attention: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G20" s="25" t="str">
+        <x:v>1) Be advised: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
+2) Attention: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
+3) For information: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="120" hidden="0" customHeight="1">
@@ -555,9 +596,12 @@
         <x:v>Doc refers they have almost done we should wait for them to return.</x:v>
       </x:c>
       <x:c r="F21" s="25" t="str">
-        <x:v>1) The doctor says they are almost finished. We should wait for their return.
-2) Be advised: the doctor says they are almost finished. We should wait for their return.
-3) Attention: the doctor says they are almost finished. We should wait for their return.</x:v>
+        <x:v>The doctor says they are almost finished. We should wait for their return.</x:v>
+      </x:c>
+      <x:c r="G21" s="25" t="str">
+        <x:v>1) Be advised: the doctor says they are almost finished. We should wait for their return.
+2) Attention: the doctor says they are almost finished. We should wait for their return.
+3) For information: the doctor says they are almost finished. We should wait for their return.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="120" hidden="0" customHeight="1">
@@ -571,9 +615,12 @@
         <x:v>Okay finished go away now go go go.</x:v>
       </x:c>
       <x:c r="F22" s="25" t="str">
-        <x:v>1) Okay, finished. Move away now; go, go, go.
-2) Be advised: okay, finished. Move away now; go, go, go.
-3) Attention: okay, finished. Move away now; go, go, go.</x:v>
+        <x:v>Okay, finished. Move away now; go, go, go.</x:v>
+      </x:c>
+      <x:c r="G22" s="25" t="str">
+        <x:v>1) Be advised: okay, finished. Move away now; go, go, go.
+2) Attention: okay, finished. Move away now; go, go, go.
+3) For information: okay, finished. Move away now; go, go, go.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="120" hidden="0" customHeight="1">
@@ -587,9 +634,12 @@
         <x:v>We're going to try and oh he i take off it will be difficult if needed be prepared for immediate evacuation.</x:v>
       </x:c>
       <x:c r="F23" s="25" t="str">
-        <x:v>1) We are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
-2) We're going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
-3) Attention: we are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.</x:v>
+        <x:v>We are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.</x:v>
+      </x:c>
+      <x:c r="G23" s="25" t="str">
+        <x:v>1) We're going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
+2) Attention: we are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.
+3) For information: we are going to attempt takeoff. It may be difficult; prepare for an immediate evacuation if required.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="120" hidden="0" customHeight="1">
@@ -603,9 +653,12 @@
         <x:v>Cabin preparation completed.</x:v>
       </x:c>
       <x:c r="F24" s="25" t="str">
-        <x:v>1) Cabin preparation completed.
-2) Be advised: cabin preparation completed.
-3) Attention: cabin preparation completed.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G24" s="25" t="str">
+        <x:v>1) Be advised: cabin preparation completed.
+2) Attention: cabin preparation completed.
+3) For information: cabin preparation completed.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="120" hidden="0" customHeight="1">
@@ -619,9 +672,12 @@
         <x:v>Cabin preparation please wait.</x:v>
       </x:c>
       <x:c r="F25" s="25" t="str">
-        <x:v>1) Cabin preparation is in progress. Please wait.
-2) Be advised: cabin preparation is in progress. Please wait.
-3) Attention: cabin preparation is in progress. Please wait.</x:v>
+        <x:v>Cabin preparation is in progress. Please wait.</x:v>
+      </x:c>
+      <x:c r="G25" s="25" t="str">
+        <x:v>1) Be advised: cabin preparation is in progress. Please wait.
+2) Attention: cabin preparation is in progress. Please wait.
+3) For information: cabin preparation is in progress. Please wait.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="120" hidden="0" customHeight="1">
@@ -635,9 +691,12 @@
         <x:v>Cabin secured ready to fly.</x:v>
       </x:c>
       <x:c r="F26" s="25" t="str">
-        <x:v>1) Cabin secured and ready for flight.
-2) Be advised: cabin secured and ready for flight.
-3) Attention: cabin secured and ready for flight.</x:v>
+        <x:v>Cabin secured and ready for flight.</x:v>
+      </x:c>
+      <x:c r="G26" s="25" t="str">
+        <x:v>1) Be advised: cabin secured and ready for flight.
+2) Attention: cabin secured and ready for flight.
+3) For information: cabin secured and ready for flight.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="120" hidden="0" customHeight="1">
@@ -651,9 +710,12 @@
         <x:v>Hoist one plus stretcher to helicopter.</x:v>
       </x:c>
       <x:c r="F27" s="25" t="str">
-        <x:v>1) Bring hoist one and the stretcher to the helicopter.
-2) Be advised: bring hoist one and the stretcher to the helicopter.
-3) Attention: bring hoist one and the stretcher to the helicopter.</x:v>
+        <x:v>Bring hoist one and the stretcher to the helicopter.</x:v>
+      </x:c>
+      <x:c r="G27" s="25" t="str">
+        <x:v>1) Be advised: bring hoist one and the stretcher to the helicopter.
+2) Attention: bring hoist one and the stretcher to the helicopter.
+3) For information: bring hoist one and the stretcher to the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="120" hidden="0" customHeight="1">
@@ -667,9 +729,12 @@
         <x:v>Hoist one to helicopter; patient and doctor will go with ambulance.</x:v>
       </x:c>
       <x:c r="F28" s="25" t="str">
-        <x:v>1) Hoist one to the helicopter. The patient and doctor will travel by ambulance.
-2) Be advised: hoist one to the helicopter. The patient and doctor will travel by ambulance.
-3) Attention: hoist one to the helicopter. The patient and doctor will travel by ambulance.</x:v>
+        <x:v>Hoist one to the helicopter. The patient and doctor will travel by ambulance.</x:v>
+      </x:c>
+      <x:c r="G28" s="25" t="str">
+        <x:v>1) Be advised: hoist one to the helicopter. The patient and doctor will travel by ambulance.
+2) Attention: hoist one to the helicopter. The patient and doctor will travel by ambulance.
+3) For information: hoist one to the helicopter. The patient and doctor will travel by ambulance.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="120" hidden="0" customHeight="1">
@@ -683,9 +748,12 @@
         <x:v>Hoist two to helicopter.</x:v>
       </x:c>
       <x:c r="F29" s="25" t="str">
-        <x:v>1) Hoist two to helicopter.
-2) Be advised: hoist two to helicopter.
-3) Attention: hoist two to helicopter.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G29" s="25" t="str">
+        <x:v>1) Be advised: hoist two to helicopter.
+2) Attention: hoist two to helicopter.
+3) For information: hoist two to helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="120" hidden="0" customHeight="1">
@@ -699,9 +767,12 @@
         <x:v>Hoist three to helicopter.</x:v>
       </x:c>
       <x:c r="F30" s="25" t="str">
-        <x:v>1) Hoist three to helicopter.
-2) Be advised: hoist three to helicopter.
-3) Attention: hoist three to helicopter.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G30" s="25" t="str">
+        <x:v>1) Be advised: hoist three to helicopter.
+2) Attention: hoist three to helicopter.
+3) For information: hoist three to helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="120" hidden="0" customHeight="1">
@@ -715,9 +786,12 @@
         <x:v>Hoist boom extended.</x:v>
       </x:c>
       <x:c r="F31" s="25" t="str">
-        <x:v>1) Hoist boom extended.
-2) Be advised: hoist boom extended.
-3) Attention: hoist boom extended.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G31" s="25" t="str">
+        <x:v>1) Be advised: hoist boom extended.
+2) Attention: hoist boom extended.
+3) For information: hoist boom extended.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="120" hidden="0" customHeight="1">
@@ -731,9 +805,12 @@
         <x:v>Hoist is clear.</x:v>
       </x:c>
       <x:c r="F32" s="25" t="str">
-        <x:v>1) Hoist is clear.
-2) Be advised: hoist is clear.
-3) Attention: hoist is clear.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G32" s="25" t="str">
+        <x:v>1) Be advised: hoist is clear.
+2) Attention: hoist is clear.
+3) For information: hoist is clear.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="120" hidden="0" customHeight="1">
@@ -747,9 +824,12 @@
         <x:v>Hoist is running down.</x:v>
       </x:c>
       <x:c r="F33" s="25" t="str">
-        <x:v>1) Hoist is running down.
-2) Be advised: hoist is running down.
-3) Attention: hoist is running down.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G33" s="25" t="str">
+        <x:v>1) Be advised: hoist is running down.
+2) Attention: hoist is running down.
+3) For information: hoist is running down.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="120" hidden="0" customHeight="1">
@@ -763,9 +843,12 @@
         <x:v>Hoist is running up.</x:v>
       </x:c>
       <x:c r="F34" s="25" t="str">
-        <x:v>1) Hoist is running up.
-2) Be advised: hoist is running up.
-3) Attention: hoist is running up.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G34" s="25" t="str">
+        <x:v>1) Be advised: hoist is running up.
+2) Attention: hoist is running up.
+3) For information: hoist is running up.</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="120" hidden="0" customHeight="1">
@@ -779,9 +862,12 @@
         <x:v>Hoist his up boom extended patient and doctor are outside hook to hoist.</x:v>
       </x:c>
       <x:c r="F35" s="25" t="str">
-        <x:v>1) Hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
-2) Be advised: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
-3) Attention: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.</x:v>
+        <x:v>Hoist is up and boom extended. The patient and doctor are clear and ready to hook on.</x:v>
+      </x:c>
+      <x:c r="G35" s="25" t="str">
+        <x:v>1) Be advised: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
+2) Attention: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.
+3) For information: hoist is up and boom extended. The patient and doctor are clear and ready to hook on.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="120" hidden="0" customHeight="1">
@@ -795,9 +881,12 @@
         <x:v>Hoist his up personnel is strapped in.</x:v>
       </x:c>
       <x:c r="F36" s="25" t="str">
-        <x:v>1) Hoist is up; personnel are strapped in.
-2) Be advised: hoist is up; personnel are strapped in.
-3) Attention: hoist is up; personnel are strapped in.</x:v>
+        <x:v>Hoist is up; personnel are strapped in.</x:v>
+      </x:c>
+      <x:c r="G36" s="25" t="str">
+        <x:v>1) Be advised: hoist is up; personnel are strapped in.
+2) Attention: hoist is up; personnel are strapped in.
+3) For information: hoist is up; personnel are strapped in.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="120" hidden="0" customHeight="1">
@@ -811,9 +900,12 @@
         <x:v>Hoist on ground personnel is getting hooked.</x:v>
       </x:c>
       <x:c r="F37" s="25" t="str">
-        <x:v>1) Hoist is on the ground. Personnel are being hooked on.
-2) Be advised: hoist is on the ground. Personnel are being hooked on.
-3) Attention: hoist is on the ground. Personnel are being hooked on.</x:v>
+        <x:v>Hoist is on the ground. Personnel are being hooked on.</x:v>
+      </x:c>
+      <x:c r="G37" s="25" t="str">
+        <x:v>1) Be advised: hoist is on the ground. Personnel are being hooked on.
+2) Attention: hoist is on the ground. Personnel are being hooked on.
+3) For information: hoist is on the ground. Personnel are being hooked on.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="120" hidden="0" customHeight="1">
@@ -827,9 +919,12 @@
         <x:v>Hold position.</x:v>
       </x:c>
       <x:c r="F38" s="25" t="str">
-        <x:v>1) Hold position.
-2) Maintain position.
-3) Maintain your position.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G38" s="25" t="str">
+        <x:v>1) Maintain position.
+2) Maintain your position.
+3) Please hold position.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="120" hidden="0" customHeight="1">
@@ -843,9 +938,12 @@
         <x:v>Hook is in hoist boomers retracted you're free to leave hover.</x:v>
       </x:c>
       <x:c r="F39" s="25" t="str">
-        <x:v>1) Hook is in and boom retracted. You are clear to leave the hover.
-2) Hook is in and boom retracted. You're clear to leave the hover.
-3) Attention: hook is in and boom retracted. You are clear to leave the hover.</x:v>
+        <x:v>Hook is in and boom retracted. You are clear to leave the hover.</x:v>
+      </x:c>
+      <x:c r="G39" s="25" t="str">
+        <x:v>1) Hook is in and boom retracted. You're clear to leave the hover.
+2) Attention: hook is in and boom retracted. You are clear to leave the hover.
+3) For information: hook is in and boom retracted. You are clear to leave the hover.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="120" hidden="0" customHeight="1">
@@ -859,9 +957,12 @@
         <x:v>Medical on ground and disconnected.</x:v>
       </x:c>
       <x:c r="F40" s="25" t="str">
-        <x:v>1) Medic is on the ground and disconnected.
-2) Be advised: medic is on the ground and disconnected.
-3) Attention: medic is on the ground and disconnected.</x:v>
+        <x:v>Medic is on the ground and disconnected.</x:v>
+      </x:c>
+      <x:c r="G40" s="25" t="str">
+        <x:v>1) Be advised: medic is on the ground and disconnected.
+2) Attention: medic is on the ground and disconnected.
+3) For information: medic is on the ground and disconnected.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="120" hidden="0" customHeight="1">
@@ -875,9 +976,12 @@
         <x:v>Patient will go with ambulance.</x:v>
       </x:c>
       <x:c r="F41" s="25" t="str">
-        <x:v>1) The patient will travel by ambulance.
-2) Be advised: the patient will travel by ambulance.
-3) Attention: the patient will travel by ambulance.</x:v>
+        <x:v>The patient will travel by ambulance.</x:v>
+      </x:c>
+      <x:c r="G41" s="25" t="str">
+        <x:v>1) Be advised: the patient will travel by ambulance.
+2) Attention: the patient will travel by ambulance.
+3) For information: the patient will travel by ambulance.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="120" hidden="0" customHeight="1">
@@ -891,9 +995,12 @@
         <x:v>Personnel on ground and disconnected.</x:v>
       </x:c>
       <x:c r="F42" s="25" t="str">
-        <x:v>1) Personnel are on the ground and disconnected.
-2) Be advised: personnel are on the ground and disconnected.
-3) Attention: personnel are on the ground and disconnected.</x:v>
+        <x:v>Personnel are on the ground and disconnected.</x:v>
+      </x:c>
+      <x:c r="G42" s="25" t="str">
+        <x:v>1) Be advised: personnel are on the ground and disconnected.
+2) Attention: personnel are on the ground and disconnected.
+3) For information: personnel are on the ground and disconnected.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="120" hidden="0" customHeight="1">
@@ -907,9 +1014,12 @@
         <x:v>Position is good.</x:v>
       </x:c>
       <x:c r="F43" s="25" t="str">
-        <x:v>1) Position is good.
-2) Be advised: position is good.
-3) Attention: position is good.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G43" s="25" t="str">
+        <x:v>1) Be advised: position is good.
+2) Attention: position is good.
+3) For information: position is good.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="120" hidden="0" customHeight="1">
@@ -923,9 +1033,12 @@
         <x:v>Hold on, hoisting preparation is in progress and almost completed.</x:v>
       </x:c>
       <x:c r="F44" s="25" t="str">
-        <x:v>1) Hold on, hoisting preparation is in progress and almost completed.
-2) Be advised: hold on, hoisting preparation is in progress and almost completed.
-3) Attention: hold on, hoisting preparation is in progress and almost completed.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G44" s="25" t="str">
+        <x:v>1) Be advised: hold on, hoisting preparation is in progress and almost completed.
+2) Attention: hold on, hoisting preparation is in progress and almost completed.
+3) Please hold on, hoisting preparation is in progress and almost completed.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="120" hidden="0" customHeight="1">
@@ -939,9 +1052,12 @@
         <x:v>Set hover conditions.</x:v>
       </x:c>
       <x:c r="F45" s="25" t="str">
-        <x:v>1) Set hover conditions.
-2) Be advised: set hover conditions.
-3) Attention: set hover conditions.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G45" s="25" t="str">
+        <x:v>1) Be advised: set hover conditions.
+2) Attention: set hover conditions.
+3) For information: set hover conditions.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="120" hidden="0" customHeight="1">
@@ -955,9 +1071,12 @@
         <x:v>That's one com check.</x:v>
       </x:c>
       <x:c r="F46" s="25" t="str">
-        <x:v>1) This is a communications check.
-2) Be advised: this is a communications check.
-3) Attention: this is a communications check.</x:v>
+        <x:v>This is a communications check.</x:v>
+      </x:c>
+      <x:c r="G46" s="25" t="str">
+        <x:v>1) Be advised: this is a communications check.
+2) Attention: this is a communications check.
+3) For information: this is a communications check.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="120" hidden="0" customHeight="1">
@@ -971,9 +1090,12 @@
         <x:v>Hoist wonder helicopter.</x:v>
       </x:c>
       <x:c r="F47" s="25" t="str">
-        <x:v>1) Hoist one to the helicopter.
-2) Be advised: hoist one to the helicopter.
-3) Attention: hoist one to the helicopter.</x:v>
+        <x:v>Hoist one to the helicopter.</x:v>
+      </x:c>
+      <x:c r="G47" s="25" t="str">
+        <x:v>1) Be advised: hoist one to the helicopter.
+2) Attention: hoist one to the helicopter.
+3) For information: hoist one to the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="120" hidden="0" customHeight="1">
@@ -987,9 +1109,12 @@
         <x:v>Ten.</x:v>
       </x:c>
       <x:c r="F48" s="25" t="str">
-        <x:v>1) Ten.
-2) Be advised: ten.
-3) Attention: ten.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G48" s="25" t="str">
+        <x:v>1) Be advised: ten.
+2) Attention: ten.
+3) For information: ten.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="120" hidden="0" customHeight="1">
@@ -1003,9 +1128,12 @@
         <x:v>Twenty.</x:v>
       </x:c>
       <x:c r="F49" s="25" t="str">
-        <x:v>1) Twenty.
-2) Be advised: twenty.
-3) Attention: twenty.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G49" s="25" t="str">
+        <x:v>1) Be advised: twenty.
+2) Attention: twenty.
+3) For information: twenty.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="120" hidden="0" customHeight="1">
@@ -1019,9 +1147,12 @@
         <x:v>Fifty meters.</x:v>
       </x:c>
       <x:c r="F50" s="25" t="str">
-        <x:v>1) Fifty meters.
-2) Be advised: fifty meters.
-3) Attention: fifty meters.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G50" s="25" t="str">
+        <x:v>1) Be advised: fifty meters.
+2) Attention: fifty meters.
+3) For information: fifty meters.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="120" hidden="0" customHeight="1">
@@ -1035,9 +1166,12 @@
         <x:v>Hey frank good morning.</x:v>
       </x:c>
       <x:c r="F51" s="25" t="str">
-        <x:v>1) Hey frank good morning.
-2) Be advised: hey frank good morning.
-3) Attention: hey frank good morning.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G51" s="25" t="str">
+        <x:v>1) Be advised: hey frank good morning.
+2) Attention: hey frank good morning.
+3) For information: hey frank good morning.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="120" hidden="0" customHeight="1">
@@ -1051,9 +1185,12 @@
         <x:v>Hi sarah how are you.</x:v>
       </x:c>
       <x:c r="F52" s="25" t="str">
-        <x:v>1) Hi sarah how are you.
-2) Be advised: hi sarah how are you.
-3) Attention: hi sarah how are you.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G52" s="25" t="str">
+        <x:v>1) Be advised: hi sarah how are you.
+2) Attention: hi sarah how are you.
+3) For information: hi sarah how are you.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="120" hidden="0" customHeight="1">
@@ -1067,9 +1204,12 @@
         <x:v>Stretcher is secure.</x:v>
       </x:c>
       <x:c r="F53" s="25" t="str">
-        <x:v>1) Stretcher is secure.
-2) Be advised: stretcher is secure.
-3) Attention: stretcher is secure.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G53" s="25" t="str">
+        <x:v>1) Be advised: stretcher is secure.
+2) Attention: stretcher is secure.
+3) For information: stretcher is secure.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="120" hidden="0" customHeight="1">
@@ -1083,9 +1223,12 @@
         <x:v>We are reasonably close said hover is appropriate.</x:v>
       </x:c>
       <x:c r="F54" s="25" t="str">
-        <x:v>1) We are close enough; set hover conditions.
-2) We're close enough; set hover conditions.
-3) Attention: we are close enough; set hover conditions.</x:v>
+        <x:v>We are close enough; set hover conditions.</x:v>
+      </x:c>
+      <x:c r="G54" s="25" t="str">
+        <x:v>1) We're close enough; set hover conditions.
+2) Attention: we are close enough; set hover conditions.
+3) For information: we are close enough; set hover conditions.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="120" hidden="0" customHeight="1">
@@ -1099,9 +1242,12 @@
         <x:v>We are reasonably close.</x:v>
       </x:c>
       <x:c r="F55" s="25" t="str">
-        <x:v>1) We are reasonably close.
-2) We're reasonably close.
-3) Attention: we are reasonably close.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G55" s="25" t="str">
+        <x:v>1) We're reasonably close.
+2) Attention: we are reasonably close.
+3) For information: we are reasonably close.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="120" hidden="0" customHeight="1">
@@ -1115,9 +1261,12 @@
         <x:v>We are too far.</x:v>
       </x:c>
       <x:c r="F56" s="25" t="str">
-        <x:v>1) We are too far.
-2) We're too far.
-3) Attention: we are too far.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G56" s="25" t="str">
+        <x:v>1) We're too far.
+2) Attention: we are too far.
+3) For information: we are too far.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="120" hidden="0" customHeight="1">
@@ -1131,9 +1280,12 @@
         <x:v>Height is good.</x:v>
       </x:c>
       <x:c r="F57" s="25" t="str">
-        <x:v>1) Height is good.
-2) Be advised: height is good.
-3) Attention: height is good.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G57" s="25" t="str">
+        <x:v>1) Be advised: height is good.
+2) Attention: height is good.
+3) For information: height is good.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="120" hidden="0" customHeight="1">
@@ -1147,9 +1299,12 @@
         <x:v>We are too high.</x:v>
       </x:c>
       <x:c r="F58" s="25" t="str">
-        <x:v>1) We are too high.
-2) We're too high.
-3) Attention: we are too high.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G58" s="25" t="str">
+        <x:v>1) We're too high.
+2) Attention: we are too high.
+3) For information: we are too high.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="120" hidden="0" customHeight="1">
@@ -1163,9 +1318,12 @@
         <x:v>We are too low.</x:v>
       </x:c>
       <x:c r="F59" s="25" t="str">
-        <x:v>1) We are too low.
-2) We're too low.
-3) Attention: we are too low.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G59" s="25" t="str">
+        <x:v>1) We're too low.
+2) Attention: we are too low.
+3) For information: we are too low.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="120" hidden="0" customHeight="1">
@@ -1179,9 +1337,12 @@
         <x:v>Doc and stretcher have been disconnected.</x:v>
       </x:c>
       <x:c r="F60" s="25" t="str">
-        <x:v>1) The doctor and stretcher are disconnected.
-2) Be advised: the doctor and stretcher are disconnected.
-3) Attention: the doctor and stretcher are disconnected.</x:v>
+        <x:v>The doctor and stretcher are disconnected.</x:v>
+      </x:c>
+      <x:c r="G60" s="25" t="str">
+        <x:v>1) Be advised: the doctor and stretcher are disconnected.
+2) Attention: the doctor and stretcher are disconnected.
+3) For information: the doctor and stretcher are disconnected.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="120" hidden="0" customHeight="1">
@@ -1195,9 +1356,12 @@
         <x:v>Doc is getting hooked.</x:v>
       </x:c>
       <x:c r="F61" s="25" t="str">
-        <x:v>1) Doc is getting hooked.
-2) Be advised: doc is getting hooked.
-3) Attention: doc is getting hooked.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G61" s="25" t="str">
+        <x:v>1) Be advised: doc is getting hooked.
+2) Attention: doc is getting hooked.
+3) For information: doc is getting hooked.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="120" hidden="0" customHeight="1">
@@ -1211,9 +1375,12 @@
         <x:v>Hoist storm extended.</x:v>
       </x:c>
       <x:c r="F62" s="25" t="str">
-        <x:v>1) Hoist boom extended.
-2) Be advised: hoist boom extended.
-3) Attention: hoist boom extended.</x:v>
+        <x:v>Hoist boom extended.</x:v>
+      </x:c>
+      <x:c r="G62" s="25" t="str">
+        <x:v>1) Be advised: hoist boom extended.
+2) Attention: hoist boom extended.
+3) For information: hoist boom extended.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="120" hidden="0" customHeight="1">
@@ -1227,9 +1394,12 @@
         <x:v>Hoist retracted door closed cabin secured.</x:v>
       </x:c>
       <x:c r="F63" s="25" t="str">
-        <x:v>1) Hoist retracted, door closed, cabin secured.
-2) Be advised: hoist retracted, door closed, cabin secured.
-3) Attention: hoist retracted, door closed, cabin secured.</x:v>
+        <x:v>Hoist retracted, door closed, cabin secured.</x:v>
+      </x:c>
+      <x:c r="G63" s="25" t="str">
+        <x:v>1) Be advised: hoist retracted, door closed, cabin secured.
+2) Attention: hoist retracted, door closed, cabin secured.
+3) For information: hoist retracted, door closed, cabin secured.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="120" hidden="0" customHeight="1">
@@ -1243,9 +1413,12 @@
         <x:v>Opening door and preparing for hoist operation.</x:v>
       </x:c>
       <x:c r="F64" s="25" t="str">
-        <x:v>1) Opening door and preparing for hoist operation.
-2) Be advised: opening door and preparing for hoist operation.
-3) Attention: opening door and preparing for hoist operation.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G64" s="25" t="str">
+        <x:v>1) Be advised: opening door and preparing for hoist operation.
+2) Attention: opening door and preparing for hoist operation.
+3) For information: opening door and preparing for hoist operation.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="120" hidden="0" customHeight="1">
@@ -1259,9 +1432,12 @@
         <x:v>Operator has been disconnected.</x:v>
       </x:c>
       <x:c r="F65" s="25" t="str">
-        <x:v>1) Operator has been disconnected.
-2) Be advised: operator has been disconnected.
-3) Attention: operator has been disconnected.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G65" s="25" t="str">
+        <x:v>1) Be advised: operator has been disconnected.
+2) Attention: operator has been disconnected.
+3) For information: operator has been disconnected.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="120" hidden="0" customHeight="1">
@@ -1275,9 +1451,12 @@
         <x:v>Operator is getting hooked.</x:v>
       </x:c>
       <x:c r="F66" s="25" t="str">
-        <x:v>1) Operator is getting hooked.
-2) Be advised: operator is getting hooked.
-3) Attention: operator is getting hooked.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G66" s="25" t="str">
+        <x:v>1) Be advised: operator is getting hooked.
+2) Attention: operator is getting hooked.
+3) For information: operator is getting hooked.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="120" hidden="0" customHeight="1">
@@ -1291,9 +1470,12 @@
         <x:v>Crew boarded cabin ready to go.</x:v>
       </x:c>
       <x:c r="F67" s="25" t="str">
-        <x:v>1) Crew boarded, cabin ready to go.
-2) Be advised: crew boarded, cabin ready to go.
-3) Attention: crew boarded, cabin ready to go.</x:v>
+        <x:v>Crew boarded, cabin ready to go.</x:v>
+      </x:c>
+      <x:c r="G67" s="25" t="str">
+        <x:v>1) Be advised: crew boarded, cabin ready to go.
+2) Attention: crew boarded, cabin ready to go.
+3) For information: crew boarded, cabin ready to go.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="24" hidden="0" customHeight="1">
@@ -1307,9 +1489,12 @@
         <x:v>Due to impervious location of accident site we should evaluate to call and board expert heli-rescuers use the tablet to decide if we continue alone or if we have to pick kelly rescuers on board.</x:v>
       </x:c>
       <x:c r="F68" s="25" t="str">
-        <x:v>1) The accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
-2) Be advised: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
-3) Attention: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.</x:v>
+        <x:v>The accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.</x:v>
+      </x:c>
+      <x:c r="G68" s="25" t="str">
+        <x:v>1) Be advised: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
+2) Attention: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.
+3) For information: the accident site is inaccessible. Use the tablet to decide whether to pick up a heli-rescuer or continue alone.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="120" hidden="0" customHeight="1">
@@ -1323,9 +1508,12 @@
         <x:v>Okay heli rescuer secure the area and the casualty we are go for hosting down the other personnel.</x:v>
       </x:c>
       <x:c r="F69" s="25" t="str">
-        <x:v>1) The heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
-2) Be advised: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
-3) Attention: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.</x:v>
+        <x:v>The heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.</x:v>
+      </x:c>
+      <x:c r="G69" s="25" t="str">
+        <x:v>1) Be advised: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
+2) Attention: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.
+3) For information: the heli-rescuer has secured the area and the casualty. Prepare to hoist the remaining personnel down.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="24" hidden="0" customHeight="1">
@@ -1339,9 +1527,12 @@
         <x:v>The proposed meeting point seems far away from accident site i believe we should arrange another feasible meeting point.</x:v>
       </x:c>
       <x:c r="F70" s="25" t="str">
-        <x:v>1) The proposed meeting point is far from the accident site. We should arrange a more practical point.
-2) Be advised: the proposed meeting point is far from the accident site. We should arrange a more practical point.
-3) Attention: the proposed meeting point is far from the accident site. We should arrange a more practical point.</x:v>
+        <x:v>The proposed meeting point is far from the accident site. We should arrange a more practical point.</x:v>
+      </x:c>
+      <x:c r="G70" s="25" t="str">
+        <x:v>1) Be advised: the proposed meeting point is far from the accident site. We should arrange a more practical point.
+2) Attention: the proposed meeting point is far from the accident site. We should arrange a more practical point.
+3) For information: the proposed meeting point is far from the accident site. We should arrange a more practical point.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="120" hidden="0" customHeight="1">
@@ -1355,9 +1546,12 @@
         <x:v>We have to hoist three to ground heli rescuer will be first to secure the area.</x:v>
       </x:c>
       <x:c r="F71" s="25" t="str">
-        <x:v>1) We need to hoist three people to the ground. The heli-rescuer will secure the area first.
-2) Be advised: we need to hoist three people to the ground. The heli-rescuer will secure the area first.
-3) Attention: we need to hoist three people to the ground. The heli-rescuer will secure the area first.</x:v>
+        <x:v>We need to hoist three people to the ground. The heli-rescuer will secure the area first.</x:v>
+      </x:c>
+      <x:c r="G71" s="25" t="str">
+        <x:v>1) Be advised: we need to hoist three people to the ground. The heli-rescuer will secure the area first.
+2) Attention: we need to hoist three people to the ground. The heli-rescuer will secure the area first.
+3) For information: we need to hoist three people to the ground. The heli-rescuer will secure the area first.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="120" hidden="0" customHeight="1">
@@ -1371,9 +1565,12 @@
         <x:v>We have to increase distance and hide until the rescue area is secure.</x:v>
       </x:c>
       <x:c r="F72" s="25" t="str">
-        <x:v>1) Increase distance and altitude until the rescue area is secure.
-2) Be advised: increase distance and altitude until the rescue area is secure.
-3) Attention: increase distance and altitude until the rescue area is secure.</x:v>
+        <x:v>Increase distance and altitude until the rescue area is secure.</x:v>
+      </x:c>
+      <x:c r="G72" s="25" t="str">
+        <x:v>1) Be advised: increase distance and altitude until the rescue area is secure.
+2) Attention: increase distance and altitude until the rescue area is secure.
+3) For information: increase distance and altitude until the rescue area is secure.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="120" hidden="0" customHeight="1">
@@ -1387,9 +1584,12 @@
         <x:v>Dark and patient will go with the ambulance to the design hospital we have to pick him at the hospital hello pat.</x:v>
       </x:c>
       <x:c r="F73" s="25" t="str">
-        <x:v>1) The doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
-2) Be advised: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
-3) Attention: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.</x:v>
+        <x:v>The doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.</x:v>
+      </x:c>
+      <x:c r="G73" s="25" t="str">
+        <x:v>1) Be advised: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
+2) Attention: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.
+3) For information: the doctor and patient will travel by ambulance to the designated hospital. We will pick up the doctor there.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="120" hidden="0" customHeight="1">
@@ -1403,9 +1603,12 @@
         <x:v>Three o'clock.</x:v>
       </x:c>
       <x:c r="F74" s="25" t="str">
-        <x:v>1) Three o'clock.
-2) Be advised: three o'clock.
-3) Attention: three o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G74" s="25" t="str">
+        <x:v>1) Be advised: three o'clock.
+2) Attention: three o'clock.
+3) For information: three o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="120" hidden="0" customHeight="1">
@@ -1419,9 +1622,12 @@
         <x:v>Four o'clock.</x:v>
       </x:c>
       <x:c r="F75" s="25" t="str">
-        <x:v>1) Four o'clock.
-2) Be advised: four o'clock.
-3) Attention: four o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G75" s="25" t="str">
+        <x:v>1) Be advised: four o'clock.
+2) Attention: four o'clock.
+3) For information: four o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="120" hidden="0" customHeight="1">
@@ -1435,9 +1641,12 @@
         <x:v>Five o'clock.</x:v>
       </x:c>
       <x:c r="F76" s="25" t="str">
-        <x:v>1) Five o'clock.
-2) Be advised: five o'clock.
-3) Attention: five o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G76" s="25" t="str">
+        <x:v>1) Be advised: five o'clock.
+2) Attention: five o'clock.
+3) For information: five o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="120" hidden="0" customHeight="1">
@@ -1451,9 +1660,12 @@
         <x:v>Six o'clock.</x:v>
       </x:c>
       <x:c r="F77" s="25" t="str">
-        <x:v>1) Six o'clock.
-2) Be advised: six o'clock.
-3) Attention: six o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G77" s="25" t="str">
+        <x:v>1) Be advised: six o'clock.
+2) Attention: six o'clock.
+3) For information: six o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="120" hidden="0" customHeight="1">
@@ -1467,9 +1679,12 @@
         <x:v>Seven o'clock.</x:v>
       </x:c>
       <x:c r="F78" s="25" t="str">
-        <x:v>1) Seven o'clock.
-2) Be advised: seven o'clock.
-3) Attention: seven o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G78" s="25" t="str">
+        <x:v>1) Be advised: seven o'clock.
+2) Attention: seven o'clock.
+3) For information: seven o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="120" hidden="0" customHeight="1">
@@ -1483,9 +1698,12 @@
         <x:v>Eight o'clock.</x:v>
       </x:c>
       <x:c r="F79" s="25" t="str">
-        <x:v>1) Eight o'clock.
-2) Be advised: eight o'clock.
-3) Attention: eight o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G79" s="25" t="str">
+        <x:v>1) Be advised: eight o'clock.
+2) Attention: eight o'clock.
+3) For information: eight o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="120" hidden="0" customHeight="1">
@@ -1499,9 +1717,12 @@
         <x:v>Nine o'clock.</x:v>
       </x:c>
       <x:c r="F80" s="25" t="str">
-        <x:v>1) Nine o'clock.
-2) Be advised: nine o'clock.
-3) Attention: nine o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G80" s="25" t="str">
+        <x:v>1) Be advised: nine o'clock.
+2) Attention: nine o'clock.
+3) For information: nine o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="120" hidden="0" customHeight="1">
@@ -1515,9 +1736,12 @@
         <x:v>Ten o'clock.</x:v>
       </x:c>
       <x:c r="F81" s="25" t="str">
-        <x:v>1) Ten o'clock.
-2) Be advised: ten o'clock.
-3) Attention: ten o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G81" s="25" t="str">
+        <x:v>1) Be advised: ten o'clock.
+2) Attention: ten o'clock.
+3) For information: ten o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="120" hidden="0" customHeight="1">
@@ -1531,9 +1755,12 @@
         <x:v>Eleven o'clock.</x:v>
       </x:c>
       <x:c r="F82" s="25" t="str">
-        <x:v>1) Eleven o'clock.
-2) Be advised: eleven o'clock.
-3) Attention: eleven o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G82" s="25" t="str">
+        <x:v>1) Be advised: eleven o'clock.
+2) Attention: eleven o'clock.
+3) For information: eleven o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="120" hidden="0" customHeight="1">
@@ -1547,9 +1774,12 @@
         <x:v>Twelve o'clock.</x:v>
       </x:c>
       <x:c r="F83" s="25" t="str">
-        <x:v>1) Twelve o'clock.
-2) Be advised: twelve o'clock.
-3) Attention: twelve o'clock.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G83" s="25" t="str">
+        <x:v>1) Be advised: twelve o'clock.
+2) Attention: twelve o'clock.
+3) For information: twelve o'clock.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="120" hidden="0" customHeight="1">
@@ -1563,9 +1793,12 @@
         <x:v>Or on the way to the accident site.</x:v>
       </x:c>
       <x:c r="F84" s="25" t="str">
-        <x:v>1) We are on the way to the accident site.
-2) We're on the way to the accident site.
-3) Attention: we are on the way to the accident site.</x:v>
+        <x:v>We are on the way to the accident site.</x:v>
+      </x:c>
+      <x:c r="G84" s="25" t="str">
+        <x:v>1) We're on the way to the accident site.
+2) Attention: we are on the way to the accident site.
+3) For information: we are on the way to the accident site.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="120" hidden="0" customHeight="1">
@@ -1579,9 +1812,12 @@
         <x:v>Check on tablet.</x:v>
       </x:c>
       <x:c r="F85" s="25" t="str">
-        <x:v>1) Check the tablet.
-2) Review the tablet.
-3) Please review the tablet.</x:v>
+        <x:v>Check the tablet.</x:v>
+      </x:c>
+      <x:c r="G85" s="25" t="str">
+        <x:v>1) Review the tablet.
+2) Please review the tablet.
+3) Please check the tablet.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="120" hidden="0" customHeight="1">
@@ -1595,9 +1831,12 @@
         <x:v>I believe we found something.</x:v>
       </x:c>
       <x:c r="F86" s="25" t="str">
-        <x:v>1) I believe we found something.
-2) Be advised: i believe we found something.
-3) Attention: i believe we found something.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G86" s="25" t="str">
+        <x:v>1) Be advised: i believe we found something.
+2) Attention: i believe we found something.
+3) For information: i believe we found something.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="120" hidden="0" customHeight="1">
@@ -1611,9 +1850,12 @@
         <x:v>It's in front of us.</x:v>
       </x:c>
       <x:c r="F87" s="25" t="str">
-        <x:v>1) It's in front of us.
-2) Be advised: it's in front of us.
-3) Attention: it's in front of us.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G87" s="25" t="str">
+        <x:v>1) Be advised: it's in front of us.
+2) Attention: it's in front of us.
+3) For information: it's in front of us.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="120" hidden="0" customHeight="1">
@@ -1627,9 +1869,12 @@
         <x:v>Yes confirmed we found our target.</x:v>
       </x:c>
       <x:c r="F88" s="25" t="str">
-        <x:v>1) Confirmed. We found the target.
-2) Be advised: confirmed. We found the target.
-3) Attention: confirmed. We found the target.</x:v>
+        <x:v>Confirmed. We found the target.</x:v>
+      </x:c>
+      <x:c r="G88" s="25" t="str">
+        <x:v>1) Be advised: confirmed. We found the target.
+2) Attention: confirmed. We found the target.
+3) For information: confirmed. We found the target.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="120" hidden="0" customHeight="1">
@@ -1643,9 +1888,12 @@
         <x:v>Helicopter clear ready to fly.</x:v>
       </x:c>
       <x:c r="F89" s="25" t="str">
-        <x:v>1) Helicopter clear and ready for flight.
-2) Be advised: helicopter clear and ready for flight.
-3) Attention: helicopter clear and ready for flight.</x:v>
+        <x:v>Helicopter clear and ready for flight.</x:v>
+      </x:c>
+      <x:c r="G89" s="25" t="str">
+        <x:v>1) Be advised: helicopter clear and ready for flight.
+2) Attention: helicopter clear and ready for flight.
+3) For information: helicopter clear and ready for flight.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="120" hidden="0" customHeight="1">
@@ -1659,9 +1907,12 @@
         <x:v>All engines started successfully.</x:v>
       </x:c>
       <x:c r="F90" s="25" t="str">
-        <x:v>1) Both engines started successfully.
-2) Be advised: both engines started successfully.
-3) Attention: both engines started successfully.</x:v>
+        <x:v>Both engines started successfully.</x:v>
+      </x:c>
+      <x:c r="G90" s="25" t="str">
+        <x:v>1) Be advised: both engines started successfully.
+2) Attention: both engines started successfully.
+3) For information: both engines started successfully.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="120" hidden="0" customHeight="1">
@@ -1675,9 +1926,12 @@
         <x:v>Okay all good.</x:v>
       </x:c>
       <x:c r="F91" s="25" t="str">
-        <x:v>1) Okay, all good.
-2) Be advised: okay, all good.
-3) Attention: okay, all good.</x:v>
+        <x:v>Okay, all good.</x:v>
+      </x:c>
+      <x:c r="G91" s="25" t="str">
+        <x:v>1) Be advised: okay, all good.
+2) Attention: okay, all good.
+3) For information: okay, all good.</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="120" hidden="0" customHeight="1">
@@ -1691,9 +1945,12 @@
         <x:v>Area clear ready to start engine one.</x:v>
       </x:c>
       <x:c r="F92" s="25" t="str">
-        <x:v>1) Area clear. Ready to start engine one.
-2) Be advised: area clear. Ready to start engine one.
-3) Attention: area clear. Ready to start engine one.</x:v>
+        <x:v>Area clear. Ready to start engine one.</x:v>
+      </x:c>
+      <x:c r="G92" s="25" t="str">
+        <x:v>1) Be advised: area clear. Ready to start engine one.
+2) Attention: area clear. Ready to start engine one.
+3) For information: area clear. Ready to start engine one.</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="120" hidden="0" customHeight="1">
@@ -1707,9 +1964,12 @@
         <x:v>Area clear ready to start engine two.</x:v>
       </x:c>
       <x:c r="F93" s="25" t="str">
-        <x:v>1) Area clear. Ready to start engine two.
-2) Be advised: area clear. Ready to start engine two.
-3) Attention: area clear. Ready to start engine two.</x:v>
+        <x:v>Area clear. Ready to start engine two.</x:v>
+      </x:c>
+      <x:c r="G93" s="25" t="str">
+        <x:v>1) Be advised: area clear. Ready to start engine two.
+2) Attention: area clear. Ready to start engine two.
+3) For information: area clear. Ready to start engine two.</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="120" hidden="0" customHeight="1">
@@ -1723,9 +1983,12 @@
         <x:v>Co pilot hh oh comm check.</x:v>
       </x:c>
       <x:c r="F94" s="25" t="str">
-        <x:v>1) Copilot here, communications check.
-2) Be advised: copilot here, communications check.
-3) Attention: copilot here, communications check.</x:v>
+        <x:v>Copilot here, communications check.</x:v>
+      </x:c>
+      <x:c r="G94" s="25" t="str">
+        <x:v>1) Be advised: copilot here, communications check.
+2) Attention: copilot here, communications check.
+3) For information: copilot here, communications check.</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="120" hidden="0" customHeight="1">
@@ -1739,9 +2002,12 @@
         <x:v>Engine clear.</x:v>
       </x:c>
       <x:c r="F95" s="25" t="str">
-        <x:v>1) Engine area clear.
-2) Be advised: engine area clear.
-3) Attention: engine area clear.</x:v>
+        <x:v>Engine area clear.</x:v>
+      </x:c>
+      <x:c r="G95" s="25" t="str">
+        <x:v>1) Be advised: engine area clear.
+2) Attention: engine area clear.
+3) For information: engine area clear.</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="120" hidden="0" customHeight="1">
@@ -1755,9 +2021,12 @@
         <x:v>Fire we have an engine fire stop engine.</x:v>
       </x:c>
       <x:c r="F96" s="25" t="str">
-        <x:v>1) Engine fire. Stop the engine.
-2) Be advised: engine fire. Stop the engine.
-3) Attention: engine fire. Stop the engine.</x:v>
+        <x:v>Engine fire. Stop the engine.</x:v>
+      </x:c>
+      <x:c r="G96" s="25" t="str">
+        <x:v>1) Be advised: engine fire. Stop the engine.
+2) Attention: engine fire. Stop the engine.
+3) For information: engine fire. Stop the engine.</x:v>
       </x:c>
     </x:row>
     <x:row r="97" ht="120" hidden="0" customHeight="1">
@@ -1771,9 +2040,12 @@
         <x:v>Engine started successfully moving to other engine.</x:v>
       </x:c>
       <x:c r="F97" s="25" t="str">
-        <x:v>1) Engine started successfully. Moving to the other engine.
-2) Be advised: engine started successfully. Moving to the other engine.
-3) Attention: engine started successfully. Moving to the other engine.</x:v>
+        <x:v>Engine started successfully. Moving to the other engine.</x:v>
+      </x:c>
+      <x:c r="G97" s="25" t="str">
+        <x:v>1) Be advised: engine started successfully. Moving to the other engine.
+2) Attention: engine started successfully. Moving to the other engine.
+3) For information: engine started successfully. Moving to the other engine.</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="120" hidden="0" customHeight="1">
@@ -1787,9 +2059,12 @@
         <x:v>Damn we have a failure.</x:v>
       </x:c>
       <x:c r="F98" s="25" t="str">
-        <x:v>1) Damn we have a failure.
-2) Be advised: damn we have a failure.
-3) Attention: damn we have a failure.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G98" s="25" t="str">
+        <x:v>1) Be advised: damn we have a failure.
+2) Attention: damn we have a failure.
+3) For information: damn we have a failure.</x:v>
       </x:c>
     </x:row>
     <x:row r="99" ht="120" hidden="0" customHeight="1">
@@ -1803,9 +2078,12 @@
         <x:v>Hold on performing leak checks.</x:v>
       </x:c>
       <x:c r="F99" s="25" t="str">
-        <x:v>1) Hold on. Performing leak checks.
-2) Be advised: hold on. Performing leak checks.
-3) Attention: hold on. Performing leak checks.</x:v>
+        <x:v>Hold on. Performing leak checks.</x:v>
+      </x:c>
+      <x:c r="G99" s="25" t="str">
+        <x:v>1) Be advised: hold on. Performing leak checks.
+2) Attention: hold on. Performing leak checks.
+3) Please hold on. Performing leak checks.</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="120" hidden="0" customHeight="1">
@@ -1819,9 +2097,12 @@
         <x:v>Rear crew prepare for ground operation.</x:v>
       </x:c>
       <x:c r="F100" s="25" t="str">
-        <x:v>1) Rear crew, prepare for ground operations.
-2) Be advised: rear crew, prepare for ground operations.
-3) Attention: rear crew, prepare for ground operations.</x:v>
+        <x:v>Rear crew, prepare for ground operations.</x:v>
+      </x:c>
+      <x:c r="G100" s="25" t="str">
+        <x:v>1) Be advised: rear crew, prepare for ground operations.
+2) Attention: rear crew, prepare for ground operations.
+3) For information: rear crew, prepare for ground operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="101" ht="120" hidden="0" customHeight="1">
@@ -1835,9 +2116,12 @@
         <x:v>Rear crew prepare for hoist operation.</x:v>
       </x:c>
       <x:c r="F101" s="25" t="str">
-        <x:v>1) Rear crew, prepare for hoist operations.
-2) Be advised: rear crew, prepare for hoist operations.
-3) Attention: rear crew, prepare for hoist operations.</x:v>
+        <x:v>Rear crew, prepare for hoist operations.</x:v>
+      </x:c>
+      <x:c r="G101" s="25" t="str">
+        <x:v>1) Be advised: rear crew, prepare for hoist operations.
+2) Attention: rear crew, prepare for hoist operations.
+3) For information: rear crew, prepare for hoist operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="120" hidden="0" customHeight="1">
@@ -1851,9 +2135,12 @@
         <x:v>Preparing for engine starting sequence one too.</x:v>
       </x:c>
       <x:c r="F102" s="25" t="str">
-        <x:v>1) Preparing for engine-start sequence one, then two.
-2) Be advised: preparing for engine-start sequence one, then two.
-3) Attention: preparing for engine-start sequence one, then two.</x:v>
+        <x:v>Preparing for engine-start sequence one, then two.</x:v>
+      </x:c>
+      <x:c r="G102" s="25" t="str">
+        <x:v>1) Be advised: preparing for engine-start sequence one, then two.
+2) Attention: preparing for engine-start sequence one, then two.
+3) For information: preparing for engine-start sequence one, then two.</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="120" hidden="0" customHeight="1">
@@ -1867,9 +2154,12 @@
         <x:v>Preparing for engine starting sequence to one.</x:v>
       </x:c>
       <x:c r="F103" s="25" t="str">
-        <x:v>1) Preparing for engine-start sequence two, then one.
-2) Be advised: preparing for engine-start sequence two, then one.
-3) Attention: preparing for engine-start sequence two, then one.</x:v>
+        <x:v>Preparing for engine-start sequence two, then one.</x:v>
+      </x:c>
+      <x:c r="G103" s="25" t="str">
+        <x:v>1) Be advised: preparing for engine-start sequence two, then one.
+2) Attention: preparing for engine-start sequence two, then one.
+3) For information: preparing for engine-start sequence two, then one.</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="120" hidden="0" customHeight="1">
@@ -1883,9 +2173,12 @@
         <x:v>Helicopter in position rear crew clear to start operation.</x:v>
       </x:c>
       <x:c r="F104" s="25" t="str">
-        <x:v>1) Helicopter in position. Rear crew, clear to start operations.
-2) Be advised: helicopter in position. Rear crew, clear to start operations.
-3) Attention: helicopter in position. Rear crew, clear to start operations.</x:v>
+        <x:v>Helicopter in position. Rear crew, clear to start operations.</x:v>
+      </x:c>
+      <x:c r="G104" s="25" t="str">
+        <x:v>1) Be advised: helicopter in position. Rear crew, clear to start operations.
+2) Attention: helicopter in position. Rear crew, clear to start operations.
+3) For information: helicopter in position. Rear crew, clear to start operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="105" ht="120" hidden="0" customHeight="1">
@@ -1899,9 +2192,12 @@
         <x:v>Rear crew we are approaching the landing site.</x:v>
       </x:c>
       <x:c r="F105" s="25" t="str">
-        <x:v>1) Rear crew, we are approaching the landing site.
-2) Be advised: rear crew, we are approaching the landing site.
-3) Attention: rear crew, we are approaching the landing site.</x:v>
+        <x:v>Rear crew, we are approaching the landing site.</x:v>
+      </x:c>
+      <x:c r="G105" s="25" t="str">
+        <x:v>1) Be advised: rear crew, we are approaching the landing site.
+2) Attention: rear crew, we are approaching the landing site.
+3) For information: rear crew, we are approaching the landing site.</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="120" hidden="0" customHeight="1">
@@ -1915,9 +2211,12 @@
         <x:v>Site is not safe for us waiting for clearance.</x:v>
       </x:c>
       <x:c r="F106" s="25" t="str">
-        <x:v>1) The site is not safe. Waiting for clearance.
-2) Be advised: the site is not safe. Waiting for clearance.
-3) Attention: the site is not safe. Waiting for clearance.</x:v>
+        <x:v>The site is not safe. Waiting for clearance.</x:v>
+      </x:c>
+      <x:c r="G106" s="25" t="str">
+        <x:v>1) Be advised: the site is not safe. Waiting for clearance.
+2) Attention: the site is not safe. Waiting for clearance.
+3) For information: the site is not safe. Waiting for clearance.</x:v>
       </x:c>
     </x:row>
     <x:row r="107" ht="120" hidden="0" customHeight="1">
@@ -1931,9 +2230,12 @@
         <x:v>Site is safer operations we can proceed.</x:v>
       </x:c>
       <x:c r="F107" s="25" t="str">
-        <x:v>1) The site is safe. Operations may proceed.
-2) Be advised: the site is safe. Operations may proceed.
-3) Attention: the site is safe. Operations may proceed.</x:v>
+        <x:v>The site is safe. Operations may proceed.</x:v>
+      </x:c>
+      <x:c r="G107" s="25" t="str">
+        <x:v>1) Be advised: the site is safe. Operations may proceed.
+2) Attention: the site is safe. Operations may proceed.
+3) For information: the site is safe. Operations may proceed.</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="120" hidden="0" customHeight="1">
@@ -1947,9 +2249,12 @@
         <x:v>Rear crew prepare for skid lending operation.</x:v>
       </x:c>
       <x:c r="F108" s="25" t="str">
-        <x:v>1) Rear crew, prepare for skid landing operations.
-2) Be advised: rear crew, prepare for skid landing operations.
-3) Attention: rear crew, prepare for skid landing operations.</x:v>
+        <x:v>Rear crew, prepare for skid landing operations.</x:v>
+      </x:c>
+      <x:c r="G108" s="25" t="str">
+        <x:v>1) Be advised: rear crew, prepare for skid landing operations.
+2) Attention: rear crew, prepare for skid landing operations.
+3) For information: rear crew, prepare for skid landing operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="120" hidden="0" customHeight="1">
@@ -1963,9 +2268,12 @@
         <x:v>Ambulance is arriving.</x:v>
       </x:c>
       <x:c r="F109" s="25" t="str">
-        <x:v>1) Ambulance is arriving.
-2) Be advised: ambulance is arriving.
-3) Attention: ambulance is arriving.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G109" s="25" t="str">
+        <x:v>1) Be advised: ambulance is arriving.
+2) Attention: ambulance is arriving.
+3) For information: ambulance is arriving.</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="120" hidden="0" customHeight="1">
@@ -1979,9 +2287,12 @@
         <x:v>Ambulance is still far away.</x:v>
       </x:c>
       <x:c r="F110" s="25" t="str">
-        <x:v>1) Ambulance is still far away.
-2) Be advised: ambulance is still far away.
-3) Attention: ambulance is still far away.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G110" s="25" t="str">
+        <x:v>1) Be advised: ambulance is still far away.
+2) Attention: ambulance is still far away.
+3) For information: ambulance is still far away.</x:v>
       </x:c>
     </x:row>
     <x:row r="111" ht="120" hidden="0" customHeight="1">
@@ -1995,9 +2306,12 @@
         <x:v>Crew prepare for operation.</x:v>
       </x:c>
       <x:c r="F111" s="25" t="str">
-        <x:v>1) Crew, prepare for operations.
-2) Be advised: crew, prepare for operations.
-3) All crew, prepare for operations.</x:v>
+        <x:v>Crew, prepare for operations.</x:v>
+      </x:c>
+      <x:c r="G111" s="25" t="str">
+        <x:v>1) Be advised: crew, prepare for operations.
+2) All crew, prepare for operations.
+3) For information: crew, prepare for operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="120" hidden="0" customHeight="1">
@@ -2011,9 +2325,12 @@
         <x:v>Good morning frank.</x:v>
       </x:c>
       <x:c r="F112" s="25" t="str">
-        <x:v>1) Good morning frank.
-2) Be advised: good morning frank.
-3) Attention: good morning frank.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G112" s="25" t="str">
+        <x:v>1) Be advised: good morning frank.
+2) Attention: good morning frank.
+3) For information: good morning frank.</x:v>
       </x:c>
     </x:row>
     <x:row r="113" ht="120" hidden="0" customHeight="1">
@@ -2027,9 +2344,12 @@
         <x:v>Destination insight medical crew is ready on landing spot.</x:v>
       </x:c>
       <x:c r="F113" s="25" t="str">
-        <x:v>1) Landing site in sight. Medical crew is ready at the landing area.
-2) Be advised: landing site in sight. Medical crew is ready at the landing area.
-3) Attention: landing site in sight. Medical crew is ready at the landing area.</x:v>
+        <x:v>Landing site in sight. Medical crew is ready at the landing area.</x:v>
+      </x:c>
+      <x:c r="G113" s="25" t="str">
+        <x:v>1) Be advised: landing site in sight. Medical crew is ready at the landing area.
+2) Attention: landing site in sight. Medical crew is ready at the landing area.
+3) For information: landing site in sight. Medical crew is ready at the landing area.</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="120" hidden="0" customHeight="1">
@@ -2043,9 +2363,12 @@
         <x:v>We have to stop engines and switch off the helicopter.</x:v>
       </x:c>
       <x:c r="F114" s="25" t="str">
-        <x:v>1) We have to stop the engines and shut down the helicopter.
-2) Be advised: we have to stop the engines and shut down the helicopter.
-3) Attention: we have to stop the engines and shut down the helicopter.</x:v>
+        <x:v>We have to stop the engines and shut down the helicopter.</x:v>
+      </x:c>
+      <x:c r="G114" s="25" t="str">
+        <x:v>1) Be advised: we have to stop the engines and shut down the helicopter.
+2) Attention: we have to stop the engines and shut down the helicopter.
+3) For information: we have to stop the engines and shut down the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="115" ht="24" hidden="0" customHeight="1">
@@ -2059,9 +2382,12 @@
         <x:v>The crew i received a call from doc due to patient conditions the ambulance arrived to an alternate hospital doc is waiting us their check location on map.</x:v>
       </x:c>
       <x:c r="F115" s="25" t="str">
-        <x:v>1) Crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
-2) Be advised: crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
-3) All crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.</x:v>
+        <x:v>Crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.</x:v>
+      </x:c>
+      <x:c r="G115" s="25" t="str">
+        <x:v>1) Be advised: crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
+2) All crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.
+3) For information: crew, the doctor reports that the ambulance has been rerouted to an alternate hospital. Check the location on the map.</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="120" hidden="0" customHeight="1">
@@ -2075,9 +2401,12 @@
         <x:v>We are above maximum hoist out speed.</x:v>
       </x:c>
       <x:c r="F116" s="25" t="str">
-        <x:v>1) We are above maximum hoist-out speed.
-2) We're above maximum hoist-out speed.
-3) Attention: we are above maximum hoist-out speed.</x:v>
+        <x:v>We are above maximum hoist-out speed.</x:v>
+      </x:c>
+      <x:c r="G116" s="25" t="str">
+        <x:v>1) We're above maximum hoist-out speed.
+2) Attention: we are above maximum hoist-out speed.
+3) For information: we are above maximum hoist-out speed.</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="120" hidden="0" customHeight="1">
@@ -2091,9 +2420,12 @@
         <x:v>Oh acceleration is over the hoist limit.</x:v>
       </x:c>
       <x:c r="F117" s="25" t="str">
-        <x:v>1) Acceleration is above the hoist limit.
-2) Be advised: acceleration is above the hoist limit.
-3) Attention: acceleration is above the hoist limit.</x:v>
+        <x:v>Acceleration is above the hoist limit.</x:v>
+      </x:c>
+      <x:c r="G117" s="25" t="str">
+        <x:v>1) Be advised: acceleration is above the hoist limit.
+2) Attention: acceleration is above the hoist limit.
+3) For information: acceleration is above the hoist limit.</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="120" hidden="0" customHeight="1">
@@ -2107,9 +2439,12 @@
         <x:v>Bank angle is too high people on hoist will have troubles if we continue.</x:v>
       </x:c>
       <x:c r="F118" s="25" t="str">
-        <x:v>1) Bank angle is too high. Continuing would endanger the patient and hoist operator.
-2) Be advised: bank angle is too high. Continuing would endanger the patient and hoist operator.
-3) Attention: bank angle is too high. Continuing would endanger the patient and hoist operator.</x:v>
+        <x:v>Bank angle is too high. Continuing would endanger the patient and hoist operator.</x:v>
+      </x:c>
+      <x:c r="G118" s="25" t="str">
+        <x:v>1) Be advised: bank angle is too high. Continuing would endanger the patient and hoist operator.
+2) Attention: bank angle is too high. Continuing would endanger the patient and hoist operator.
+3) For information: bank angle is too high. Continuing would endanger the patient and hoist operator.</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="120" hidden="0" customHeight="1">
@@ -2123,9 +2458,12 @@
         <x:v>Keep bank angled within limits.</x:v>
       </x:c>
       <x:c r="F119" s="25" t="str">
-        <x:v>1) Keep the bank angle within limits.
-2) Be advised: keep the bank angle within limits.
-3) Attention: keep the bank angle within limits.</x:v>
+        <x:v>Keep the bank angle within limits.</x:v>
+      </x:c>
+      <x:c r="G119" s="25" t="str">
+        <x:v>1) Be advised: keep the bank angle within limits.
+2) Attention: keep the bank angle within limits.
+3) Please keep the bank angle within limits.</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="120" hidden="0" customHeight="1">
@@ -2139,9 +2477,12 @@
         <x:v>We are too fast sir we risk our patient and operator life moreover we are damaging the helicopter.</x:v>
       </x:c>
       <x:c r="F120" s="25" t="str">
-        <x:v>1) We are too fast. We risk the patient, the operator, and the helicopter.
-2) We're too fast. We risk the patient, the operator, and the helicopter.
-3) Attention: we are too fast. We risk the patient, the operator, and the helicopter.</x:v>
+        <x:v>We are too fast. We risk the patient, the operator, and the helicopter.</x:v>
+      </x:c>
+      <x:c r="G120" s="25" t="str">
+        <x:v>1) We're too fast. We risk the patient, the operator, and the helicopter.
+2) Attention: we are too fast. We risk the patient, the operator, and the helicopter.
+3) For information: we are too fast. We risk the patient, the operator, and the helicopter.</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="120" hidden="0" customHeight="1">
@@ -2155,9 +2496,12 @@
         <x:v>Fuck sir we have to abort mission now.</x:v>
       </x:c>
       <x:c r="F121" s="25" t="str">
-        <x:v>1) We have to abort the mission now.
-2) Be advised: we have to abort the mission now.
-3) Attention: we have to abort the mission now.</x:v>
+        <x:v>We have to abort the mission now.</x:v>
+      </x:c>
+      <x:c r="G121" s="25" t="str">
+        <x:v>1) Be advised: we have to abort the mission now.
+2) Attention: we have to abort the mission now.
+3) For information: we have to abort the mission now.</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="120" hidden="0" customHeight="1">
@@ -2171,9 +2515,12 @@
         <x:v>What the fuck we lost patient and doc what are you doing.</x:v>
       </x:c>
       <x:c r="F122" s="25" t="str">
-        <x:v>1) We lost the doctor and patient. What are you doing?
-2) Can you confirm: we lost the doctor and patient. What are you doing?
-3) Please confirm: we lost the doctor and patient. What are you doing?</x:v>
+        <x:v>We lost the doctor and patient. What are you doing?</x:v>
+      </x:c>
+      <x:c r="G122" s="25" t="str">
+        <x:v>1) Can you confirm: we lost the doctor and patient. What are you doing?
+2) Please confirm: we lost the doctor and patient. What are you doing?
+3) Message update: we lost the doctor and patient. What are you doing?</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="120" hidden="0" customHeight="1">
@@ -2187,9 +2534,12 @@
         <x:v>Ah are we doing acrobatic maneuvers with a patient on board are you serious.</x:v>
       </x:c>
       <x:c r="F123" s="25" t="str">
-        <x:v>1) Are we doing aerobatics with a patient on board?
-2) Can you confirm: are we doing aerobatics with a patient on board?
-3) Please confirm: are we doing aerobatics with a patient on board?</x:v>
+        <x:v>Are we doing aerobatics with a patient on board?</x:v>
+      </x:c>
+      <x:c r="G123" s="25" t="str">
+        <x:v>1) Can you confirm: are we doing aerobatics with a patient on board?
+2) Please confirm: are we doing aerobatics with a patient on board?
+3) Message update: are we doing aerobatics with a patient on board?</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="24" hidden="0" customHeight="1">
@@ -2203,9 +2553,12 @@
         <x:v>Doc refers the ground operations are almost done we can either go back and have or as soon as possible or stay here and proceed with ground operation.</x:v>
       </x:c>
       <x:c r="F124" s="25" t="str">
-        <x:v>1) The doctor says ground operations are almost complete. We can return to base or wait to proceed.
-2) Be advised: the doctor says ground operations are almost complete. We can return to base or wait to proceed.
-3) Attention: the doctor says ground operations are almost complete. We can return to base or wait to proceed.</x:v>
+        <x:v>The doctor says ground operations are almost complete. We can return to base or wait to proceed.</x:v>
+      </x:c>
+      <x:c r="G124" s="25" t="str">
+        <x:v>1) Be advised: the doctor says ground operations are almost complete. We can return to base or wait to proceed.
+2) Attention: the doctor says ground operations are almost complete. We can return to base or wait to proceed.
+3) For information: the doctor says ground operations are almost complete. We can return to base or wait to proceed.</x:v>
       </x:c>
     </x:row>
     <x:row r="125" ht="24" hidden="0" customHeight="1">
@@ -2219,9 +2572,12 @@
         <x:v>Round operations will take time we can leave hover and find a safe landing spot we will be advised when operations are done.</x:v>
       </x:c>
       <x:c r="F125" s="25" t="str">
-        <x:v>1) Ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
-2) Be advised: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
-3) Attention: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.</x:v>
+        <x:v>Ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.</x:v>
+      </x:c>
+      <x:c r="G125" s="25" t="str">
+        <x:v>1) Be advised: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
+2) Attention: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.
+3) For information: ground operations will take time. We can leave the hover and find a safe landing spot; they will advise us when finished.</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="120" hidden="0" customHeight="1">
@@ -2235,9 +2591,12 @@
         <x:v>Ouch it was hard landing this time sarah won't be happy.</x:v>
       </x:c>
       <x:c r="F126" s="25" t="str">
-        <x:v>1) That was a hard landing. Sarah will not be happy.
-2) Be advised: that was a hard landing. Sarah will not be happy.
-3) Attention: that was a hard landing. Sarah will not be happy.</x:v>
+        <x:v>That was a hard landing. Sarah will not be happy.</x:v>
+      </x:c>
+      <x:c r="G126" s="25" t="str">
+        <x:v>1) Be advised: that was a hard landing. Sarah will not be happy.
+2) Attention: that was a hard landing. Sarah will not be happy.
+3) For information: that was a hard landing. Sarah will not be happy.</x:v>
       </x:c>
     </x:row>
     <x:row r="127" ht="120" hidden="0" customHeight="1">
@@ -2251,9 +2610,12 @@
         <x:v>Hey it was a hard touch.</x:v>
       </x:c>
       <x:c r="F127" s="25" t="str">
-        <x:v>1) That was a hard touch.
-2) Be advised: that was a hard touch.
-3) Attention: that was a hard touch.</x:v>
+        <x:v>That was a hard touch.</x:v>
+      </x:c>
+      <x:c r="G127" s="25" t="str">
+        <x:v>1) Be advised: that was a hard touch.
+2) Attention: that was a hard touch.
+3) For information: that was a hard touch.</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="120" hidden="0" customHeight="1">
@@ -2267,9 +2629,12 @@
         <x:v>Wow nice touch captain.</x:v>
       </x:c>
       <x:c r="F128" s="25" t="str">
-        <x:v>1) Wow nice touch captain.
-2) Be advised: wow nice touch captain.
-3) Attention: wow nice touch captain.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G128" s="25" t="str">
+        <x:v>1) Be advised: wow nice touch captain.
+2) Attention: wow nice touch captain.
+3) For information: wow nice touch captain.</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="120" hidden="0" customHeight="1">
@@ -2283,9 +2648,12 @@
         <x:v>VNE.</x:v>
       </x:c>
       <x:c r="F129" s="25" t="str">
-        <x:v>1) VNE.
-2) Be advised: vNE.
-3) Attention: vNE.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G129" s="25" t="str">
+        <x:v>1) Be advised: vNE.
+2) Attention: vNE.
+3) For information: vNE.</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="120" hidden="0" customHeight="1">
@@ -2299,9 +2667,12 @@
         <x:v>VTOSS.</x:v>
       </x:c>
       <x:c r="F130" s="25" t="str">
-        <x:v>1) VTOSS.
-2) Be advised: vTOSS.
-3) Attention: vTOSS.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G130" s="25" t="str">
+        <x:v>1) Be advised: vTOSS.
+2) Attention: vTOSS.
+3) For information: vTOSS.</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="120" hidden="0" customHeight="1">
@@ -2315,9 +2686,12 @@
         <x:v>Vy.</x:v>
       </x:c>
       <x:c r="F131" s="25" t="str">
-        <x:v>1) Vy.
-2) Be advised: vy.
-3) Attention: vy.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G131" s="25" t="str">
+        <x:v>1) Be advised: vy.
+2) Attention: vy.
+3) For information: vy.</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="120" hidden="0" customHeight="1">
@@ -2331,9 +2705,12 @@
         <x:v>The a what we crashed are you all okay.</x:v>
       </x:c>
       <x:c r="F132" s="25" t="str">
-        <x:v>1) We crashed. Is everyone okay?
-2) Can you confirm: we crashed. Is everyone okay?
-3) Please confirm: we crashed. Is everyone okay?</x:v>
+        <x:v>We crashed. Is everyone okay?</x:v>
+      </x:c>
+      <x:c r="G132" s="25" t="str">
+        <x:v>1) Can you confirm: we crashed. Is everyone okay?
+2) Please confirm: we crashed. Is everyone okay?
+3) Message update: we crashed. Is everyone okay?</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="120" hidden="0" customHeight="1">
@@ -2347,9 +2724,12 @@
         <x:v>Hey hey captain that's not and aerobatic helicopter please keep calm.</x:v>
       </x:c>
       <x:c r="F133" s="25" t="str">
-        <x:v>1) Captain, this is not an aerobatic helicopter. Please keep it calm.
-2) Be advised: captain, this is not an aerobatic helicopter. Please keep it calm.
-3) Attention: captain, this is not an aerobatic helicopter. Please keep it calm.</x:v>
+        <x:v>Captain, this is not an aerobatic helicopter. Please keep it calm.</x:v>
+      </x:c>
+      <x:c r="G133" s="25" t="str">
+        <x:v>1) Be advised: captain, this is not an aerobatic helicopter. Please keep it calm.
+2) Attention: captain, this is not an aerobatic helicopter. Please keep it calm.
+3) For information: captain, this is not an aerobatic helicopter. Please keep it calm.</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="36" hidden="0" customHeight="1">
@@ -2363,9 +2743,12 @@
         <x:v>Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
       <x:c r="F134" s="25" t="str">
-        <x:v>1) Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
-2) Be advised: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
-3) Attention: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G134" s="25" t="str">
+        <x:v>1) Be advised: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
+2) Attention: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
+3) For information: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
     </x:row>
     <x:row r="135" ht="24" hidden="0" customHeight="1">
@@ -2379,9 +2762,12 @@
         <x:v>Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
       <x:c r="F135" s="25" t="str">
-        <x:v>1) Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
-2) Be advised: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
-3) Attention: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G135" s="25" t="str">
+        <x:v>1) Be advised: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
+2) Attention: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
+3) For information: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
     </x:row>
     <x:row r="136" ht="120" hidden="0" customHeight="1">
@@ -2395,9 +2781,12 @@
         <x:v>Watch out reduce collective now.</x:v>
       </x:c>
       <x:c r="F136" s="25" t="str">
-        <x:v>1) Watch out. Reduce collective now.
-2) Be advised: watch out. Reduce collective now.
-3) Attention: watch out. Reduce collective now.</x:v>
+        <x:v>Watch out. Reduce collective now.</x:v>
+      </x:c>
+      <x:c r="G136" s="25" t="str">
+        <x:v>1) Be advised: watch out. Reduce collective now.
+2) Attention: watch out. Reduce collective now.
+3) For information: watch out. Reduce collective now.</x:v>
       </x:c>
     </x:row>
     <x:row r="137" ht="24" hidden="0" customHeight="1">
@@ -2411,9 +2800,12 @@
         <x:v>A crew i just received a call from doc the ambulance has been rerouted to another hospital it seems to be better for patient conditions we have to modify our root for the new picking point location.</x:v>
       </x:c>
       <x:c r="F137" s="25" t="str">
-        <x:v>1) Crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
-2) Be advised: crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
-3) All crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.</x:v>
+        <x:v>Crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.</x:v>
+      </x:c>
+      <x:c r="G137" s="25" t="str">
+        <x:v>1) Be advised: crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
+2) All crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.
+3) For information: crew, the doctor reports that the ambulance has been rerouted to another hospital. We must change our route to the new pickup point.</x:v>
       </x:c>
     </x:row>
     <x:row r="138" ht="120" hidden="0" customHeight="1">
@@ -2427,9 +2819,12 @@
         <x:v>Medical crew was starting ground loading procedures we have to wait here.</x:v>
       </x:c>
       <x:c r="F138" s="25" t="str">
-        <x:v>1) Medical crew has started ground-loading procedures. We must wait here.
-2) Be advised: medical crew has started ground-loading procedures. We must wait here.
-3) Attention: medical crew has started ground-loading procedures. We must wait here.</x:v>
+        <x:v>Medical crew has started ground-loading procedures. We must wait here.</x:v>
+      </x:c>
+      <x:c r="G138" s="25" t="str">
+        <x:v>1) Be advised: medical crew has started ground-loading procedures. We must wait here.
+2) Attention: medical crew has started ground-loading procedures. We must wait here.
+3) For information: medical crew has started ground-loading procedures. We must wait here.</x:v>
       </x:c>
     </x:row>
     <x:row r="139" ht="120" hidden="0" customHeight="1">
@@ -2443,9 +2838,12 @@
         <x:v>Medical crew informs the due to distance we need to proceed with hoist operation crew was ready waiting us.</x:v>
       </x:c>
       <x:c r="F139" s="25" t="str">
-        <x:v>1) Medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
-2) Be advised: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
-3) Attention: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.</x:v>
+        <x:v>Medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.</x:v>
+      </x:c>
+      <x:c r="G139" s="25" t="str">
+        <x:v>1) Be advised: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
+2) Attention: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.
+3) For information: medical crew reports that distance requires a hoist operation. The crew is ready and waiting for us.</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="120" hidden="0" customHeight="1">
@@ -2459,9 +2857,12 @@
         <x:v>Medical crew was ready for hoist operation.</x:v>
       </x:c>
       <x:c r="F140" s="25" t="str">
-        <x:v>1) Medical crew is ready for hoist operations.
-2) Be advised: medical crew is ready for hoist operations.
-3) Attention: medical crew is ready for hoist operations.</x:v>
+        <x:v>Medical crew is ready for hoist operations.</x:v>
+      </x:c>
+      <x:c r="G140" s="25" t="str">
+        <x:v>1) Be advised: medical crew is ready for hoist operations.
+2) Attention: medical crew is ready for hoist operations.
+3) For information: medical crew is ready for hoist operations.</x:v>
       </x:c>
     </x:row>
     <x:row r="141" ht="120" hidden="0" customHeight="1">
@@ -2475,9 +2876,12 @@
         <x:v>Patient and doctor will be transported by ambulance and we have to pick doc and hospital.</x:v>
       </x:c>
       <x:c r="F141" s="25" t="str">
-        <x:v>1) The patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
-2) Be advised: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
-3) Attention: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.</x:v>
+        <x:v>The patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.</x:v>
+      </x:c>
+      <x:c r="G141" s="25" t="str">
+        <x:v>1) Be advised: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
+2) Attention: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.
+3) For information: the patient and doctor will travel by ambulance. We will pick up the doctor at the hospital.</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="120" hidden="0" customHeight="1">
@@ -2491,9 +2895,12 @@
         <x:v>Patient will be transported by ambulance we completed our task.</x:v>
       </x:c>
       <x:c r="F142" s="25" t="str">
-        <x:v>1) The patient will travel by ambulance. Our task is complete.
-2) Be advised: the patient will travel by ambulance. Our task is complete.
-3) Attention: the patient will travel by ambulance. Our task is complete.</x:v>
+        <x:v>The patient will travel by ambulance. Our task is complete.</x:v>
+      </x:c>
+      <x:c r="G142" s="25" t="str">
+        <x:v>1) Be advised: the patient will travel by ambulance. Our task is complete.
+2) Attention: the patient will travel by ambulance. Our task is complete.
+3) For information: the patient will travel by ambulance. Our task is complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="143" ht="120" hidden="0" customHeight="1">
@@ -2507,9 +2914,12 @@
         <x:v>Patient will be transported by us.</x:v>
       </x:c>
       <x:c r="F143" s="25" t="str">
-        <x:v>1) The patient will be transported by us.
-2) Be advised: the patient will be transported by us.
-3) Attention: the patient will be transported by us.</x:v>
+        <x:v>The patient will be transported by us.</x:v>
+      </x:c>
+      <x:c r="G143" s="25" t="str">
+        <x:v>1) Be advised: the patient will be transported by us.
+2) Attention: the patient will be transported by us.
+3) For information: the patient will be transported by us.</x:v>
       </x:c>
     </x:row>
     <x:row r="144" ht="120" hidden="0" customHeight="1">
@@ -2523,9 +2933,12 @@
         <x:v>Rescue team identified a valid landing spot a marshal or is waiting us.</x:v>
       </x:c>
       <x:c r="F144" s="25" t="str">
-        <x:v>1) The rescue team identified a valid landing spot. A marshal is waiting for us.
-2) Be advised: the rescue team identified a valid landing spot. A marshal is waiting for us.
-3) Attention: the rescue team identified a valid landing spot. A marshal is waiting for us.</x:v>
+        <x:v>The rescue team identified a valid landing spot. A marshal is waiting for us.</x:v>
+      </x:c>
+      <x:c r="G144" s="25" t="str">
+        <x:v>1) Be advised: the rescue team identified a valid landing spot. A marshal is waiting for us.
+2) Attention: the rescue team identified a valid landing spot. A marshal is waiting for us.
+3) For information: the rescue team identified a valid landing spot. A marshal is waiting for us.</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="120" hidden="0" customHeight="1">
@@ -2539,9 +2952,12 @@
         <x:v>Hey we cannot take off with fuel hose attached.</x:v>
       </x:c>
       <x:c r="F145" s="25" t="str">
-        <x:v>1) We cannot take off with the fuel hose attached.
-2) We can't take off with the fuel hose attached.
-3) Attention: we cannot take off with the fuel hose attached.</x:v>
+        <x:v>We cannot take off with the fuel hose attached.</x:v>
+      </x:c>
+      <x:c r="G145" s="25" t="str">
+        <x:v>1) We can't take off with the fuel hose attached.
+2) Attention: we cannot take off with the fuel hose attached.
+3) For information: we cannot take off with the fuel hose attached.</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="120" hidden="0" customHeight="1">
@@ -2555,9 +2971,12 @@
         <x:v>Crew is ready on landing spot we can proceed.</x:v>
       </x:c>
       <x:c r="F146" s="25" t="str">
-        <x:v>1) Crew is ready at the landing site. We can proceed.
-2) Be advised: crew is ready at the landing site. We can proceed.
-3) Attention: crew is ready at the landing site. We can proceed.</x:v>
+        <x:v>Crew is ready at the landing site. We can proceed.</x:v>
+      </x:c>
+      <x:c r="G146" s="25" t="str">
+        <x:v>1) Be advised: crew is ready at the landing site. We can proceed.
+2) Attention: crew is ready at the landing site. We can proceed.
+3) For information: crew is ready at the landing site. We can proceed.</x:v>
       </x:c>
     </x:row>
     <x:row r="147" ht="15" hidden="0" customHeight="1">
@@ -2582,9 +3001,12 @@
         <x:v>This is the default hoist pack enjoy.</x:v>
       </x:c>
       <x:c r="F148" s="25" t="str">
-        <x:v>1) This is the default hoist pack enjoy.
-2) Be advised: this is the default hoist pack enjoy.
-3) Attention: this is the default hoist pack enjoy.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G148" s="25" t="str">
+        <x:v>1) Be advised: this is the default hoist pack enjoy.
+2) Attention: this is the default hoist pack enjoy.
+3) For information: this is the default hoist pack enjoy.</x:v>
       </x:c>
     </x:row>
     <x:row r="149" ht="120" hidden="0" customHeight="1">
@@ -2598,9 +3020,12 @@
         <x:v>Through comm check please.</x:v>
       </x:c>
       <x:c r="F149" s="25" t="str">
-        <x:v>1) Pilot, communications check.
-2) Be advised: pilot, communications check.
-3) Attention: pilot, communications check.</x:v>
+        <x:v>Pilot, communications check.</x:v>
+      </x:c>
+      <x:c r="G149" s="25" t="str">
+        <x:v>1) Be advised: pilot, communications check.
+2) Attention: pilot, communications check.
+3) For information: pilot, communications check.</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="120" hidden="0" customHeight="1">
@@ -2614,9 +3039,12 @@
         <x:v>Landed crew aboard authorized.</x:v>
       </x:c>
       <x:c r="F150" s="25" t="str">
-        <x:v>1) Landed. Crew, board when authorized.
-2) Be advised: landed. Crew, board when authorized.
-3) Attention: landed. Crew, board when authorized.</x:v>
+        <x:v>Landed. Crew, board when authorized.</x:v>
+      </x:c>
+      <x:c r="G150" s="25" t="str">
+        <x:v>1) Be advised: landed. Crew, board when authorized.
+2) Attention: landed. Crew, board when authorized.
+3) For information: landed. Crew, board when authorized.</x:v>
       </x:c>
     </x:row>
     <x:row r="151" ht="120" hidden="0" customHeight="1">
@@ -2630,9 +3058,12 @@
         <x:v>Evacuate helicopter now.</x:v>
       </x:c>
       <x:c r="F151" s="25" t="str">
-        <x:v>1) Evacuate helicopter now.
-2) Be advised: evacuate helicopter now.
-3) Attention: evacuate helicopter now.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G151" s="25" t="str">
+        <x:v>1) Be advised: evacuate helicopter now.
+2) Attention: evacuate helicopter now.
+3) For information: evacuate helicopter now.</x:v>
       </x:c>
     </x:row>
     <x:row r="152" ht="120" hidden="0" customHeight="1">
@@ -2646,9 +3077,12 @@
         <x:v>Hi sarah how you helicopter is good fuel needs to be refilled.</x:v>
       </x:c>
       <x:c r="F152" s="25" t="str">
-        <x:v>1) Hi Sarah, how are you? The helicopter is good, but it needs refuelling.
-2) Be advised: hi Sarah, how are you? The helicopter is good, but it needs refuelling.
-3) Attention: hi Sarah, how are you? The helicopter is good, but it needs refuelling.</x:v>
+        <x:v>Hi Sarah, how are you? The helicopter is good, but it needs refuelling.</x:v>
+      </x:c>
+      <x:c r="G152" s="25" t="str">
+        <x:v>1) Be advised: hi Sarah, how are you? The helicopter is good, but it needs refuelling.
+2) Attention: hi Sarah, how are you? The helicopter is good, but it needs refuelling.
+3) For information: hi Sarah, how are you? The helicopter is good, but it needs refuelling.</x:v>
       </x:c>
     </x:row>
     <x:row r="153" ht="120" hidden="0" customHeight="1">
@@ -2662,9 +3096,12 @@
         <x:v>I'll check.</x:v>
       </x:c>
       <x:c r="F153" s="25" t="str">
-        <x:v>1) I'll check.
-2) Be advised: i'll check.
-3) Attention: i'll check.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G153" s="25" t="str">
+        <x:v>1) Be advised: i'll check.
+2) Attention: i'll check.
+3) For information: i'll check.</x:v>
       </x:c>
     </x:row>
     <x:row r="154" ht="120" hidden="0" customHeight="1">
@@ -2678,9 +3115,12 @@
         <x:v>Mission accomplished.</x:v>
       </x:c>
       <x:c r="F154" s="25" t="str">
-        <x:v>1) Mission accomplished.
-2) Be advised: mission accomplished.
-3) Attention: mission accomplished.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G154" s="25" t="str">
+        <x:v>1) Be advised: mission accomplished.
+2) Attention: mission accomplished.
+3) For information: mission accomplished.</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="120" hidden="0" customHeight="1">
@@ -2694,9 +3134,12 @@
         <x:v>Thank you.</x:v>
       </x:c>
       <x:c r="F155" s="25" t="str">
-        <x:v>1) Thank you.
-2) Be advised: thank you.
-3) Attention: thank you.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G155" s="25" t="str">
+        <x:v>1) Be advised: thank you.
+2) Attention: thank you.
+3) For information: thank you.</x:v>
       </x:c>
     </x:row>
     <x:row r="156" ht="120" hidden="0" customHeight="1">
@@ -2710,9 +3153,12 @@
         <x:v>Thank you frank.</x:v>
       </x:c>
       <x:c r="F156" s="25" t="str">
-        <x:v>1) Thank you, Frank.
-2) Be advised: thank you, Frank.
-3) Attention: thank you, Frank.</x:v>
+        <x:v>Thank you, Frank.</x:v>
+      </x:c>
+      <x:c r="G156" s="25" t="str">
+        <x:v>1) Be advised: thank you, Frank.
+2) Attention: thank you, Frank.
+3) For information: thank you, Frank.</x:v>
       </x:c>
     </x:row>
     <x:row r="157" ht="120" hidden="0" customHeight="1">
@@ -2726,9 +3172,12 @@
         <x:v>We did our best unfortunately we cannot save all patients.</x:v>
       </x:c>
       <x:c r="F157" s="25" t="str">
-        <x:v>1) We did our best. Unfortunately, we could not save every patient.
-2) Be advised: we did our best. Unfortunately, we could not save every patient.
-3) Attention: we did our best. Unfortunately, we could not save every patient.</x:v>
+        <x:v>We did our best. Unfortunately, we could not save every patient.</x:v>
+      </x:c>
+      <x:c r="G157" s="25" t="str">
+        <x:v>1) Be advised: we did our best. Unfortunately, we could not save every patient.
+2) Attention: we did our best. Unfortunately, we could not save every patient.
+3) For information: we did our best. Unfortunately, we could not save every patient.</x:v>
       </x:c>
     </x:row>
     <x:row r="158" ht="120" hidden="0" customHeight="1">
@@ -2742,9 +3191,12 @@
         <x:v>Well done.</x:v>
       </x:c>
       <x:c r="F158" s="25" t="str">
-        <x:v>1) Well done.
-2) Be advised: well done.
-3) Attention: well done.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G158" s="25" t="str">
+        <x:v>1) Be advised: well done.
+2) Attention: well done.
+3) For information: well done.</x:v>
       </x:c>
     </x:row>
     <x:row r="159" ht="120" hidden="0" customHeight="1">
@@ -2758,9 +3210,12 @@
         <x:v>Two nautical miles from accident area.</x:v>
       </x:c>
       <x:c r="F159" s="25" t="str">
-        <x:v>1) Two nautical miles from the accident area.
-2) Be advised: two nautical miles from the accident area.
-3) Attention: two nautical miles from the accident area.</x:v>
+        <x:v>Two nautical miles from the accident area.</x:v>
+      </x:c>
+      <x:c r="G159" s="25" t="str">
+        <x:v>1) Be advised: two nautical miles from the accident area.
+2) Attention: two nautical miles from the accident area.
+3) For information: two nautical miles from the accident area.</x:v>
       </x:c>
     </x:row>
     <x:row r="160" ht="120" hidden="0" customHeight="1">
@@ -2774,9 +3229,12 @@
         <x:v>Two nautical miles from our base.</x:v>
       </x:c>
       <x:c r="F160" s="25" t="str">
-        <x:v>1) Two nautical miles from our base.
-2) Be advised: two nautical miles from our base.
-3) Attention: two nautical miles from our base.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G160" s="25" t="str">
+        <x:v>1) Be advised: two nautical miles from our base.
+2) Attention: two nautical miles from our base.
+3) For information: two nautical miles from our base.</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="120" hidden="0" customHeight="1">
@@ -2790,9 +3248,12 @@
         <x:v>Two nautical miles from hospital.</x:v>
       </x:c>
       <x:c r="F161" s="25" t="str">
-        <x:v>1) Two nautical miles from hospital.
-2) Be advised: two nautical miles from hospital.
-3) Attention: two nautical miles from hospital.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G161" s="25" t="str">
+        <x:v>1) Be advised: two nautical miles from hospital.
+2) Attention: two nautical miles from hospital.
+3) For information: two nautical miles from hospital.</x:v>
       </x:c>
     </x:row>
     <x:row r="162" ht="120" hidden="0" customHeight="1">
@@ -2806,9 +3267,12 @@
         <x:v>Two nautical miles from loading area.</x:v>
       </x:c>
       <x:c r="F162" s="25" t="str">
-        <x:v>1) Two nautical miles from the loading area.
-2) Be advised: two nautical miles from the loading area.
-3) Attention: two nautical miles from the loading area.</x:v>
+        <x:v>Two nautical miles from the loading area.</x:v>
+      </x:c>
+      <x:c r="G162" s="25" t="str">
+        <x:v>1) Be advised: two nautical miles from the loading area.
+2) Attention: two nautical miles from the loading area.
+3) For information: two nautical miles from the loading area.</x:v>
       </x:c>
     </x:row>
     <x:row r="163" ht="120" hidden="0" customHeight="1">
@@ -2822,9 +3286,12 @@
         <x:v>Engine parameters when not good.</x:v>
       </x:c>
       <x:c r="F163" s="25" t="str">
-        <x:v>1) Engine parameters are not good.
-2) Be advised: engine parameters are not good.
-3) Attention: engine parameters are not good.</x:v>
+        <x:v>Engine parameters are not good.</x:v>
+      </x:c>
+      <x:c r="G163" s="25" t="str">
+        <x:v>1) Be advised: engine parameters are not good.
+2) Attention: engine parameters are not good.
+3) For information: engine parameters are not good.</x:v>
       </x:c>
     </x:row>
     <x:row r="164" ht="120" hidden="0" customHeight="1">
@@ -2838,9 +3305,12 @@
         <x:v>We exceeded VNE.</x:v>
       </x:c>
       <x:c r="F164" s="25" t="str">
-        <x:v>1) We exceeded VNE.
-2) Be advised: we exceeded VNE.
-3) Attention: we exceeded VNE.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G164" s="25" t="str">
+        <x:v>1) Be advised: we exceeded VNE.
+2) Attention: we exceeded VNE.
+3) For information: we exceeded VNE.</x:v>
       </x:c>
     </x:row>
     <x:row r="165" ht="120" hidden="0" customHeight="1">
@@ -2854,9 +3324,12 @@
         <x:v>We exceeded the torque limits.</x:v>
       </x:c>
       <x:c r="F165" s="25" t="str">
-        <x:v>1) We exceeded the torque limits.
-2) Be advised: we exceeded the torque limits.
-3) Attention: we exceeded the torque limits.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G165" s="25" t="str">
+        <x:v>1) Be advised: we exceeded the torque limits.
+2) Attention: we exceeded the torque limits.
+3) For information: we exceeded the torque limits.</x:v>
       </x:c>
     </x:row>
     <x:row r="166" ht="120" hidden="0" customHeight="1">
@@ -2870,9 +3343,12 @@
         <x:v>Hi sarah i'm sorry we have some bad news for you.</x:v>
       </x:c>
       <x:c r="F166" s="25" t="str">
-        <x:v>1) Hi sarah i'm sorry we have some bad news for you.
-2) Be advised: hi sarah i'm sorry we have some bad news for you.
-3) Attention: hi sarah i'm sorry we have some bad news for you.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G166" s="25" t="str">
+        <x:v>1) Be advised: hi sarah i'm sorry we have some bad news for you.
+2) Attention: hi sarah i'm sorry we have some bad news for you.
+3) For information: hi sarah i'm sorry we have some bad news for you.</x:v>
       </x:c>
     </x:row>
     <x:row r="167" ht="120" hidden="0" customHeight="1">
@@ -2886,9 +3362,12 @@
         <x:v>Main gearbox parameters were high and we felt hi vibrations.</x:v>
       </x:c>
       <x:c r="F167" s="25" t="str">
-        <x:v>1) Main gearbox parameters were high, and we felt strong vibrations.
-2) Be advised: main gearbox parameters were high, and we felt strong vibrations.
-3) Attention: main gearbox parameters were high, and we felt strong vibrations.</x:v>
+        <x:v>Main gearbox parameters were high, and we felt strong vibrations.</x:v>
+      </x:c>
+      <x:c r="G167" s="25" t="str">
+        <x:v>1) Be advised: main gearbox parameters were high, and we felt strong vibrations.
+2) Attention: main gearbox parameters were high, and we felt strong vibrations.
+3) For information: main gearbox parameters were high, and we felt strong vibrations.</x:v>
       </x:c>
     </x:row>
     <x:row r="168" ht="120" hidden="0" customHeight="1">
@@ -2902,9 +3381,12 @@
         <x:v>We had tail rotor gearbox parameters fluctuations.</x:v>
       </x:c>
       <x:c r="F168" s="25" t="str">
-        <x:v>1) Tail-rotor gearbox parameters fluctuated.
-2) Be advised: tail-rotor gearbox parameters fluctuated.
-3) Attention: tail-rotor gearbox parameters fluctuated.</x:v>
+        <x:v>Tail-rotor gearbox parameters fluctuated.</x:v>
+      </x:c>
+      <x:c r="G168" s="25" t="str">
+        <x:v>1) Be advised: tail-rotor gearbox parameters fluctuated.
+2) Attention: tail-rotor gearbox parameters fluctuated.
+3) For information: tail-rotor gearbox parameters fluctuated.</x:v>
       </x:c>
     </x:row>
     <x:row r="169" ht="120" hidden="0" customHeight="1">
@@ -2918,9 +3400,12 @@
         <x:v>We had failures they are reported in the technical log book.</x:v>
       </x:c>
       <x:c r="F169" s="25" t="str">
-        <x:v>1) We had failures. They are recorded in the technical logbook.
-2) Be advised: we had failures. They are recorded in the technical logbook.
-3) Attention: we had failures. They are recorded in the technical logbook.</x:v>
+        <x:v>We had failures. They are recorded in the technical logbook.</x:v>
+      </x:c>
+      <x:c r="G169" s="25" t="str">
+        <x:v>1) Be advised: we had failures. They are recorded in the technical logbook.
+2) Attention: we had failures. They are recorded in the technical logbook.
+3) For information: we had failures. They are recorded in the technical logbook.</x:v>
       </x:c>
     </x:row>
     <x:row r="170" ht="120" hidden="0" customHeight="1">
@@ -2934,9 +3419,12 @@
         <x:v>We had a hard landing.</x:v>
       </x:c>
       <x:c r="F170" s="25" t="str">
-        <x:v>1) We had a hard landing.
-2) Be advised: we had a hard landing.
-3) Attention: we had a hard landing.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G170" s="25" t="str">
+        <x:v>1) Be advised: we had a hard landing.
+2) Attention: we had a hard landing.
+3) For information: we had a hard landing.</x:v>
       </x:c>
     </x:row>
     <x:row r="171" ht="120" hidden="0" customHeight="1">
@@ -2950,9 +3438,12 @@
         <x:v>Two nautical miles from pick up location.</x:v>
       </x:c>
       <x:c r="F171" s="25" t="str">
-        <x:v>1) Two nautical miles from the pickup location.
-2) Be advised: two nautical miles from the pickup location.
-3) Attention: two nautical miles from the pickup location.</x:v>
+        <x:v>Two nautical miles from the pickup location.</x:v>
+      </x:c>
+      <x:c r="G171" s="25" t="str">
+        <x:v>1) Be advised: two nautical miles from the pickup location.
+2) Attention: two nautical miles from the pickup location.
+3) For information: two nautical miles from the pickup location.</x:v>
       </x:c>
     </x:row>
     <x:row r="172" ht="120" hidden="0" customHeight="1">
@@ -2966,9 +3457,12 @@
         <x:v>Hr we are now approaching to drop point thanks for the help and see you next time.</x:v>
       </x:c>
       <x:c r="F172" s="25" t="str">
-        <x:v>1) Heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
-2) Be advised: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
-3) Attention: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.</x:v>
+        <x:v>Heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.</x:v>
+      </x:c>
+      <x:c r="G172" s="25" t="str">
+        <x:v>1) Be advised: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
+2) Attention: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.
+3) For information: heli-rescuer, we are approaching the drop point. Thanks for the help; see you next time.</x:v>
       </x:c>
     </x:row>
     <x:row r="173" ht="120" hidden="0" customHeight="1">
@@ -2982,9 +3476,12 @@
         <x:v>We are entering into designated SAR area it's time to start our search for the casualties.</x:v>
       </x:c>
       <x:c r="F173" s="25" t="str">
-        <x:v>1) We are entering the designated SAR area. Start the search for casualties.
-2) We're entering the designated SAR area. Start the search for casualties.
-3) Attention: we are entering the designated SAR area. Start the search for casualties.</x:v>
+        <x:v>We are entering the designated SAR area. Start the search for casualties.</x:v>
+      </x:c>
+      <x:c r="G173" s="25" t="str">
+        <x:v>1) We're entering the designated SAR area. Start the search for casualties.
+2) Attention: we are entering the designated SAR area. Start the search for casualties.
+3) For information: we are entering the designated SAR area. Start the search for casualties.</x:v>
       </x:c>
     </x:row>
     <x:row r="174" ht="120" hidden="0" customHeight="1">
@@ -2998,9 +3495,12 @@
         <x:v>SAR area starts here watch out and let's find our signed casualties.</x:v>
       </x:c>
       <x:c r="F174" s="25" t="str">
-        <x:v>1) The SAR area starts here. Stay alert and search for casualties.
-2) Be advised: the SAR area starts here. Stay alert and search for casualties.
-3) Attention: the SAR area starts here. Stay alert and search for casualties.</x:v>
+        <x:v>The SAR area starts here. Stay alert and search for casualties.</x:v>
+      </x:c>
+      <x:c r="G174" s="25" t="str">
+        <x:v>1) Be advised: the SAR area starts here. Stay alert and search for casualties.
+2) Attention: the SAR area starts here. Stay alert and search for casualties.
+3) For information: the SAR area starts here. Stay alert and search for casualties.</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="120" hidden="0" customHeight="1">
@@ -3014,9 +3514,12 @@
         <x:v>Crew please stop searching for the survivor now we are entering in the assigned area.</x:v>
       </x:c>
       <x:c r="F175" s="25" t="str">
-        <x:v>1) Crew, stop searching. We are now entering the assigned area.
-2) Crew, stop searching. We're now entering the assigned area.
-3) All crew, stop searching. We are now entering the assigned area.</x:v>
+        <x:v>Crew, stop searching. We are now entering the assigned area.</x:v>
+      </x:c>
+      <x:c r="G175" s="25" t="str">
+        <x:v>1) Crew, stop searching. We're now entering the assigned area.
+2) All crew, stop searching. We are now entering the assigned area.
+3) For information: crew, stop searching. We are now entering the assigned area.</x:v>
       </x:c>
     </x:row>
     <x:row r="176" ht="120" hidden="0" customHeight="1">
@@ -3030,9 +3533,12 @@
         <x:v>Confirmed solve every of established the clock is ticking let's find the casualties now.</x:v>
       </x:c>
       <x:c r="F176" s="25" t="str">
-        <x:v>1) Confirmed. The clock is ticking; start the search now.
-2) Be advised: confirmed. The clock is ticking; start the search now.
-3) Attention: confirmed. The clock is ticking; start the search now.</x:v>
+        <x:v>Confirmed. The clock is ticking; start the search now.</x:v>
+      </x:c>
+      <x:c r="G176" s="25" t="str">
+        <x:v>1) Be advised: confirmed. The clock is ticking; start the search now.
+2) Attention: confirmed. The clock is ticking; start the search now.
+3) For information: confirmed. The clock is ticking; start the search now.</x:v>
       </x:c>
     </x:row>
     <x:row r="177" ht="120" hidden="0" customHeight="1">
@@ -3046,9 +3552,12 @@
         <x:v>The boundary crossed let's execute the search plan and locate the survivors.</x:v>
       </x:c>
       <x:c r="F177" s="25" t="str">
-        <x:v>1) Boundary crossed. Execute the search plan and locate the survivors.
-2) Be advised: boundary crossed. Execute the search plan and locate the survivors.
-3) Attention: boundary crossed. Execute the search plan and locate the survivors.</x:v>
+        <x:v>Boundary crossed. Execute the search plan and locate the survivors.</x:v>
+      </x:c>
+      <x:c r="G177" s="25" t="str">
+        <x:v>1) Be advised: boundary crossed. Execute the search plan and locate the survivors.
+2) Attention: boundary crossed. Execute the search plan and locate the survivors.
+3) For information: boundary crossed. Execute the search plan and locate the survivors.</x:v>
       </x:c>
     </x:row>
     <x:row r="178" ht="120" hidden="0" customHeight="1">
@@ -3062,9 +3571,12 @@
         <x:v>We have reached the search and rescue zone initiate the search pattern for survivors.</x:v>
       </x:c>
       <x:c r="F178" s="25" t="str">
-        <x:v>1) We have reached the search-and-rescue zone. Begin the search pattern for survivors.
-2) We've reached the search-and-rescue zone. Begin the search pattern for survivors.
-3) Attention: we have reached the search-and-rescue zone. Begin the search pattern for survivors.</x:v>
+        <x:v>We have reached the search-and-rescue zone. Begin the search pattern for survivors.</x:v>
+      </x:c>
+      <x:c r="G178" s="25" t="str">
+        <x:v>1) We've reached the search-and-rescue zone. Begin the search pattern for survivors.
+2) Attention: we have reached the search-and-rescue zone. Begin the search pattern for survivors.
+3) For information: we have reached the search-and-rescue zone. Begin the search pattern for survivors.</x:v>
       </x:c>
     </x:row>
     <x:row r="179" ht="120" hidden="0" customHeight="1">
@@ -3078,9 +3590,12 @@
         <x:v>Crew is cutting back.</x:v>
       </x:c>
       <x:c r="F179" s="25" t="str">
-        <x:v>1) Crew is coming back.
-2) Be advised: crew is coming back.
-3) Attention: crew is coming back.</x:v>
+        <x:v>Crew is coming back.</x:v>
+      </x:c>
+      <x:c r="G179" s="25" t="str">
+        <x:v>1) Be advised: crew is coming back.
+2) Attention: crew is coming back.
+3) For information: crew is coming back.</x:v>
       </x:c>
     </x:row>
     <x:row r="180" ht="120" hidden="0" customHeight="1">
@@ -3094,9 +3609,12 @@
         <x:v>Let's go.</x:v>
       </x:c>
       <x:c r="F180" s="25" t="str">
-        <x:v>1) Let's go.
-2) Be advised: let's go.
-3) Attention: let's go.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G180" s="25" t="str">
+        <x:v>1) Be advised: let's go.
+2) Attention: let's go.
+3) For information: let's go.</x:v>
       </x:c>
     </x:row>
     <x:row r="181" ht="120" hidden="0" customHeight="1">
@@ -3110,9 +3628,12 @@
         <x:v>We're crew are we able to accept a new dispatch or do we need to come back to base.</x:v>
       </x:c>
       <x:c r="F181" s="25" t="str">
-        <x:v>1) Crew, can we accept a new dispatch, or do we need to return to base?
-2) Can you confirm: crew, can we accept a new dispatch, or do we need to return to base?
-3) All crew, can we accept a new dispatch, or do we need to return to base?</x:v>
+        <x:v>Crew, can we accept a new dispatch, or do we need to return to base?</x:v>
+      </x:c>
+      <x:c r="G181" s="25" t="str">
+        <x:v>1) Can you confirm: crew, can we accept a new dispatch, or do we need to return to base?
+2) All crew, can we accept a new dispatch, or do we need to return to base?
+3) Please confirm: crew, can we accept a new dispatch, or do we need to return to base?</x:v>
       </x:c>
     </x:row>
     <x:row r="182" ht="120" hidden="0" customHeight="1">
@@ -3126,9 +3647,12 @@
         <x:v>I believe we must go back to the base before we accept new dispatches.</x:v>
       </x:c>
       <x:c r="F182" s="25" t="str">
-        <x:v>1) I believe we should return to base before accepting another dispatch.
-2) Be advised: i believe we should return to base before accepting another dispatch.
-3) Attention: i believe we should return to base before accepting another dispatch.</x:v>
+        <x:v>I believe we should return to base before accepting another dispatch.</x:v>
+      </x:c>
+      <x:c r="G182" s="25" t="str">
+        <x:v>1) Be advised: i believe we should return to base before accepting another dispatch.
+2) Attention: i believe we should return to base before accepting another dispatch.
+3) For information: i believe we should return to base before accepting another dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="120" hidden="0" customHeight="1">
@@ -3142,9 +3666,12 @@
         <x:v>Hey we have a new dispatch.</x:v>
       </x:c>
       <x:c r="F183" s="25" t="str">
-        <x:v>1) We have a new dispatch.
-2) Be advised: we have a new dispatch.
-3) Attention: we have a new dispatch.</x:v>
+        <x:v>We have a new dispatch.</x:v>
+      </x:c>
+      <x:c r="G183" s="25" t="str">
+        <x:v>1) Be advised: we have a new dispatch.
+2) Attention: we have a new dispatch.
+3) For information: we have a new dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="120" hidden="0" customHeight="1">
@@ -3158,9 +3685,12 @@
         <x:v>How crew we have a new assignment.</x:v>
       </x:c>
       <x:c r="F184" s="25" t="str">
-        <x:v>1) Crew, we have a new assignment.
-2) Be advised: crew, we have a new assignment.
-3) All crew, we have a new assignment.</x:v>
+        <x:v>Crew, we have a new assignment.</x:v>
+      </x:c>
+      <x:c r="G184" s="25" t="str">
+        <x:v>1) Be advised: crew, we have a new assignment.
+2) All crew, we have a new assignment.
+3) For information: crew, we have a new assignment.</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="120" hidden="0" customHeight="1">
@@ -3174,9 +3704,12 @@
         <x:v>How we have another dispatch.</x:v>
       </x:c>
       <x:c r="F185" s="25" t="str">
-        <x:v>1) We have another dispatch.
-2) Be advised: we have another dispatch.
-3) Attention: we have another dispatch.</x:v>
+        <x:v>We have another dispatch.</x:v>
+      </x:c>
+      <x:c r="G185" s="25" t="str">
+        <x:v>1) Be advised: we have another dispatch.
+2) Attention: we have another dispatch.
+3) For information: we have another dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="186" ht="120" hidden="0" customHeight="1">
@@ -3190,9 +3723,12 @@
         <x:v>Busy day we received a new dispatch.</x:v>
       </x:c>
       <x:c r="F186" s="25" t="str">
-        <x:v>1) Busy day we received a new dispatch.
-2) Be advised: busy day we received a new dispatch.
-3) Attention: busy day we received a new dispatch.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G186" s="25" t="str">
+        <x:v>1) Be advised: busy day we received a new dispatch.
+2) Attention: busy day we received a new dispatch.
+3) For information: busy day we received a new dispatch.</x:v>
       </x:c>
     </x:row>
     <x:row r="187" ht="120" hidden="0" customHeight="1">
@@ -3206,9 +3742,12 @@
         <x:v>Looks set to drop point.</x:v>
       </x:c>
       <x:c r="F187" s="25" t="str">
-        <x:v>1) Route set to the drop point.
-2) Be advised: route set to the drop point.
-3) Attention: route set to the drop point.</x:v>
+        <x:v>Route set to the drop point.</x:v>
+      </x:c>
+      <x:c r="G187" s="25" t="str">
+        <x:v>1) Be advised: route set to the drop point.
+2) Attention: route set to the drop point.
+3) For information: route set to the drop point.</x:v>
       </x:c>
     </x:row>
     <x:row r="188" ht="120" hidden="0" customHeight="1">
@@ -3222,9 +3761,12 @@
         <x:v>Group set to the pick up point.</x:v>
       </x:c>
       <x:c r="F188" s="25" t="str">
-        <x:v>1) Route set to the pickup point.
-2) Be advised: route set to the pickup point.
-3) Attention: route set to the pickup point.</x:v>
+        <x:v>Route set to the pickup point.</x:v>
+      </x:c>
+      <x:c r="G188" s="25" t="str">
+        <x:v>1) Be advised: route set to the pickup point.
+2) Attention: route set to the pickup point.
+3) For information: route set to the pickup point.</x:v>
       </x:c>
     </x:row>
     <x:row r="189" ht="120" hidden="0" customHeight="1">
@@ -3238,9 +3780,12 @@
         <x:v>Copy paramedic here comm check.</x:v>
       </x:c>
       <x:c r="F189" s="25" t="str">
-        <x:v>1) Copy, paramedic here. Communications check.
-2) Be advised: copy, paramedic here. Communications check.
-3) Attention: copy, paramedic here. Communications check.</x:v>
+        <x:v>Copy, paramedic here. Communications check.</x:v>
+      </x:c>
+      <x:c r="G189" s="25" t="str">
+        <x:v>1) Be advised: copy, paramedic here. Communications check.
+2) Attention: copy, paramedic here. Communications check.
+3) For information: copy, paramedic here. Communications check.</x:v>
       </x:c>
     </x:row>
     <x:row r="190" ht="120" hidden="0" customHeight="1">
@@ -3254,9 +3799,12 @@
         <x:v>Hi anna nice to meet you again are you free for lunch tomorrow.</x:v>
       </x:c>
       <x:c r="F190" s="25" t="str">
-        <x:v>1) Hi Anna, nice to meet you again. Are you free for lunch tomorrow?
-2) Can you confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?
-3) Please confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?</x:v>
+        <x:v>Hi Anna, nice to meet you again. Are you free for lunch tomorrow?</x:v>
+      </x:c>
+      <x:c r="G190" s="25" t="str">
+        <x:v>1) Can you confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?
+2) Please confirm: hi Anna, nice to meet you again. Are you free for lunch tomorrow?
+3) Message update: hi Anna, nice to meet you again. Are you free for lunch tomorrow?</x:v>
       </x:c>
     </x:row>
     <x:row r="191" ht="120" hidden="0" customHeight="1">
@@ -3270,9 +3818,12 @@
         <x:v>Stretches secured.</x:v>
       </x:c>
       <x:c r="F191" s="25" t="str">
-        <x:v>1) Stretcher secured.
-2) Be advised: stretcher secured.
-3) Attention: stretcher secured.</x:v>
+        <x:v>Stretcher secured.</x:v>
+      </x:c>
+      <x:c r="G191" s="25" t="str">
+        <x:v>1) Be advised: stretcher secured.
+2) Attention: stretcher secured.
+3) For information: stretcher secured.</x:v>
       </x:c>
     </x:row>
     <x:row r="192" ht="120" hidden="0" customHeight="1">
@@ -3286,9 +3837,12 @@
         <x:v>The ambulance with no paramedic.</x:v>
       </x:c>
       <x:c r="F192" s="25" t="str">
-        <x:v>1) An ambulance is on scene, but no paramedic is present.
-2) Be advised: an ambulance is on scene, but no paramedic is present.
-3) Attention: an ambulance is on scene, but no paramedic is present.</x:v>
+        <x:v>An ambulance is on scene, but no paramedic is present.</x:v>
+      </x:c>
+      <x:c r="G192" s="25" t="str">
+        <x:v>1) Be advised: an ambulance is on scene, but no paramedic is present.
+2) Attention: an ambulance is on scene, but no paramedic is present.
+3) For information: an ambulance is on scene, but no paramedic is present.</x:v>
       </x:c>
     </x:row>
     <x:row r="193" ht="120" hidden="0" customHeight="1">
@@ -3302,9 +3856,12 @@
         <x:v>Duck here comm check.</x:v>
       </x:c>
       <x:c r="F193" s="25" t="str">
-        <x:v>1) Medic here. Communications check.
-2) Be advised: medic here. Communications check.
-3) Attention: medic here. Communications check.</x:v>
+        <x:v>Medic here. Communications check.</x:v>
+      </x:c>
+      <x:c r="G193" s="25" t="str">
+        <x:v>1) Be advised: medic here. Communications check.
+2) Attention: medic here. Communications check.
+3) For information: medic here. Communications check.</x:v>
       </x:c>
     </x:row>
     <x:row r="194" ht="120" hidden="0" customHeight="1">
@@ -3318,9 +3875,12 @@
         <x:v>Confirmed on scene.</x:v>
       </x:c>
       <x:c r="F194" s="25" t="str">
-        <x:v>1) Confirmed on scene.
-2) Be advised: confirmed on scene.
-3) Attention: confirmed on scene.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G194" s="25" t="str">
+        <x:v>1) Be advised: confirmed on scene.
+2) Attention: confirmed on scene.
+3) For information: confirmed on scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="195" ht="120" hidden="0" customHeight="1">
@@ -3334,9 +3894,12 @@
         <x:v>Fire engine.</x:v>
       </x:c>
       <x:c r="F195" s="25" t="str">
-        <x:v>1) Fire engine.
-2) Be advised: fire engine.
-3) Attention: fire engine.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G195" s="25" t="str">
+        <x:v>1) Be advised: fire engine.
+2) Attention: fire engine.
+3) For information: fire engine.</x:v>
       </x:c>
     </x:row>
     <x:row r="196" ht="120" hidden="0" customHeight="1">
@@ -3350,9 +3913,12 @@
         <x:v>We need time for ground operations please stand by.</x:v>
       </x:c>
       <x:c r="F196" s="25" t="str">
-        <x:v>1) We need time for ground operations. Please stand by.
-2) Be advised: we need time for ground operations. Please stand by.
-3) Attention: we need time for ground operations. Please stand by.</x:v>
+        <x:v>We need time for ground operations. Please stand by.</x:v>
+      </x:c>
+      <x:c r="G196" s="25" t="str">
+        <x:v>1) Be advised: we need time for ground operations. Please stand by.
+2) Attention: we need time for ground operations. Please stand by.
+3) For information: we need time for ground operations. Please stand by.</x:v>
       </x:c>
     </x:row>
     <x:row r="197" ht="120" hidden="0" customHeight="1">
@@ -3366,9 +3932,12 @@
         <x:v>I said of possible hospital destination for our patient info available on tablet we can confirm or change later.</x:v>
       </x:c>
       <x:c r="F197" s="25" t="str">
-        <x:v>1) A possible hospital destination is available on the tablet. We can confirm or change it later.
-2) Be advised: a possible hospital destination is available on the tablet. We can confirm or change it later.
-3) Attention: a possible hospital destination is available on the tablet. We can confirm or change it later.</x:v>
+        <x:v>A possible hospital destination is available on the tablet. We can confirm or change it later.</x:v>
+      </x:c>
+      <x:c r="G197" s="25" t="str">
+        <x:v>1) Be advised: a possible hospital destination is available on the tablet. We can confirm or change it later.
+2) Attention: a possible hospital destination is available on the tablet. We can confirm or change it later.
+3) For information: a possible hospital destination is available on the tablet. We can confirm or change it later.</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="120" hidden="0" customHeight="1">
@@ -3382,9 +3951,12 @@
         <x:v>Patient has died.</x:v>
       </x:c>
       <x:c r="F198" s="25" t="str">
-        <x:v>1) Patient has died.
-2) Be advised: patient has died.
-3) Attention: patient has died.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G198" s="25" t="str">
+        <x:v>1) Be advised: patient has died.
+2) Attention: patient has died.
+3) For information: patient has died.</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="120" hidden="0" customHeight="1">
@@ -3398,9 +3970,12 @@
         <x:v>Patient life signs of fading.</x:v>
       </x:c>
       <x:c r="F199" s="25" t="str">
-        <x:v>1) The patient's vital signs are fading.
-2) Be advised: the patient's vital signs are fading.
-3) Attention: the patient's vital signs are fading.</x:v>
+        <x:v>The patient's vital signs are fading.</x:v>
+      </x:c>
+      <x:c r="G199" s="25" t="str">
+        <x:v>1) Be advised: the patient's vital signs are fading.
+2) Attention: the patient's vital signs are fading.
+3) For information: the patient's vital signs are fading.</x:v>
       </x:c>
     </x:row>
     <x:row r="200" ht="24" hidden="0" customHeight="1">
@@ -3414,9 +3989,12 @@
         <x:v>Patient location is far away ambulance crew on seen may transport patient to the meeting point proposed on tablet please confirm if we want to meet midway.</x:v>
       </x:c>
       <x:c r="F200" s="25" t="str">
-        <x:v>1) The patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
-2) Be advised: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
-3) Attention: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.</x:v>
+        <x:v>The patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.</x:v>
+      </x:c>
+      <x:c r="G200" s="25" t="str">
+        <x:v>1) Be advised: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
+2) Attention: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.
+3) For information: the patient is far away. The ambulance crew may transport the patient to the meeting point shown on the tablet. Confirm whether we should meet midway.</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="120" hidden="0" customHeight="1">
@@ -3430,9 +4008,12 @@
         <x:v>Patient on board take care.</x:v>
       </x:c>
       <x:c r="F201" s="25" t="str">
-        <x:v>1) Patient on board. Take care.
-2) Be advised: patient on board. Take care.
-3) The patient is on board. Take care.</x:v>
+        <x:v>Patient on board. Take care.</x:v>
+      </x:c>
+      <x:c r="G201" s="25" t="str">
+        <x:v>1) Be advised: patient on board. Take care.
+2) The patient is on board. Take care.
+3) For information: patient on board. Take care.</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="120" hidden="0" customHeight="1">
@@ -3446,9 +4027,12 @@
         <x:v>Patient has been the board to the hospital key is safe.</x:v>
       </x:c>
       <x:c r="F202" s="25" t="str">
-        <x:v>1) The patient has been delivered to the hospital and is safe.
-2) Be advised: the patient has been delivered to the hospital and is safe.
-3) Attention: the patient has been delivered to the hospital and is safe.</x:v>
+        <x:v>The patient has been delivered to the hospital and is safe.</x:v>
+      </x:c>
+      <x:c r="G202" s="25" t="str">
+        <x:v>1) Be advised: the patient has been delivered to the hospital and is safe.
+2) Attention: the patient has been delivered to the hospital and is safe.
+3) For information: the patient has been delivered to the hospital and is safe.</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="120" hidden="0" customHeight="1">
@@ -3462,9 +4046,12 @@
         <x:v>Police.</x:v>
       </x:c>
       <x:c r="F203" s="25" t="str">
-        <x:v>1) Police.
-2) Be advised: police.
-3) Attention: police.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G203" s="25" t="str">
+        <x:v>1) Be advised: police.
+2) Attention: police.
+3) For information: police.</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="120" hidden="0" customHeight="1">
@@ -3478,9 +4065,12 @@
         <x:v>Patients has been deboarded to the hospital.</x:v>
       </x:c>
       <x:c r="F204" s="25" t="str">
-        <x:v>1) The patient has been deboarded at the hospital.
-2) Be advised: the patient has been deboarded at the hospital.
-3) Attention: the patient has been deboarded at the hospital.</x:v>
+        <x:v>The patient has been deboarded at the hospital.</x:v>
+      </x:c>
+      <x:c r="G204" s="25" t="str">
+        <x:v>1) Be advised: the patient has been deboarded at the hospital.
+2) Attention: the patient has been deboarded at the hospital.
+3) For information: the patient has been deboarded at the hospital.</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="120" hidden="0" customHeight="1">
@@ -3494,9 +4084,12 @@
         <x:v>We will be first on scene.</x:v>
       </x:c>
       <x:c r="F205" s="25" t="str">
-        <x:v>1) We will be first on scene.
-2) Be advised: we will be first on scene.
-3) Attention: we will be first on scene.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G205" s="25" t="str">
+        <x:v>1) Be advised: we will be first on scene.
+2) Attention: we will be first on scene.
+3) For information: we will be first on scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="120" hidden="0" customHeight="1">
@@ -3510,9 +4103,12 @@
         <x:v>We will find an ambulance not far away from accident site they are unable to reach the site.</x:v>
       </x:c>
       <x:c r="F206" s="25" t="str">
-        <x:v>1) We will find an ambulance near the accident site; it cannot reach the scene.
-2) We will find an ambulance near the accident site; it can't reach the scene.
-3) Attention: we will find an ambulance near the accident site; it cannot reach the scene.</x:v>
+        <x:v>We will find an ambulance near the accident site; it cannot reach the scene.</x:v>
+      </x:c>
+      <x:c r="G206" s="25" t="str">
+        <x:v>1) We will find an ambulance near the accident site; it can't reach the scene.
+2) Attention: we will find an ambulance near the accident site; it cannot reach the scene.
+3) For information: we will find an ambulance near the accident site; it cannot reach the scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="207" ht="120" hidden="0" customHeight="1">
@@ -3526,9 +4122,12 @@
         <x:v>Cpr in progress please stand by it may take time.</x:v>
       </x:c>
       <x:c r="F207" s="25" t="str">
-        <x:v>1) CPR in progress. Please stand by; it may take time.
-2) Be advised: cPR in progress. Please stand by; it may take time.
-3) Attention: cPR in progress. Please stand by; it may take time.</x:v>
+        <x:v>CPR in progress. Please stand by; it may take time.</x:v>
+      </x:c>
+      <x:c r="G207" s="25" t="str">
+        <x:v>1) Be advised: cPR in progress. Please stand by; it may take time.
+2) Attention: cPR in progress. Please stand by; it may take time.
+3) For information: cPR in progress. Please stand by; it may take time.</x:v>
       </x:c>
     </x:row>
     <x:row r="208" ht="120" hidden="0" customHeight="1">
@@ -3542,9 +4141,12 @@
         <x:v>We lost the patient we have to record the time of the death please stand by until we secure the cabin.</x:v>
       </x:c>
       <x:c r="F208" s="25" t="str">
-        <x:v>1) We lost the patient. Record the time of death and stand by while we secure the cabin.
-2) Be advised: we lost the patient. Record the time of death and stand by while we secure the cabin.
-3) Attention: we lost the patient. Record the time of death and stand by while we secure the cabin.</x:v>
+        <x:v>We lost the patient. Record the time of death and stand by while we secure the cabin.</x:v>
+      </x:c>
+      <x:c r="G208" s="25" t="str">
+        <x:v>1) Be advised: we lost the patient. Record the time of death and stand by while we secure the cabin.
+2) Attention: we lost the patient. Record the time of death and stand by while we secure the cabin.
+3) For information: we lost the patient. Record the time of death and stand by while we secure the cabin.</x:v>
       </x:c>
     </x:row>
     <x:row r="209" ht="120" hidden="0" customHeight="1">
@@ -3558,9 +4160,12 @@
         <x:v>Good cpr successfully reanimated patient we are now securing him for the flight please wait for clearance.</x:v>
       </x:c>
       <x:c r="F209" s="25" t="str">
-        <x:v>1) CPR was successful. The patient has been resuscitated; we are securing them for flight.
-2) Be advised: cPR was successful. The patient has been resuscitated; we are securing them for flight.
-3) Attention: cPR was successful. The patient has been resuscitated; we are securing them for flight.</x:v>
+        <x:v>CPR was successful. The patient has been resuscitated; we are securing them for flight.</x:v>
+      </x:c>
+      <x:c r="G209" s="25" t="str">
+        <x:v>1) Be advised: cPR was successful. The patient has been resuscitated; we are securing them for flight.
+2) Attention: cPR was successful. The patient has been resuscitated; we are securing them for flight.
+3) For information: cPR was successful. The patient has been resuscitated; we are securing them for flight.</x:v>
       </x:c>
     </x:row>
     <x:row r="210" ht="120" hidden="0" customHeight="1">
@@ -3574,9 +4179,12 @@
         <x:v>Patient conditions are critical we need extra time to stabilize for transport please wait.</x:v>
       </x:c>
       <x:c r="F210" s="25" t="str">
-        <x:v>1) The patient is critical. We need extra time to stabilize them for transport.
-2) Be advised: the patient is critical. We need extra time to stabilize them for transport.
-3) Attention: the patient is critical. We need extra time to stabilize them for transport.</x:v>
+        <x:v>The patient is critical. We need extra time to stabilize them for transport.</x:v>
+      </x:c>
+      <x:c r="G210" s="25" t="str">
+        <x:v>1) Be advised: the patient is critical. We need extra time to stabilize them for transport.
+2) Attention: the patient is critical. We need extra time to stabilize them for transport.
+3) For information: the patient is critical. We need extra time to stabilize them for transport.</x:v>
       </x:c>
     </x:row>
     <x:row r="211" ht="120" hidden="0" customHeight="1">
@@ -3590,9 +4198,12 @@
         <x:v>I believe we lost the organ it's too degraded.</x:v>
       </x:c>
       <x:c r="F211" s="25" t="str">
-        <x:v>1) We lost the organ; it is too degraded.
-2) Be advised: we lost the organ; it is too degraded.
-3) Attention: we lost the organ; it is too degraded.</x:v>
+        <x:v>We lost the organ; it is too degraded.</x:v>
+      </x:c>
+      <x:c r="G211" s="25" t="str">
+        <x:v>1) Be advised: we lost the organ; it is too degraded.
+2) Attention: we lost the organ; it is too degraded.
+3) For information: we lost the organ; it is too degraded.</x:v>
       </x:c>
     </x:row>
     <x:row r="212" ht="120" hidden="0" customHeight="1">
@@ -3606,9 +4217,12 @@
         <x:v>Organs data seems to be degrading.</x:v>
       </x:c>
       <x:c r="F212" s="25" t="str">
-        <x:v>1) The organ's condition is deteriorating.
-2) Be advised: the organ's condition is deteriorating.
-3) Attention: the organ's condition is deteriorating.</x:v>
+        <x:v>The organ's condition is deteriorating.</x:v>
+      </x:c>
+      <x:c r="G212" s="25" t="str">
+        <x:v>1) Be advised: the organ's condition is deteriorating.
+2) Attention: the organ's condition is deteriorating.
+3) For information: the organ's condition is deteriorating.</x:v>
       </x:c>
     </x:row>
     <x:row r="213" ht="36" hidden="0" customHeight="1">
@@ -3622,9 +4236,12 @@
         <x:v>Let's proceed with a small briefing about our next operations as soon as we arrive h i will proceed to the scene securing the area after their clearance our crew will join them to perform the medical operation at the end of rescue operations the medical cruel board followed by hr in case the engine has to be transported with hoist out i will be boarded first all clear.</x:v>
       </x:c>
       <x:c r="F213" s="25" t="str">
-        <x:v>1) Briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
-2) Be advised: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
-3) Attention: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.</x:v>
+        <x:v>Briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.</x:v>
+      </x:c>
+      <x:c r="G213" s="25" t="str">
+        <x:v>1) Be advised: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
+2) Attention: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.
+3) For information: briefing: on arrival, I will secure the scene. After clearance, the crew will join for medical operations. At the end, the medical crew boards first; the heli-rescuer boards first if hoist extraction is required.</x:v>
       </x:c>
     </x:row>
     <x:row r="214" ht="120" hidden="0" customHeight="1">
@@ -3638,9 +4255,12 @@
         <x:v>Welcome onboard hello his viewers.</x:v>
       </x:c>
       <x:c r="F214" s="25" t="str">
-        <x:v>1) Welcome on board, heli-rescuer.
-2) Be advised: welcome on board, heli-rescuer.
-3) Attention: welcome on board, heli-rescuer.</x:v>
+        <x:v>Welcome on board, heli-rescuer.</x:v>
+      </x:c>
+      <x:c r="G214" s="25" t="str">
+        <x:v>1) Be advised: welcome on board, heli-rescuer.
+2) Attention: welcome on board, heli-rescuer.
+3) For information: welcome on board, heli-rescuer.</x:v>
       </x:c>
     </x:row>
     <x:row r="215" ht="120" hidden="0" customHeight="1">
@@ -3654,9 +4274,12 @@
         <x:v>If you need refueling please ask.</x:v>
       </x:c>
       <x:c r="F215" s="25" t="str">
-        <x:v>1) If you need refueling please ask.
-2) Be advised: if you need refueling please ask.
-3) Attention: if you need refueling please ask.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G215" s="25" t="str">
+        <x:v>1) Be advised: if you need refueling please ask.
+2) Attention: if you need refueling please ask.
+3) For information: if you need refueling please ask.</x:v>
       </x:c>
     </x:row>
     <x:row r="216" ht="120" hidden="0" customHeight="1">
@@ -3670,9 +4293,12 @@
         <x:v>Fuel is as you requested.</x:v>
       </x:c>
       <x:c r="F216" s="25" t="str">
-        <x:v>1) Fuel is as you requested.
-2) Be advised: fuel is as you requested.
-3) Attention: fuel is as you requested.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G216" s="25" t="str">
+        <x:v>1) Be advised: fuel is as you requested.
+2) Attention: fuel is as you requested.
+3) For information: fuel is as you requested.</x:v>
       </x:c>
     </x:row>
     <x:row r="217" ht="120" hidden="0" customHeight="1">
@@ -3686,9 +4312,12 @@
         <x:v>Fuel tanks are almost full.</x:v>
       </x:c>
       <x:c r="F217" s="25" t="str">
-        <x:v>1) Fuel tanks are almost full.
-2) Be advised: fuel tanks are almost full.
-3) Attention: fuel tanks are almost full.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G217" s="25" t="str">
+        <x:v>1) Be advised: fuel tanks are almost full.
+2) Attention: fuel tanks are almost full.
+3) For information: fuel tanks are almost full.</x:v>
       </x:c>
     </x:row>
     <x:row r="218" ht="120" hidden="0" customHeight="1">
@@ -3702,9 +4331,12 @@
         <x:v>Refueling has not been performed and fuel level is low.</x:v>
       </x:c>
       <x:c r="F218" s="25" t="str">
-        <x:v>1) Refueling has not been performed and fuel level is low.
-2) Be advised: refueling has not been performed and fuel level is low.
-3) Attention: refueling has not been performed and fuel level is low.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G218" s="25" t="str">
+        <x:v>1) Be advised: refueling has not been performed and fuel level is low.
+2) Attention: refueling has not been performed and fuel level is low.
+3) For information: refueling has not been performed and fuel level is low.</x:v>
       </x:c>
     </x:row>
     <x:row r="219" ht="120" hidden="0" customHeight="1">
@@ -3718,9 +4350,12 @@
         <x:v>Gp you disconnected ready to go good day.</x:v>
       </x:c>
       <x:c r="F219" s="25" t="str">
-        <x:v>1) GPU disconnected. Ready to go. Good day.
-2) Be advised: gPU disconnected. Ready to go. Good day.
-3) Attention: gPU disconnected. Ready to go. Good day.</x:v>
+        <x:v>GPU disconnected. Ready to go. Good day.</x:v>
+      </x:c>
+      <x:c r="G219" s="25" t="str">
+        <x:v>1) Be advised: gPU disconnected. Ready to go. Good day.
+2) Attention: gPU disconnected. Ready to go. Good day.
+3) For information: gPU disconnected. Ready to go. Good day.</x:v>
       </x:c>
     </x:row>
     <x:row r="220" ht="120" hidden="0" customHeight="1">
@@ -3734,9 +4369,12 @@
         <x:v>I kept captain helicopter is ready to fly law book filled and signed.</x:v>
       </x:c>
       <x:c r="F220" s="25" t="str">
-        <x:v>1) Captain, the helicopter is ready for flight. The logbook is completed and signed.
-2) Be advised: captain, the helicopter is ready for flight. The logbook is completed and signed.
-3) Attention: captain, the helicopter is ready for flight. The logbook is completed and signed.</x:v>
+        <x:v>Captain, the helicopter is ready for flight. The logbook is completed and signed.</x:v>
+      </x:c>
+      <x:c r="G220" s="25" t="str">
+        <x:v>1) Be advised: captain, the helicopter is ready for flight. The logbook is completed and signed.
+2) Attention: captain, the helicopter is ready for flight. The logbook is completed and signed.
+3) For information: captain, the helicopter is ready for flight. The logbook is completed and signed.</x:v>
       </x:c>
     </x:row>
     <x:row r="221" ht="120" hidden="0" customHeight="1">
@@ -3750,9 +4388,12 @@
         <x:v>Hey good morning all ready for the missions.</x:v>
       </x:c>
       <x:c r="F221" s="25" t="str">
-        <x:v>1) Good morning, everyone. Ready for the mission?
-2) Can you confirm: good morning, everyone. Ready for the mission?
-3) Please confirm: good morning, everyone. Ready for the mission?</x:v>
+        <x:v>Good morning, everyone. Ready for the mission?</x:v>
+      </x:c>
+      <x:c r="G221" s="25" t="str">
+        <x:v>1) Can you confirm: good morning, everyone. Ready for the mission?
+2) Please confirm: good morning, everyone. Ready for the mission?
+3) Message update: good morning, everyone. Ready for the mission?</x:v>
       </x:c>
     </x:row>
     <x:row r="222" ht="120" hidden="0" customHeight="1">
@@ -3766,9 +4407,12 @@
         <x:v>Really to supply external power at your request.</x:v>
       </x:c>
       <x:c r="F222" s="25" t="str">
-        <x:v>1) Ready to provide external power at your request.
-2) Be advised: ready to provide external power at your request.
-3) Attention: ready to provide external power at your request.</x:v>
+        <x:v>Ready to provide external power at your request.</x:v>
+      </x:c>
+      <x:c r="G222" s="25" t="str">
+        <x:v>1) Be advised: ready to provide external power at your request.
+2) Attention: ready to provide external power at your request.
+3) For information: ready to provide external power at your request.</x:v>
       </x:c>
     </x:row>
     <x:row r="223" ht="120" hidden="0" customHeight="1">
@@ -3782,9 +4426,12 @@
         <x:v>Bye see you tomorrow.</x:v>
       </x:c>
       <x:c r="F223" s="25" t="str">
-        <x:v>1) Bye see you tomorrow.
-2) Be advised: bye see you tomorrow.
-3) Attention: bye see you tomorrow.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G223" s="25" t="str">
+        <x:v>1) Be advised: bye see you tomorrow.
+2) Attention: bye see you tomorrow.
+3) For information: bye see you tomorrow.</x:v>
       </x:c>
     </x:row>
     <x:row r="224" ht="120" hidden="0" customHeight="1">
@@ -3798,9 +4445,12 @@
         <x:v>How was the last mission was everything good with the helicopter.</x:v>
       </x:c>
       <x:c r="F224" s="25" t="str">
-        <x:v>1) How was the last mission? Was everything all right with the helicopter?
-2) Can you confirm: how was the last mission? Was everything all right with the helicopter?
-3) Please confirm: how was the last mission? Was everything all right with the helicopter?</x:v>
+        <x:v>How was the last mission? Was everything all right with the helicopter?</x:v>
+      </x:c>
+      <x:c r="G224" s="25" t="str">
+        <x:v>1) Can you confirm: how was the last mission? Was everything all right with the helicopter?
+2) Please confirm: how was the last mission? Was everything all right with the helicopter?
+3) Message update: how was the last mission? Was everything all right with the helicopter?</x:v>
       </x:c>
     </x:row>
     <x:row r="225" ht="120" hidden="0" customHeight="1">
@@ -3814,9 +4464,12 @@
         <x:v>Don't worry the helicopter is now in my precious hands it will be ready to fly for the next mission.</x:v>
       </x:c>
       <x:c r="F225" s="25" t="str">
-        <x:v>1) Do not worry; the helicopter is in good hands and will be ready for the next mission.
-2) Be advised: do not worry; the helicopter is in good hands and will be ready for the next mission.
-3) Attention: do not worry; the helicopter is in good hands and will be ready for the next mission.</x:v>
+        <x:v>Do not worry; the helicopter is in good hands and will be ready for the next mission.</x:v>
+      </x:c>
+      <x:c r="G225" s="25" t="str">
+        <x:v>1) Be advised: do not worry; the helicopter is in good hands and will be ready for the next mission.
+2) Attention: do not worry; the helicopter is in good hands and will be ready for the next mission.
+3) Please do not worry; the helicopter is in good hands and will be ready for the next mission.</x:v>
       </x:c>
     </x:row>
     <x:row r="226" ht="120" hidden="0" customHeight="1">
@@ -3830,9 +4483,12 @@
         <x:v>Oh my preferred cray hi guys.</x:v>
       </x:c>
       <x:c r="F226" s="25" t="str">
-        <x:v>1) Hi, guys.
-2) Be advised: hi, guys.
-3) Attention: hi, guys.</x:v>
+        <x:v>Hi, guys.</x:v>
+      </x:c>
+      <x:c r="G226" s="25" t="str">
+        <x:v>1) Be advised: hi, guys.
+2) Attention: hi, guys.
+3) For information: hi, guys.</x:v>
       </x:c>
     </x:row>
     <x:row r="227" ht="120" hidden="0" customHeight="1">
@@ -3846,9 +4502,12 @@
         <x:v>It seems i have to work a lot on it.</x:v>
       </x:c>
       <x:c r="F227" s="25" t="str">
-        <x:v>1) It looks like I have a lot of work to do.
-2) Be advised: it looks like I have a lot of work to do.
-3) Attention: it looks like I have a lot of work to do.</x:v>
+        <x:v>It looks like I have a lot of work to do.</x:v>
+      </x:c>
+      <x:c r="G227" s="25" t="str">
+        <x:v>1) Be advised: it looks like I have a lot of work to do.
+2) Attention: it looks like I have a lot of work to do.
+3) For information: it looks like I have a lot of work to do.</x:v>
       </x:c>
     </x:row>
     <x:row r="228" ht="120" hidden="0" customHeight="1">
@@ -3862,9 +4521,12 @@
         <x:v>Hi tomorrow okay there is a good restaurant just out of here.</x:v>
       </x:c>
       <x:c r="F228" s="25" t="str">
-        <x:v>1) Tomorrow there is a good restaurant just outside. Would you like to go?
-2) Can you confirm: tomorrow there is a good restaurant just outside. Would you like to go?
-3) Please confirm: tomorrow there is a good restaurant just outside. Would you like to go?</x:v>
+        <x:v>Tomorrow there is a good restaurant just outside. Would you like to go?</x:v>
+      </x:c>
+      <x:c r="G228" s="25" t="str">
+        <x:v>1) Can you confirm: tomorrow there is a good restaurant just outside. Would you like to go?
+2) Please confirm: tomorrow there is a good restaurant just outside. Would you like to go?
+3) Message update: tomorrow there is a good restaurant just outside. Would you like to go?</x:v>
       </x:c>
     </x:row>
     <x:row r="229" ht="120" hidden="0" customHeight="1">
@@ -3878,9 +4540,12 @@
         <x:v>Hey what you did to the helicopter.</x:v>
       </x:c>
       <x:c r="F229" s="25" t="str">
-        <x:v>1) What did you do to the helicopter?
-2) Can you confirm: what did you do to the helicopter?
-3) Please confirm: what did you do to the helicopter?</x:v>
+        <x:v>What did you do to the helicopter?</x:v>
+      </x:c>
+      <x:c r="G229" s="25" t="str">
+        <x:v>1) Can you confirm: what did you do to the helicopter?
+2) Please confirm: what did you do to the helicopter?
+3) Message update: what did you do to the helicopter?</x:v>
       </x:c>
     </x:row>
     <x:row r="230" ht="15" hidden="0" customHeight="1">
@@ -3911,9 +4576,12 @@
         <x:v>Shared marshall/pisteur3 controller selects the left correction.</x:v>
       </x:c>
       <x:c r="F231" s="25" t="str">
-        <x:v>1) Move left slowly.
-2) Be advised: move left slowly.
-3) Attention: move left slowly.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G231" s="25" t="str">
+        <x:v>1) Be advised: move left slowly.
+2) Attention: move left slowly.
+3) Please move left slowly.</x:v>
       </x:c>
     </x:row>
     <x:row r="232" ht="120" customHeight="1">
@@ -3933,9 +4601,12 @@
         <x:v>Shared marshall/pisteur3 controller selects the right correction.</x:v>
       </x:c>
       <x:c r="F232" s="25" t="str">
-        <x:v>1) Move right slowly.
-2) Be advised: move right slowly.
-3) Attention: move right slowly.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G232" s="25" t="str">
+        <x:v>1) Be advised: move right slowly.
+2) Attention: move right slowly.
+3) Please move right slowly.</x:v>
       </x:c>
     </x:row>
     <x:row r="233" ht="120" customHeight="1">
@@ -3955,9 +4626,12 @@
         <x:v>Shared marshal controller commands the forward approach.</x:v>
       </x:c>
       <x:c r="F233" s="25" t="str">
-        <x:v>1) Come forward slowly.
-2) Be advised: come forward slowly.
-3) Attention: come forward slowly.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G233" s="25" t="str">
+        <x:v>1) Be advised: come forward slowly.
+2) Attention: come forward slowly.
+3) For information: come forward slowly.</x:v>
       </x:c>
     </x:row>
     <x:row r="234" ht="120" customHeight="1">
@@ -3977,9 +4651,12 @@
         <x:v>Marshal controller enters the hold or safety-buffer state.</x:v>
       </x:c>
       <x:c r="F234" s="25" t="str">
-        <x:v>1) Hold position.
-2) Maintain position.
-3) Maintain your position.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G234" s="25" t="str">
+        <x:v>1) Maintain position.
+2) Maintain your position.
+3) Please hold position.</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="120" customHeight="1">
@@ -3999,9 +4676,12 @@
         <x:v>A valid landing is committed inside the configured landing area.</x:v>
       </x:c>
       <x:c r="F235" s="25" t="str">
-        <x:v>1) Landing area clear. You are cleared to land.
-2) Landing area clear. You're cleared to land.
-3) Attention: landing area clear. You are cleared to land.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G235" s="25" t="str">
+        <x:v>1) Landing area clear. You're cleared to land.
+2) Attention: landing area clear. You are cleared to land.
+3) For information: landing area clear. You are cleared to land.</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="120" customHeight="1">
@@ -4021,9 +4701,12 @@
         <x:v>Crew visit begins and the tablet starts revealing clinical data.</x:v>
       </x:c>
       <x:c r="F236" s="25" t="str">
-        <x:v>1) Patient assessment in progress. Stand by for the treatment decision.
-2) Be advised: patient assessment in progress. Stand by for the treatment decision.
-3) Attention: patient assessment in progress. Stand by for the treatment decision.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G236" s="25" t="str">
+        <x:v>1) Be advised: patient assessment in progress. Stand by for the treatment decision.
+2) Attention: patient assessment in progress. Stand by for the treatment decision.
+3) For information: patient assessment in progress. Stand by for the treatment decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="237" ht="120" customHeight="1">
@@ -4043,9 +4726,12 @@
         <x:v>Critical-vitals indicators turn red, patient deterioration requires an urgent transport decision.</x:v>
       </x:c>
       <x:c r="F237" s="25" t="str">
-        <x:v>1) Critical vital signs. Prepare for immediate transport.
-2) Be advised: critical vital signs. Prepare for immediate transport.
-3) Attention: critical vital signs. Prepare for immediate transport.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G237" s="25" t="str">
+        <x:v>1) Be advised: critical vital signs. Prepare for immediate transport.
+2) Attention: critical vital signs. Prepare for immediate transport.
+3) For information: critical vital signs. Prepare for immediate transport.</x:v>
       </x:c>
     </x:row>
     <x:row r="238" ht="120" customHeight="1">
@@ -4065,9 +4751,12 @@
         <x:v>Treatment result allows the loading or transport branch to start.</x:v>
       </x:c>
       <x:c r="F238" s="25" t="str">
-        <x:v>1) Patient stabilized for transport. Prepare the cabin for loading.
-2) Be advised: patient stabilized for transport. Prepare the cabin for loading.
-3) Attention: patient stabilized for transport. Prepare the cabin for loading.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G238" s="25" t="str">
+        <x:v>1) Be advised: patient stabilized for transport. Prepare the cabin for loading.
+2) Attention: patient stabilized for transport. Prepare the cabin for loading.
+3) For information: patient stabilized for transport. Prepare the cabin for loading.</x:v>
       </x:c>
     </x:row>
     <x:row r="239" ht="120" customHeight="1">
@@ -4087,9 +4776,12 @@
         <x:v>L:CPR becomes 1 while airborne and MCPR_ONBOARD is disabled.</x:v>
       </x:c>
       <x:c r="F239" s="25" t="str">
-        <x:v>1) CPR is required. Land as soon as safely possible before treatment can start.
-2) Be advised: cPR is required. Land as soon as safely possible before treatment can start.
-3) Attention: cPR is required. Land as soon as safely possible before treatment can start.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G239" s="25" t="str">
+        <x:v>1) Be advised: cPR is required. Land as soon as safely possible before treatment can start.
+2) Attention: cPR is required. Land as soon as safely possible before treatment can start.
+3) For information: cPR is required. Land as soon as safely possible before treatment can start.</x:v>
       </x:c>
     </x:row>
     <x:row r="240" ht="120" customHeight="1">
@@ -4109,9 +4801,12 @@
         <x:v>The tablet STOP CPR action sets L:CPR to 5.</x:v>
       </x:c>
       <x:c r="F240" s="25" t="str">
-        <x:v>1) CPR has been stopped. Continue monitoring and follow the clinical plan.
-2) Be advised: cPR has been stopped. Continue monitoring and follow the clinical plan.
-3) Attention: cPR has been stopped. Continue monitoring and follow the clinical plan.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G240" s="25" t="str">
+        <x:v>1) Be advised: cPR has been stopped. Continue monitoring and follow the clinical plan.
+2) Attention: cPR has been stopped. Continue monitoring and follow the clinical plan.
+3) For information: cPR has been stopped. Continue monitoring and follow the clinical plan.</x:v>
       </x:c>
     </x:row>
     <x:row r="241" ht="120" customHeight="1">
@@ -4131,9 +4826,12 @@
         <x:v>Ambulance arrival completes, before the patient-transfer branch begins.</x:v>
       </x:c>
       <x:c r="F241" s="25" t="str">
-        <x:v>1) Ambulance is on scene. Prepare for patient handover.
-2) Be advised: ambulance is on scene. Prepare for patient handover.
-3) Attention: ambulance is on scene. Prepare for patient handover.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G241" s="25" t="str">
+        <x:v>1) Be advised: ambulance is on scene. Prepare for patient handover.
+2) Attention: ambulance is on scene. Prepare for patient handover.
+3) For information: ambulance is on scene. Prepare for patient handover.</x:v>
       </x:c>
     </x:row>
     <x:row r="242" ht="120" customHeight="1">
@@ -4153,9 +4851,12 @@
         <x:v>Secondary-rescue flow assigns ambulance 2 to patient 2 or patient 3.</x:v>
       </x:c>
       <x:c r="F242" s="25" t="str">
-        <x:v>1) A second ambulance is managing another patient. Keep the landing area clear.
-2) Be advised: a second ambulance is managing another patient. Keep the landing area clear.
-3) Attention: a second ambulance is managing another patient. Keep the landing area clear.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G242" s="25" t="str">
+        <x:v>1) Be advised: a second ambulance is managing another patient. Keep the landing area clear.
+2) Attention: a second ambulance is managing another patient. Keep the landing area clear.
+3) For information: a second ambulance is managing another patient. Keep the landing area clear.</x:v>
       </x:c>
     </x:row>
     <x:row r="243" ht="120" customHeight="1">
@@ -4175,9 +4876,12 @@
         <x:v>Police arrival and the scene-security/privacy-screen path begin.</x:v>
       </x:c>
       <x:c r="F243" s="25" t="str">
-        <x:v>1) Police are securing the scene. Stay clear until the area is released.
-2) Be advised: police are securing the scene. Stay clear until the area is released.
-3) Attention: police are securing the scene. Stay clear until the area is released.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G243" s="25" t="str">
+        <x:v>1) Be advised: police are securing the scene. Stay clear until the area is released.
+2) Attention: police are securing the scene. Stay clear until the area is released.
+3) For information: police are securing the scene. Stay clear until the area is released.</x:v>
       </x:c>
     </x:row>
     <x:row r="244" ht="120" customHeight="1">
@@ -4197,9 +4901,12 @@
         <x:v>Fire-engine or fire-hazard branch is active.</x:v>
       </x:c>
       <x:c r="F244" s="25" t="str">
-        <x:v>1) Fire service is controlling a hazard. Do not land until cleared.
-2) Be advised: fire service is controlling a hazard. Do not land until cleared.
-3) Attention: fire service is controlling a hazard. Do not land until cleared.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G244" s="25" t="str">
+        <x:v>1) Be advised: fire service is controlling a hazard. Do not land until cleared.
+2) Attention: fire service is controlling a hazard. Do not land until cleared.
+3) For information: fire service is controlling a hazard. Do not land until cleared.</x:v>
       </x:c>
     </x:row>
     <x:row r="245" ht="120" customHeight="1">
@@ -4219,9 +4926,12 @@
         <x:v>ops_progress_warning becomes 1 after 120 seconds without progress; tablet shows the orange Dispatch warning.</x:v>
       </x:c>
       <x:c r="F245" s="25" t="str">
-        <x:v>1) Ground operations are delayed. Check the Dispatch page for the current status.
-2) Be advised: ground operations are delayed. Check the Dispatch page for the current status.
-3) Attention: ground operations are delayed. Check the Dispatch page for the current status.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G245" s="25" t="str">
+        <x:v>1) Be advised: ground operations are delayed. Check the Dispatch page for the current status.
+2) Attention: ground operations are delayed. Check the Dispatch page for the current status.
+3) For information: ground operations are delayed. Check the Dispatch page for the current status.</x:v>
       </x:c>
     </x:row>
     <x:row r="246" ht="120" customHeight="1">
@@ -4241,9 +4951,12 @@
         <x:v>A speed, acceleration, or bank-angle limit requires a temporary hoist pause.</x:v>
       </x:c>
       <x:c r="F246" s="25" t="str">
-        <x:v>1) Hold position. Hoist operation is paused until the aircraft is stable.
-2) Maintain position. Hoist operation is paused until the aircraft is stable.
-3) Maintain your position. Hoist operation is paused until the aircraft is stable.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G246" s="25" t="str">
+        <x:v>1) Maintain position. Hoist operation is paused until the aircraft is stable.
+2) Maintain your position. Hoist operation is paused until the aircraft is stable.
+3) Please hold position. Hoist operation is paused until the aircraft is stable.</x:v>
       </x:c>
     </x:row>
     <x:row r="247" ht="120" customHeight="1">
@@ -4263,9 +4976,12 @@
         <x:v>An unsafe hoist state requires abort and recovery rather than continuation.</x:v>
       </x:c>
       <x:c r="F247" s="25" t="str">
-        <x:v>1) Abort the hoist operation. Recover the crew only when conditions are safe.
-2) Be advised: abort the hoist operation. Recover the crew only when conditions are safe.
-3) Attention: abort the hoist operation. Recover the crew only when conditions are safe.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G247" s="25" t="str">
+        <x:v>1) Be advised: abort the hoist operation. Recover the crew only when conditions are safe.
+2) Attention: abort the hoist operation. Recover the crew only when conditions are safe.
+3) Please abort the hoist operation. Recover the crew only when conditions are safe.</x:v>
       </x:c>
     </x:row>
     <x:row r="248" ht="120" customHeight="1">
@@ -4285,9 +5001,12 @@
         <x:v>routeupdate records a missing or failed destination after its retry.</x:v>
       </x:c>
       <x:c r="F248" s="25" t="str">
-        <x:v>1) Route is unavailable. Select or confirm the destination on the tablet.
-2) Be advised: route is unavailable. Select or confirm the destination on the tablet.
-3) Attention: route is unavailable. Select or confirm the destination on the tablet.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G248" s="25" t="str">
+        <x:v>1) Be advised: route is unavailable. Select or confirm the destination on the tablet.
+2) Attention: route is unavailable. Select or confirm the destination on the tablet.
+3) For information: route is unavailable. Select or confirm the destination on the tablet.</x:v>
       </x:c>
     </x:row>
     <x:row r="249" ht="120" customHeight="1">
@@ -4307,9 +5026,12 @@
         <x:v>Hospital, pickup, or custom target changes and the route is recalculated.</x:v>
       </x:c>
       <x:c r="F249" s="25" t="str">
-        <x:v>1) Destination changed. Check the revised route on the tablet.
-2) Be advised: destination changed. Check the revised route on the tablet.
-3) Attention: destination changed. Check the revised route on the tablet.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G249" s="25" t="str">
+        <x:v>1) Be advised: destination changed. Check the revised route on the tablet.
+2) Attention: destination changed. Check the revised route on the tablet.
+3) For information: destination changed. Check the revised route on the tablet.</x:v>
       </x:c>
     </x:row>
     <x:row r="250" ht="120" customHeight="1">
@@ -4329,9 +5051,12 @@
         <x:v>Cancellation criteria end the current dispatch; HEMS must not continue intervention.</x:v>
       </x:c>
       <x:c r="F250" s="25" t="str">
-        <x:v>1) Dispatch cancelled. Follow the instructions on the tablet and await reassignment.
-2) Be advised: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
-3) Attention: dispatch cancelled. Follow the instructions on the tablet and await reassignment.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G250" s="25" t="str">
+        <x:v>1) Be advised: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
+2) Attention: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
+3) For information: dispatch cancelled. Follow the instructions on the tablet and await reassignment.</x:v>
       </x:c>
     </x:row>
     <x:row r="251" ht="120" customHeight="1">
@@ -4351,9 +5076,12 @@
         <x:v>marshall_ground_ops_active or pisteur3_guidance_active blocks a first-pump start request.</x:v>
       </x:c>
       <x:c r="F251" s="25" t="str">
-        <x:v>1) Hold engine start. Ground operations are still in progress.
-2) Be advised: hold engine start. Ground operations are still in progress.
-3) Attention: hold engine start. Ground operations are still in progress.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G251" s="25" t="str">
+        <x:v>1) Be advised: hold engine start. Ground operations are still in progress.
+2) Attention: hold engine start. Ground operations are still in progress.
+3) Please hold engine start. Ground operations are still in progress.</x:v>
       </x:c>
     </x:row>
     <x:row r="252" ht="120" customHeight="1">
@@ -4373,9 +5101,12 @@
         <x:v>A failure or hard landing requires inspection before the next release.</x:v>
       </x:c>
       <x:c r="F252" s="25" t="str">
-        <x:v>1) Aircraft requires inspection. Do not depart until maintenance releases it.
-2) Be advised: aircraft requires inspection. Do not depart until maintenance releases it.
-3) Attention: aircraft requires inspection. Do not depart until maintenance releases it.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G252" s="25" t="str">
+        <x:v>1) Be advised: aircraft requires inspection. Do not depart until maintenance releases it.
+2) Attention: aircraft requires inspection. Do not depart until maintenance releases it.
+3) For information: aircraft requires inspection. Do not depart until maintenance releases it.</x:v>
       </x:c>
     </x:row>
     <x:row r="253" ht="120" customHeight="1">
@@ -4395,9 +5126,12 @@
         <x:v>Patient 2 or 3 remains active, or secondary rescue begins.</x:v>
       </x:c>
       <x:c r="F253" s="25" t="str">
-        <x:v>1) Additional patients remain on scene. Await tasking before departure.
-2) Be advised: additional patients remain on scene. Await tasking before departure.
-3) Attention: additional patients remain on scene. Await tasking before departure.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G253" s="25" t="str">
+        <x:v>1) Be advised: additional patients remain on scene. Await tasking before departure.
+2) Attention: additional patients remain on scene. Await tasking before departure.
+3) For information: additional patients remain on scene. Await tasking before departure.</x:v>
       </x:c>
     </x:row>
     <x:row r="254" ht="120" customHeight="1">
@@ -4417,9 +5151,12 @@
         <x:v>Post-visit, post-load, or post-hoist crew-return flow begins.</x:v>
       </x:c>
       <x:c r="F254" s="26" t="str">
-        <x:v>1) Ground crew is returning to the aircraft. Keep the landing area clear.
-2) Be advised: ground crew is returning to the aircraft. Keep the landing area clear.
-3) Attention: ground crew is returning to the aircraft. Keep the landing area clear.</x:v>
+        <x:v/>
+      </x:c>
+      <x:c r="G254" s="26" t="str">
+        <x:v>1) Be advised: ground crew is returning to the aircraft. Keep the landing area clear.
+2) Attention: ground crew is returning to the aircraft. Keep the landing area clear.
+3) For information: ground crew is returning to the aircraft. Keep the landing area clear.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Assign proposed voice cues to crew LVAR prefixes
</commit_message>
<xml_diff>
--- a/docs/AND_voice_messages.xlsx
+++ b/docs/AND_voice_messages.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet name="Voci AND" sheetId="1" r:id="rId1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci AND" sheetId="1" r:id="R21192e1e95734eca"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -47,7 +51,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9D9D9"/>
-        <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -244,6 +247,197 @@
 </x:table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+  <a:themeElements>
+    <a:clrScheme name="ChatGPT">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="ChatGPT">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -519,9 +713,7 @@
       <x:c r="C17" s="12" t="str">
         <x:v>What the hell is happening here.</x:v>
       </x:c>
-      <x:c r="F17" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F17" s="25" t="str"/>
       <x:c r="G17" s="25" t="str">
         <x:v>1) Be advised: what the hell is happening here.
 2) Attention: what the hell is happening here.
@@ -576,9 +768,7 @@
       <x:c r="C20" s="12" t="str">
         <x:v>We need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.</x:v>
       </x:c>
-      <x:c r="F20" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F20" s="25" t="str"/>
       <x:c r="G20" s="25" t="str">
         <x:v>1) Be advised: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
 2) Attention: we need to abort, guys. Please check whether we are still good to proceed; if not, we need to abort ASAP.
@@ -652,9 +842,7 @@
       <x:c r="C24" s="12" t="str">
         <x:v>Cabin preparation completed.</x:v>
       </x:c>
-      <x:c r="F24" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F24" s="25" t="str"/>
       <x:c r="G24" s="25" t="str">
         <x:v>1) Be advised: cabin preparation completed.
 2) Attention: cabin preparation completed.
@@ -747,9 +935,7 @@
       <x:c r="C29" s="12" t="str">
         <x:v>Hoist two to helicopter.</x:v>
       </x:c>
-      <x:c r="F29" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F29" s="25" t="str"/>
       <x:c r="G29" s="25" t="str">
         <x:v>1) Be advised: hoist two to helicopter.
 2) Attention: hoist two to helicopter.
@@ -766,9 +952,7 @@
       <x:c r="C30" s="12" t="str">
         <x:v>Hoist three to helicopter.</x:v>
       </x:c>
-      <x:c r="F30" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F30" s="25" t="str"/>
       <x:c r="G30" s="25" t="str">
         <x:v>1) Be advised: hoist three to helicopter.
 2) Attention: hoist three to helicopter.
@@ -785,9 +969,7 @@
       <x:c r="C31" s="12" t="str">
         <x:v>Hoist boom extended.</x:v>
       </x:c>
-      <x:c r="F31" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F31" s="25" t="str"/>
       <x:c r="G31" s="25" t="str">
         <x:v>1) Be advised: hoist boom extended.
 2) Attention: hoist boom extended.
@@ -804,9 +986,7 @@
       <x:c r="C32" s="12" t="str">
         <x:v>Hoist is clear.</x:v>
       </x:c>
-      <x:c r="F32" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F32" s="25" t="str"/>
       <x:c r="G32" s="25" t="str">
         <x:v>1) Be advised: hoist is clear.
 2) Attention: hoist is clear.
@@ -823,9 +1003,7 @@
       <x:c r="C33" s="12" t="str">
         <x:v>Hoist is running down.</x:v>
       </x:c>
-      <x:c r="F33" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F33" s="25" t="str"/>
       <x:c r="G33" s="25" t="str">
         <x:v>1) Be advised: hoist is running down.
 2) Attention: hoist is running down.
@@ -842,9 +1020,7 @@
       <x:c r="C34" s="12" t="str">
         <x:v>Hoist is running up.</x:v>
       </x:c>
-      <x:c r="F34" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F34" s="25" t="str"/>
       <x:c r="G34" s="25" t="str">
         <x:v>1) Be advised: hoist is running up.
 2) Attention: hoist is running up.
@@ -918,9 +1094,7 @@
       <x:c r="C38" s="12" t="str">
         <x:v>Hold position.</x:v>
       </x:c>
-      <x:c r="F38" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F38" s="25" t="str"/>
       <x:c r="G38" s="25" t="str">
         <x:v>1) Maintain position.
 2) Maintain your position.
@@ -1013,9 +1187,7 @@
       <x:c r="C43" s="12" t="str">
         <x:v>Position is good.</x:v>
       </x:c>
-      <x:c r="F43" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F43" s="25" t="str"/>
       <x:c r="G43" s="25" t="str">
         <x:v>1) Be advised: position is good.
 2) Attention: position is good.
@@ -1032,9 +1204,7 @@
       <x:c r="C44" s="12" t="str">
         <x:v>Hold on, hoisting preparation is in progress and almost completed.</x:v>
       </x:c>
-      <x:c r="F44" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F44" s="25" t="str"/>
       <x:c r="G44" s="25" t="str">
         <x:v>1) Be advised: hold on, hoisting preparation is in progress and almost completed.
 2) Attention: hold on, hoisting preparation is in progress and almost completed.
@@ -1051,9 +1221,7 @@
       <x:c r="C45" s="12" t="str">
         <x:v>Set hover conditions.</x:v>
       </x:c>
-      <x:c r="F45" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F45" s="25" t="str"/>
       <x:c r="G45" s="25" t="str">
         <x:v>1) Be advised: set hover conditions.
 2) Attention: set hover conditions.
@@ -1108,9 +1276,7 @@
       <x:c r="C48" s="12" t="str">
         <x:v>Ten.</x:v>
       </x:c>
-      <x:c r="F48" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F48" s="25" t="str"/>
       <x:c r="G48" s="25" t="str">
         <x:v>1) Be advised: ten.
 2) Attention: ten.
@@ -1127,9 +1293,7 @@
       <x:c r="C49" s="12" t="str">
         <x:v>Twenty.</x:v>
       </x:c>
-      <x:c r="F49" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F49" s="25" t="str"/>
       <x:c r="G49" s="25" t="str">
         <x:v>1) Be advised: twenty.
 2) Attention: twenty.
@@ -1146,9 +1310,7 @@
       <x:c r="C50" s="12" t="str">
         <x:v>Fifty meters.</x:v>
       </x:c>
-      <x:c r="F50" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F50" s="25" t="str"/>
       <x:c r="G50" s="25" t="str">
         <x:v>1) Be advised: fifty meters.
 2) Attention: fifty meters.
@@ -1165,9 +1327,7 @@
       <x:c r="C51" s="12" t="str">
         <x:v>Hey frank good morning.</x:v>
       </x:c>
-      <x:c r="F51" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F51" s="25" t="str"/>
       <x:c r="G51" s="25" t="str">
         <x:v>1) Be advised: hey frank good morning.
 2) Attention: hey frank good morning.
@@ -1184,9 +1344,7 @@
       <x:c r="C52" s="12" t="str">
         <x:v>Hi sarah how are you.</x:v>
       </x:c>
-      <x:c r="F52" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F52" s="25" t="str"/>
       <x:c r="G52" s="25" t="str">
         <x:v>1) Be advised: hi sarah how are you.
 2) Attention: hi sarah how are you.
@@ -1203,9 +1361,7 @@
       <x:c r="C53" s="12" t="str">
         <x:v>Stretcher is secure.</x:v>
       </x:c>
-      <x:c r="F53" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F53" s="25" t="str"/>
       <x:c r="G53" s="25" t="str">
         <x:v>1) Be advised: stretcher is secure.
 2) Attention: stretcher is secure.
@@ -1241,9 +1397,7 @@
       <x:c r="C55" s="12" t="str">
         <x:v>We are reasonably close.</x:v>
       </x:c>
-      <x:c r="F55" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F55" s="25" t="str"/>
       <x:c r="G55" s="25" t="str">
         <x:v>1) We're reasonably close.
 2) Attention: we are reasonably close.
@@ -1260,9 +1414,7 @@
       <x:c r="C56" s="12" t="str">
         <x:v>We are too far.</x:v>
       </x:c>
-      <x:c r="F56" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F56" s="25" t="str"/>
       <x:c r="G56" s="25" t="str">
         <x:v>1) We're too far.
 2) Attention: we are too far.
@@ -1279,9 +1431,7 @@
       <x:c r="C57" s="12" t="str">
         <x:v>Height is good.</x:v>
       </x:c>
-      <x:c r="F57" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F57" s="25" t="str"/>
       <x:c r="G57" s="25" t="str">
         <x:v>1) Be advised: height is good.
 2) Attention: height is good.
@@ -1298,9 +1448,7 @@
       <x:c r="C58" s="12" t="str">
         <x:v>We are too high.</x:v>
       </x:c>
-      <x:c r="F58" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F58" s="25" t="str"/>
       <x:c r="G58" s="25" t="str">
         <x:v>1) We're too high.
 2) Attention: we are too high.
@@ -1317,9 +1465,7 @@
       <x:c r="C59" s="12" t="str">
         <x:v>We are too low.</x:v>
       </x:c>
-      <x:c r="F59" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F59" s="25" t="str"/>
       <x:c r="G59" s="25" t="str">
         <x:v>1) We're too low.
 2) Attention: we are too low.
@@ -1355,9 +1501,7 @@
       <x:c r="C61" s="12" t="str">
         <x:v>Doc is getting hooked.</x:v>
       </x:c>
-      <x:c r="F61" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F61" s="25" t="str"/>
       <x:c r="G61" s="25" t="str">
         <x:v>1) Be advised: doc is getting hooked.
 2) Attention: doc is getting hooked.
@@ -1412,9 +1556,7 @@
       <x:c r="C64" s="12" t="str">
         <x:v>Opening door and preparing for hoist operation.</x:v>
       </x:c>
-      <x:c r="F64" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F64" s="25" t="str"/>
       <x:c r="G64" s="25" t="str">
         <x:v>1) Be advised: opening door and preparing for hoist operation.
 2) Attention: opening door and preparing for hoist operation.
@@ -1431,9 +1573,7 @@
       <x:c r="C65" s="12" t="str">
         <x:v>Operator has been disconnected.</x:v>
       </x:c>
-      <x:c r="F65" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F65" s="25" t="str"/>
       <x:c r="G65" s="25" t="str">
         <x:v>1) Be advised: operator has been disconnected.
 2) Attention: operator has been disconnected.
@@ -1450,9 +1590,7 @@
       <x:c r="C66" s="12" t="str">
         <x:v>Operator is getting hooked.</x:v>
       </x:c>
-      <x:c r="F66" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F66" s="25" t="str"/>
       <x:c r="G66" s="25" t="str">
         <x:v>1) Be advised: operator is getting hooked.
 2) Attention: operator is getting hooked.
@@ -1602,9 +1740,7 @@
       <x:c r="C74" s="12" t="str">
         <x:v>Three o'clock.</x:v>
       </x:c>
-      <x:c r="F74" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F74" s="25" t="str"/>
       <x:c r="G74" s="25" t="str">
         <x:v>1) Be advised: three o'clock.
 2) Attention: three o'clock.
@@ -1621,9 +1757,7 @@
       <x:c r="C75" s="12" t="str">
         <x:v>Four o'clock.</x:v>
       </x:c>
-      <x:c r="F75" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F75" s="25" t="str"/>
       <x:c r="G75" s="25" t="str">
         <x:v>1) Be advised: four o'clock.
 2) Attention: four o'clock.
@@ -1640,9 +1774,7 @@
       <x:c r="C76" s="12" t="str">
         <x:v>Five o'clock.</x:v>
       </x:c>
-      <x:c r="F76" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F76" s="25" t="str"/>
       <x:c r="G76" s="25" t="str">
         <x:v>1) Be advised: five o'clock.
 2) Attention: five o'clock.
@@ -1659,9 +1791,7 @@
       <x:c r="C77" s="12" t="str">
         <x:v>Six o'clock.</x:v>
       </x:c>
-      <x:c r="F77" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F77" s="25" t="str"/>
       <x:c r="G77" s="25" t="str">
         <x:v>1) Be advised: six o'clock.
 2) Attention: six o'clock.
@@ -1678,9 +1808,7 @@
       <x:c r="C78" s="12" t="str">
         <x:v>Seven o'clock.</x:v>
       </x:c>
-      <x:c r="F78" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F78" s="25" t="str"/>
       <x:c r="G78" s="25" t="str">
         <x:v>1) Be advised: seven o'clock.
 2) Attention: seven o'clock.
@@ -1697,9 +1825,7 @@
       <x:c r="C79" s="12" t="str">
         <x:v>Eight o'clock.</x:v>
       </x:c>
-      <x:c r="F79" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F79" s="25" t="str"/>
       <x:c r="G79" s="25" t="str">
         <x:v>1) Be advised: eight o'clock.
 2) Attention: eight o'clock.
@@ -1716,9 +1842,7 @@
       <x:c r="C80" s="12" t="str">
         <x:v>Nine o'clock.</x:v>
       </x:c>
-      <x:c r="F80" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F80" s="25" t="str"/>
       <x:c r="G80" s="25" t="str">
         <x:v>1) Be advised: nine o'clock.
 2) Attention: nine o'clock.
@@ -1735,9 +1859,7 @@
       <x:c r="C81" s="12" t="str">
         <x:v>Ten o'clock.</x:v>
       </x:c>
-      <x:c r="F81" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F81" s="25" t="str"/>
       <x:c r="G81" s="25" t="str">
         <x:v>1) Be advised: ten o'clock.
 2) Attention: ten o'clock.
@@ -1754,9 +1876,7 @@
       <x:c r="C82" s="12" t="str">
         <x:v>Eleven o'clock.</x:v>
       </x:c>
-      <x:c r="F82" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F82" s="25" t="str"/>
       <x:c r="G82" s="25" t="str">
         <x:v>1) Be advised: eleven o'clock.
 2) Attention: eleven o'clock.
@@ -1773,9 +1893,7 @@
       <x:c r="C83" s="12" t="str">
         <x:v>Twelve o'clock.</x:v>
       </x:c>
-      <x:c r="F83" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F83" s="25" t="str"/>
       <x:c r="G83" s="25" t="str">
         <x:v>1) Be advised: twelve o'clock.
 2) Attention: twelve o'clock.
@@ -1830,9 +1948,7 @@
       <x:c r="C86" s="12" t="str">
         <x:v>I believe we found something.</x:v>
       </x:c>
-      <x:c r="F86" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F86" s="25" t="str"/>
       <x:c r="G86" s="25" t="str">
         <x:v>1) Be advised: i believe we found something.
 2) Attention: i believe we found something.
@@ -1849,9 +1965,7 @@
       <x:c r="C87" s="12" t="str">
         <x:v>It's in front of us.</x:v>
       </x:c>
-      <x:c r="F87" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F87" s="25" t="str"/>
       <x:c r="G87" s="25" t="str">
         <x:v>1) Be advised: it's in front of us.
 2) Attention: it's in front of us.
@@ -2058,9 +2172,7 @@
       <x:c r="C98" s="12" t="str">
         <x:v>Damn we have a failure.</x:v>
       </x:c>
-      <x:c r="F98" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F98" s="25" t="str"/>
       <x:c r="G98" s="25" t="str">
         <x:v>1) Be advised: damn we have a failure.
 2) Attention: damn we have a failure.
@@ -2267,9 +2379,7 @@
       <x:c r="C109" s="12" t="str">
         <x:v>Ambulance is arriving.</x:v>
       </x:c>
-      <x:c r="F109" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F109" s="25" t="str"/>
       <x:c r="G109" s="25" t="str">
         <x:v>1) Be advised: ambulance is arriving.
 2) Attention: ambulance is arriving.
@@ -2286,9 +2396,7 @@
       <x:c r="C110" s="12" t="str">
         <x:v>Ambulance is still far away.</x:v>
       </x:c>
-      <x:c r="F110" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F110" s="25" t="str"/>
       <x:c r="G110" s="25" t="str">
         <x:v>1) Be advised: ambulance is still far away.
 2) Attention: ambulance is still far away.
@@ -2324,9 +2432,7 @@
       <x:c r="C112" s="12" t="str">
         <x:v>Good morning frank.</x:v>
       </x:c>
-      <x:c r="F112" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F112" s="25" t="str"/>
       <x:c r="G112" s="25" t="str">
         <x:v>1) Be advised: good morning frank.
 2) Attention: good morning frank.
@@ -2628,9 +2734,7 @@
       <x:c r="C128" s="12" t="str">
         <x:v>Wow nice touch captain.</x:v>
       </x:c>
-      <x:c r="F128" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F128" s="25" t="str"/>
       <x:c r="G128" s="25" t="str">
         <x:v>1) Be advised: wow nice touch captain.
 2) Attention: wow nice touch captain.
@@ -2647,9 +2751,7 @@
       <x:c r="C129" s="12" t="str">
         <x:v>VNE.</x:v>
       </x:c>
-      <x:c r="F129" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F129" s="25" t="str"/>
       <x:c r="G129" s="25" t="str">
         <x:v>1) Be advised: vNE.
 2) Attention: vNE.
@@ -2666,9 +2768,7 @@
       <x:c r="C130" s="12" t="str">
         <x:v>VTOSS.</x:v>
       </x:c>
-      <x:c r="F130" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F130" s="25" t="str"/>
       <x:c r="G130" s="25" t="str">
         <x:v>1) Be advised: vTOSS.
 2) Attention: vTOSS.
@@ -2685,9 +2785,7 @@
       <x:c r="C131" s="12" t="str">
         <x:v>Vy.</x:v>
       </x:c>
-      <x:c r="F131" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F131" s="25" t="str"/>
       <x:c r="G131" s="25" t="str">
         <x:v>1) Be advised: vy.
 2) Attention: vy.
@@ -2742,9 +2840,7 @@
       <x:c r="C134" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
-      <x:c r="F134" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F134" s="25" t="str"/>
       <x:c r="G134" s="25" t="str">
         <x:v>1) Be advised: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
 2) Attention: ground crew was doing last operations before leaving the scene said engines to fly condition and take off as soon as possible for continuing with hoist operations if in your opinion the landing spot is good for ground loading we can stay here.
@@ -2761,9 +2857,7 @@
       <x:c r="C135" s="12" t="str">
         <x:v>Ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.</x:v>
       </x:c>
-      <x:c r="F135" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F135" s="25" t="str"/>
       <x:c r="G135" s="25" t="str">
         <x:v>1) Be advised: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
 2) Attention: ground crew was doing last operations before leaving the scene start engines and take off as soon as possible for continuing with hoist operations if landing spot is good for ground loading we can stay here.
@@ -3000,9 +3094,7 @@
       <x:c r="C148" s="12" t="str">
         <x:v>This is the default hoist pack enjoy.</x:v>
       </x:c>
-      <x:c r="F148" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F148" s="25" t="str"/>
       <x:c r="G148" s="25" t="str">
         <x:v>1) Be advised: this is the default hoist pack enjoy.
 2) Attention: this is the default hoist pack enjoy.
@@ -3057,9 +3149,7 @@
       <x:c r="C151" s="12" t="str">
         <x:v>Evacuate helicopter now.</x:v>
       </x:c>
-      <x:c r="F151" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F151" s="25" t="str"/>
       <x:c r="G151" s="25" t="str">
         <x:v>1) Be advised: evacuate helicopter now.
 2) Attention: evacuate helicopter now.
@@ -3095,9 +3185,7 @@
       <x:c r="C153" s="12" t="str">
         <x:v>I'll check.</x:v>
       </x:c>
-      <x:c r="F153" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F153" s="25" t="str"/>
       <x:c r="G153" s="25" t="str">
         <x:v>1) Be advised: i'll check.
 2) Attention: i'll check.
@@ -3114,9 +3202,7 @@
       <x:c r="C154" s="12" t="str">
         <x:v>Mission accomplished.</x:v>
       </x:c>
-      <x:c r="F154" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F154" s="25" t="str"/>
       <x:c r="G154" s="25" t="str">
         <x:v>1) Be advised: mission accomplished.
 2) Attention: mission accomplished.
@@ -3133,9 +3219,7 @@
       <x:c r="C155" s="12" t="str">
         <x:v>Thank you.</x:v>
       </x:c>
-      <x:c r="F155" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F155" s="25" t="str"/>
       <x:c r="G155" s="25" t="str">
         <x:v>1) Be advised: thank you.
 2) Attention: thank you.
@@ -3190,9 +3274,7 @@
       <x:c r="C158" s="12" t="str">
         <x:v>Well done.</x:v>
       </x:c>
-      <x:c r="F158" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F158" s="25" t="str"/>
       <x:c r="G158" s="25" t="str">
         <x:v>1) Be advised: well done.
 2) Attention: well done.
@@ -3228,9 +3310,7 @@
       <x:c r="C160" s="12" t="str">
         <x:v>Two nautical miles from our base.</x:v>
       </x:c>
-      <x:c r="F160" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F160" s="25" t="str"/>
       <x:c r="G160" s="25" t="str">
         <x:v>1) Be advised: two nautical miles from our base.
 2) Attention: two nautical miles from our base.
@@ -3247,9 +3327,7 @@
       <x:c r="C161" s="12" t="str">
         <x:v>Two nautical miles from hospital.</x:v>
       </x:c>
-      <x:c r="F161" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F161" s="25" t="str"/>
       <x:c r="G161" s="25" t="str">
         <x:v>1) Be advised: two nautical miles from hospital.
 2) Attention: two nautical miles from hospital.
@@ -3304,9 +3382,7 @@
       <x:c r="C164" s="12" t="str">
         <x:v>We exceeded VNE.</x:v>
       </x:c>
-      <x:c r="F164" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F164" s="25" t="str"/>
       <x:c r="G164" s="25" t="str">
         <x:v>1) Be advised: we exceeded VNE.
 2) Attention: we exceeded VNE.
@@ -3323,9 +3399,7 @@
       <x:c r="C165" s="12" t="str">
         <x:v>We exceeded the torque limits.</x:v>
       </x:c>
-      <x:c r="F165" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F165" s="25" t="str"/>
       <x:c r="G165" s="25" t="str">
         <x:v>1) Be advised: we exceeded the torque limits.
 2) Attention: we exceeded the torque limits.
@@ -3342,9 +3416,7 @@
       <x:c r="C166" s="12" t="str">
         <x:v>Hi sarah i'm sorry we have some bad news for you.</x:v>
       </x:c>
-      <x:c r="F166" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F166" s="25" t="str"/>
       <x:c r="G166" s="25" t="str">
         <x:v>1) Be advised: hi sarah i'm sorry we have some bad news for you.
 2) Attention: hi sarah i'm sorry we have some bad news for you.
@@ -3418,9 +3490,7 @@
       <x:c r="C170" s="12" t="str">
         <x:v>We had a hard landing.</x:v>
       </x:c>
-      <x:c r="F170" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F170" s="25" t="str"/>
       <x:c r="G170" s="25" t="str">
         <x:v>1) Be advised: we had a hard landing.
 2) Attention: we had a hard landing.
@@ -3608,9 +3678,7 @@
       <x:c r="C180" s="12" t="str">
         <x:v>Let's go.</x:v>
       </x:c>
-      <x:c r="F180" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F180" s="25" t="str"/>
       <x:c r="G180" s="25" t="str">
         <x:v>1) Be advised: let's go.
 2) Attention: let's go.
@@ -3722,9 +3790,7 @@
       <x:c r="C186" s="12" t="str">
         <x:v>Busy day we received a new dispatch.</x:v>
       </x:c>
-      <x:c r="F186" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F186" s="25" t="str"/>
       <x:c r="G186" s="25" t="str">
         <x:v>1) Be advised: busy day we received a new dispatch.
 2) Attention: busy day we received a new dispatch.
@@ -3874,9 +3940,7 @@
       <x:c r="C194" s="12" t="str">
         <x:v>Confirmed on scene.</x:v>
       </x:c>
-      <x:c r="F194" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F194" s="25" t="str"/>
       <x:c r="G194" s="25" t="str">
         <x:v>1) Be advised: confirmed on scene.
 2) Attention: confirmed on scene.
@@ -3893,9 +3957,7 @@
       <x:c r="C195" s="12" t="str">
         <x:v>Fire engine.</x:v>
       </x:c>
-      <x:c r="F195" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F195" s="25" t="str"/>
       <x:c r="G195" s="25" t="str">
         <x:v>1) Be advised: fire engine.
 2) Attention: fire engine.
@@ -3950,9 +4012,7 @@
       <x:c r="C198" s="12" t="str">
         <x:v>Patient has died.</x:v>
       </x:c>
-      <x:c r="F198" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F198" s="25" t="str"/>
       <x:c r="G198" s="25" t="str">
         <x:v>1) Be advised: patient has died.
 2) Attention: patient has died.
@@ -4045,9 +4105,7 @@
       <x:c r="C203" s="12" t="str">
         <x:v>Police.</x:v>
       </x:c>
-      <x:c r="F203" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F203" s="25" t="str"/>
       <x:c r="G203" s="25" t="str">
         <x:v>1) Be advised: police.
 2) Attention: police.
@@ -4083,9 +4141,7 @@
       <x:c r="C205" s="12" t="str">
         <x:v>We will be first on scene.</x:v>
       </x:c>
-      <x:c r="F205" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F205" s="25" t="str"/>
       <x:c r="G205" s="25" t="str">
         <x:v>1) Be advised: we will be first on scene.
 2) Attention: we will be first on scene.
@@ -4273,9 +4329,7 @@
       <x:c r="C215" s="12" t="str">
         <x:v>If you need refueling please ask.</x:v>
       </x:c>
-      <x:c r="F215" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F215" s="25" t="str"/>
       <x:c r="G215" s="25" t="str">
         <x:v>1) Be advised: if you need refueling please ask.
 2) Attention: if you need refueling please ask.
@@ -4292,9 +4346,7 @@
       <x:c r="C216" s="12" t="str">
         <x:v>Fuel is as you requested.</x:v>
       </x:c>
-      <x:c r="F216" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F216" s="25" t="str"/>
       <x:c r="G216" s="25" t="str">
         <x:v>1) Be advised: fuel is as you requested.
 2) Attention: fuel is as you requested.
@@ -4311,9 +4363,7 @@
       <x:c r="C217" s="12" t="str">
         <x:v>Fuel tanks are almost full.</x:v>
       </x:c>
-      <x:c r="F217" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F217" s="25" t="str"/>
       <x:c r="G217" s="25" t="str">
         <x:v>1) Be advised: fuel tanks are almost full.
 2) Attention: fuel tanks are almost full.
@@ -4330,9 +4380,7 @@
       <x:c r="C218" s="12" t="str">
         <x:v>Refueling has not been performed and fuel level is low.</x:v>
       </x:c>
-      <x:c r="F218" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F218" s="25" t="str"/>
       <x:c r="G218" s="25" t="str">
         <x:v>1) Be advised: refueling has not been performed and fuel level is low.
 2) Attention: refueling has not been performed and fuel level is low.
@@ -4425,9 +4473,7 @@
       <x:c r="C223" s="12" t="str">
         <x:v>Bye see you tomorrow.</x:v>
       </x:c>
-      <x:c r="F223" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F223" s="25" t="str"/>
       <x:c r="G223" s="25" t="str">
         <x:v>1) Be advised: bye see you tomorrow.
 2) Attention: bye see you tomorrow.
@@ -4561,7 +4607,7 @@
     </x:row>
     <x:row r="231" ht="120" customHeight="1">
       <x:c r="A231" s="19" t="str">
-        <x:v>L:ANDMARSHALLEFT</x:v>
+        <x:v>L:MARAND1</x:v>
       </x:c>
       <x:c r="B231" s="20" t="str">
         <x:v>AND.marshal.move.left.wav</x:v>
@@ -4570,14 +4616,12 @@
         <x:v>Move left slowly.</x:v>
       </x:c>
       <x:c r="D231" s="20" t="str">
-        <x:v>Marshal</x:v>
+        <x:v>Marshal / MAR</x:v>
       </x:c>
       <x:c r="E231" s="20" t="str">
         <x:v>Shared marshall/pisteur3 controller selects the left correction.</x:v>
       </x:c>
-      <x:c r="F231" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F231" s="25" t="str"/>
       <x:c r="G231" s="25" t="str">
         <x:v>1) Be advised: move left slowly.
 2) Attention: move left slowly.
@@ -4586,7 +4630,7 @@
     </x:row>
     <x:row r="232" ht="120" customHeight="1">
       <x:c r="A232" s="19" t="str">
-        <x:v>L:ANDMARSHALRIGHT</x:v>
+        <x:v>L:MARAND2</x:v>
       </x:c>
       <x:c r="B232" s="20" t="str">
         <x:v>AND.marshal.move.right.wav</x:v>
@@ -4595,14 +4639,12 @@
         <x:v>Move right slowly.</x:v>
       </x:c>
       <x:c r="D232" s="20" t="str">
-        <x:v>Marshal</x:v>
+        <x:v>Marshal / MAR</x:v>
       </x:c>
       <x:c r="E232" s="20" t="str">
         <x:v>Shared marshall/pisteur3 controller selects the right correction.</x:v>
       </x:c>
-      <x:c r="F232" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F232" s="25" t="str"/>
       <x:c r="G232" s="25" t="str">
         <x:v>1) Be advised: move right slowly.
 2) Attention: move right slowly.
@@ -4611,7 +4653,7 @@
     </x:row>
     <x:row r="233" ht="120" customHeight="1">
       <x:c r="A233" s="19" t="str">
-        <x:v>L:ANDMARSHALFORWARD</x:v>
+        <x:v>L:MARAND3</x:v>
       </x:c>
       <x:c r="B233" s="20" t="str">
         <x:v>AND.marshal.come.forward.wav</x:v>
@@ -4620,14 +4662,12 @@
         <x:v>Come forward slowly.</x:v>
       </x:c>
       <x:c r="D233" s="20" t="str">
-        <x:v>Marshal</x:v>
+        <x:v>Marshal / MAR</x:v>
       </x:c>
       <x:c r="E233" s="20" t="str">
         <x:v>Shared marshal controller commands the forward approach.</x:v>
       </x:c>
-      <x:c r="F233" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F233" s="25" t="str"/>
       <x:c r="G233" s="25" t="str">
         <x:v>1) Be advised: come forward slowly.
 2) Attention: come forward slowly.
@@ -4636,7 +4676,7 @@
     </x:row>
     <x:row r="234" ht="120" customHeight="1">
       <x:c r="A234" s="19" t="str">
-        <x:v>L:ANDMARSHALHOLD</x:v>
+        <x:v>L:MARAND4</x:v>
       </x:c>
       <x:c r="B234" s="20" t="str">
         <x:v>AND.marshal.hold.position.wav</x:v>
@@ -4645,14 +4685,12 @@
         <x:v>Hold position.</x:v>
       </x:c>
       <x:c r="D234" s="20" t="str">
-        <x:v>Marshal</x:v>
+        <x:v>Marshal / MAR</x:v>
       </x:c>
       <x:c r="E234" s="20" t="str">
         <x:v>Marshal controller enters the hold or safety-buffer state.</x:v>
       </x:c>
-      <x:c r="F234" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F234" s="25" t="str"/>
       <x:c r="G234" s="25" t="str">
         <x:v>1) Maintain position.
 2) Maintain your position.
@@ -4661,7 +4699,7 @@
     </x:row>
     <x:row r="235" ht="120" customHeight="1">
       <x:c r="A235" s="19" t="str">
-        <x:v>L:ANDMARSHALLANDCLEAR</x:v>
+        <x:v>L:MARAND5</x:v>
       </x:c>
       <x:c r="B235" s="20" t="str">
         <x:v>AND.marshal.landing.area.clear.wav</x:v>
@@ -4670,14 +4708,12 @@
         <x:v>Landing area clear. You are cleared to land.</x:v>
       </x:c>
       <x:c r="D235" s="20" t="str">
-        <x:v>Marshal</x:v>
+        <x:v>Marshal / MAR</x:v>
       </x:c>
       <x:c r="E235" s="20" t="str">
         <x:v>A valid landing is committed inside the configured landing area.</x:v>
       </x:c>
-      <x:c r="F235" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F235" s="25" t="str"/>
       <x:c r="G235" s="25" t="str">
         <x:v>1) Landing area clear. You're cleared to land.
 2) Attention: landing area clear. You are cleared to land.
@@ -4686,7 +4722,7 @@
     </x:row>
     <x:row r="236" ht="120" customHeight="1">
       <x:c r="A236" s="19" t="str">
-        <x:v>L:ANDMEDASSESSMENT</x:v>
+        <x:v>L:PAX3AND27</x:v>
       </x:c>
       <x:c r="B236" s="20" t="str">
         <x:v>AND.medical.assessment.in.progress.wav</x:v>
@@ -4695,14 +4731,12 @@
         <x:v>Patient assessment in progress. Stand by for the treatment decision.</x:v>
       </x:c>
       <x:c r="D236" s="20" t="str">
-        <x:v>Medical crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E236" s="20" t="str">
         <x:v>Crew visit begins and the tablet starts revealing clinical data.</x:v>
       </x:c>
-      <x:c r="F236" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F236" s="25" t="str"/>
       <x:c r="G236" s="25" t="str">
         <x:v>1) Be advised: patient assessment in progress. Stand by for the treatment decision.
 2) Attention: patient assessment in progress. Stand by for the treatment decision.
@@ -4711,7 +4745,7 @@
     </x:row>
     <x:row r="237" ht="120" customHeight="1">
       <x:c r="A237" s="19" t="str">
-        <x:v>L:ANDMEDCRITICAL</x:v>
+        <x:v>L:PAX3AND28</x:v>
       </x:c>
       <x:c r="B237" s="20" t="str">
         <x:v>AND.medical.critical.vital.signs.wav</x:v>
@@ -4720,14 +4754,12 @@
         <x:v>Critical vital signs. Prepare for immediate transport.</x:v>
       </x:c>
       <x:c r="D237" s="20" t="str">
-        <x:v>Medical crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E237" s="20" t="str">
         <x:v>Critical-vitals indicators turn red, patient deterioration requires an urgent transport decision.</x:v>
       </x:c>
-      <x:c r="F237" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F237" s="25" t="str"/>
       <x:c r="G237" s="25" t="str">
         <x:v>1) Be advised: critical vital signs. Prepare for immediate transport.
 2) Attention: critical vital signs. Prepare for immediate transport.
@@ -4736,7 +4768,7 @@
     </x:row>
     <x:row r="238" ht="120" customHeight="1">
       <x:c r="A238" s="19" t="str">
-        <x:v>L:ANDMEDTRANSPORT</x:v>
+        <x:v>L:PAX3AND29</x:v>
       </x:c>
       <x:c r="B238" s="20" t="str">
         <x:v>AND.medical.patient.ready.for.transport.wav</x:v>
@@ -4745,14 +4777,12 @@
         <x:v>Patient stabilized for transport. Prepare the cabin for loading.</x:v>
       </x:c>
       <x:c r="D238" s="20" t="str">
-        <x:v>Medical crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E238" s="20" t="str">
         <x:v>Treatment result allows the loading or transport branch to start.</x:v>
       </x:c>
-      <x:c r="F238" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F238" s="25" t="str"/>
       <x:c r="G238" s="25" t="str">
         <x:v>1) Be advised: patient stabilized for transport. Prepare the cabin for loading.
 2) Attention: patient stabilized for transport. Prepare the cabin for loading.
@@ -4761,7 +4791,7 @@
     </x:row>
     <x:row r="239" ht="120" customHeight="1">
       <x:c r="A239" s="19" t="str">
-        <x:v>L:ANDCPRAWAITLAND</x:v>
+        <x:v>L:PAX3AND30</x:v>
       </x:c>
       <x:c r="B239" s="20" t="str">
         <x:v>AND.medical.cpr.awaiting.landing.wav</x:v>
@@ -4770,14 +4800,12 @@
         <x:v>CPR is required. Land as soon as safely possible before treatment can start.</x:v>
       </x:c>
       <x:c r="D239" s="20" t="str">
-        <x:v>Medical crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E239" s="20" t="str">
         <x:v>L:CPR becomes 1 while airborne and MCPR_ONBOARD is disabled.</x:v>
       </x:c>
-      <x:c r="F239" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F239" s="25" t="str"/>
       <x:c r="G239" s="25" t="str">
         <x:v>1) Be advised: cPR is required. Land as soon as safely possible before treatment can start.
 2) Attention: cPR is required. Land as soon as safely possible before treatment can start.
@@ -4786,7 +4814,7 @@
     </x:row>
     <x:row r="240" ht="120" customHeight="1">
       <x:c r="A240" s="19" t="str">
-        <x:v>L:ANDCPRSTOPPED</x:v>
+        <x:v>L:PAX3AND31</x:v>
       </x:c>
       <x:c r="B240" s="20" t="str">
         <x:v>AND.medical.cpr.stopped.wav</x:v>
@@ -4795,14 +4823,12 @@
         <x:v>CPR has been stopped. Continue monitoring and follow the clinical plan.</x:v>
       </x:c>
       <x:c r="D240" s="20" t="str">
-        <x:v>Medical crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E240" s="20" t="str">
         <x:v>The tablet STOP CPR action sets L:CPR to 5.</x:v>
       </x:c>
-      <x:c r="F240" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F240" s="25" t="str"/>
       <x:c r="G240" s="25" t="str">
         <x:v>1) Be advised: cPR has been stopped. Continue monitoring and follow the clinical plan.
 2) Attention: cPR has been stopped. Continue monitoring and follow the clinical plan.
@@ -4811,7 +4837,7 @@
     </x:row>
     <x:row r="241" ht="120" customHeight="1">
       <x:c r="A241" s="19" t="str">
-        <x:v>L:ANDAMBUHANDOVER</x:v>
+        <x:v>L:PAX3AND32</x:v>
       </x:c>
       <x:c r="B241" s="20" t="str">
         <x:v>AND.ground.ambulance.handover.ready.wav</x:v>
@@ -4820,14 +4846,12 @@
         <x:v>Ambulance is on scene. Prepare for patient handover.</x:v>
       </x:c>
       <x:c r="D241" s="20" t="str">
-        <x:v>Ground support</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E241" s="20" t="str">
         <x:v>Ambulance arrival completes, before the patient-transfer branch begins.</x:v>
       </x:c>
-      <x:c r="F241" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F241" s="25" t="str"/>
       <x:c r="G241" s="25" t="str">
         <x:v>1) Be advised: ambulance is on scene. Prepare for patient handover.
 2) Attention: ambulance is on scene. Prepare for patient handover.
@@ -4836,7 +4860,7 @@
     </x:row>
     <x:row r="242" ht="120" customHeight="1">
       <x:c r="A242" s="19" t="str">
-        <x:v>L:ANDSECONDAMBULANCE</x:v>
+        <x:v>L:PAX3AND33</x:v>
       </x:c>
       <x:c r="B242" s="20" t="str">
         <x:v>AND.ground.second.ambulance.assigned.wav</x:v>
@@ -4845,14 +4869,12 @@
         <x:v>A second ambulance is managing another patient. Keep the landing area clear.</x:v>
       </x:c>
       <x:c r="D242" s="20" t="str">
-        <x:v>Ground support</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E242" s="20" t="str">
         <x:v>Secondary-rescue flow assigns ambulance 2 to patient 2 or patient 3.</x:v>
       </x:c>
-      <x:c r="F242" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F242" s="25" t="str"/>
       <x:c r="G242" s="25" t="str">
         <x:v>1) Be advised: a second ambulance is managing another patient. Keep the landing area clear.
 2) Attention: a second ambulance is managing another patient. Keep the landing area clear.
@@ -4861,7 +4883,7 @@
     </x:row>
     <x:row r="243" ht="120" customHeight="1">
       <x:c r="A243" s="19" t="str">
-        <x:v>L:ANDPOLICESECURING</x:v>
+        <x:v>L:PAX3AND34</x:v>
       </x:c>
       <x:c r="B243" s="20" t="str">
         <x:v>AND.ground.police.securing.scene.wav</x:v>
@@ -4870,14 +4892,12 @@
         <x:v>Police are securing the scene. Stay clear until the area is released.</x:v>
       </x:c>
       <x:c r="D243" s="20" t="str">
-        <x:v>Ground support</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E243" s="20" t="str">
         <x:v>Police arrival and the scene-security/privacy-screen path begin.</x:v>
       </x:c>
-      <x:c r="F243" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F243" s="25" t="str"/>
       <x:c r="G243" s="25" t="str">
         <x:v>1) Be advised: police are securing the scene. Stay clear until the area is released.
 2) Attention: police are securing the scene. Stay clear until the area is released.
@@ -4886,7 +4906,7 @@
     </x:row>
     <x:row r="244" ht="120" customHeight="1">
       <x:c r="A244" s="19" t="str">
-        <x:v>L:ANDFIREHAZARD</x:v>
+        <x:v>L:PAX3AND35</x:v>
       </x:c>
       <x:c r="B244" s="20" t="str">
         <x:v>AND.ground.fire.service.hazard.wav</x:v>
@@ -4895,14 +4915,12 @@
         <x:v>Fire service is controlling a hazard. Do not land until cleared.</x:v>
       </x:c>
       <x:c r="D244" s="20" t="str">
-        <x:v>Ground support</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E244" s="20" t="str">
         <x:v>Fire-engine or fire-hazard branch is active.</x:v>
       </x:c>
-      <x:c r="F244" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F244" s="25" t="str"/>
       <x:c r="G244" s="25" t="str">
         <x:v>1) Be advised: fire service is controlling a hazard. Do not land until cleared.
 2) Attention: fire service is controlling a hazard. Do not land until cleared.
@@ -4911,7 +4929,7 @@
     </x:row>
     <x:row r="245" ht="120" customHeight="1">
       <x:c r="A245" s="19" t="str">
-        <x:v>L:ANDOPSGROUNDDELAY</x:v>
+        <x:v>L:PAX3AND36</x:v>
       </x:c>
       <x:c r="B245" s="20" t="str">
         <x:v>AND.ops.ground.operations.delayed.wav</x:v>
@@ -4920,14 +4938,12 @@
         <x:v>Ground operations are delayed. Check the Dispatch page for the current status.</x:v>
       </x:c>
       <x:c r="D245" s="20" t="str">
-        <x:v>Flight or ground crew</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E245" s="20" t="str">
         <x:v>ops_progress_warning becomes 1 after 120 seconds without progress; tablet shows the orange Dispatch warning.</x:v>
       </x:c>
-      <x:c r="F245" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F245" s="25" t="str"/>
       <x:c r="G245" s="25" t="str">
         <x:v>1) Be advised: ground operations are delayed. Check the Dispatch page for the current status.
 2) Attention: ground operations are delayed. Check the Dispatch page for the current status.
@@ -4936,7 +4952,7 @@
     </x:row>
     <x:row r="246" ht="120" customHeight="1">
       <x:c r="A246" s="19" t="str">
-        <x:v>L:ANDHOISTPAUSE</x:v>
+        <x:v>L:PAX2AND5</x:v>
       </x:c>
       <x:c r="B246" s="20" t="str">
         <x:v>AND.hoist.operation.paused.wav</x:v>
@@ -4945,14 +4961,12 @@
         <x:v>Hold position. Hoist operation is paused until the aircraft is stable.</x:v>
       </x:c>
       <x:c r="D246" s="20" t="str">
-        <x:v>Hoist operator</x:v>
+        <x:v>Hoist operator / PAX2</x:v>
       </x:c>
       <x:c r="E246" s="20" t="str">
         <x:v>A speed, acceleration, or bank-angle limit requires a temporary hoist pause.</x:v>
       </x:c>
-      <x:c r="F246" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F246" s="25" t="str"/>
       <x:c r="G246" s="25" t="str">
         <x:v>1) Maintain position. Hoist operation is paused until the aircraft is stable.
 2) Maintain your position. Hoist operation is paused until the aircraft is stable.
@@ -4961,7 +4975,7 @@
     </x:row>
     <x:row r="247" ht="120" customHeight="1">
       <x:c r="A247" s="19" t="str">
-        <x:v>L:ANDHOISTABORT</x:v>
+        <x:v>L:PAX2AND6</x:v>
       </x:c>
       <x:c r="B247" s="20" t="str">
         <x:v>AND.hoist.operation.abort.wav</x:v>
@@ -4970,14 +4984,12 @@
         <x:v>Abort the hoist operation. Recover the crew only when conditions are safe.</x:v>
       </x:c>
       <x:c r="D247" s="20" t="str">
-        <x:v>Hoist operator</x:v>
+        <x:v>Hoist operator / PAX2</x:v>
       </x:c>
       <x:c r="E247" s="20" t="str">
         <x:v>An unsafe hoist state requires abort and recovery rather than continuation.</x:v>
       </x:c>
-      <x:c r="F247" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F247" s="25" t="str"/>
       <x:c r="G247" s="25" t="str">
         <x:v>1) Be advised: abort the hoist operation. Recover the crew only when conditions are safe.
 2) Attention: abort the hoist operation. Recover the crew only when conditions are safe.
@@ -4986,7 +4998,7 @@
     </x:row>
     <x:row r="248" ht="120" customHeight="1">
       <x:c r="A248" s="19" t="str">
-        <x:v>L:ANDROUTEUNAVAILABLE</x:v>
+        <x:v>L:CPLAND62</x:v>
       </x:c>
       <x:c r="B248" s="20" t="str">
         <x:v>AND.route.unavailable.check.tablet.wav</x:v>
@@ -4995,14 +5007,12 @@
         <x:v>Route is unavailable. Select or confirm the destination on the tablet.</x:v>
       </x:c>
       <x:c r="D248" s="20" t="str">
-        <x:v>Pilot or copilot</x:v>
+        <x:v>Copilot / CPL</x:v>
       </x:c>
       <x:c r="E248" s="20" t="str">
         <x:v>routeupdate records a missing or failed destination after its retry.</x:v>
       </x:c>
-      <x:c r="F248" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F248" s="25" t="str"/>
       <x:c r="G248" s="25" t="str">
         <x:v>1) Be advised: route is unavailable. Select or confirm the destination on the tablet.
 2) Attention: route is unavailable. Select or confirm the destination on the tablet.
@@ -5011,7 +5021,7 @@
     </x:row>
     <x:row r="249" ht="120" customHeight="1">
       <x:c r="A249" s="19" t="str">
-        <x:v>L:ANDROUTECHANGED</x:v>
+        <x:v>L:CPLAND63</x:v>
       </x:c>
       <x:c r="B249" s="20" t="str">
         <x:v>AND.route.changed.check.tablet.wav</x:v>
@@ -5020,14 +5030,12 @@
         <x:v>Destination changed. Check the revised route on the tablet.</x:v>
       </x:c>
       <x:c r="D249" s="20" t="str">
-        <x:v>Pilot or copilot</x:v>
+        <x:v>Copilot / CPL</x:v>
       </x:c>
       <x:c r="E249" s="20" t="str">
         <x:v>Hospital, pickup, or custom target changes and the route is recalculated.</x:v>
       </x:c>
-      <x:c r="F249" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F249" s="25" t="str"/>
       <x:c r="G249" s="25" t="str">
         <x:v>1) Be advised: destination changed. Check the revised route on the tablet.
 2) Attention: destination changed. Check the revised route on the tablet.
@@ -5036,7 +5044,7 @@
     </x:row>
     <x:row r="250" ht="120" customHeight="1">
       <x:c r="A250" s="19" t="str">
-        <x:v>L:ANDDISPATCHCANCELLED</x:v>
+        <x:v>L:PLTAND46</x:v>
       </x:c>
       <x:c r="B250" s="20" t="str">
         <x:v>AND.dispatch.cancelled.await.tasking.wav</x:v>
@@ -5045,14 +5053,12 @@
         <x:v>Dispatch cancelled. Follow the instructions on the tablet and await reassignment.</x:v>
       </x:c>
       <x:c r="D250" s="20" t="str">
-        <x:v>Dispatch</x:v>
+        <x:v>Pilot / PLT</x:v>
       </x:c>
       <x:c r="E250" s="20" t="str">
         <x:v>Cancellation criteria end the current dispatch; HEMS must not continue intervention.</x:v>
       </x:c>
-      <x:c r="F250" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F250" s="25" t="str"/>
       <x:c r="G250" s="25" t="str">
         <x:v>1) Be advised: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
 2) Attention: dispatch cancelled. Follow the instructions on the tablet and await reassignment.
@@ -5061,7 +5067,7 @@
     </x:row>
     <x:row r="251" ht="120" customHeight="1">
       <x:c r="A251" s="19" t="str">
-        <x:v>L:ANDSTARTUPBLOCKED</x:v>
+        <x:v>L:CPLAND64</x:v>
       </x:c>
       <x:c r="B251" s="20" t="str">
         <x:v>AND.cockpit.engine.start.hold.wav</x:v>
@@ -5070,14 +5076,12 @@
         <x:v>Hold engine start. Ground operations are still in progress.</x:v>
       </x:c>
       <x:c r="D251" s="20" t="str">
-        <x:v>Pilot or copilot</x:v>
+        <x:v>Copilot / CPL</x:v>
       </x:c>
       <x:c r="E251" s="20" t="str">
         <x:v>marshall_ground_ops_active or pisteur3_guidance_active blocks a first-pump start request.</x:v>
       </x:c>
-      <x:c r="F251" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F251" s="25" t="str"/>
       <x:c r="G251" s="25" t="str">
         <x:v>1) Be advised: hold engine start. Ground operations are still in progress.
 2) Attention: hold engine start. Ground operations are still in progress.
@@ -5086,7 +5090,7 @@
     </x:row>
     <x:row r="252" ht="120" customHeight="1">
       <x:c r="A252" s="19" t="str">
-        <x:v>L:ANDMAINTENANCEHOLD</x:v>
+        <x:v>L:FRAAND9</x:v>
       </x:c>
       <x:c r="B252" s="20" t="str">
         <x:v>AND.technical.inspection.required.wav</x:v>
@@ -5095,14 +5099,12 @@
         <x:v>Aircraft requires inspection. Do not depart until maintenance releases it.</x:v>
       </x:c>
       <x:c r="D252" s="20" t="str">
-        <x:v>Technician</x:v>
+        <x:v>Technician / FRA</x:v>
       </x:c>
       <x:c r="E252" s="20" t="str">
         <x:v>A failure or hard landing requires inspection before the next release.</x:v>
       </x:c>
-      <x:c r="F252" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F252" s="25" t="str"/>
       <x:c r="G252" s="25" t="str">
         <x:v>1) Be advised: aircraft requires inspection. Do not depart until maintenance releases it.
 2) Attention: aircraft requires inspection. Do not depart until maintenance releases it.
@@ -5111,7 +5113,7 @@
     </x:row>
     <x:row r="253" ht="120" customHeight="1">
       <x:c r="A253" s="19" t="str">
-        <x:v>L:ANDMULTIPLEPATIENTS</x:v>
+        <x:v>L:PAX3AND37</x:v>
       </x:c>
       <x:c r="B253" s="20" t="str">
         <x:v>AND.medical.additional.patients.on.scene.wav</x:v>
@@ -5120,14 +5122,12 @@
         <x:v>Additional patients remain on scene. Await tasking before departure.</x:v>
       </x:c>
       <x:c r="D253" s="20" t="str">
-        <x:v>Crew chief</x:v>
+        <x:v>Medical crew / PAX3</x:v>
       </x:c>
       <x:c r="E253" s="20" t="str">
         <x:v>Patient 2 or 3 remains active, or secondary rescue begins.</x:v>
       </x:c>
-      <x:c r="F253" s="25" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F253" s="25" t="str"/>
       <x:c r="G253" s="25" t="str">
         <x:v>1) Be advised: additional patients remain on scene. Await tasking before departure.
 2) Attention: additional patients remain on scene. Await tasking before departure.
@@ -5136,7 +5136,7 @@
     </x:row>
     <x:row r="254" ht="120" customHeight="1">
       <x:c r="A254" s="22" t="str">
-        <x:v>L:ANDCREWRETURNING</x:v>
+        <x:v>L:AND82</x:v>
       </x:c>
       <x:c r="B254" s="23" t="str">
         <x:v>AND.crew.returning.to.aircraft.wav</x:v>
@@ -5145,14 +5145,12 @@
         <x:v>Ground crew is returning to the aircraft. Keep the landing area clear.</x:v>
       </x:c>
       <x:c r="D254" s="23" t="str">
-        <x:v>Crew chief</x:v>
+        <x:v>Crew chief / PAX1 (no prefix)</x:v>
       </x:c>
       <x:c r="E254" s="23" t="str">
         <x:v>Post-visit, post-load, or post-hoist crew-return flow begins.</x:v>
       </x:c>
-      <x:c r="F254" s="26" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="F254" s="26" t="str"/>
       <x:c r="G254" s="26" t="str">
         <x:v>1) Be advised: ground crew is returning to the aircraft. Keep the landing area clear.
 2) Attention: ground crew is returning to the aircraft. Keep the landing area clear.
@@ -5162,7 +5160,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9adf0640d8884837"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>